<commit_message>
Agregar verdulería 17/09/2026 $34.000 en Almacén CIUDAD
Carga COMIDA · VERDULERÍA en Almacen Detalle (Importe Sol) y regenera el maestro SOL.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -61383,15 +61383,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B356" s="17" t="n"/>
-      <c r="C356" s="14" t="n"/>
-      <c r="D356" s="27" t="n"/>
+      <c r="B356" s="17" t="n">
+        <v>46282</v>
+      </c>
+      <c r="C356" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · VERDULERÍA</t>
+        </is>
+      </c>
+      <c r="D356" s="27" t="n">
+        <v>34000</v>
+      </c>
       <c r="E356" s="28" t="n"/>
       <c r="F356" s="15">
-        <f>IF(OR(D340&lt;&gt;"",E340&lt;&gt;""),IF(D340="",0,D340)+IF(E340="",0,E340),"")</f>
-        <v/>
-      </c>
-      <c r="G356" s="14" t="n"/>
+        <f>IF(OR(D356&lt;&gt;"",E356&lt;&gt;""),IF(D356="",0,D356)+IF(E356="",0,E356),"")</f>
+        <v/>
+      </c>
+      <c r="G356" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · VERDULERÍA</t>
+        </is>
+      </c>
     </row>
     <row r="357">
       <c r="A357" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Cargar movimientos MP dinero en cuenta septiembre 2026
Transcribe 107 movimientos de capturas MP, categoriza Almacén/GPS/
Limpieza/ABL/OHIGGINS, excluye cuotas y transferencias propias, y
regenera el maestro SOL.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -1037,7 +1037,9 @@
         <v>26175</v>
       </c>
       <c r="K9" s="5" t="n"/>
-      <c r="L9" s="5" t="n"/>
+      <c r="L9" s="5" t="n">
+        <v>27635</v>
+      </c>
       <c r="M9" s="5" t="n"/>
       <c r="N9" s="5" t="n"/>
       <c r="O9" s="5" t="n"/>
@@ -1084,7 +1086,9 @@
         <v>400640</v>
       </c>
       <c r="K10" s="9" t="n"/>
-      <c r="L10" s="9" t="n"/>
+      <c r="L10" s="9" t="n">
+        <v>835200</v>
+      </c>
       <c r="M10" s="9" t="n"/>
       <c r="N10" s="9" t="n"/>
       <c r="O10" s="9" t="n"/>
@@ -1567,7 +1571,6 @@
         <v/>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
@@ -3726,7 +3729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F833"/>
+  <dimension ref="A1:F898"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25971,6 +25974,1826 @@
       <c r="F833" t="inlineStr">
         <is>
           <t>COMIDA · Oficina · Copetin Catering · Gmail Pago aprobado · REVISAR vs settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" s="52" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>TRANSFERENCIAS</t>
+        </is>
+      </c>
+      <c r="D834" t="n">
+        <v>45000</v>
+      </c>
+      <c r="E834" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F834" t="inlineStr">
+        <is>
+          <t>Facundo Lisandro Marin · Transferencia enviada · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" s="52" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B835" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>SUSCRIPCIONES · Apple</t>
+        </is>
+      </c>
+      <c r="D835" t="n">
+        <v>81961</v>
+      </c>
+      <c r="E835" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F835" t="inlineStr">
+        <is>
+          <t>SUSCRIPCIONES · Apple · Mercado Pago · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" s="52" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber</t>
+        </is>
+      </c>
+      <c r="D836" t="n">
+        <v>6094</v>
+      </c>
+      <c r="E836" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F836" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber · Ebanx (=Uber) · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" s="52" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Didi</t>
+        </is>
+      </c>
+      <c r="D837" t="n">
+        <v>7600</v>
+      </c>
+      <c r="E837" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F837" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Didi · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" s="52" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B838" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C838" t="inlineStr">
+        <is>
+          <t>TRANSFERENCIAS</t>
+        </is>
+      </c>
+      <c r="D838" t="n">
+        <v>863600</v>
+      </c>
+      <c r="E838" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F838" t="inlineStr">
+        <is>
+          <t>Neira Martina · Transferencia enviada · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" s="52" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B839" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C839" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber</t>
+        </is>
+      </c>
+      <c r="D839" t="n">
+        <v>6607</v>
+      </c>
+      <c r="E839" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F839" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber · Ebanx (=Uber) · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" s="52" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B840" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C840" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber</t>
+        </is>
+      </c>
+      <c r="D840" t="n">
+        <v>6607</v>
+      </c>
+      <c r="E840" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F840" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber · Ebanx (=Uber) · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" s="52" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B841" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C841" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D841" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E841" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F841" t="inlineStr">
+        <is>
+          <t>COMPRAS · Kiosk Store · gasto personal Sol · REVISAR ítem · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" s="52" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B842" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C842" t="inlineStr">
+        <is>
+          <t>ENVÍOS</t>
+        </is>
+      </c>
+      <c r="D842" t="n">
+        <v>24000</v>
+      </c>
+      <c r="E842" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F842" t="inlineStr">
+        <is>
+          <t>ENVÍOS · Correo Oficial · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" s="52" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C843" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber</t>
+        </is>
+      </c>
+      <c r="D843" t="n">
+        <v>7520</v>
+      </c>
+      <c r="E843" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F843" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber · Ebanx (=Uber) · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" s="52" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C844" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Didi</t>
+        </is>
+      </c>
+      <c r="D844" t="n">
+        <v>4900</v>
+      </c>
+      <c r="E844" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F844" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Didi · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" s="52" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C845" t="inlineStr">
+        <is>
+          <t>TRANSFERENCIAS</t>
+        </is>
+      </c>
+      <c r="D845" t="n">
+        <v>10800</v>
+      </c>
+      <c r="E845" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F845" t="inlineStr">
+        <is>
+          <t>Digno Lopez · Transferencia enviada · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" s="52" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C846" t="inlineStr">
+        <is>
+          <t>IMPUESTOS · ARCA</t>
+        </is>
+      </c>
+      <c r="D846" t="n">
+        <v>10000</v>
+      </c>
+      <c r="E846" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F846" t="inlineStr">
+        <is>
+          <t>IMPUESTOS · ARCA / AFIP · MP 2026-09-05 · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" s="52" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr">
+        <is>
+          <t>IMPUESTOS · ARCA</t>
+        </is>
+      </c>
+      <c r="D847" t="n">
+        <v>10000</v>
+      </c>
+      <c r="E847" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F847" t="inlineStr">
+        <is>
+          <t>IMPUESTOS · ARCA / AFIP · MP 2026-09-05 · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" s="52" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr">
+        <is>
+          <t>Servicio - Telefonía</t>
+        </is>
+      </c>
+      <c r="D848" t="n">
+        <v>18300</v>
+      </c>
+      <c r="E848" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F848" t="inlineStr">
+        <is>
+          <t>Servicio - Telefonía · Tuenti · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" s="52" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · SUBE</t>
+        </is>
+      </c>
+      <c r="D849" t="n">
+        <v>987</v>
+      </c>
+      <c r="E849" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F849" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · SUBE · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" s="52" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber</t>
+        </is>
+      </c>
+      <c r="D850" t="n">
+        <v>6948</v>
+      </c>
+      <c r="E850" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F850" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber · Ebanx (=Uber) · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" s="52" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C851" t="inlineStr">
+        <is>
+          <t>COMIDA · Oficina</t>
+        </is>
+      </c>
+      <c r="D851" t="n">
+        <v>1350</v>
+      </c>
+      <c r="E851" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F851" t="inlineStr">
+        <is>
+          <t>COMIDA · Oficina · Feed · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" s="52" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C852" t="inlineStr">
+        <is>
+          <t>IMPUESTOS · ARCA</t>
+        </is>
+      </c>
+      <c r="D852" t="n">
+        <v>58118</v>
+      </c>
+      <c r="E852" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F852" t="inlineStr">
+        <is>
+          <t>IMPUESTOS · ARCA / AFIP · MP 2026-09-07 · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" s="52" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C853" t="inlineStr">
+        <is>
+          <t>IMPUESTOS · ARCA</t>
+        </is>
+      </c>
+      <c r="D853" t="n">
+        <v>43038</v>
+      </c>
+      <c r="E853" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F853" t="inlineStr">
+        <is>
+          <t>IMPUESTOS · ARCA / AFIP · MP 2026-09-07 · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" s="52" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C854" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Didi</t>
+        </is>
+      </c>
+      <c r="D854" t="n">
+        <v>6700</v>
+      </c>
+      <c r="E854" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F854" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Didi · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" s="52" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C855" t="inlineStr">
+        <is>
+          <t>IMPUESTOS · ARCA</t>
+        </is>
+      </c>
+      <c r="D855" t="n">
+        <v>4866</v>
+      </c>
+      <c r="E855" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F855" t="inlineStr">
+        <is>
+          <t>IMPUESTOS · ARCA / AFIP · MP 2026-09-08 · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" s="52" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C856" t="inlineStr">
+        <is>
+          <t>VESTIMENTA</t>
+        </is>
+      </c>
+      <c r="D856" t="n">
+        <v>28199</v>
+      </c>
+      <c r="E856" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F856" t="inlineStr">
+        <is>
+          <t>VESTIMENTA · OZZ · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" s="52" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C857" t="inlineStr">
+        <is>
+          <t>IMPUESTOS · ARCA</t>
+        </is>
+      </c>
+      <c r="D857" t="n">
+        <v>43083</v>
+      </c>
+      <c r="E857" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F857" t="inlineStr">
+        <is>
+          <t>IMPUESTOS · ARCA / AFIP · MP 2026-09-10 · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" s="52" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C858" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber</t>
+        </is>
+      </c>
+      <c r="D858" t="n">
+        <v>5612</v>
+      </c>
+      <c r="E858" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F858" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber · Ebanx (=Uber) · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" s="52" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B859" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C859" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber</t>
+        </is>
+      </c>
+      <c r="D859" t="n">
+        <v>7155</v>
+      </c>
+      <c r="E859" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F859" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber · Ebanx (=Uber) · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" s="52" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C860" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber</t>
+        </is>
+      </c>
+      <c r="D860" t="n">
+        <v>81</v>
+      </c>
+      <c r="E860" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F860" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber · Ebanx (=Uber) · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" s="52" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C861" t="inlineStr">
+        <is>
+          <t>TRANSFERENCIAS</t>
+        </is>
+      </c>
+      <c r="D861" t="n">
+        <v>131000</v>
+      </c>
+      <c r="E861" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F861" t="inlineStr">
+        <is>
+          <t>Cova Abreu Gibiana Del Valle · Transferencia enviada · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" s="52" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C862" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D862" t="n">
+        <v>163350</v>
+      </c>
+      <c r="E862" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F862" t="inlineStr">
+        <is>
+          <t>COMPRAS · ZILVER SA · gasto personal Sol · REVISAR ítem · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" s="52" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C863" t="inlineStr">
+        <is>
+          <t>SUSCRIPCIONES · Apple</t>
+        </is>
+      </c>
+      <c r="D863" t="n">
+        <v>29331</v>
+      </c>
+      <c r="E863" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F863" t="inlineStr">
+        <is>
+          <t>SUSCRIPCIONES · Apple · Mercado Pago · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" s="52" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C864" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Didi</t>
+        </is>
+      </c>
+      <c r="D864" t="n">
+        <v>5800</v>
+      </c>
+      <c r="E864" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F864" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Didi · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" s="52" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C865" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Didi</t>
+        </is>
+      </c>
+      <c r="D865" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E865" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F865" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Didi · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" s="52" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C866" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber</t>
+        </is>
+      </c>
+      <c r="D866" t="n">
+        <v>7758</v>
+      </c>
+      <c r="E866" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F866" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber · Ebanx (=Uber) · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" s="52" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C867" t="inlineStr">
+        <is>
+          <t>TRANSFERENCIAS</t>
+        </is>
+      </c>
+      <c r="D867" t="n">
+        <v>185288</v>
+      </c>
+      <c r="E867" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F867" t="inlineStr">
+        <is>
+          <t>Sanbras oficial · Transferencia enviada · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" s="52" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B868" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C868" t="inlineStr">
+        <is>
+          <t>TRANSFERENCIAS</t>
+        </is>
+      </c>
+      <c r="D868" t="n">
+        <v>135000</v>
+      </c>
+      <c r="E868" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F868" t="inlineStr">
+        <is>
+          <t>Paula Carolina Fasanella · Transferencia enviada · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" s="52" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B869" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C869" t="inlineStr">
+        <is>
+          <t>SUSCRIPCIONES · Apple</t>
+        </is>
+      </c>
+      <c r="D869" t="n">
+        <v>19749</v>
+      </c>
+      <c r="E869" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F869" t="inlineStr">
+        <is>
+          <t>SUSCRIPCIONES · Apple · Mercado Pago · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" s="52" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B870" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C870" t="inlineStr">
+        <is>
+          <t>TRANSFERENCIAS</t>
+        </is>
+      </c>
+      <c r="D870" t="n">
+        <v>140000</v>
+      </c>
+      <c r="E870" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F870" t="inlineStr">
+        <is>
+          <t>Eva Graciela Zarate Valdovino · Transferencia enviada · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" s="52" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B871" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C871" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D871" t="n">
+        <v>176509</v>
+      </c>
+      <c r="E871" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F871" t="inlineStr">
+        <is>
+          <t>COMPRAS · El Bazar Digital · gasto personal Sol · REVISAR ítem · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" s="52" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B872" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C872" t="inlineStr">
+        <is>
+          <t>PELUQUERÍA</t>
+        </is>
+      </c>
+      <c r="D872" t="n">
+        <v>12720</v>
+      </c>
+      <c r="E872" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F872" t="inlineStr">
+        <is>
+          <t>PELUQUERÍA · Megapeluquerías CABA · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" s="52" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B873" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C873" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D873" t="n">
+        <v>71250</v>
+      </c>
+      <c r="E873" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F873" t="inlineStr">
+        <is>
+          <t>Pago · Pago · gasto personal Sol · REVISAR ítem · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" s="52" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B874" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C874" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D874" t="n">
+        <v>76742</v>
+      </c>
+      <c r="E874" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F874" t="inlineStr">
+        <is>
+          <t>Pago · Pago · gasto personal Sol · REVISAR ítem · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" s="52" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B875" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C875" t="inlineStr">
+        <is>
+          <t>TRANSFERENCIAS</t>
+        </is>
+      </c>
+      <c r="D875" t="n">
+        <v>85000</v>
+      </c>
+      <c r="E875" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F875" t="inlineStr">
+        <is>
+          <t>Maria Celeste Gonzalez · Transferencia enviada · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" s="52" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B876" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C876" t="inlineStr">
+        <is>
+          <t>TRANSFERENCIAS</t>
+        </is>
+      </c>
+      <c r="D876" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E876" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F876" t="inlineStr">
+        <is>
+          <t>Mariano Morales · Transferencia enviada · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" s="52" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B877" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C877" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber</t>
+        </is>
+      </c>
+      <c r="D877" t="n">
+        <v>4980</v>
+      </c>
+      <c r="E877" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F877" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber · Ebanx (=Uber) · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" s="52" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B878" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C878" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D878" t="n">
+        <v>40900</v>
+      </c>
+      <c r="E878" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F878" t="inlineStr">
+        <is>
+          <t>COMPRAS · Happy buy · gasto personal Sol · REVISAR ítem · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" s="52" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B879" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C879" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Didi</t>
+        </is>
+      </c>
+      <c r="D879" t="n">
+        <v>5500</v>
+      </c>
+      <c r="E879" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F879" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Didi · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" s="52" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B880" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C880" t="inlineStr">
+        <is>
+          <t>IMPUESTOS · Epagos</t>
+        </is>
+      </c>
+      <c r="D880" t="n">
+        <v>10150</v>
+      </c>
+      <c r="E880" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F880" t="inlineStr">
+        <is>
+          <t>IMPUESTOS · Epagos · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" s="52" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B881" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C881" t="inlineStr">
+        <is>
+          <t>TRANSFERENCIAS</t>
+        </is>
+      </c>
+      <c r="D881" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E881" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F881" t="inlineStr">
+        <is>
+          <t>Gaston Osvaldo Roca · Transferencia enviada · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" s="52" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B882" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C882" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber</t>
+        </is>
+      </c>
+      <c r="D882" t="n">
+        <v>7257</v>
+      </c>
+      <c r="E882" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F882" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber · Ebanx (=Uber) · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" s="52" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B883" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C883" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Didi</t>
+        </is>
+      </c>
+      <c r="D883" t="n">
+        <v>6200</v>
+      </c>
+      <c r="E883" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F883" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Didi · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" s="52" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B884" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C884" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber</t>
+        </is>
+      </c>
+      <c r="D884" t="n">
+        <v>6053</v>
+      </c>
+      <c r="E884" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F884" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber · Ebanx (=Uber) · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" s="52" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B885" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C885" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Didi</t>
+        </is>
+      </c>
+      <c r="D885" t="n">
+        <v>4900</v>
+      </c>
+      <c r="E885" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F885" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Didi · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" s="52" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B886" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C886" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber</t>
+        </is>
+      </c>
+      <c r="D886" t="n">
+        <v>6478</v>
+      </c>
+      <c r="E886" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F886" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber · Ebanx (=Uber) · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" s="52" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B887" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C887" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · SUBE</t>
+        </is>
+      </c>
+      <c r="D887" t="n">
+        <v>862</v>
+      </c>
+      <c r="E887" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F887" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · SUBE · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" s="52" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B888" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C888" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber</t>
+        </is>
+      </c>
+      <c r="D888" t="n">
+        <v>5393</v>
+      </c>
+      <c r="E888" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F888" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber · Ebanx (=Uber) · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" s="52" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B889" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C889" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Didi</t>
+        </is>
+      </c>
+      <c r="D889" t="n">
+        <v>3300</v>
+      </c>
+      <c r="E889" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F889" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Didi · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" s="52" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B890" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C890" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D890" t="n">
+        <v>63514</v>
+      </c>
+      <c r="E890" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F890" t="inlineStr">
+        <is>
+          <t>Randy Kopeles · Pago · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" s="52" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B891" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C891" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber</t>
+        </is>
+      </c>
+      <c r="D891" t="n">
+        <v>7016</v>
+      </c>
+      <c r="E891" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F891" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber · Ebanx (=Uber) · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" s="52" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B892" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C892" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber</t>
+        </is>
+      </c>
+      <c r="D892" t="n">
+        <v>153</v>
+      </c>
+      <c r="E892" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F892" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber · Ebanx (=Uber) · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" s="52" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B893" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C893" t="inlineStr">
+        <is>
+          <t>SALUD</t>
+        </is>
+      </c>
+      <c r="D893" t="n">
+        <v>50000</v>
+      </c>
+      <c r="E893" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F893" t="inlineStr">
+        <is>
+          <t>SALUD · Clinicas Altamirao · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" s="52" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B894" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C894" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Didi</t>
+        </is>
+      </c>
+      <c r="D894" t="n">
+        <v>3200</v>
+      </c>
+      <c r="E894" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F894" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Didi · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" s="52" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B895" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C895" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D895" t="n">
+        <v>72999</v>
+      </c>
+      <c r="E895" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F895" t="inlineStr">
+        <is>
+          <t>Tatiana Aylén Gonzalez · Pago · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" s="52" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B896" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C896" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Didi</t>
+        </is>
+      </c>
+      <c r="D896" t="n">
+        <v>4800</v>
+      </c>
+      <c r="E896" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F896" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Didi · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" s="52" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B897" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C897" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Didi</t>
+        </is>
+      </c>
+      <c r="D897" t="n">
+        <v>6800</v>
+      </c>
+      <c r="E897" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F897" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Didi · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" s="52" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B898" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C898" t="inlineStr">
+        <is>
+          <t>ENVÍOS</t>
+        </is>
+      </c>
+      <c r="D898" t="n">
+        <v>13288</v>
+      </c>
+      <c r="E898" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F898" t="inlineStr">
+        <is>
+          <t>ENVÍOS · DHL Express · gasto personal Sol · dinero en cuenta MP screenshot</t>
         </is>
       </c>
     </row>
@@ -57849,6 +59672,7 @@
       </c>
       <c r="G176" s="22" t="n"/>
     </row>
+    <row r="177"/>
     <row r="178">
       <c r="A178" s="14" t="inlineStr">
         <is>
@@ -59131,6 +60955,7 @@
       </c>
       <c r="G228" s="22" t="n"/>
     </row>
+    <row r="229"/>
     <row r="230">
       <c r="A230" s="14" t="inlineStr">
         <is>
@@ -60169,6 +61994,7 @@
       </c>
       <c r="G273" s="22" t="n"/>
     </row>
+    <row r="274"/>
     <row r="275">
       <c r="A275" s="14" t="inlineStr">
         <is>
@@ -60936,6 +62762,7 @@
       </c>
       <c r="G312" s="22" t="n"/>
     </row>
+    <row r="313"/>
     <row r="314">
       <c r="A314" s="14" t="inlineStr">
         <is>
@@ -61602,6 +63429,7 @@
       </c>
       <c r="G354" s="22" t="n"/>
     </row>
+    <row r="355"/>
     <row r="356">
       <c r="A356" s="14" t="inlineStr">
         <is>
@@ -61692,15 +63520,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B359" s="17" t="n"/>
-      <c r="C359" s="14" t="n"/>
-      <c r="D359" s="27" t="n"/>
+      <c r="B359" s="17" t="n">
+        <v>46268</v>
+      </c>
+      <c r="C359" s="14" t="inlineStr">
+        <is>
+          <t>PEDIDOS YA · COMIDA</t>
+        </is>
+      </c>
+      <c r="D359" s="27" t="n">
+        <v>16149</v>
+      </c>
       <c r="E359" s="28" t="n"/>
       <c r="F359" s="15">
-        <f>IF(OR(D343&lt;&gt;"",E343&lt;&gt;""),IF(D343="",0,D343)+IF(E343="",0,E343),"")</f>
-        <v/>
-      </c>
-      <c r="G359" s="14" t="n"/>
+        <f>IF(OR(D359&lt;&gt;"",E359&lt;&gt;""),IF(D359="",0,D359)+IF(E359="",0,E359),"")</f>
+        <v/>
+      </c>
+      <c r="G359" s="14" t="inlineStr">
+        <is>
+          <t>PEDIDOS YA · COMIDA · screenshot · REVISAR si Market · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
     </row>
     <row r="360">
       <c r="A360" s="14" t="inlineStr">
@@ -61708,15 +63548,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B360" s="17" t="n"/>
-      <c r="C360" s="14" t="n"/>
-      <c r="D360" s="27" t="n"/>
+      <c r="B360" s="17" t="n">
+        <v>46268</v>
+      </c>
+      <c r="C360" s="14" t="inlineStr">
+        <is>
+          <t>PEDIDOS YA · COMIDA · propina</t>
+        </is>
+      </c>
+      <c r="D360" s="27" t="n">
+        <v>800</v>
+      </c>
       <c r="E360" s="28" t="n"/>
       <c r="F360" s="15">
-        <f>IF(OR(D344&lt;&gt;"",E344&lt;&gt;""),IF(D344="",0,D344)+IF(E344="",0,E344),"")</f>
-        <v/>
-      </c>
-      <c r="G360" s="14" t="n"/>
+        <f>IF(OR(D360&lt;&gt;"",E360&lt;&gt;""),IF(D360="",0,D360)+IF(E360="",0,E360),"")</f>
+        <v/>
+      </c>
+      <c r="G360" s="14" t="inlineStr">
+        <is>
+          <t>PEDIDOS YA · COMIDA · propina · screenshot · REVISAR si Market · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
     </row>
     <row r="361">
       <c r="A361" s="14" t="inlineStr">
@@ -61724,15 +63576,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B361" s="17" t="n"/>
-      <c r="C361" s="14" t="n"/>
-      <c r="D361" s="27" t="n"/>
+      <c r="B361" s="17" t="n">
+        <v>46271</v>
+      </c>
+      <c r="C361" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · AL PASO</t>
+        </is>
+      </c>
+      <c r="D361" s="27" t="n">
+        <v>8700</v>
+      </c>
       <c r="E361" s="28" t="n"/>
       <c r="F361" s="15">
-        <f>IF(OR(D345&lt;&gt;"",E345&lt;&gt;""),IF(D345="",0,D345)+IF(E345="",0,E345),"")</f>
-        <v/>
-      </c>
-      <c r="G361" s="14" t="n"/>
+        <f>IF(OR(D361&lt;&gt;"",E361&lt;&gt;""),IF(D361="",0,D361)+IF(E361="",0,E361),"")</f>
+        <v/>
+      </c>
+      <c r="G361" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · AL PASO · Mercado Pago · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
     </row>
     <row r="362">
       <c r="A362" s="14" t="inlineStr">
@@ -61740,15 +63604,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B362" s="17" t="n"/>
-      <c r="C362" s="14" t="n"/>
-      <c r="D362" s="27" t="n"/>
+      <c r="B362" s="17" t="n">
+        <v>46272</v>
+      </c>
+      <c r="C362" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · McDonald's</t>
+        </is>
+      </c>
+      <c r="D362" s="27" t="n">
+        <v>2040</v>
+      </c>
       <c r="E362" s="28" t="n"/>
       <c r="F362" s="15">
-        <f>IF(OR(D346&lt;&gt;"",E346&lt;&gt;""),IF(D346="",0,D346)+IF(E346="",0,E346),"")</f>
-        <v/>
-      </c>
-      <c r="G362" s="14" t="n"/>
+        <f>IF(OR(D362&lt;&gt;"",E362&lt;&gt;""),IF(D362="",0,D362)+IF(E362="",0,E362),"")</f>
+        <v/>
+      </c>
+      <c r="G362" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · McDonald's · Mercado Pago · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
     </row>
     <row r="363">
       <c r="A363" s="14" t="inlineStr">
@@ -61756,15 +63632,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B363" s="17" t="n"/>
-      <c r="C363" s="14" t="n"/>
-      <c r="D363" s="27" t="n"/>
+      <c r="B363" s="17" t="n">
+        <v>46273</v>
+      </c>
+      <c r="C363" s="14" t="inlineStr">
+        <is>
+          <t>ENTRETENIMIENTO · Social</t>
+        </is>
+      </c>
+      <c r="D363" s="27" t="n">
+        <v>8248</v>
+      </c>
       <c r="E363" s="28" t="n"/>
       <c r="F363" s="15">
-        <f>IF(OR(D347&lt;&gt;"",E347&lt;&gt;""),IF(D347="",0,D347)+IF(E347="",0,E347),"")</f>
-        <v/>
-      </c>
-      <c r="G363" s="14" t="n"/>
+        <f>IF(OR(D363&lt;&gt;"",E363&lt;&gt;""),IF(D363="",0,D363)+IF(E363="",0,E363),"")</f>
+        <v/>
+      </c>
+      <c r="G363" s="14" t="inlineStr">
+        <is>
+          <t>ENTRETENIMIENTO · Social · la monumental · Mercado Pago · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
     </row>
     <row r="364">
       <c r="A364" s="14" t="inlineStr">
@@ -61772,15 +63660,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B364" s="17" t="n"/>
-      <c r="C364" s="14" t="n"/>
-      <c r="D364" s="27" t="n"/>
+      <c r="B364" s="17" t="n">
+        <v>46274</v>
+      </c>
+      <c r="C364" s="14" t="inlineStr">
+        <is>
+          <t>PEDIDOS YA · COMIDA</t>
+        </is>
+      </c>
+      <c r="D364" s="27" t="n">
+        <v>39819</v>
+      </c>
       <c r="E364" s="28" t="n"/>
       <c r="F364" s="15">
-        <f>IF(OR(D348&lt;&gt;"",E348&lt;&gt;""),IF(D348="",0,D348)+IF(E348="",0,E348),"")</f>
-        <v/>
-      </c>
-      <c r="G364" s="14" t="n"/>
+        <f>IF(OR(D364&lt;&gt;"",E364&lt;&gt;""),IF(D364="",0,D364)+IF(E364="",0,E364),"")</f>
+        <v/>
+      </c>
+      <c r="G364" s="14" t="inlineStr">
+        <is>
+          <t>PEDIDOS YA · COMIDA · screenshot · REVISAR si Market · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
     </row>
     <row r="365">
       <c r="A365" s="14" t="inlineStr">
@@ -61788,15 +63688,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B365" s="17" t="n"/>
-      <c r="C365" s="14" t="n"/>
-      <c r="D365" s="27" t="n"/>
+      <c r="B365" s="17" t="n">
+        <v>46274</v>
+      </c>
+      <c r="C365" s="14" t="inlineStr">
+        <is>
+          <t>PEDIDOS YA · COMIDA · propina</t>
+        </is>
+      </c>
+      <c r="D365" s="27" t="n">
+        <v>900</v>
+      </c>
       <c r="E365" s="28" t="n"/>
       <c r="F365" s="15">
-        <f>IF(OR(D349&lt;&gt;"",E349&lt;&gt;""),IF(D349="",0,D349)+IF(E349="",0,E349),"")</f>
-        <v/>
-      </c>
-      <c r="G365" s="14" t="n"/>
+        <f>IF(OR(D365&lt;&gt;"",E365&lt;&gt;""),IF(D365="",0,D365)+IF(E365="",0,E365),"")</f>
+        <v/>
+      </c>
+      <c r="G365" s="14" t="inlineStr">
+        <is>
+          <t>PEDIDOS YA · COMIDA · propina · screenshot · REVISAR si Market · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
     </row>
     <row r="366">
       <c r="A366" s="14" t="inlineStr">
@@ -61804,15 +63716,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B366" s="17" t="n"/>
-      <c r="C366" s="14" t="n"/>
-      <c r="D366" s="27" t="n"/>
+      <c r="B366" s="17" t="n">
+        <v>46277</v>
+      </c>
+      <c r="C366" s="14" t="inlineStr">
+        <is>
+          <t>PEDIDOS YA · COMIDA</t>
+        </is>
+      </c>
+      <c r="D366" s="27" t="n">
+        <v>38099</v>
+      </c>
       <c r="E366" s="28" t="n"/>
       <c r="F366" s="15">
-        <f>IF(OR(D350&lt;&gt;"",E350&lt;&gt;""),IF(D350="",0,D350)+IF(E350="",0,E350),"")</f>
-        <v/>
-      </c>
-      <c r="G366" s="14" t="n"/>
+        <f>IF(OR(D366&lt;&gt;"",E366&lt;&gt;""),IF(D366="",0,D366)+IF(E366="",0,E366),"")</f>
+        <v/>
+      </c>
+      <c r="G366" s="14" t="inlineStr">
+        <is>
+          <t>PEDIDOS YA · COMIDA · screenshot · REVISAR si Market · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
     </row>
     <row r="367">
       <c r="A367" s="14" t="inlineStr">
@@ -61820,15 +63744,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B367" s="17" t="n"/>
-      <c r="C367" s="14" t="n"/>
-      <c r="D367" s="27" t="n"/>
+      <c r="B367" s="17" t="n">
+        <v>46277</v>
+      </c>
+      <c r="C367" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · McDonald's</t>
+        </is>
+      </c>
+      <c r="D367" s="27" t="n">
+        <v>8010</v>
+      </c>
       <c r="E367" s="28" t="n"/>
       <c r="F367" s="15">
-        <f>IF(OR(D351&lt;&gt;"",E351&lt;&gt;""),IF(D351="",0,D351)+IF(E351="",0,E351),"")</f>
-        <v/>
-      </c>
-      <c r="G367" s="14" t="n"/>
+        <f>IF(OR(D367&lt;&gt;"",E367&lt;&gt;""),IF(D367="",0,D367)+IF(E367="",0,E367),"")</f>
+        <v/>
+      </c>
+      <c r="G367" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · McDonald's · Mercado Pago · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
     </row>
     <row r="368">
       <c r="A368" s="14" t="inlineStr">
@@ -61836,15 +63772,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B368" s="17" t="n"/>
-      <c r="C368" s="14" t="n"/>
-      <c r="D368" s="27" t="n"/>
+      <c r="B368" s="17" t="n">
+        <v>46278</v>
+      </c>
+      <c r="C368" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · VERDULERÍA</t>
+        </is>
+      </c>
+      <c r="D368" s="27" t="n">
+        <v>5900</v>
+      </c>
       <c r="E368" s="28" t="n"/>
       <c r="F368" s="15">
-        <f>IF(OR(D352&lt;&gt;"",E352&lt;&gt;""),IF(D352="",0,D352)+IF(E352="",0,E352),"")</f>
-        <v/>
-      </c>
-      <c r="G368" s="14" t="n"/>
+        <f>IF(OR(D368&lt;&gt;"",E368&lt;&gt;""),IF(D368="",0,D368)+IF(E368="",0,E368),"")</f>
+        <v/>
+      </c>
+      <c r="G368" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · VERDULERÍA · Noelia Caballero · Mercado Pago · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
     </row>
     <row r="369">
       <c r="A369" s="14" t="inlineStr">
@@ -61852,15 +63800,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B369" s="17" t="n"/>
-      <c r="C369" s="14" t="n"/>
-      <c r="D369" s="27" t="n"/>
+      <c r="B369" s="17" t="n">
+        <v>46280</v>
+      </c>
+      <c r="C369" s="14" t="inlineStr">
+        <is>
+          <t>PEDIDOS YA · COMIDA</t>
+        </is>
+      </c>
+      <c r="D369" s="27" t="n">
+        <v>26019</v>
+      </c>
       <c r="E369" s="28" t="n"/>
       <c r="F369" s="15">
-        <f>IF(OR(D353&lt;&gt;"",E353&lt;&gt;""),IF(D353="",0,D353)+IF(E353="",0,E353),"")</f>
-        <v/>
-      </c>
-      <c r="G369" s="14" t="n"/>
+        <f>IF(OR(D369&lt;&gt;"",E369&lt;&gt;""),IF(D369="",0,D369)+IF(E369="",0,E369),"")</f>
+        <v/>
+      </c>
+      <c r="G369" s="14" t="inlineStr">
+        <is>
+          <t>PEDIDOS YA · COMIDA · screenshot · REVISAR si Market · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
     </row>
     <row r="370">
       <c r="A370" s="14" t="inlineStr">
@@ -61868,15 +63828,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B370" s="17" t="n"/>
-      <c r="C370" s="14" t="n"/>
-      <c r="D370" s="27" t="n"/>
+      <c r="B370" s="17" t="n">
+        <v>46280</v>
+      </c>
+      <c r="C370" s="14" t="inlineStr">
+        <is>
+          <t>PEDIDOS YA · COMIDA · propina</t>
+        </is>
+      </c>
+      <c r="D370" s="27" t="n">
+        <v>1050</v>
+      </c>
       <c r="E370" s="28" t="n"/>
       <c r="F370" s="15">
-        <f>IF(OR(D354&lt;&gt;"",E354&lt;&gt;""),IF(D354="",0,D354)+IF(E354="",0,E354),"")</f>
-        <v/>
-      </c>
-      <c r="G370" s="14" t="n"/>
+        <f>IF(OR(D370&lt;&gt;"",E370&lt;&gt;""),IF(D370="",0,D370)+IF(E370="",0,E370),"")</f>
+        <v/>
+      </c>
+      <c r="G370" s="14" t="inlineStr">
+        <is>
+          <t>PEDIDOS YA · COMIDA · propina · screenshot · REVISAR si Market · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
     </row>
     <row r="371">
       <c r="A371" s="14" t="inlineStr">
@@ -61884,15 +63856,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B371" s="17" t="n"/>
-      <c r="C371" s="14" t="n"/>
-      <c r="D371" s="27" t="n"/>
+      <c r="B371" s="17" t="n">
+        <v>46280</v>
+      </c>
+      <c r="C371" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · CASAARISTOBULO017</t>
+        </is>
+      </c>
+      <c r="D371" s="27" t="n">
+        <v>43667</v>
+      </c>
       <c r="E371" s="28" t="n"/>
       <c r="F371" s="15">
-        <f>IF(OR(D355&lt;&gt;"",E355&lt;&gt;""),IF(D355="",0,D355)+IF(E355="",0,E355),"")</f>
-        <v/>
-      </c>
-      <c r="G371" s="14" t="n"/>
+        <f>IF(OR(D371&lt;&gt;"",E371&lt;&gt;""),IF(D371="",0,D371)+IF(E371="",0,E371),"")</f>
+        <v/>
+      </c>
+      <c r="G371" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · CASAARISTOBULO017 · QR · Mercado Pago · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
     </row>
     <row r="372">
       <c r="A372" s="14" t="inlineStr">
@@ -61900,15 +63884,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B372" s="17" t="n"/>
-      <c r="C372" s="14" t="n"/>
-      <c r="D372" s="27" t="n"/>
+      <c r="B372" s="17" t="n">
+        <v>46282</v>
+      </c>
+      <c r="C372" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · McDonald's</t>
+        </is>
+      </c>
+      <c r="D372" s="27" t="n">
+        <v>1900</v>
+      </c>
       <c r="E372" s="28" t="n"/>
       <c r="F372" s="15">
-        <f>IF(OR(D356&lt;&gt;"",E356&lt;&gt;""),IF(D356="",0,D356)+IF(E356="",0,E356),"")</f>
-        <v/>
-      </c>
-      <c r="G372" s="14" t="n"/>
+        <f>IF(OR(D372&lt;&gt;"",E372&lt;&gt;""),IF(D372="",0,D372)+IF(E372="",0,E372),"")</f>
+        <v/>
+      </c>
+      <c r="G372" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · McDonald's · Mercado Pago · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
     </row>
     <row r="373">
       <c r="A373" s="14" t="inlineStr">
@@ -61916,15 +63912,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B373" s="17" t="n"/>
-      <c r="C373" s="14" t="n"/>
-      <c r="D373" s="27" t="n"/>
+      <c r="B373" s="17" t="n">
+        <v>46284</v>
+      </c>
+      <c r="C373" s="14" t="inlineStr">
+        <is>
+          <t>ENTRETENIMIENTO · Social</t>
+        </is>
+      </c>
+      <c r="D373" s="27" t="n">
+        <v>33359</v>
+      </c>
       <c r="E373" s="28" t="n"/>
       <c r="F373" s="15">
-        <f>IF(OR(D357&lt;&gt;"",E357&lt;&gt;""),IF(D357="",0,D357)+IF(E357="",0,E357),"")</f>
-        <v/>
-      </c>
-      <c r="G373" s="14" t="n"/>
+        <f>IF(OR(D373&lt;&gt;"",E373&lt;&gt;""),IF(D373="",0,D373)+IF(E373="",0,E373),"")</f>
+        <v/>
+      </c>
+      <c r="G373" s="14" t="inlineStr">
+        <is>
+          <t>ENTRETENIMIENTO · Social · la monumental · Mercado Pago · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
     </row>
     <row r="374">
       <c r="A374" s="14" t="inlineStr">
@@ -61932,15 +63940,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B374" s="17" t="n"/>
-      <c r="C374" s="14" t="n"/>
-      <c r="D374" s="27" t="n"/>
+      <c r="B374" s="17" t="n">
+        <v>46288</v>
+      </c>
+      <c r="C374" s="14" t="inlineStr">
+        <is>
+          <t>PEDIDOS YA · COMIDA</t>
+        </is>
+      </c>
+      <c r="D374" s="27" t="n">
+        <v>23964</v>
+      </c>
       <c r="E374" s="28" t="n"/>
       <c r="F374" s="15">
-        <f>IF(OR(D358&lt;&gt;"",E358&lt;&gt;""),IF(D358="",0,D358)+IF(E358="",0,E358),"")</f>
-        <v/>
-      </c>
-      <c r="G374" s="14" t="n"/>
+        <f>IF(OR(D374&lt;&gt;"",E374&lt;&gt;""),IF(D374="",0,D374)+IF(E374="",0,E374),"")</f>
+        <v/>
+      </c>
+      <c r="G374" s="14" t="inlineStr">
+        <is>
+          <t>PEDIDOS YA · COMIDA · screenshot · REVISAR si Market · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
     </row>
     <row r="375">
       <c r="A375" s="14" t="inlineStr">
@@ -61948,15 +63968,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B375" s="17" t="n"/>
-      <c r="C375" s="14" t="n"/>
-      <c r="D375" s="27" t="n"/>
+      <c r="B375" s="17" t="n">
+        <v>46288</v>
+      </c>
+      <c r="C375" s="14" t="inlineStr">
+        <is>
+          <t>PEDIDOS YA · COMIDA · propina</t>
+        </is>
+      </c>
+      <c r="D375" s="27" t="n">
+        <v>850</v>
+      </c>
       <c r="E375" s="28" t="n"/>
       <c r="F375" s="15">
-        <f>IF(OR(D359&lt;&gt;"",E359&lt;&gt;""),IF(D359="",0,D359)+IF(E359="",0,E359),"")</f>
-        <v/>
-      </c>
-      <c r="G375" s="14" t="n"/>
+        <f>IF(OR(D375&lt;&gt;"",E375&lt;&gt;""),IF(D375="",0,D375)+IF(E375="",0,E375),"")</f>
+        <v/>
+      </c>
+      <c r="G375" s="14" t="inlineStr">
+        <is>
+          <t>PEDIDOS YA · COMIDA · propina · screenshot · REVISAR si Market · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
     </row>
     <row r="376">
       <c r="A376" s="14" t="inlineStr">
@@ -61964,15 +63996,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B376" s="17" t="n"/>
-      <c r="C376" s="14" t="n"/>
-      <c r="D376" s="27" t="n"/>
+      <c r="B376" s="17" t="n">
+        <v>46288</v>
+      </c>
+      <c r="C376" s="14" t="inlineStr">
+        <is>
+          <t>ENTRETENIMIENTO · Salidas comida</t>
+        </is>
+      </c>
+      <c r="D376" s="27" t="n">
+        <v>16598</v>
+      </c>
       <c r="E376" s="28" t="n"/>
       <c r="F376" s="15">
-        <f>IF(OR(D360&lt;&gt;"",E360&lt;&gt;""),IF(D360="",0,D360)+IF(E360="",0,E360),"")</f>
-        <v/>
-      </c>
-      <c r="G376" s="14" t="n"/>
+        <f>IF(OR(D376&lt;&gt;"",E376&lt;&gt;""),IF(D376="",0,D376)+IF(E376="",0,E376),"")</f>
+        <v/>
+      </c>
+      <c r="G376" s="14" t="inlineStr">
+        <is>
+          <t>ENTRETENIMIENTO · Salidas comida · Estancia San Francisco Devoto · Mercado Pago · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
     </row>
     <row r="377">
       <c r="A377" s="14" t="inlineStr">
@@ -61980,15 +64024,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B377" s="17" t="n"/>
-      <c r="C377" s="14" t="n"/>
-      <c r="D377" s="27" t="n"/>
+      <c r="B377" s="17" t="n">
+        <v>46290</v>
+      </c>
+      <c r="C377" s="14" t="inlineStr">
+        <is>
+          <t>RAMON · Otros</t>
+        </is>
+      </c>
+      <c r="D377" s="27" t="n">
+        <v>47900</v>
+      </c>
       <c r="E377" s="28" t="n"/>
       <c r="F377" s="15">
-        <f>IF(OR(D361&lt;&gt;"",E361&lt;&gt;""),IF(D361="",0,D361)+IF(E361="",0,E361),"")</f>
-        <v/>
-      </c>
-      <c r="G377" s="14" t="n"/>
+        <f>IF(OR(D377&lt;&gt;"",E377&lt;&gt;""),IF(D377="",0,D377)+IF(E377="",0,E377),"")</f>
+        <v/>
+      </c>
+      <c r="G377" s="14" t="inlineStr">
+        <is>
+          <t>RAMON · Otros · Paws Pet Market · Mercado Pago · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
     </row>
     <row r="378">
       <c r="A378" s="14" t="inlineStr">
@@ -61996,15 +64052,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B378" s="17" t="n"/>
-      <c r="C378" s="14" t="n"/>
-      <c r="D378" s="27" t="n"/>
+      <c r="B378" s="17" t="n">
+        <v>46292</v>
+      </c>
+      <c r="C378" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · Open 25</t>
+        </is>
+      </c>
+      <c r="D378" s="27" t="n">
+        <v>6700</v>
+      </c>
       <c r="E378" s="28" t="n"/>
       <c r="F378" s="15">
-        <f>IF(OR(D362&lt;&gt;"",E362&lt;&gt;""),IF(D362="",0,D362)+IF(E362="",0,E362),"")</f>
-        <v/>
-      </c>
-      <c r="G378" s="14" t="n"/>
+        <f>IF(OR(D378&lt;&gt;"",E378&lt;&gt;""),IF(D378="",0,D378)+IF(E378="",0,E378),"")</f>
+        <v/>
+      </c>
+      <c r="G378" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · Open 25 · Mercado Pago · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
     </row>
     <row r="379">
       <c r="A379" s="14" t="inlineStr">
@@ -62304,6 +64372,7 @@
       </c>
       <c r="G396" s="22" t="n"/>
     </row>
+    <row r="397"/>
     <row r="398">
       <c r="A398" s="14" t="inlineStr">
         <is>
@@ -62970,6 +65039,7 @@
       </c>
       <c r="G438" s="22" t="n"/>
     </row>
+    <row r="439"/>
     <row r="440">
       <c r="A440" s="14" t="inlineStr">
         <is>
@@ -63636,6 +65706,7 @@
       </c>
       <c r="G480" s="22" t="n"/>
     </row>
+    <row r="481"/>
     <row r="482">
       <c r="A482" s="14" t="inlineStr">
         <is>
@@ -64367,7 +66438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I79"/>
+  <dimension ref="A1:I81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -66822,6 +68893,72 @@
         </is>
       </c>
       <c r="I79" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="52" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>LIMPIEZA CASA</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Limpieza Susana — Septiembre 2026 (consolidado MP)</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>835200</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>7 transferencias Susana Carmen Ortiz · dinero en cuenta MP · no duplicar</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="52" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>IMPUESTOS</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>ABL — partida 397789 · AGIP</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>27635</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>AGIP ABL GCBA · MP 2026-09-14 · partida 397789 (≤80k=CIUDAD)</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
         <is>
           <t>Septiembre</t>
         </is>

</xml_diff>

<commit_message>
Cargar resumen TC Mercado Pago septiembre 2026
Consumos y reembolsos del cierre 12/09 (Enerfit, HBO Max, cuotas,
Aerolíneas, Zara refund, etc.), pagos de resumen ago en MP No Gasto,
y actualización del catálogo TC MP + maestro SOL.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -689,7 +689,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:P49"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -1873,7 +1873,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G148"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -3729,8 +3729,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F898"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:F925"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -25889,7 +25889,7 @@
       </c>
       <c r="F830" t="inlineStr">
         <is>
-          <t>SALUD · Vitaminas · Promarine · TC Mercado Pago · 6 cuotas · Gmail Pago aprobado · REVISAR vs resumen TC MP</t>
+          <t>SALUD · Vitaminas · Promarine · TC Mercado Pago · 6 cuotas · Gmail Pago aprobado · REVISAR vs resumen TC MP · post-cierre 12/09 → confirmar en resumen TC MP octubre</t>
         </is>
       </c>
     </row>
@@ -25917,7 +25917,7 @@
       </c>
       <c r="F831" t="inlineStr">
         <is>
-          <t>VESTIMENTA · Itsclassic · TC Mercado Pago · Gmail Pago aprobado · REVISAR (también alerta BBVA MERPAGO*ITSCLASSIC)</t>
+          <t>VESTIMENTA · Itsclassic · TC Mercado Pago · Gmail Pago aprobado · REVISAR (también alerta BBVA MERPAGO*ITSCLASSIC) · post-cierre 12/09 → confirmar en resumen TC MP octubre</t>
         </is>
       </c>
     </row>
@@ -25945,7 +25945,7 @@
       </c>
       <c r="F832" t="inlineStr">
         <is>
-          <t>EDUCACIÓN · EducaciónIT · Automatización Claude · TC Mercado Pago · 3 cuotas · Gmail</t>
+          <t>EDUCACIÓN · EducaciónIT · Automatización Claude · TC Mercado Pago · 3 cuotas · Gmail · post-cierre 12/09 → confirmar en resumen TC MP octubre</t>
         </is>
       </c>
     </row>
@@ -27794,6 +27794,762 @@
       <c r="F898" t="inlineStr">
         <is>
           <t>ENVÍOS · DHL Express · gasto personal Sol · dinero en cuenta MP screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" s="52" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B899" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C899" t="inlineStr">
+        <is>
+          <t>ROPA</t>
+        </is>
+      </c>
+      <c r="D899" t="n">
+        <v>41715</v>
+      </c>
+      <c r="E899" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F899" t="inlineStr">
+        <is>
+          <t>ROPA · Loccitane · TC Mercado Pago · C.6/6 · compra 2026-03-20 · cierre 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" s="52" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B900" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C900" t="inlineStr">
+        <is>
+          <t>ROPA</t>
+        </is>
+      </c>
+      <c r="D900" t="n">
+        <v>23000</v>
+      </c>
+      <c r="E900" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F900" t="inlineStr">
+        <is>
+          <t>ROPA · Adidas · TC Mercado Pago · C.6/6 · compra 2026-03-23 · cierre 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" s="52" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B901" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C901" t="inlineStr">
+        <is>
+          <t>ROPA</t>
+        </is>
+      </c>
+      <c r="D901" t="n">
+        <v>67112</v>
+      </c>
+      <c r="E901" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F901" t="inlineStr">
+        <is>
+          <t>ROPA · Awada · TC Mercado Pago · C.6/9 · compra 2026-03-23 · cierre 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" s="52" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B902" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C902" t="inlineStr">
+        <is>
+          <t>ROPA</t>
+        </is>
+      </c>
+      <c r="D902" t="n">
+        <v>41345</v>
+      </c>
+      <c r="E902" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F902" t="inlineStr">
+        <is>
+          <t>ROPA · Laparfumerie · TC Mercado Pago · C.6/6 · compra 2026-03-30 · cierre 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" s="52" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B903" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C903" t="inlineStr">
+        <is>
+          <t>SALUD · Vitaminas</t>
+        </is>
+      </c>
+      <c r="D903" t="n">
+        <v>87900</v>
+      </c>
+      <c r="E903" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F903" t="inlineStr">
+        <is>
+          <t>SALUD · Vitaminas · Promarine · TC Mercado Pago · C.6/6 · compra 2026-04-04 · cierre 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" s="52" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B904" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C904" t="inlineStr">
+        <is>
+          <t>SALUD</t>
+        </is>
+      </c>
+      <c r="D904" t="n">
+        <v>55707</v>
+      </c>
+      <c r="E904" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F904" t="inlineStr">
+        <is>
+          <t>SALUD · Laboratorio · TC Mercado Pago · C.3/9 · compra 2026-06-23 · cierre 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" s="52" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B905" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C905" t="inlineStr">
+        <is>
+          <t>SALUD</t>
+        </is>
+      </c>
+      <c r="D905" t="n">
+        <v>58334</v>
+      </c>
+      <c r="E905" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F905" t="inlineStr">
+        <is>
+          <t>SALUD · Biodepot · TC Mercado Pago · C.3/3 · compra 2026-06-25 · cierre 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" s="52" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B906" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C906" t="inlineStr">
+        <is>
+          <t>ROPA</t>
+        </is>
+      </c>
+      <c r="D906" t="n">
+        <v>297891</v>
+      </c>
+      <c r="E906" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F906" t="inlineStr">
+        <is>
+          <t>ROPA · Pandora · TC Mercado Pago · C.3/6 · compra 2026-07-09 · cierre 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" s="52" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B907" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C907" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D907" t="n">
+        <v>31450</v>
+      </c>
+      <c r="E907" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F907" t="inlineStr">
+        <is>
+          <t>COMPRAS · PPNL · TC Mercado Pago · C.2/2 · REVISAR ítem · compra 2026-07-16 · cierre 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" s="52" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B908" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C908" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D908" t="n">
+        <v>126325</v>
+      </c>
+      <c r="E908" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F908" t="inlineStr">
+        <is>
+          <t>COMPRAS · LG Distribuidor · TC Mercado Pago · C.2/3 · REVISAR ítem · compra 2026-07-29 · cierre 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" s="52" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B909" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C909" t="inlineStr">
+        <is>
+          <t>REGALOS</t>
+        </is>
+      </c>
+      <c r="D909" t="n">
+        <v>33500</v>
+      </c>
+      <c r="E909" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F909" t="inlineStr">
+        <is>
+          <t>REGALOS · Regalos Dalila · TC Mercado Pago · C.2/2 · compra 2026-07-31 · cierre 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" s="52" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B910" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C910" t="inlineStr">
+        <is>
+          <t>REGALOS</t>
+        </is>
+      </c>
+      <c r="D910" t="n">
+        <v>546850</v>
+      </c>
+      <c r="E910" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F910" t="inlineStr">
+        <is>
+          <t>REGALOS · Regalos Dalila · TC Mercado Pago · C.2/2 · compra 2026-07-31 · cierre 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" s="52" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B911" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C911" t="inlineStr">
+        <is>
+          <t>REGALOS</t>
+        </is>
+      </c>
+      <c r="D911" t="n">
+        <v>62500</v>
+      </c>
+      <c r="E911" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F911" t="inlineStr">
+        <is>
+          <t>REGALOS · Regalos Dalila · TC Mercado Pago · C.2/2 · compra 2026-07-31 · cierre 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" s="52" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B912" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C912" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D912" t="n">
+        <v>58430</v>
+      </c>
+      <c r="E912" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F912" t="inlineStr">
+        <is>
+          <t>COMPRAS · Central Store · TC Mercado Pago · C.2/6 · compra 2026-08-01 · cierre 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" s="52" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B913" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C913" t="inlineStr">
+        <is>
+          <t>ROPA</t>
+        </is>
+      </c>
+      <c r="D913" t="n">
+        <v>82742</v>
+      </c>
+      <c r="E913" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F913" t="inlineStr">
+        <is>
+          <t>ROPA · Monofuk · TC Mercado Pago · C.2/12 · compra 2026-08-04 · cierre 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" s="52" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B914" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C914" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D914" t="n">
+        <v>290000</v>
+      </c>
+      <c r="E914" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F914" t="inlineStr">
+        <is>
+          <t>COMPRAS · Mac Station · TC Mercado Pago · C.1/2 · compra 2026-08-13 · cierre 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" s="52" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B915" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C915" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D915" t="n">
+        <v>52624</v>
+      </c>
+      <c r="E915" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F915" t="inlineStr">
+        <is>
+          <t>COMPRAS · Mac Station · TC Mercado Pago · C.1/2 · compra 2026-08-13 · cierre 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" s="52" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B916" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C916" t="inlineStr">
+        <is>
+          <t>HOGAR</t>
+        </is>
+      </c>
+      <c r="D916" t="n">
+        <v>256862</v>
+      </c>
+      <c r="E916" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F916" t="inlineStr">
+        <is>
+          <t>HOGAR · Banchero Sanitarios · TC Mercado Pago · C.1/3 · compra 2026-08-18 · cierre 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" s="52" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B917" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C917" t="inlineStr">
+        <is>
+          <t>VIAJES</t>
+        </is>
+      </c>
+      <c r="D917" t="n">
+        <v>1633555</v>
+      </c>
+      <c r="E917" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F917" t="inlineStr">
+        <is>
+          <t>VIAJES · Aerolíneas Argentinas · TC Mercado Pago · compra 2026-08-22 · cierre 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" s="52" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B918" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C918" t="inlineStr">
+        <is>
+          <t>MERCADO LIBRE</t>
+        </is>
+      </c>
+      <c r="D918" t="n">
+        <v>107500</v>
+      </c>
+      <c r="E918" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F918" t="inlineStr">
+        <is>
+          <t>Mercado Libre · TC Mercado Pago · C.1/2 · compra 2026-08-22 · cierre 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" s="52" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B919" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C919" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D919" t="n">
+        <v>40000</v>
+      </c>
+      <c r="E919" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F919" t="inlineStr">
+        <is>
+          <t>COMPRAS · Celugadgets · TC Mercado Pago · compra 2026-08-22 · cierre 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" s="52" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B920" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C920" t="inlineStr">
+        <is>
+          <t>VESTIMENTA</t>
+        </is>
+      </c>
+      <c r="D920" t="n">
+        <v>72000</v>
+      </c>
+      <c r="E920" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F920" t="inlineStr">
+        <is>
+          <t>VESTIMENTA · Etiqueta Negra · TC Mercado Pago · C.1/6 · compra 2026-08-25 · cierre 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" s="52" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B921" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C921" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D921" t="n">
+        <v>57725</v>
+      </c>
+      <c r="E921" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F921" t="inlineStr">
+        <is>
+          <t>COMPRAS · Juan Cornacchi · TC Mercado Pago · REVISAR ítem · compra 2026-08-27 · cierre 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" s="52" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B922" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C922" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D922" t="n">
+        <v>39000</v>
+      </c>
+      <c r="E922" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F922" t="inlineStr">
+        <is>
+          <t>COMPRAS · Megaventas HM · TC Mercado Pago · compra 2026-08-27 · cierre 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" s="52" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B923" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C923" t="inlineStr">
+        <is>
+          <t>ROPA</t>
+        </is>
+      </c>
+      <c r="D923" t="n">
+        <v>418000</v>
+      </c>
+      <c r="E923" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F923" t="inlineStr">
+        <is>
+          <t>ROPA · Galeon Joyas · TC Mercado Pago · C.1/3 · compra 2026-09-10 · cierre 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" s="52" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B924" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C924" t="inlineStr">
+        <is>
+          <t>ROPA</t>
+        </is>
+      </c>
+      <c r="D924" t="n">
+        <v>-795614</v>
+      </c>
+      <c r="E924" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F924" t="inlineStr">
+        <is>
+          <t>REEMBOLSO · ROPA · Zara · TC Mercado Pago · compra 2026-08-19 · cierre 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" s="52" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B925" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C925" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D925" t="n">
+        <v>-39000</v>
+      </c>
+      <c r="E925" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F925" t="inlineStr">
+        <is>
+          <t>REEMBOLSO · COMPRAS · Megaventas HM · TC Mercado Pago · compra 2026-08-27 · cierre 2026-09-12</t>
         </is>
       </c>
     </row>
@@ -27813,7 +28569,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L282"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -55122,7 +55878,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G524"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -64084,15 +64840,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B379" s="17" t="n"/>
-      <c r="C379" s="14" t="n"/>
-      <c r="D379" s="27" t="n"/>
+      <c r="B379" s="17" t="n">
+        <v>46277</v>
+      </c>
+      <c r="C379" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · Barritas proteicas</t>
+        </is>
+      </c>
+      <c r="D379" s="27" t="n">
+        <v>66527</v>
+      </c>
       <c r="E379" s="28" t="n"/>
       <c r="F379" s="15">
-        <f>IF(OR(D363&lt;&gt;"",E363&lt;&gt;""),IF(D363="",0,D363)+IF(E363="",0,E363),"")</f>
-        <v/>
-      </c>
-      <c r="G379" s="14" t="n"/>
+        <f>IF(OR(D379&lt;&gt;"",E379&lt;&gt;""),IF(D379="",0,D379)+IF(E379="",0,E379),"")</f>
+        <v/>
+      </c>
+      <c r="G379" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · Barritas proteicas · Enerfit · TC Mercado Pago · C.10/12 · compra 2025-11-26 · cierre 2026-09-12</t>
+        </is>
+      </c>
     </row>
     <row r="380">
       <c r="A380" s="14" t="inlineStr">
@@ -64100,15 +64868,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B380" s="17" t="n"/>
-      <c r="C380" s="14" t="n"/>
-      <c r="D380" s="27" t="n"/>
+      <c r="B380" s="17" t="n">
+        <v>46277</v>
+      </c>
+      <c r="C380" s="14" t="inlineStr">
+        <is>
+          <t>STREAMING TV</t>
+        </is>
+      </c>
+      <c r="D380" s="27" t="n">
+        <v>97393</v>
+      </c>
       <c r="E380" s="28" t="n"/>
       <c r="F380" s="15">
-        <f>IF(OR(D364&lt;&gt;"",E364&lt;&gt;""),IF(D364="",0,D364)+IF(E364="",0,E364),"")</f>
-        <v/>
-      </c>
-      <c r="G380" s="14" t="n"/>
+        <f>IF(OR(D380&lt;&gt;"",E380&lt;&gt;""),IF(D380="",0,D380)+IF(E380="",0,E380),"")</f>
+        <v/>
+      </c>
+      <c r="G380" s="14" t="inlineStr">
+        <is>
+          <t>STREAMING TV · HBO Max · TC Mercado Pago · compra 2026-09-05 · cierre 2026-09-12</t>
+        </is>
+      </c>
     </row>
     <row r="381">
       <c r="A381" s="14" t="inlineStr">
@@ -66440,7 +67220,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I81"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -68978,7 +69758,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F142"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -70378,8 +71158,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:H53"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -71660,6 +72440,72 @@
       <c r="H51" t="inlineStr">
         <is>
           <t>Reserva automática · − · 17:15 · NUNCA almacén</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="52" t="n">
+        <v>46253</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Pago de resumen TC</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Tarjeta de crédito Mercado Pago</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="52" t="n">
+        <v>46253</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Pago de resumen TC</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Tarjeta de crédito Mercado Pago</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>1225483</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
         </is>
       </c>
     </row>
@@ -71680,7 +72526,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J223"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -74569,7 +75415,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F172"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -76429,7 +77275,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -76608,6 +77454,7 @@
         <v/>
       </c>
     </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
         <is>
@@ -76784,6 +77631,62 @@
       <c r="F27" t="inlineStr">
         <is>
           <t>Pago de resumen · ceil 576241.18 · hoja Pago de Tarjetas / MP No Gasto</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="52" t="n">
+        <v>46253</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Tarjeta de crédito</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Pago de resumen · $1.200.000 · composición resumen TC MP sep</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="52" t="n">
+        <v>46253</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Tarjeta de crédito</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>1225483</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Pago de resumen · $1.225.482,78 ceil · composición resumen TC MP sep</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Armar septiembre 2026: alertas BBVA faltantes y resumen
Completa GPS con USD IA (ChatGPT/Cursor/Google One), dhgate,
Markova/Luxodia/Luna Hogar, Yenny/Vienna; corrige Telecentro en
Detalle; registra pago AVA en Expensas Consorcios; deja resumen
consolidado del mes.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -689,7 +689,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:P49"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -1873,7 +1873,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G148"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -2797,13 +2797,37 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="17" t="n"/>
-      <c r="B47" s="14" t="n"/>
-      <c r="C47" s="14" t="n"/>
-      <c r="D47" s="14" t="n"/>
-      <c r="E47" s="15" t="n"/>
-      <c r="F47" s="14" t="n"/>
-      <c r="G47" s="14" t="n"/>
+      <c r="A47" s="17" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B47" s="14" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C47" s="14" t="inlineStr">
+        <is>
+          <t>Fideicomiso Ava Palpa</t>
+        </is>
+      </c>
+      <c r="D47" s="14" t="inlineStr">
+        <is>
+          <t>AVA</t>
+        </is>
+      </c>
+      <c r="E47" s="15" t="n">
+        <v>6269440</v>
+      </c>
+      <c r="F47" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Transferencia enviada</t>
+        </is>
+      </c>
+      <c r="G47" s="14" t="inlineStr">
+        <is>
+          <t>AVA cuota 10 · pagado 07/09 · total $6.269.440 · 50% Sol ya en GPS</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="17" t="n"/>
@@ -3729,8 +3753,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F925"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:F937"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -28550,6 +28574,342 @@
       <c r="F925" t="inlineStr">
         <is>
           <t>REEMBOLSO · COMPRAS · Megaventas HM · TC Mercado Pago · compra 2026-08-27 · cierre 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" s="52" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B926" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C926" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D926" t="n">
+        <v>580320</v>
+      </c>
+      <c r="E926" t="inlineStr">
+        <is>
+          <t>BBVA VISA</t>
+        </is>
+      </c>
+      <c r="F926" t="inlineStr">
+        <is>
+          <t>COMPRAS · dhgate.com · BBVA VISA · USD 380.44 × TC MEP 1525.39 · importación · alerta Gmail Compra aprobada · REVISAR vs resumen BBVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" s="52" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B927" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C927" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D927" t="n">
+        <v>629985</v>
+      </c>
+      <c r="E927" t="inlineStr">
+        <is>
+          <t>BBVA VISA</t>
+        </is>
+      </c>
+      <c r="F927" t="inlineStr">
+        <is>
+          <t>COMPRAS · dhgate.com · BBVA VISA · USD 409.57 × TC MEP 1538.16 · importación · MEP 11/09 (13/09 domingo) · alerta Gmail Compra aprobada · REVISAR vs resumen BBVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" s="52" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B928" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C928" t="inlineStr">
+        <is>
+          <t>SUSCRIPCIONES · IA</t>
+        </is>
+      </c>
+      <c r="D928" t="n">
+        <v>7668</v>
+      </c>
+      <c r="E928" t="inlineStr">
+        <is>
+          <t>BBVA VISA</t>
+        </is>
+      </c>
+      <c r="F928" t="inlineStr">
+        <is>
+          <t>SUSCRIPCIONES · IA · Google One / Gemini · BBVA VISA · USD 4.99 × TC MEP 1536.51 · alerta Gmail Compra aprobada · REVISAR vs resumen BBVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" s="52" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B929" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C929" t="inlineStr">
+        <is>
+          <t>SUSCRIPCIONES · IA</t>
+        </is>
+      </c>
+      <c r="D929" t="n">
+        <v>93150</v>
+      </c>
+      <c r="E929" t="inlineStr">
+        <is>
+          <t>BBVA VISA</t>
+        </is>
+      </c>
+      <c r="F929" t="inlineStr">
+        <is>
+          <t>SUSCRIPCIONES · IA · Cursor · BBVA VISA · USD 60.00 × TC MEP 1552.5 · MEP 25/09 (27/09 domingo) · alerta Gmail Compra aprobada · REVISAR vs resumen BBVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" s="52" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B930" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C930" t="inlineStr">
+        <is>
+          <t>SUSCRIPCIONES · IA</t>
+        </is>
+      </c>
+      <c r="D930" t="n">
+        <v>30852</v>
+      </c>
+      <c r="E930" t="inlineStr">
+        <is>
+          <t>BBVA VISA</t>
+        </is>
+      </c>
+      <c r="F930" t="inlineStr">
+        <is>
+          <t>SUSCRIPCIONES · IA · ChatGPT / OpenAI · BBVA VISA · USD 20.00 × TC MEP 1542.56 · alerta Gmail Compra aprobada · REVISAR vs resumen BBVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" s="52" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B931" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C931" t="inlineStr">
+        <is>
+          <t>VESTIMENTA</t>
+        </is>
+      </c>
+      <c r="D931" t="n">
+        <v>809200</v>
+      </c>
+      <c r="E931" t="inlineStr">
+        <is>
+          <t>BBVA VISA</t>
+        </is>
+      </c>
+      <c r="F931" t="inlineStr">
+        <is>
+          <t>VESTIMENTA · Markova · BBVA VISA · MERPAGO*MARKOVA · alerta Gmail · REVISAR ítem</t>
+        </is>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" s="52" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B932" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C932" t="inlineStr">
+        <is>
+          <t>HOGAR</t>
+        </is>
+      </c>
+      <c r="D932" t="n">
+        <v>186300</v>
+      </c>
+      <c r="E932" t="inlineStr">
+        <is>
+          <t>BBVA VISA</t>
+        </is>
+      </c>
+      <c r="F932" t="inlineStr">
+        <is>
+          <t>HOGAR · Luna Hogar · BBVA VISA · MERPAGO*LUNAHOGAR · alerta Gmail</t>
+        </is>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" s="52" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B933" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C933" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D933" t="n">
+        <v>8520</v>
+      </c>
+      <c r="E933" t="inlineStr">
+        <is>
+          <t>BBVA VISA</t>
+        </is>
+      </c>
+      <c r="F933" t="inlineStr">
+        <is>
+          <t>COMPRAS · La Obanesad · BBVA VISA · MERPAGO*LAOBANESAD · alerta Gmail · REVISAR ítem</t>
+        </is>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" s="52" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B934" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C934" t="inlineStr">
+        <is>
+          <t>VESTIMENTA</t>
+        </is>
+      </c>
+      <c r="D934" t="n">
+        <v>334288</v>
+      </c>
+      <c r="E934" t="inlineStr">
+        <is>
+          <t>BBVA VISA</t>
+        </is>
+      </c>
+      <c r="F934" t="inlineStr">
+        <is>
+          <t>VESTIMENTA · Luxodia · BBVA VISA · MERPAGO*LUXODIA · alerta Gmail · REVISAR ítem</t>
+        </is>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" s="52" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B935" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C935" t="inlineStr">
+        <is>
+          <t>VESTIMENTA</t>
+        </is>
+      </c>
+      <c r="D935" t="n">
+        <v>49492</v>
+      </c>
+      <c r="E935" t="inlineStr">
+        <is>
+          <t>BBVA VISA</t>
+        </is>
+      </c>
+      <c r="F935" t="inlineStr">
+        <is>
+          <t>VESTIMENTA · Luxodia · BBVA VISA · MERPAGO*LUXODIA · alerta Gmail · REVISAR ítem</t>
+        </is>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" s="52" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B936" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C936" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D936" t="n">
+        <v>89998</v>
+      </c>
+      <c r="E936" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F936" t="inlineStr">
+        <is>
+          <t>COMPRAS · Yenny El Ateneo · TC Mercado Pago · Gmail Pago aprobado · post-cierre 12/09 → confirmar resumen octubre</t>
+        </is>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" s="52" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B937" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C937" t="inlineStr">
+        <is>
+          <t>HOGAR</t>
+        </is>
+      </c>
+      <c r="D937" t="n">
+        <v>134572</v>
+      </c>
+      <c r="E937" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F937" t="inlineStr">
+        <is>
+          <t>HOGAR · ViennaHogar · TC Mercado Pago · 3 cuotas · Gmail Pago aprobado · post-cierre 12/09 → confirmar resumen octubre</t>
         </is>
       </c>
     </row>
@@ -28569,7 +28929,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L282"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -55878,7 +56238,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G524"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -67220,7 +67580,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I81"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -68371,18 +68731,22 @@
       </c>
       <c r="C36" s="14" t="inlineStr">
         <is>
-          <t>Telecentro CIUDAD — servicio mensual 09/2026</t>
+          <t>Telecentro CIUDAD — débito BBVA 25/09/2026 (reemplaza placeholder $50.000)</t>
         </is>
       </c>
       <c r="D36" s="15" t="n">
-        <v>50000</v>
-      </c>
-      <c r="E36" s="14" t="inlineStr"/>
+        <v>69659</v>
+      </c>
+      <c r="E36" s="14" t="inlineStr">
+        <is>
+          <t>Débito BBVA</t>
+        </is>
+      </c>
       <c r="F36" s="18" t="inlineStr"/>
       <c r="G36" s="18" t="inlineStr"/>
       <c r="H36" s="14" t="inlineStr">
         <is>
-          <t>Recurrente $50.000/mes hasta nuevo aviso</t>
+          <t>Oficial $69.659 · mes=cobro · supersede recurrent placeholder</t>
         </is>
       </c>
       <c r="I36" s="14" t="inlineStr">
@@ -69758,7 +70122,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F142"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -71159,7 +71523,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H53"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -72526,7 +72890,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J223"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -75415,7 +75779,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F172"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -77454,7 +77818,6 @@
         <v/>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Confirmar PedidosYa septiembre como COMIDA en Almacén
Sol confirma que PedidosYa es comida: se mantienen en Almacen Detalle
como PEDIDOS YA · COMIDA (+ propina) y se quitan las notas REVISAR Market.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -60797,6 +60797,7 @@
       </c>
       <c r="G176" s="22" t="n"/>
     </row>
+    <row r="177"/>
     <row r="178">
       <c r="A178" s="14" t="inlineStr">
         <is>
@@ -62079,6 +62080,7 @@
       </c>
       <c r="G228" s="22" t="n"/>
     </row>
+    <row r="229"/>
     <row r="230">
       <c r="A230" s="14" t="inlineStr">
         <is>
@@ -63117,6 +63119,7 @@
       </c>
       <c r="G273" s="22" t="n"/>
     </row>
+    <row r="274"/>
     <row r="275">
       <c r="A275" s="14" t="inlineStr">
         <is>
@@ -63884,6 +63887,7 @@
       </c>
       <c r="G312" s="22" t="n"/>
     </row>
+    <row r="313"/>
     <row r="314">
       <c r="A314" s="14" t="inlineStr">
         <is>
@@ -64550,6 +64554,7 @@
       </c>
       <c r="G354" s="22" t="n"/>
     </row>
+    <row r="355"/>
     <row r="356">
       <c r="A356" s="14" t="inlineStr">
         <is>
@@ -64658,7 +64663,7 @@
       </c>
       <c r="G359" s="14" t="inlineStr">
         <is>
-          <t>PEDIDOS YA · COMIDA · screenshot · REVISAR si Market · dinero en cuenta MP screenshot</t>
+          <t>PEDIDOS YA · COMIDA · screenshot · dinero en cuenta MP screenshot</t>
         </is>
       </c>
     </row>
@@ -64686,7 +64691,7 @@
       </c>
       <c r="G360" s="14" t="inlineStr">
         <is>
-          <t>PEDIDOS YA · COMIDA · propina · screenshot · REVISAR si Market · dinero en cuenta MP screenshot</t>
+          <t>PEDIDOS YA · COMIDA · propina · screenshot · dinero en cuenta MP screenshot</t>
         </is>
       </c>
     </row>
@@ -64798,7 +64803,7 @@
       </c>
       <c r="G364" s="14" t="inlineStr">
         <is>
-          <t>PEDIDOS YA · COMIDA · screenshot · REVISAR si Market · dinero en cuenta MP screenshot</t>
+          <t>PEDIDOS YA · COMIDA · screenshot · dinero en cuenta MP screenshot</t>
         </is>
       </c>
     </row>
@@ -64826,7 +64831,7 @@
       </c>
       <c r="G365" s="14" t="inlineStr">
         <is>
-          <t>PEDIDOS YA · COMIDA · propina · screenshot · REVISAR si Market · dinero en cuenta MP screenshot</t>
+          <t>PEDIDOS YA · COMIDA · propina · screenshot · dinero en cuenta MP screenshot</t>
         </is>
       </c>
     </row>
@@ -64854,7 +64859,7 @@
       </c>
       <c r="G366" s="14" t="inlineStr">
         <is>
-          <t>PEDIDOS YA · COMIDA · screenshot · REVISAR si Market · dinero en cuenta MP screenshot</t>
+          <t>PEDIDOS YA · COMIDA · screenshot · dinero en cuenta MP screenshot</t>
         </is>
       </c>
     </row>
@@ -64938,7 +64943,7 @@
       </c>
       <c r="G369" s="14" t="inlineStr">
         <is>
-          <t>PEDIDOS YA · COMIDA · screenshot · REVISAR si Market · dinero en cuenta MP screenshot</t>
+          <t>PEDIDOS YA · COMIDA · screenshot · dinero en cuenta MP screenshot</t>
         </is>
       </c>
     </row>
@@ -64966,7 +64971,7 @@
       </c>
       <c r="G370" s="14" t="inlineStr">
         <is>
-          <t>PEDIDOS YA · COMIDA · propina · screenshot · REVISAR si Market · dinero en cuenta MP screenshot</t>
+          <t>PEDIDOS YA · COMIDA · propina · screenshot · dinero en cuenta MP screenshot</t>
         </is>
       </c>
     </row>
@@ -65078,7 +65083,7 @@
       </c>
       <c r="G374" s="14" t="inlineStr">
         <is>
-          <t>PEDIDOS YA · COMIDA · screenshot · REVISAR si Market · dinero en cuenta MP screenshot</t>
+          <t>PEDIDOS YA · COMIDA · screenshot · dinero en cuenta MP screenshot</t>
         </is>
       </c>
     </row>
@@ -65106,7 +65111,7 @@
       </c>
       <c r="G375" s="14" t="inlineStr">
         <is>
-          <t>PEDIDOS YA · COMIDA · propina · screenshot · REVISAR si Market · dinero en cuenta MP screenshot</t>
+          <t>PEDIDOS YA · COMIDA · propina · screenshot · dinero en cuenta MP screenshot</t>
         </is>
       </c>
     </row>
@@ -65516,6 +65521,7 @@
       </c>
       <c r="G396" s="22" t="n"/>
     </row>
+    <row r="397"/>
     <row r="398">
       <c r="A398" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Quitar Telecentro duplicado en Detalle de septiembre
La matriz ya tenía el débito BBVA $69.659; se anula el placeholder
repetido para no confundir el detalle de servicios.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -60797,7 +60797,6 @@
       </c>
       <c r="G176" s="22" t="n"/>
     </row>
-    <row r="177"/>
     <row r="178">
       <c r="A178" s="14" t="inlineStr">
         <is>
@@ -62080,7 +62079,6 @@
       </c>
       <c r="G228" s="22" t="n"/>
     </row>
-    <row r="229"/>
     <row r="230">
       <c r="A230" s="14" t="inlineStr">
         <is>
@@ -63119,7 +63117,6 @@
       </c>
       <c r="G273" s="22" t="n"/>
     </row>
-    <row r="274"/>
     <row r="275">
       <c r="A275" s="14" t="inlineStr">
         <is>
@@ -63887,7 +63884,6 @@
       </c>
       <c r="G312" s="22" t="n"/>
     </row>
-    <row r="313"/>
     <row r="314">
       <c r="A314" s="14" t="inlineStr">
         <is>
@@ -64554,7 +64550,6 @@
       </c>
       <c r="G354" s="22" t="n"/>
     </row>
-    <row r="355"/>
     <row r="356">
       <c r="A356" s="14" t="inlineStr">
         <is>
@@ -65521,7 +65516,6 @@
       </c>
       <c r="G396" s="22" t="n"/>
     </row>
-    <row r="397"/>
     <row r="398">
       <c r="A398" s="14" t="inlineStr">
         <is>
@@ -68737,12 +68731,10 @@
       </c>
       <c r="C36" s="14" t="inlineStr">
         <is>
-          <t>Telecentro CIUDAD — débito BBVA 25/09/2026 (reemplaza placeholder $50.000)</t>
-        </is>
-      </c>
-      <c r="D36" s="15" t="n">
-        <v>69659</v>
-      </c>
+          <t>(duplicado) ver fila débito BBVA 25/09 — no sumar</t>
+        </is>
+      </c>
+      <c r="D36" s="15" t="n"/>
       <c r="E36" s="14" t="inlineStr">
         <is>
           <t>Débito BBVA</t>
@@ -68752,7 +68744,7 @@
       <c r="G36" s="18" t="inlineStr"/>
       <c r="H36" s="14" t="inlineStr">
         <is>
-          <t>Oficial $69.659 · mes=cobro · supersede recurrent placeholder</t>
+          <t>SUPERSEDE · Telecentro Sept está en Detalle débito 25/09 $69.659</t>
         </is>
       </c>
       <c r="I36" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Crear Sol Dollar Mdp y excluir compras USD Mastercard
Nueva hoja de stock USD (saldo 0 al 2026-10-04). Los consumos/compras
de dólar con BBVA Mastercard dejan de imputarse como gasto en GPS.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -19,6 +19,7 @@
     <sheet name="Expensas Consorcios" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Gasto Personal Sol" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Cashflow Compromisos" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Sol Dollar Mdp" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Detalle'!$A$3:$I$51</definedName>
@@ -37,7 +38,7 @@
     <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
     <numFmt numFmtId="168" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -115,8 +116,13 @@
       <color rgb="0017365D"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -161,6 +167,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="0017365D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2F0D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005B9BD5"/>
       </patternFill>
     </fill>
   </fills>
@@ -248,7 +264,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -323,6 +339,21 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="11" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="10" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="10" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -12140,7 +12171,7 @@
       </c>
       <c r="F337" t="inlineStr">
         <is>
-          <t>ROPA · gasto personal Sol · monto en USD (no convertido a ARS)</t>
+          <t>ROPA · gasto personal Sol · monto en USD (no convertido a ARS) · NO ES GASTO · consumo/compra USD BBVA Mastercard · ver hoja Sol Dollar Mdp</t>
         </is>
       </c>
     </row>
@@ -12270,9 +12301,6 @@
           <t>SUSCRIPCIONES · IA</t>
         </is>
       </c>
-      <c r="D342" t="n">
-        <v>28593</v>
-      </c>
       <c r="E342" t="inlineStr">
         <is>
           <t>BBVA Mastercard · USD</t>
@@ -12280,7 +12308,7 @@
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t>SUSCRIPCIONES · IA · Vercel · gasto personal Sol · USD 20.00 × TC MEP 1429.65 · suscripción · gasto personal Sol</t>
+          <t>SUSCRIPCIONES · IA · Vercel · gasto personal Sol · USD 20.00 × TC MEP 1429.65 · suscripción · gasto personal Sol · NO ES GASTO · consumo/compra USD BBVA Mastercard · ver hoja Sol Dollar Mdp</t>
         </is>
       </c>
     </row>
@@ -12298,9 +12326,6 @@
           <t>SUSCRIPCIONES · IA</t>
         </is>
       </c>
-      <c r="D343" t="n">
-        <v>42890</v>
-      </c>
       <c r="E343" t="inlineStr">
         <is>
           <t>BBVA Mastercard · USD</t>
@@ -12308,7 +12333,7 @@
       </c>
       <c r="F343" t="inlineStr">
         <is>
-          <t>SUSCRIPCIONES · IA · Vercel · gasto personal Sol · USD 30.00 × TC MEP 1429.65 · suscripción · gasto personal Sol</t>
+          <t>SUSCRIPCIONES · IA · Vercel · gasto personal Sol · USD 30.00 × TC MEP 1429.65 · suscripción · gasto personal Sol · NO ES GASTO · consumo/compra USD BBVA Mastercard · ver hoja Sol Dollar Mdp</t>
         </is>
       </c>
     </row>
@@ -12438,9 +12463,6 @@
           <t>SUSCRIPCIONES · IA</t>
         </is>
       </c>
-      <c r="D348" t="n">
-        <v>43740</v>
-      </c>
       <c r="E348" t="inlineStr">
         <is>
           <t>BBVA Mastercard · USD</t>
@@ -12448,7 +12470,7 @@
       </c>
       <c r="F348" t="inlineStr">
         <is>
-          <t>SUSCRIPCIONES · IA · Vercel · gasto personal Sol · USD 30.00 × TC MEP 1458.0 · suscripción · gasto personal Sol</t>
+          <t>SUSCRIPCIONES · IA · Vercel · gasto personal Sol · USD 30.00 × TC MEP 1458.0 · suscripción · gasto personal Sol · NO ES GASTO · consumo/compra USD BBVA Mastercard · ver hoja Sol Dollar Mdp</t>
         </is>
       </c>
     </row>
@@ -12550,9 +12572,6 @@
           <t>SUSCRIPCIONES · IA</t>
         </is>
       </c>
-      <c r="D352" t="n">
-        <v>30110</v>
-      </c>
       <c r="E352" t="inlineStr">
         <is>
           <t>BBVA Mastercard · USD</t>
@@ -12560,7 +12579,7 @@
       </c>
       <c r="F352" t="inlineStr">
         <is>
-          <t>SUSCRIPCIONES · IA · Google One / Gemini · gasto personal Sol · USD 19.99 × TC MEP 1506.21 · Gemini Advanced / Google One · gasto personal Sol</t>
+          <t>SUSCRIPCIONES · IA · Google One / Gemini · gasto personal Sol · USD 19.99 × TC MEP 1506.21 · Gemini Advanced / Google One · gasto personal Sol · NO ES GASTO · consumo/compra USD BBVA Mastercard · ver hoja Sol Dollar Mdp</t>
         </is>
       </c>
     </row>
@@ -12578,9 +12597,6 @@
           <t>SUSCRIPCIONES · IA</t>
         </is>
       </c>
-      <c r="D353" t="n">
-        <v>29193</v>
-      </c>
       <c r="E353" t="inlineStr">
         <is>
           <t>BBVA Mastercard · USD</t>
@@ -12588,7 +12604,7 @@
       </c>
       <c r="F353" t="inlineStr">
         <is>
-          <t>SUSCRIPCIONES · IA · Google One / Gemini · gasto personal Sol · USD 19.99 × TC MEP 1460.38 · Gemini Advanced / Google One · gasto personal Sol</t>
+          <t>SUSCRIPCIONES · IA · Google One / Gemini · gasto personal Sol · USD 19.99 × TC MEP 1460.38 · Gemini Advanced / Google One · gasto personal Sol · NO ES GASTO · consumo/compra USD BBVA Mastercard · ver hoja Sol Dollar Mdp</t>
         </is>
       </c>
     </row>
@@ -12606,9 +12622,6 @@
           <t>SUSCRIPCIONES · IA</t>
         </is>
       </c>
-      <c r="D354" t="n">
-        <v>28668</v>
-      </c>
       <c r="E354" t="inlineStr">
         <is>
           <t>BBVA Mastercard · USD</t>
@@ -12616,7 +12629,7 @@
       </c>
       <c r="F354" t="inlineStr">
         <is>
-          <t>SUSCRIPCIONES · IA · Google One / Gemini · gasto personal Sol · USD 19.99 × TC MEP 1434.11 · Gemini Advanced / Google One · gasto personal Sol</t>
+          <t>SUSCRIPCIONES · IA · Google One / Gemini · gasto personal Sol · USD 19.99 × TC MEP 1434.11 · Gemini Advanced / Google One · gasto personal Sol · NO ES GASTO · consumo/compra USD BBVA Mastercard · ver hoja Sol Dollar Mdp</t>
         </is>
       </c>
     </row>
@@ -12634,9 +12647,6 @@
           <t>SUSCRIPCIONES · IA</t>
         </is>
       </c>
-      <c r="D355" t="n">
-        <v>28667</v>
-      </c>
       <c r="E355" t="inlineStr">
         <is>
           <t>BBVA Mastercard · USD</t>
@@ -12644,7 +12654,7 @@
       </c>
       <c r="F355" t="inlineStr">
         <is>
-          <t>SUSCRIPCIONES · IA · Google One / Gemini · gasto personal Sol · USD 19.99 × TC MEP 1434.04 · Gemini Advanced / Google One · gasto personal Sol</t>
+          <t>SUSCRIPCIONES · IA · Google One / Gemini · gasto personal Sol · USD 19.99 × TC MEP 1434.04 · Gemini Advanced / Google One · gasto personal Sol · NO ES GASTO · consumo/compra USD BBVA Mastercard · ver hoja Sol Dollar Mdp</t>
         </is>
       </c>
     </row>
@@ -24307,9 +24317,7 @@
           <t>SUSCRIPCIONES · IA</t>
         </is>
       </c>
-      <c r="D773" s="34" t="n">
-        <v>29208</v>
-      </c>
+      <c r="D773" s="34" t="n"/>
       <c r="E773" s="34" t="inlineStr">
         <is>
           <t>BBVA</t>
@@ -24317,7 +24325,7 @@
       </c>
       <c r="F773" s="34" t="inlineStr">
         <is>
-          <t>SUSCRIPCIONES · IA · ChatGPT / OpenAI · gasto personal Sol</t>
+          <t>SUSCRIPCIONES · IA · ChatGPT / OpenAI · gasto personal Sol · NO ES GASTO · consumo/compra USD BBVA Mastercard · ver hoja Sol Dollar Mdp</t>
         </is>
       </c>
     </row>
@@ -24335,9 +24343,7 @@
           <t>SUSCRIPCIONES · IA</t>
         </is>
       </c>
-      <c r="D774" s="34" t="n">
-        <v>29208</v>
-      </c>
+      <c r="D774" s="34" t="n"/>
       <c r="E774" s="34" t="inlineStr">
         <is>
           <t>BBVA</t>
@@ -24345,7 +24351,7 @@
       </c>
       <c r="F774" s="34" t="inlineStr">
         <is>
-          <t>SUSCRIPCIONES · IA · ChatGPT / OpenAI · gasto personal Sol</t>
+          <t>SUSCRIPCIONES · IA · ChatGPT / OpenAI · gasto personal Sol · NO ES GASTO · consumo/compra USD BBVA Mastercard · ver hoja Sol Dollar Mdp</t>
         </is>
       </c>
     </row>
@@ -24363,9 +24369,7 @@
           <t>SUSCRIPCIONES · IA</t>
         </is>
       </c>
-      <c r="D775" s="34" t="n">
-        <v>28681</v>
-      </c>
+      <c r="D775" s="34" t="n"/>
       <c r="E775" s="34" t="inlineStr">
         <is>
           <t>BBVA</t>
@@ -24373,7 +24377,7 @@
       </c>
       <c r="F775" s="34" t="inlineStr">
         <is>
-          <t>SUSCRIPCIONES · IA · ChatGPT / OpenAI · gasto personal Sol</t>
+          <t>SUSCRIPCIONES · IA · ChatGPT / OpenAI · gasto personal Sol · NO ES GASTO · consumo/compra USD BBVA Mastercard · ver hoja Sol Dollar Mdp</t>
         </is>
       </c>
     </row>
@@ -25763,9 +25767,7 @@
           <t>SUSCRIPCIONES · IA</t>
         </is>
       </c>
-      <c r="D825" s="34" t="n">
-        <v>29</v>
-      </c>
+      <c r="D825" s="34" t="n"/>
       <c r="E825" s="34" t="inlineStr">
         <is>
           <t>BBVA MASTERCARD</t>
@@ -25773,7 +25775,7 @@
       </c>
       <c r="F825" s="34" t="inlineStr">
         <is>
-          <t>SUSCRIPCIONES · IA · metricscheck.com · REVISAR · metricscheck.com · posible cargo prueba USD · gasto personal Sol</t>
+          <t>SUSCRIPCIONES · IA · metricscheck.com · REVISAR · metricscheck.com · posible cargo prueba USD · gasto personal Sol · NO ES GASTO · consumo/compra USD BBVA Mastercard · ver hoja Sol Dollar Mdp</t>
         </is>
       </c>
     </row>
@@ -25791,9 +25793,7 @@
           <t>SUSCRIPCIONES · IA</t>
         </is>
       </c>
-      <c r="D826" s="34" t="n">
-        <v>1</v>
-      </c>
+      <c r="D826" s="34" t="n"/>
       <c r="E826" s="34" t="inlineStr">
         <is>
           <t>BBVA MASTERCARD</t>
@@ -25801,7 +25801,7 @@
       </c>
       <c r="F826" s="34" t="inlineStr">
         <is>
-          <t>SUSCRIPCIONES · IA · metricscheck.com · REVISAR · metricscheck.com · posible cargo prueba USD · gasto personal Sol</t>
+          <t>SUSCRIPCIONES · IA · metricscheck.com · REVISAR · metricscheck.com · posible cargo prueba USD · gasto personal Sol · NO ES GASTO · consumo/compra USD BBVA Mastercard · ver hoja Sol Dollar Mdp</t>
         </is>
       </c>
     </row>
@@ -43773,6 +43773,477 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="55" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="64" t="inlineStr">
+        <is>
+          <t>Sol Dollar Mdp</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Stock de dólares de Sol. Las compras de dólar con BBVA Mastercard NO son gasto (no van a Gasto Personal Sol ni a la matriz 2026). Consumos USD de MC tampoco se imputan como gasto ARS. Percepciones USD (RG 5617 / IVA / IIBB) sí siguen en GPS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Saldo USD a la fecha</t>
+        </is>
+      </c>
+      <c r="B4" s="54" t="n">
+        <v>46299</v>
+      </c>
+      <c r="C4" s="65" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Confirmado por Sol · no hay dólares en stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="59" t="inlineStr">
+        <is>
+          <t>Detalle de movimientos</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="66" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B7" s="66" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C7" s="66" t="inlineStr">
+        <is>
+          <t>Origen</t>
+        </is>
+      </c>
+      <c r="D7" s="66" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
+      <c r="E7" s="66" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="F7" s="66" t="inlineStr">
+        <is>
+          <t>TC MEP</t>
+        </is>
+      </c>
+      <c r="G7" s="66" t="inlineStr">
+        <is>
+          <t>ARS informativo (no es gasto)</t>
+        </is>
+      </c>
+      <c r="H7" s="66" t="inlineStr">
+        <is>
+          <t>Saldo USD</t>
+        </is>
+      </c>
+      <c r="I7" s="66" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="67" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B8" s="68" t="inlineStr">
+        <is>
+          <t>Saldo inicial</t>
+        </is>
+      </c>
+      <c r="C8" s="68" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D8" s="68" t="inlineStr">
+        <is>
+          <t>Stock USD Sol</t>
+        </is>
+      </c>
+      <c r="E8" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="68" t="n"/>
+      <c r="G8" s="68" t="n"/>
+      <c r="H8" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="68" t="inlineStr">
+        <is>
+          <t>A la fecha hay cero dólares · planilla lista para compras/ventas futuras</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Consumos USD Mastercard excluidos de GPS (no mueven el stock; stock = 0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="70" t="inlineStr">
+        <is>
+          <t>Fecha GPS</t>
+        </is>
+      </c>
+      <c r="B11" s="70" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="C11" s="70" t="inlineStr">
+        <is>
+          <t>USD / nota</t>
+        </is>
+      </c>
+      <c r="D11" s="70" t="inlineStr">
+        <is>
+          <t>ARS que se sacó de GPS</t>
+        </is>
+      </c>
+      <c r="E11" s="70" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="71" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B12" s="72" t="inlineStr">
+        <is>
+          <t>ROPA</t>
+        </is>
+      </c>
+      <c r="C12" s="72" t="inlineStr">
+        <is>
+          <t>ROPA · gasto personal Sol · monto en USD (no convertido a AR</t>
+        </is>
+      </c>
+      <c r="D12" s="72" t="n"/>
+      <c r="E12" s="72" t="inlineStr">
+        <is>
+          <t>BBVA Mastercard · USD 3.807,01 (EUR 3.250)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="71" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B13" s="72" t="inlineStr">
+        <is>
+          <t>SUSCRIPCIONES · IA</t>
+        </is>
+      </c>
+      <c r="C13" s="73" t="n">
+        <v>20</v>
+      </c>
+      <c r="D13" s="74" t="n">
+        <v>28593</v>
+      </c>
+      <c r="E13" s="72" t="inlineStr">
+        <is>
+          <t>BBVA Mastercard · USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="71" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B14" s="72" t="inlineStr">
+        <is>
+          <t>SUSCRIPCIONES · IA</t>
+        </is>
+      </c>
+      <c r="C14" s="73" t="n">
+        <v>30</v>
+      </c>
+      <c r="D14" s="74" t="n">
+        <v>42890</v>
+      </c>
+      <c r="E14" s="72" t="inlineStr">
+        <is>
+          <t>BBVA Mastercard · USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="71" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B15" s="72" t="inlineStr">
+        <is>
+          <t>SUSCRIPCIONES · IA</t>
+        </is>
+      </c>
+      <c r="C15" s="73" t="n">
+        <v>30</v>
+      </c>
+      <c r="D15" s="74" t="n">
+        <v>43740</v>
+      </c>
+      <c r="E15" s="72" t="inlineStr">
+        <is>
+          <t>BBVA Mastercard · USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="71" t="n">
+        <v>46029</v>
+      </c>
+      <c r="B16" s="72" t="inlineStr">
+        <is>
+          <t>SUSCRIPCIONES · IA</t>
+        </is>
+      </c>
+      <c r="C16" s="73" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="D16" s="74" t="n">
+        <v>30110</v>
+      </c>
+      <c r="E16" s="72" t="inlineStr">
+        <is>
+          <t>BBVA Mastercard · USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="71" t="n">
+        <v>46060</v>
+      </c>
+      <c r="B17" s="72" t="inlineStr">
+        <is>
+          <t>SUSCRIPCIONES · IA</t>
+        </is>
+      </c>
+      <c r="C17" s="73" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="D17" s="74" t="n">
+        <v>29193</v>
+      </c>
+      <c r="E17" s="72" t="inlineStr">
+        <is>
+          <t>BBVA Mastercard · USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="71" t="n">
+        <v>46088</v>
+      </c>
+      <c r="B18" s="72" t="inlineStr">
+        <is>
+          <t>SUSCRIPCIONES · IA</t>
+        </is>
+      </c>
+      <c r="C18" s="73" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="D18" s="74" t="n">
+        <v>28668</v>
+      </c>
+      <c r="E18" s="72" t="inlineStr">
+        <is>
+          <t>BBVA Mastercard · USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="71" t="n">
+        <v>46119</v>
+      </c>
+      <c r="B19" s="72" t="inlineStr">
+        <is>
+          <t>SUSCRIPCIONES · IA</t>
+        </is>
+      </c>
+      <c r="C19" s="73" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="D19" s="74" t="n">
+        <v>28667</v>
+      </c>
+      <c r="E19" s="72" t="inlineStr">
+        <is>
+          <t>BBVA Mastercard · USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="71" t="n">
+        <v>46057</v>
+      </c>
+      <c r="B20" s="72" t="inlineStr">
+        <is>
+          <t>SUSCRIPCIONES · IA</t>
+        </is>
+      </c>
+      <c r="C20" s="72" t="inlineStr">
+        <is>
+          <t>SUSCRIPCIONES · IA · ChatGPT / OpenAI · gasto personal Sol</t>
+        </is>
+      </c>
+      <c r="D20" s="74" t="n">
+        <v>29208</v>
+      </c>
+      <c r="E20" s="72" t="inlineStr">
+        <is>
+          <t>BBVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="71" t="n">
+        <v>46081</v>
+      </c>
+      <c r="B21" s="72" t="inlineStr">
+        <is>
+          <t>SUSCRIPCIONES · IA</t>
+        </is>
+      </c>
+      <c r="C21" s="72" t="inlineStr">
+        <is>
+          <t>SUSCRIPCIONES · IA · ChatGPT / OpenAI · gasto personal Sol</t>
+        </is>
+      </c>
+      <c r="D21" s="74" t="n">
+        <v>29208</v>
+      </c>
+      <c r="E21" s="72" t="inlineStr">
+        <is>
+          <t>BBVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="71" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B22" s="72" t="inlineStr">
+        <is>
+          <t>SUSCRIPCIONES · IA</t>
+        </is>
+      </c>
+      <c r="C22" s="72" t="inlineStr">
+        <is>
+          <t>SUSCRIPCIONES · IA · ChatGPT / OpenAI · gasto personal Sol</t>
+        </is>
+      </c>
+      <c r="D22" s="74" t="n">
+        <v>28681</v>
+      </c>
+      <c r="E22" s="72" t="inlineStr">
+        <is>
+          <t>BBVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="71" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B23" s="72" t="inlineStr">
+        <is>
+          <t>SUSCRIPCIONES · IA</t>
+        </is>
+      </c>
+      <c r="C23" s="72" t="inlineStr">
+        <is>
+          <t>SUSCRIPCIONES · IA · metricscheck.com · REVISAR · metricsche</t>
+        </is>
+      </c>
+      <c r="D23" s="74" t="n">
+        <v>29</v>
+      </c>
+      <c r="E23" s="72" t="inlineStr">
+        <is>
+          <t>BBVA MASTERCARD</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="71" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B24" s="72" t="inlineStr">
+        <is>
+          <t>SUSCRIPCIONES · IA</t>
+        </is>
+      </c>
+      <c r="C24" s="72" t="inlineStr">
+        <is>
+          <t>SUSCRIPCIONES · IA · metricscheck.com · REVISAR · metricsche</t>
+        </is>
+      </c>
+      <c r="D24" s="74" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="72" t="inlineStr">
+        <is>
+          <t>BBVA MASTERCARD</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A10:I10"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Categorizar Kelly (30/09) como Sol Estética en GPS
Las transferencias MP a Kelly de $20.000 y $86.000 quedan en Gasto Personal Sol
con categoría Sol Estética (ya no TRANSFERENCIAS REVISAR).

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -28961,7 +28961,7 @@
       </c>
       <c r="C942" t="inlineStr">
         <is>
-          <t>TRANSFERENCIAS</t>
+          <t>Sol Estética</t>
         </is>
       </c>
       <c r="D942" t="n">
@@ -28974,7 +28974,7 @@
       </c>
       <c r="F942" t="inlineStr">
         <is>
-          <t>TRANSFERENCIAS · Kelly · REVISAR ítem · resumen oficial cuenta MP 1–30 sep 2026</t>
+          <t>Sol Estética · Kelly · $20.000 · resumen oficial cuenta MP 1–30 sep 2026</t>
         </is>
       </c>
     </row>
@@ -28989,7 +28989,7 @@
       </c>
       <c r="C943" t="inlineStr">
         <is>
-          <t>TRANSFERENCIAS</t>
+          <t>Sol Estética</t>
         </is>
       </c>
       <c r="D943" t="n">
@@ -29002,7 +29002,7 @@
       </c>
       <c r="F943" t="inlineStr">
         <is>
-          <t>TRANSFERENCIAS · Kelly · REVISAR ítem · resumen oficial cuenta MP 1–30 sep 2026</t>
+          <t>Sol Estética · Kelly · $86.000 · resumen oficial cuenta MP 1–30 sep 2026</t>
         </is>
       </c>
     </row>
@@ -43872,7 +43872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I79"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -43900,7 +43900,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
@@ -43924,7 +43923,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="59" t="inlineStr">
         <is>
@@ -44340,7 +44338,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
@@ -44658,51 +44655,6 @@
         </is>
       </c>
     </row>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
Almacén: Café Illy ML $232.140 en agosto
Compra Mercado Libre (6×250gr) Mastercard ****7470; fecha comprobante 6/10,
asignada a mes Agosto por instrucción de Sol. Regenera maestro SOL.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -57624,6 +57624,7 @@
       </c>
       <c r="G176" s="22" t="n"/>
     </row>
+    <row r="177"/>
     <row r="178">
       <c r="A178" s="14" t="inlineStr">
         <is>
@@ -58906,6 +58907,7 @@
       </c>
       <c r="G228" s="22" t="n"/>
     </row>
+    <row r="229"/>
     <row r="230">
       <c r="A230" s="14" t="inlineStr">
         <is>
@@ -59944,6 +59946,7 @@
       </c>
       <c r="G273" s="22" t="n"/>
     </row>
+    <row r="274"/>
     <row r="275">
       <c r="A275" s="14" t="inlineStr">
         <is>
@@ -60711,21 +60714,34 @@
       </c>
       <c r="G312" s="22" t="n"/>
     </row>
+    <row r="313"/>
     <row r="314">
       <c r="A314" s="14" t="inlineStr">
         <is>
           <t>Agosto</t>
         </is>
       </c>
-      <c r="B314" s="17" t="n"/>
-      <c r="C314" s="14" t="n"/>
-      <c r="D314" s="27" t="n"/>
+      <c r="B314" s="17" t="n">
+        <v>46301</v>
+      </c>
+      <c r="C314" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · Café Illy</t>
+        </is>
+      </c>
+      <c r="D314" s="27" t="n">
+        <v>232140</v>
+      </c>
       <c r="E314" s="28" t="n"/>
       <c r="F314" s="15">
-        <f>IF(OR(D298&lt;&gt;"",E298&lt;&gt;""),IF(D298="",0,D298)+IF(E298="",0,E298),"")</f>
-        <v/>
-      </c>
-      <c r="G314" s="14" t="n"/>
+        <f>IF(OR(D314&lt;&gt;"",E314&lt;&gt;""),IF(D314="",0,D314)+IF(E314="",0,E314),"")</f>
+        <v/>
+      </c>
+      <c r="G314" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Libre · Café Illy Grano Espresso 6×250gr · Mastercard ****7470 · #2000015383852975 · mes Agosto (instrucción Sol)</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Almacén: Café Illy ML $232.140 con fecha 30/09
Mueve la compra a Septiembre (30/09/2026) según instrucción de Sol;
limpia el intento previo en Agosto. Regenera maestro SOL.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -60721,27 +60721,15 @@
           <t>Agosto</t>
         </is>
       </c>
-      <c r="B314" s="17" t="n">
-        <v>46301</v>
-      </c>
-      <c r="C314" s="14" t="inlineStr">
-        <is>
-          <t>COMIDA · Café Illy</t>
-        </is>
-      </c>
-      <c r="D314" s="27" t="n">
-        <v>232140</v>
-      </c>
+      <c r="B314" s="17" t="n"/>
+      <c r="C314" s="14" t="n"/>
+      <c r="D314" s="27" t="n"/>
       <c r="E314" s="28" t="n"/>
       <c r="F314" s="15">
         <f>IF(OR(D314&lt;&gt;"",E314&lt;&gt;""),IF(D314="",0,D314)+IF(E314="",0,E314),"")</f>
         <v/>
       </c>
-      <c r="G314" s="14" t="inlineStr">
-        <is>
-          <t>Mercado Libre · Café Illy Grano Espresso 6×250gr · Mastercard ****7470 · #2000015383852975 · mes Agosto (instrucción Sol)</t>
-        </is>
-      </c>
+      <c r="G314" s="14" t="n"/>
     </row>
     <row r="315">
       <c r="A315" s="14" t="inlineStr">
@@ -61393,6 +61381,7 @@
       </c>
       <c r="G354" s="22" t="n"/>
     </row>
+    <row r="355"/>
     <row r="356">
       <c r="A356" s="14" t="inlineStr">
         <is>
@@ -61427,15 +61416,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B357" s="17" t="n"/>
-      <c r="C357" s="14" t="n"/>
-      <c r="D357" s="27" t="n"/>
+      <c r="B357" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C357" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · Café Illy</t>
+        </is>
+      </c>
+      <c r="D357" s="27" t="n">
+        <v>232140</v>
+      </c>
       <c r="E357" s="28" t="n"/>
       <c r="F357" s="15">
-        <f>IF(OR(D341&lt;&gt;"",E341&lt;&gt;""),IF(D341="",0,D341)+IF(E341="",0,E341),"")</f>
-        <v/>
-      </c>
-      <c r="G357" s="14" t="n"/>
+        <f>IF(OR(D357&lt;&gt;"",E357&lt;&gt;""),IF(D357="",0,D357)+IF(E357="",0,E357),"")</f>
+        <v/>
+      </c>
+      <c r="G357" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Libre · Café Illy Grano Espresso 6×250gr · Mastercard ****7470 · #2000015383852975</t>
+        </is>
+      </c>
     </row>
     <row r="358">
       <c r="A358" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Almacén: mover Café Illy $232.140 a agosto
Reasigna la compra ML a mes Agosto (fecha 6/08) según instrucción de Sol.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -57624,7 +57624,6 @@
       </c>
       <c r="G176" s="22" t="n"/>
     </row>
-    <row r="177"/>
     <row r="178">
       <c r="A178" s="14" t="inlineStr">
         <is>
@@ -58907,7 +58906,6 @@
       </c>
       <c r="G228" s="22" t="n"/>
     </row>
-    <row r="229"/>
     <row r="230">
       <c r="A230" s="14" t="inlineStr">
         <is>
@@ -59946,7 +59944,6 @@
       </c>
       <c r="G273" s="22" t="n"/>
     </row>
-    <row r="274"/>
     <row r="275">
       <c r="A275" s="14" t="inlineStr">
         <is>
@@ -60714,22 +60711,33 @@
       </c>
       <c r="G312" s="22" t="n"/>
     </row>
-    <row r="313"/>
     <row r="314">
       <c r="A314" s="14" t="inlineStr">
         <is>
           <t>Agosto</t>
         </is>
       </c>
-      <c r="B314" s="17" t="n"/>
-      <c r="C314" s="14" t="n"/>
-      <c r="D314" s="27" t="n"/>
+      <c r="B314" s="17" t="n">
+        <v>46240</v>
+      </c>
+      <c r="C314" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · Café Illy</t>
+        </is>
+      </c>
+      <c r="D314" s="27" t="n">
+        <v>232140</v>
+      </c>
       <c r="E314" s="28" t="n"/>
       <c r="F314" s="15">
         <f>IF(OR(D314&lt;&gt;"",E314&lt;&gt;""),IF(D314="",0,D314)+IF(E314="",0,E314),"")</f>
         <v/>
       </c>
-      <c r="G314" s="14" t="n"/>
+      <c r="G314" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Libre · Café Illy Grano Espresso 6×250gr · Mastercard ****7470 · #2000015383852975</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" s="14" t="inlineStr">
@@ -61381,7 +61389,6 @@
       </c>
       <c r="G354" s="22" t="n"/>
     </row>
-    <row r="355"/>
     <row r="356">
       <c r="A356" s="14" t="inlineStr">
         <is>
@@ -61416,27 +61423,15 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B357" s="17" t="n">
-        <v>46295</v>
-      </c>
-      <c r="C357" s="14" t="inlineStr">
-        <is>
-          <t>COMIDA · Café Illy</t>
-        </is>
-      </c>
-      <c r="D357" s="27" t="n">
-        <v>232140</v>
-      </c>
+      <c r="B357" s="17" t="n"/>
+      <c r="C357" s="14" t="n"/>
+      <c r="D357" s="27" t="n"/>
       <c r="E357" s="28" t="n"/>
       <c r="F357" s="15">
         <f>IF(OR(D357&lt;&gt;"",E357&lt;&gt;""),IF(D357="",0,D357)+IF(E357="",0,E357),"")</f>
         <v/>
       </c>
-      <c r="G357" s="14" t="inlineStr">
-        <is>
-          <t>Mercado Libre · Café Illy Grano Espresso 6×250gr · Mastercard ****7470 · #2000015383852975</t>
-        </is>
-      </c>
+      <c r="G357" s="14" t="n"/>
     </row>
     <row r="358">
       <c r="A358" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Almacén: Café Illy $232.140 con fecha 30/09
Reasigna la compra ML a Septiembre 30/09/2026 según instrucción de Sol.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -57624,6 +57624,7 @@
       </c>
       <c r="G176" s="22" t="n"/>
     </row>
+    <row r="177"/>
     <row r="178">
       <c r="A178" s="14" t="inlineStr">
         <is>
@@ -58906,6 +58907,7 @@
       </c>
       <c r="G228" s="22" t="n"/>
     </row>
+    <row r="229"/>
     <row r="230">
       <c r="A230" s="14" t="inlineStr">
         <is>
@@ -59944,6 +59946,7 @@
       </c>
       <c r="G273" s="22" t="n"/>
     </row>
+    <row r="274"/>
     <row r="275">
       <c r="A275" s="14" t="inlineStr">
         <is>
@@ -60711,33 +60714,22 @@
       </c>
       <c r="G312" s="22" t="n"/>
     </row>
+    <row r="313"/>
     <row r="314">
       <c r="A314" s="14" t="inlineStr">
         <is>
           <t>Agosto</t>
         </is>
       </c>
-      <c r="B314" s="17" t="n">
-        <v>46240</v>
-      </c>
-      <c r="C314" s="14" t="inlineStr">
-        <is>
-          <t>COMIDA · Café Illy</t>
-        </is>
-      </c>
-      <c r="D314" s="27" t="n">
-        <v>232140</v>
-      </c>
+      <c r="B314" s="17" t="n"/>
+      <c r="C314" s="14" t="n"/>
+      <c r="D314" s="27" t="n"/>
       <c r="E314" s="28" t="n"/>
       <c r="F314" s="15">
         <f>IF(OR(D314&lt;&gt;"",E314&lt;&gt;""),IF(D314="",0,D314)+IF(E314="",0,E314),"")</f>
         <v/>
       </c>
-      <c r="G314" s="14" t="inlineStr">
-        <is>
-          <t>Mercado Libre · Café Illy Grano Espresso 6×250gr · Mastercard ****7470 · #2000015383852975</t>
-        </is>
-      </c>
+      <c r="G314" s="14" t="n"/>
     </row>
     <row r="315">
       <c r="A315" s="14" t="inlineStr">
@@ -61389,6 +61381,7 @@
       </c>
       <c r="G354" s="22" t="n"/>
     </row>
+    <row r="355"/>
     <row r="356">
       <c r="A356" s="14" t="inlineStr">
         <is>
@@ -61423,15 +61416,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B357" s="17" t="n"/>
-      <c r="C357" s="14" t="n"/>
-      <c r="D357" s="27" t="n"/>
+      <c r="B357" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C357" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · Café Illy</t>
+        </is>
+      </c>
+      <c r="D357" s="27" t="n">
+        <v>232140</v>
+      </c>
       <c r="E357" s="28" t="n"/>
       <c r="F357" s="15">
         <f>IF(OR(D357&lt;&gt;"",E357&lt;&gt;""),IF(D357="",0,D357)+IF(E357="",0,E357),"")</f>
         <v/>
       </c>
-      <c r="G357" s="14" t="n"/>
+      <c r="G357" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Libre · Café Illy Grano Espresso 6×250gr · Mastercard ****7470 · #2000015383852975</t>
+        </is>
+      </c>
     </row>
     <row r="358">
       <c r="A358" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Load Metrogas CIUDAD Oct 2026 from invoice (cobro 19/10, $106.267).
Cliente 30010996459 / medidor 40049923; mes = fecha de cobro, not consumption period.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -948,7 +948,9 @@
       <c r="L7" s="5" t="n">
         <v>105839</v>
       </c>
-      <c r="M7" s="5" t="n"/>
+      <c r="M7" s="5" t="n">
+        <v>106267</v>
+      </c>
       <c r="N7" s="5" t="n"/>
       <c r="O7" s="5" t="n"/>
       <c r="P7" s="7">
@@ -64530,7 +64532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I79"/>
+  <dimension ref="A1:I80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -66936,6 +66938,49 @@
       <c r="E79" t="inlineStr">
         <is>
           <t>BBVA Visa</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="52" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Metrogas</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Metrogas CIUDAD · cobro/venc. 19/10/2026 (fecha de cobro, no período consumo) · emisión 06/10/2026 · período 06/08–04/09/2026 · 395,24 m3 · débito automático</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>106267</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Débito automático BBVA Visa</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>30010996459</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>40049923</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Ciudad de la Paz 1132 1 A PTA: 34 · lectura real · Gmail factura 06/10/2026</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Octubre</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fill Metrogas gaps: CIUDAD Aug BBVA debits and OHIGGINS Aug–Oct invoices.
CIUDAD Agosto = two débitos (05/08 + 17/08); Julio sin cobro. OHIGGINS facturas by vencimiento (pago MP pendiente Ago–Oct).

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -944,7 +944,9 @@
         <v>30643</v>
       </c>
       <c r="J7" s="5" t="n"/>
-      <c r="K7" s="5" t="n"/>
+      <c r="K7" s="5" t="n">
+        <v>146882</v>
+      </c>
       <c r="L7" s="5" t="n">
         <v>105839</v>
       </c>
@@ -64532,7 +64534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I80"/>
+  <dimension ref="A1:I82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -66981,6 +66983,92 @@
       <c r="I80" t="inlineStr">
         <is>
           <t>Octubre</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="52" t="n">
+        <v>46239</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Metrogas</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Metrogas CIUDAD · cobro BBVA 05/08/2026 (fecha de cobro, no período consumo) · emisión 16/07 · período 08/05–05/06 · 259,13 m3</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>73695</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Débito automático BBVA Visa</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>30010996459</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>40049923</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>BBVA Compra aprobada 05/08 · ARS 73.694,19</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="52" t="n">
+        <v>46251</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Metrogas</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Metrogas CIUDAD · cobro BBVA 17/08/2026 (fecha de cobro, no período consumo) · emisión 05/08 · período 06/06–07/07 · 259,13 m3</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>73187</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Débito automático BBVA Visa</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>30010996459</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>40049923</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>BBVA Compra aprobada 17/08 · ARS 73.186,92</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Agosto</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Expensas CIUDAD septiembre $328.200 (pago MP 10-oct)
Carga período septiembre en matriz 2026, Detalle y Expensas Consorcios
(Consorcio De Propiet / Patagonia). Regenera maestro SOL.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -839,7 +839,9 @@
       </c>
       <c r="J5" s="5" t="n"/>
       <c r="K5" s="5" t="n"/>
-      <c r="L5" s="5" t="n"/>
+      <c r="L5" s="5" t="n">
+        <v>328200</v>
+      </c>
       <c r="M5" s="5" t="n"/>
       <c r="N5" s="5" t="n"/>
       <c r="O5" s="5" t="n"/>
@@ -1715,7 +1717,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>• Expensas: abr $235.210 (banco 7-abr → Consorcio De Propiet Patagonia); may/jun desde MP con período Gmail (pago jun=mayo, pago jul=junio). Julio período pendiente.</t>
+          <t>• Expensas: abr $235.210 (banco 7-abr → Consorcio De Propiet Patagonia); may/jun desde MP con período Gmail (pago jun=mayo, pago jul=junio); sept $328.200 (pago MP 10-oct → Consorcio De Propiet Patagonia). Julio/agosto período pendiente.</t>
         </is>
       </c>
     </row>
@@ -2682,13 +2684,37 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="17" t="n"/>
-      <c r="B44" s="14" t="n"/>
-      <c r="C44" s="14" t="n"/>
-      <c r="D44" s="14" t="n"/>
-      <c r="E44" s="15" t="n"/>
-      <c r="F44" s="14" t="n"/>
-      <c r="G44" s="14" t="n"/>
+      <c r="A44" s="17" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B44" s="14" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C44" s="14" t="inlineStr">
+        <is>
+          <t>Consorcio De Propiet</t>
+        </is>
+      </c>
+      <c r="D44" s="14" t="inlineStr">
+        <is>
+          <t>CIUDAD 1132</t>
+        </is>
+      </c>
+      <c r="E44" s="15" t="n">
+        <v>328200</v>
+      </c>
+      <c r="F44" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Transferencia enviada</t>
+        </is>
+      </c>
+      <c r="G44" s="14" t="inlineStr">
+        <is>
+          <t>Pago de Expensas · CIUDAD 1132 · Patagonia CBU 0340116900116010765007 / CUIL 30714962473 · período septiembre 2026 · pago MP 10-oct · op 183430766214</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="17" t="n"/>
@@ -57624,7 +57650,6 @@
       </c>
       <c r="G176" s="22" t="n"/>
     </row>
-    <row r="177"/>
     <row r="178">
       <c r="A178" s="14" t="inlineStr">
         <is>
@@ -58907,7 +58932,6 @@
       </c>
       <c r="G228" s="22" t="n"/>
     </row>
-    <row r="229"/>
     <row r="230">
       <c r="A230" s="14" t="inlineStr">
         <is>
@@ -59946,7 +59970,6 @@
       </c>
       <c r="G273" s="22" t="n"/>
     </row>
-    <row r="274"/>
     <row r="275">
       <c r="A275" s="14" t="inlineStr">
         <is>
@@ -60714,7 +60737,6 @@
       </c>
       <c r="G312" s="22" t="n"/>
     </row>
-    <row r="313"/>
     <row r="314">
       <c r="A314" s="14" t="inlineStr">
         <is>
@@ -61381,7 +61403,6 @@
       </c>
       <c r="G354" s="22" t="n"/>
     </row>
-    <row r="355"/>
     <row r="356">
       <c r="A356" s="14" t="inlineStr">
         <is>
@@ -66295,12 +66316,38 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="53" t="n"/>
-      <c r="B70" s="14" t="n"/>
-      <c r="C70" s="14" t="n"/>
-      <c r="D70" s="15" t="n"/>
-      <c r="E70" s="14" t="n"/>
+      <c r="A70" s="17" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B70" s="14" t="inlineStr">
+        <is>
+          <t>Expensas</t>
+        </is>
+      </c>
+      <c r="C70" s="14" t="inlineStr">
+        <is>
+          <t>Expensas — Septiembre 2026</t>
+        </is>
+      </c>
+      <c r="D70" s="15" t="n">
+        <v>328200</v>
+      </c>
+      <c r="E70" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Transferencia enviada</t>
+        </is>
+      </c>
       <c r="F70" s="18" t="n"/>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Consorcio de Propietarios · Pagado · período septiembre 2026 · pago 10-oct · op MP 183430766214 · CBU Patagonia 0340116900116010765007</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="53" t="n">

</xml_diff>

<commit_message>
Expensas OHIGGINS septiembre $722.978 (pago MP 10-oct)
Carga período septiembre (ceil desde $722.977,08) en Excel OHIGGINS
y espejo en Expensas Consorcios CIUDAD.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -2717,13 +2717,37 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="17" t="n"/>
-      <c r="B45" s="14" t="n"/>
-      <c r="C45" s="14" t="n"/>
-      <c r="D45" s="14" t="n"/>
-      <c r="E45" s="15" t="n"/>
-      <c r="F45" s="14" t="n"/>
-      <c r="G45" s="14" t="n"/>
+      <c r="A45" s="17" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B45" s="14" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C45" s="14" t="inlineStr">
+        <is>
+          <t>Consorcio De Copropietarios O Higgins 22</t>
+        </is>
+      </c>
+      <c r="D45" s="14" t="inlineStr">
+        <is>
+          <t>OHIGGINS</t>
+        </is>
+      </c>
+      <c r="E45" s="15" t="n">
+        <v>722978</v>
+      </c>
+      <c r="F45" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Transferencia enviada</t>
+        </is>
+      </c>
+      <c r="G45" s="14" t="inlineStr">
+        <is>
+          <t>Pago de Expensas · OHIGGINS 2219 piso 8 · período septiembre 2026 · pago MP 10-oct · Galicia CBU 0070692220000003412822 · CUIT 30-60701536-4 · op 183430574930 · ceil desde $722.977,08</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="17" t="n"/>

</xml_diff>

<commit_message>
Expensas sept: marcar MP dinero en cuenta en las 3 propiedades
Unifica medio de pago CIUDAD / OHIGGINS / BONORINO (período septiembre,
pago 10-oct) como Mercado Pago — Dinero en cuenta.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -2707,12 +2707,12 @@
       </c>
       <c r="F44" s="14" t="inlineStr">
         <is>
-          <t>Mercado Pago — Transferencia enviada</t>
+          <t>Mercado Pago — Dinero en cuenta</t>
         </is>
       </c>
       <c r="G44" s="14" t="inlineStr">
         <is>
-          <t>Pago de Expensas · CIUDAD 1132 · Patagonia CBU 0340116900116010765007 / CUIL 30714962473 · período septiembre 2026 · pago MP 10-oct · op 183430766214</t>
+          <t>Pago de Expensas · CIUDAD 1132 · Patagonia CBU 0340116900116010765007 / CUIL 30714962473 · período septiembre 2026 · pago MP 10-oct · op 183430766214 · MP dinero en cuenta</t>
         </is>
       </c>
     </row>
@@ -2740,12 +2740,12 @@
       </c>
       <c r="F45" s="14" t="inlineStr">
         <is>
-          <t>Mercado Pago — Transferencia enviada</t>
+          <t>Mercado Pago — Dinero en cuenta</t>
         </is>
       </c>
       <c r="G45" s="14" t="inlineStr">
         <is>
-          <t>Pago de Expensas · OHIGGINS 2219 piso 8 · período septiembre 2026 · pago MP 10-oct · Galicia CBU 0070692220000003412822 · CUIT 30-60701536-4 · op 183430574930 · ceil desde $722.977,08</t>
+          <t>Pago de Expensas · OHIGGINS 2219 piso 8 · período septiembre 2026 · pago MP 10-oct · Galicia CBU 0070692220000003412822 · CUIT 30-60701536-4 · op 183430574930 · ceil desde $722.977,08 · MP dinero en cuenta</t>
         </is>
       </c>
     </row>
@@ -2773,7 +2773,7 @@
       </c>
       <c r="F46" s="14" t="inlineStr">
         <is>
-          <t>Mercado Pago — Transferencia enviada</t>
+          <t>Mercado Pago — Dinero en cuenta</t>
         </is>
       </c>
       <c r="G46" s="14" t="inlineStr">
@@ -66382,13 +66382,13 @@
       </c>
       <c r="E70" s="14" t="inlineStr">
         <is>
-          <t>Mercado Pago — Transferencia enviada</t>
+          <t>Mercado Pago — Dinero en cuenta</t>
         </is>
       </c>
       <c r="F70" s="18" t="n"/>
       <c r="H70" t="inlineStr">
         <is>
-          <t>Consorcio de Propietarios · Pagado · período septiembre 2026 · pago 10-oct · op MP 183430766214 · CBU Patagonia 0340116900116010765007</t>
+          <t>Consorcio de Propietarios · Pagado · período septiembre 2026 · pago 10-oct · op MP 183430766214 · CBU Patagonia 0340116900116010765007 · MP dinero en cuenta</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">

</xml_diff>

<commit_message>
Load Chris September almacén line items into CIUDAD.
Add 23 Almacen Detalle rows (Importe Chris) for Coto, Día, verdulería, pollo, PedidosYa, vinos, plus unlabeled 48960 as REVISAR; fix Septiembre Total formulas on filled rows.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -61383,15 +61383,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B356" s="17" t="n"/>
-      <c r="C356" s="14" t="n"/>
+      <c r="B356" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C356" s="14" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Coto</t>
+        </is>
+      </c>
       <c r="D356" s="27" t="n"/>
-      <c r="E356" s="28" t="n"/>
+      <c r="E356" s="28" t="n">
+        <v>11436</v>
+      </c>
       <c r="F356" s="15">
-        <f>IF(OR(D340&lt;&gt;"",E340&lt;&gt;""),IF(D340="",0,D340)+IF(E340="",0,E340),"")</f>
-        <v/>
-      </c>
-      <c r="G356" s="14" t="n"/>
+        <f>IF(OR(D356&lt;&gt;"",E356&lt;&gt;""),IF(D356="",0,D356)+IF(E356="",0,E356),"")</f>
+        <v/>
+      </c>
+      <c r="G356" s="14" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Coto · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="357">
       <c r="A357" s="14" t="inlineStr">
@@ -61399,15 +61411,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B357" s="17" t="n"/>
-      <c r="C357" s="14" t="n"/>
+      <c r="B357" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C357" s="14" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Día</t>
+        </is>
+      </c>
       <c r="D357" s="27" t="n"/>
-      <c r="E357" s="28" t="n"/>
+      <c r="E357" s="28" t="n">
+        <v>7264</v>
+      </c>
       <c r="F357" s="15">
-        <f>IF(OR(D341&lt;&gt;"",E341&lt;&gt;""),IF(D341="",0,D341)+IF(E341="",0,E341),"")</f>
-        <v/>
-      </c>
-      <c r="G357" s="14" t="n"/>
+        <f>IF(OR(D357&lt;&gt;"",E357&lt;&gt;""),IF(D357="",0,D357)+IF(E357="",0,E357),"")</f>
+        <v/>
+      </c>
+      <c r="G357" s="14" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Día · SUPERDIA · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="358">
       <c r="A358" s="14" t="inlineStr">
@@ -61415,15 +61439,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B358" s="17" t="n"/>
-      <c r="C358" s="14" t="n"/>
+      <c r="B358" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C358" s="14" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Coto</t>
+        </is>
+      </c>
       <c r="D358" s="27" t="n"/>
-      <c r="E358" s="28" t="n"/>
+      <c r="E358" s="28" t="n">
+        <v>10000</v>
+      </c>
       <c r="F358" s="15">
-        <f>IF(OR(D342&lt;&gt;"",E342&lt;&gt;""),IF(D342="",0,D342)+IF(E342="",0,E342),"")</f>
-        <v/>
-      </c>
-      <c r="G358" s="14" t="n"/>
+        <f>IF(OR(D358&lt;&gt;"",E358&lt;&gt;""),IF(D358="",0,D358)+IF(E358="",0,E358),"")</f>
+        <v/>
+      </c>
+      <c r="G358" s="14" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Coto · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="359">
       <c r="A359" s="14" t="inlineStr">
@@ -61431,15 +61467,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B359" s="17" t="n"/>
-      <c r="C359" s="14" t="n"/>
+      <c r="B359" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C359" s="14" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Coto</t>
+        </is>
+      </c>
       <c r="D359" s="27" t="n"/>
-      <c r="E359" s="28" t="n"/>
+      <c r="E359" s="28" t="n">
+        <v>11993</v>
+      </c>
       <c r="F359" s="15">
-        <f>IF(OR(D343&lt;&gt;"",E343&lt;&gt;""),IF(D343="",0,D343)+IF(E343="",0,E343),"")</f>
-        <v/>
-      </c>
-      <c r="G359" s="14" t="n"/>
+        <f>IF(OR(D359&lt;&gt;"",E359&lt;&gt;""),IF(D359="",0,D359)+IF(E359="",0,E359),"")</f>
+        <v/>
+      </c>
+      <c r="G359" s="14" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Coto · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="360">
       <c r="A360" s="14" t="inlineStr">
@@ -61447,15 +61495,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B360" s="17" t="n"/>
-      <c r="C360" s="14" t="n"/>
+      <c r="B360" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C360" s="14" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Día</t>
+        </is>
+      </c>
       <c r="D360" s="27" t="n"/>
-      <c r="E360" s="28" t="n"/>
+      <c r="E360" s="28" t="n">
+        <v>9980</v>
+      </c>
       <c r="F360" s="15">
-        <f>IF(OR(D344&lt;&gt;"",E344&lt;&gt;""),IF(D344="",0,D344)+IF(E344="",0,E344),"")</f>
-        <v/>
-      </c>
-      <c r="G360" s="14" t="n"/>
+        <f>IF(OR(D360&lt;&gt;"",E360&lt;&gt;""),IF(D360="",0,D360)+IF(E360="",0,E360),"")</f>
+        <v/>
+      </c>
+      <c r="G360" s="14" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Día · SUPERDIA · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="361">
       <c r="A361" s="14" t="inlineStr">
@@ -61463,15 +61523,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B361" s="17" t="n"/>
-      <c r="C361" s="14" t="n"/>
+      <c r="B361" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C361" s="14" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Día</t>
+        </is>
+      </c>
       <c r="D361" s="27" t="n"/>
-      <c r="E361" s="28" t="n"/>
+      <c r="E361" s="28" t="n">
+        <v>4152</v>
+      </c>
       <c r="F361" s="15">
-        <f>IF(OR(D345&lt;&gt;"",E345&lt;&gt;""),IF(D345="",0,D345)+IF(E345="",0,E345),"")</f>
-        <v/>
-      </c>
-      <c r="G361" s="14" t="n"/>
+        <f>IF(OR(D361&lt;&gt;"",E361&lt;&gt;""),IF(D361="",0,D361)+IF(E361="",0,E361),"")</f>
+        <v/>
+      </c>
+      <c r="G361" s="14" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Día · SUPERDIA · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="362">
       <c r="A362" s="14" t="inlineStr">
@@ -61479,15 +61551,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B362" s="17" t="n"/>
-      <c r="C362" s="14" t="n"/>
+      <c r="B362" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C362" s="14" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Día</t>
+        </is>
+      </c>
       <c r="D362" s="27" t="n"/>
-      <c r="E362" s="28" t="n"/>
+      <c r="E362" s="28" t="n">
+        <v>7488</v>
+      </c>
       <c r="F362" s="15">
-        <f>IF(OR(D346&lt;&gt;"",E346&lt;&gt;""),IF(D346="",0,D346)+IF(E346="",0,E346),"")</f>
-        <v/>
-      </c>
-      <c r="G362" s="14" t="n"/>
+        <f>IF(OR(D362&lt;&gt;"",E362&lt;&gt;""),IF(D362="",0,D362)+IF(E362="",0,E362),"")</f>
+        <v/>
+      </c>
+      <c r="G362" s="14" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Día · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="363">
       <c r="A363" s="14" t="inlineStr">
@@ -61495,15 +61579,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B363" s="17" t="n"/>
-      <c r="C363" s="14" t="n"/>
+      <c r="B363" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C363" s="14" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Coto</t>
+        </is>
+      </c>
       <c r="D363" s="27" t="n"/>
-      <c r="E363" s="28" t="n"/>
+      <c r="E363" s="28" t="n">
+        <v>1999</v>
+      </c>
       <c r="F363" s="15">
-        <f>IF(OR(D347&lt;&gt;"",E347&lt;&gt;""),IF(D347="",0,D347)+IF(E347="",0,E347),"")</f>
-        <v/>
-      </c>
-      <c r="G363" s="14" t="n"/>
+        <f>IF(OR(D363&lt;&gt;"",E363&lt;&gt;""),IF(D363="",0,D363)+IF(E363="",0,E363),"")</f>
+        <v/>
+      </c>
+      <c r="G363" s="14" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Coto · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="364">
       <c r="A364" s="14" t="inlineStr">
@@ -61511,15 +61607,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B364" s="17" t="n"/>
-      <c r="C364" s="14" t="n"/>
+      <c r="B364" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C364" s="14" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Día</t>
+        </is>
+      </c>
       <c r="D364" s="27" t="n"/>
-      <c r="E364" s="28" t="n"/>
+      <c r="E364" s="28" t="n">
+        <v>5680</v>
+      </c>
       <c r="F364" s="15">
-        <f>IF(OR(D348&lt;&gt;"",E348&lt;&gt;""),IF(D348="",0,D348)+IF(E348="",0,E348),"")</f>
-        <v/>
-      </c>
-      <c r="G364" s="14" t="n"/>
+        <f>IF(OR(D364&lt;&gt;"",E364&lt;&gt;""),IF(D364="",0,D364)+IF(E364="",0,E364),"")</f>
+        <v/>
+      </c>
+      <c r="G364" s="14" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Día · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="365">
       <c r="A365" s="14" t="inlineStr">
@@ -61527,15 +61635,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B365" s="17" t="n"/>
-      <c r="C365" s="14" t="n"/>
+      <c r="B365" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C365" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · VERDULERÍA</t>
+        </is>
+      </c>
       <c r="D365" s="27" t="n"/>
-      <c r="E365" s="28" t="n"/>
+      <c r="E365" s="28" t="n">
+        <v>4101</v>
+      </c>
       <c r="F365" s="15">
-        <f>IF(OR(D349&lt;&gt;"",E349&lt;&gt;""),IF(D349="",0,D349)+IF(E349="",0,E349),"")</f>
-        <v/>
-      </c>
-      <c r="G365" s="14" t="n"/>
+        <f>IF(OR(D365&lt;&gt;"",E365&lt;&gt;""),IF(D365="",0,D365)+IF(E365="",0,E365),"")</f>
+        <v/>
+      </c>
+      <c r="G365" s="14" t="inlineStr">
+        <is>
+          <t>Chris · COMIDA · VERDULERÍA · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="366">
       <c r="A366" s="14" t="inlineStr">
@@ -61543,15 +61663,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B366" s="17" t="n"/>
-      <c r="C366" s="14" t="n"/>
+      <c r="B366" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C366" s="14" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Coto</t>
+        </is>
+      </c>
       <c r="D366" s="27" t="n"/>
-      <c r="E366" s="28" t="n"/>
+      <c r="E366" s="28" t="n">
+        <v>7610</v>
+      </c>
       <c r="F366" s="15">
-        <f>IF(OR(D350&lt;&gt;"",E350&lt;&gt;""),IF(D350="",0,D350)+IF(E350="",0,E350),"")</f>
-        <v/>
-      </c>
-      <c r="G366" s="14" t="n"/>
+        <f>IF(OR(D366&lt;&gt;"",E366&lt;&gt;""),IF(D366="",0,D366)+IF(E366="",0,E366),"")</f>
+        <v/>
+      </c>
+      <c r="G366" s="14" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Coto · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="367">
       <c r="A367" s="14" t="inlineStr">
@@ -61559,15 +61691,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B367" s="17" t="n"/>
-      <c r="C367" s="14" t="n"/>
+      <c r="B367" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C367" s="14" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Día</t>
+        </is>
+      </c>
       <c r="D367" s="27" t="n"/>
-      <c r="E367" s="28" t="n"/>
+      <c r="E367" s="28" t="n">
+        <v>4796</v>
+      </c>
       <c r="F367" s="15">
-        <f>IF(OR(D351&lt;&gt;"",E351&lt;&gt;""),IF(D351="",0,D351)+IF(E351="",0,E351),"")</f>
-        <v/>
-      </c>
-      <c r="G367" s="14" t="n"/>
+        <f>IF(OR(D367&lt;&gt;"",E367&lt;&gt;""),IF(D367="",0,D367)+IF(E367="",0,E367),"")</f>
+        <v/>
+      </c>
+      <c r="G367" s="14" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Día · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="368">
       <c r="A368" s="14" t="inlineStr">
@@ -61575,15 +61719,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B368" s="17" t="n"/>
-      <c r="C368" s="14" t="n"/>
+      <c r="B368" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C368" s="14" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Día</t>
+        </is>
+      </c>
       <c r="D368" s="27" t="n"/>
-      <c r="E368" s="28" t="n"/>
+      <c r="E368" s="28" t="n">
+        <v>3952</v>
+      </c>
       <c r="F368" s="15">
-        <f>IF(OR(D352&lt;&gt;"",E352&lt;&gt;""),IF(D352="",0,D352)+IF(E352="",0,E352),"")</f>
-        <v/>
-      </c>
-      <c r="G368" s="14" t="n"/>
+        <f>IF(OR(D368&lt;&gt;"",E368&lt;&gt;""),IF(D368="",0,D368)+IF(E368="",0,E368),"")</f>
+        <v/>
+      </c>
+      <c r="G368" s="14" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Día · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="369">
       <c r="A369" s="14" t="inlineStr">
@@ -61591,15 +61747,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B369" s="17" t="n"/>
-      <c r="C369" s="14" t="n"/>
+      <c r="B369" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C369" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · pollo</t>
+        </is>
+      </c>
       <c r="D369" s="27" t="n"/>
-      <c r="E369" s="28" t="n"/>
+      <c r="E369" s="28" t="n">
+        <v>10295</v>
+      </c>
       <c r="F369" s="15">
-        <f>IF(OR(D353&lt;&gt;"",E353&lt;&gt;""),IF(D353="",0,D353)+IF(E353="",0,E353),"")</f>
-        <v/>
-      </c>
-      <c r="G369" s="14" t="n"/>
+        <f>IF(OR(D369&lt;&gt;"",E369&lt;&gt;""),IF(D369="",0,D369)+IF(E369="",0,E369),"")</f>
+        <v/>
+      </c>
+      <c r="G369" s="14" t="inlineStr">
+        <is>
+          <t>Chris · COMIDA · pollo · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="370">
       <c r="A370" s="14" t="inlineStr">
@@ -61607,15 +61775,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B370" s="17" t="n"/>
-      <c r="C370" s="14" t="n"/>
+      <c r="B370" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C370" s="14" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Día</t>
+        </is>
+      </c>
       <c r="D370" s="27" t="n"/>
-      <c r="E370" s="28" t="n"/>
+      <c r="E370" s="28" t="n">
+        <v>6480</v>
+      </c>
       <c r="F370" s="15">
-        <f>IF(OR(D354&lt;&gt;"",E354&lt;&gt;""),IF(D354="",0,D354)+IF(E354="",0,E354),"")</f>
-        <v/>
-      </c>
-      <c r="G370" s="14" t="n"/>
+        <f>IF(OR(D370&lt;&gt;"",E370&lt;&gt;""),IF(D370="",0,D370)+IF(E370="",0,E370),"")</f>
+        <v/>
+      </c>
+      <c r="G370" s="14" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Día · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="371">
       <c r="A371" s="14" t="inlineStr">
@@ -61623,15 +61803,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B371" s="17" t="n"/>
-      <c r="C371" s="14" t="n"/>
+      <c r="B371" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C371" s="14" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Día</t>
+        </is>
+      </c>
       <c r="D371" s="27" t="n"/>
-      <c r="E371" s="28" t="n"/>
+      <c r="E371" s="28" t="n">
+        <v>4739</v>
+      </c>
       <c r="F371" s="15">
-        <f>IF(OR(D355&lt;&gt;"",E355&lt;&gt;""),IF(D355="",0,D355)+IF(E355="",0,E355),"")</f>
-        <v/>
-      </c>
-      <c r="G371" s="14" t="n"/>
+        <f>IF(OR(D371&lt;&gt;"",E371&lt;&gt;""),IF(D371="",0,D371)+IF(E371="",0,E371),"")</f>
+        <v/>
+      </c>
+      <c r="G371" s="14" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Día · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="372">
       <c r="A372" s="14" t="inlineStr">
@@ -61639,15 +61831,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B372" s="17" t="n"/>
-      <c r="C372" s="14" t="n"/>
+      <c r="B372" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C372" s="14" t="inlineStr">
+        <is>
+          <t>PEDIDOS YA · COMIDA</t>
+        </is>
+      </c>
       <c r="D372" s="27" t="n"/>
-      <c r="E372" s="28" t="n"/>
+      <c r="E372" s="28" t="n">
+        <v>23424</v>
+      </c>
       <c r="F372" s="15">
-        <f>IF(OR(D356&lt;&gt;"",E356&lt;&gt;""),IF(D356="",0,D356)+IF(E356="",0,E356),"")</f>
-        <v/>
-      </c>
-      <c r="G372" s="14" t="n"/>
+        <f>IF(OR(D372&lt;&gt;"",E372&lt;&gt;""),IF(D372="",0,D372)+IF(E372="",0,E372),"")</f>
+        <v/>
+      </c>
+      <c r="G372" s="14" t="inlineStr">
+        <is>
+          <t>Chris · PEDIDOS YA · COMIDA · sin fecha día · REVISAR · confirmar si Market</t>
+        </is>
+      </c>
     </row>
     <row r="373">
       <c r="A373" s="14" t="inlineStr">
@@ -61655,15 +61859,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B373" s="17" t="n"/>
-      <c r="C373" s="14" t="n"/>
+      <c r="B373" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C373" s="14" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Día</t>
+        </is>
+      </c>
       <c r="D373" s="27" t="n"/>
-      <c r="E373" s="28" t="n"/>
+      <c r="E373" s="28" t="n">
+        <v>7439</v>
+      </c>
       <c r="F373" s="15">
-        <f>IF(OR(D357&lt;&gt;"",E357&lt;&gt;""),IF(D357="",0,D357)+IF(E357="",0,E357),"")</f>
-        <v/>
-      </c>
-      <c r="G373" s="14" t="n"/>
+        <f>IF(OR(D373&lt;&gt;"",E373&lt;&gt;""),IF(D373="",0,D373)+IF(E373="",0,E373),"")</f>
+        <v/>
+      </c>
+      <c r="G373" s="14" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Día · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="374">
       <c r="A374" s="14" t="inlineStr">
@@ -61671,15 +61887,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B374" s="17" t="n"/>
-      <c r="C374" s="14" t="n"/>
+      <c r="B374" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C374" s="14" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Día</t>
+        </is>
+      </c>
       <c r="D374" s="27" t="n"/>
-      <c r="E374" s="28" t="n"/>
+      <c r="E374" s="28" t="n">
+        <v>5716</v>
+      </c>
       <c r="F374" s="15">
-        <f>IF(OR(D358&lt;&gt;"",E358&lt;&gt;""),IF(D358="",0,D358)+IF(E358="",0,E358),"")</f>
-        <v/>
-      </c>
-      <c r="G374" s="14" t="n"/>
+        <f>IF(OR(D374&lt;&gt;"",E374&lt;&gt;""),IF(D374="",0,D374)+IF(E374="",0,E374),"")</f>
+        <v/>
+      </c>
+      <c r="G374" s="14" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Día · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="375">
       <c r="A375" s="14" t="inlineStr">
@@ -61687,15 +61915,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B375" s="17" t="n"/>
-      <c r="C375" s="14" t="n"/>
+      <c r="B375" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C375" s="14" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Día</t>
+        </is>
+      </c>
       <c r="D375" s="27" t="n"/>
-      <c r="E375" s="28" t="n"/>
+      <c r="E375" s="28" t="n">
+        <v>3768</v>
+      </c>
       <c r="F375" s="15">
-        <f>IF(OR(D359&lt;&gt;"",E359&lt;&gt;""),IF(D359="",0,D359)+IF(E359="",0,E359),"")</f>
-        <v/>
-      </c>
-      <c r="G375" s="14" t="n"/>
+        <f>IF(OR(D375&lt;&gt;"",E375&lt;&gt;""),IF(D375="",0,D375)+IF(E375="",0,E375),"")</f>
+        <v/>
+      </c>
+      <c r="G375" s="14" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Día · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="376">
       <c r="A376" s="14" t="inlineStr">
@@ -61703,15 +61943,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B376" s="17" t="n"/>
-      <c r="C376" s="14" t="n"/>
+      <c r="B376" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C376" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · Vinos</t>
+        </is>
+      </c>
       <c r="D376" s="27" t="n"/>
-      <c r="E376" s="28" t="n"/>
+      <c r="E376" s="28" t="n">
+        <v>17780</v>
+      </c>
       <c r="F376" s="15">
-        <f>IF(OR(D360&lt;&gt;"",E360&lt;&gt;""),IF(D360="",0,D360)+IF(E360="",0,E360),"")</f>
-        <v/>
-      </c>
-      <c r="G376" s="14" t="n"/>
+        <f>IF(OR(D376&lt;&gt;"",E376&lt;&gt;""),IF(D376="",0,D376)+IF(E376="",0,E376),"")</f>
+        <v/>
+      </c>
+      <c r="G376" s="14" t="inlineStr">
+        <is>
+          <t>Chris · COMIDA · Vinos · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="377">
       <c r="A377" s="14" t="inlineStr">
@@ -61719,15 +61971,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B377" s="17" t="n"/>
-      <c r="C377" s="14" t="n"/>
+      <c r="B377" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C377" s="14" t="inlineStr">
+        <is>
+          <t>REVISAR · sin comercio</t>
+        </is>
+      </c>
       <c r="D377" s="27" t="n"/>
-      <c r="E377" s="28" t="n"/>
+      <c r="E377" s="28" t="n">
+        <v>48960</v>
+      </c>
       <c r="F377" s="15">
-        <f>IF(OR(D361&lt;&gt;"",E361&lt;&gt;""),IF(D361="",0,D361)+IF(E361="",0,E361),"")</f>
-        <v/>
-      </c>
-      <c r="G377" s="14" t="n"/>
+        <f>IF(OR(D377&lt;&gt;"",E377&lt;&gt;""),IF(D377="",0,D377)+IF(E377="",0,E377),"")</f>
+        <v/>
+      </c>
+      <c r="G377" s="14" t="inlineStr">
+        <is>
+          <t>Chris · REVISAR · monto sin comercio en listado · sin fecha día</t>
+        </is>
+      </c>
     </row>
     <row r="378">
       <c r="A378" s="14" t="inlineStr">
@@ -61735,15 +61999,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B378" s="17" t="n"/>
-      <c r="C378" s="14" t="n"/>
+      <c r="B378" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C378" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · VERDULERÍA</t>
+        </is>
+      </c>
       <c r="D378" s="27" t="n"/>
-      <c r="E378" s="28" t="n"/>
+      <c r="E378" s="28" t="n">
+        <v>7912</v>
+      </c>
       <c r="F378" s="15">
-        <f>IF(OR(D362&lt;&gt;"",E362&lt;&gt;""),IF(D362="",0,D362)+IF(E362="",0,E362),"")</f>
-        <v/>
-      </c>
-      <c r="G378" s="14" t="n"/>
+        <f>IF(OR(D378&lt;&gt;"",E378&lt;&gt;""),IF(D378="",0,D378)+IF(E378="",0,E378),"")</f>
+        <v/>
+      </c>
+      <c r="G378" s="14" t="inlineStr">
+        <is>
+          <t>Chris · COMIDA · VERDULERÍA · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="379">
       <c r="A379" s="14" t="inlineStr">
@@ -61756,7 +62032,7 @@
       <c r="D379" s="27" t="n"/>
       <c r="E379" s="28" t="n"/>
       <c r="F379" s="15">
-        <f>IF(OR(D363&lt;&gt;"",E363&lt;&gt;""),IF(D363="",0,D363)+IF(E363="",0,E363),"")</f>
+        <f>IF(OR(D379&lt;&gt;"",E379&lt;&gt;""),IF(D379="",0,D379)+IF(E379="",0,E379),"")</f>
         <v/>
       </c>
       <c r="G379" s="14" t="n"/>
@@ -61772,7 +62048,7 @@
       <c r="D380" s="27" t="n"/>
       <c r="E380" s="28" t="n"/>
       <c r="F380" s="15">
-        <f>IF(OR(D364&lt;&gt;"",E364&lt;&gt;""),IF(D364="",0,D364)+IF(E364="",0,E364),"")</f>
+        <f>IF(OR(D380&lt;&gt;"",E380&lt;&gt;""),IF(D380="",0,D380)+IF(E380="",0,E380),"")</f>
         <v/>
       </c>
       <c r="G380" s="14" t="n"/>
@@ -61788,7 +62064,7 @@
       <c r="D381" s="27" t="n"/>
       <c r="E381" s="28" t="n"/>
       <c r="F381" s="15">
-        <f>IF(OR(D365&lt;&gt;"",E365&lt;&gt;""),IF(D365="",0,D365)+IF(E365="",0,E365),"")</f>
+        <f>IF(OR(D381&lt;&gt;"",E381&lt;&gt;""),IF(D381="",0,D381)+IF(E381="",0,E381),"")</f>
         <v/>
       </c>
       <c r="G381" s="14" t="n"/>
@@ -61804,7 +62080,7 @@
       <c r="D382" s="27" t="n"/>
       <c r="E382" s="28" t="n"/>
       <c r="F382" s="15">
-        <f>IF(OR(D366&lt;&gt;"",E366&lt;&gt;""),IF(D366="",0,D366)+IF(E366="",0,E366),"")</f>
+        <f>IF(OR(D382&lt;&gt;"",E382&lt;&gt;""),IF(D382="",0,D382)+IF(E382="",0,E382),"")</f>
         <v/>
       </c>
       <c r="G382" s="14" t="n"/>
@@ -61820,7 +62096,7 @@
       <c r="D383" s="27" t="n"/>
       <c r="E383" s="28" t="n"/>
       <c r="F383" s="15">
-        <f>IF(OR(D367&lt;&gt;"",E367&lt;&gt;""),IF(D367="",0,D367)+IF(E367="",0,E367),"")</f>
+        <f>IF(OR(D383&lt;&gt;"",E383&lt;&gt;""),IF(D383="",0,D383)+IF(E383="",0,E383),"")</f>
         <v/>
       </c>
       <c r="G383" s="14" t="n"/>
@@ -61836,7 +62112,7 @@
       <c r="D384" s="27" t="n"/>
       <c r="E384" s="28" t="n"/>
       <c r="F384" s="15">
-        <f>IF(OR(D368&lt;&gt;"",E368&lt;&gt;""),IF(D368="",0,D368)+IF(E368="",0,E368),"")</f>
+        <f>IF(OR(D384&lt;&gt;"",E384&lt;&gt;""),IF(D384="",0,D384)+IF(E384="",0,E384),"")</f>
         <v/>
       </c>
       <c r="G384" s="14" t="n"/>
@@ -61852,7 +62128,7 @@
       <c r="D385" s="27" t="n"/>
       <c r="E385" s="28" t="n"/>
       <c r="F385" s="15">
-        <f>IF(OR(D369&lt;&gt;"",E369&lt;&gt;""),IF(D369="",0,D369)+IF(E369="",0,E369),"")</f>
+        <f>IF(OR(D385&lt;&gt;"",E385&lt;&gt;""),IF(D385="",0,D385)+IF(E385="",0,E385),"")</f>
         <v/>
       </c>
       <c r="G385" s="14" t="n"/>
@@ -61868,7 +62144,7 @@
       <c r="D386" s="27" t="n"/>
       <c r="E386" s="28" t="n"/>
       <c r="F386" s="15">
-        <f>IF(OR(D370&lt;&gt;"",E370&lt;&gt;""),IF(D370="",0,D370)+IF(E370="",0,E370),"")</f>
+        <f>IF(OR(D386&lt;&gt;"",E386&lt;&gt;""),IF(D386="",0,D386)+IF(E386="",0,E386),"")</f>
         <v/>
       </c>
       <c r="G386" s="14" t="n"/>
@@ -61884,7 +62160,7 @@
       <c r="D387" s="27" t="n"/>
       <c r="E387" s="28" t="n"/>
       <c r="F387" s="15">
-        <f>IF(OR(D371&lt;&gt;"",E371&lt;&gt;""),IF(D371="",0,D371)+IF(E371="",0,E371),"")</f>
+        <f>IF(OR(D387&lt;&gt;"",E387&lt;&gt;""),IF(D387="",0,D387)+IF(E387="",0,E387),"")</f>
         <v/>
       </c>
       <c r="G387" s="14" t="n"/>
@@ -61900,7 +62176,7 @@
       <c r="D388" s="27" t="n"/>
       <c r="E388" s="28" t="n"/>
       <c r="F388" s="15">
-        <f>IF(OR(D372&lt;&gt;"",E372&lt;&gt;""),IF(D372="",0,D372)+IF(E372="",0,E372),"")</f>
+        <f>IF(OR(D388&lt;&gt;"",E388&lt;&gt;""),IF(D388="",0,D388)+IF(E388="",0,E388),"")</f>
         <v/>
       </c>
       <c r="G388" s="14" t="n"/>
@@ -61916,7 +62192,7 @@
       <c r="D389" s="27" t="n"/>
       <c r="E389" s="28" t="n"/>
       <c r="F389" s="15">
-        <f>IF(OR(D373&lt;&gt;"",E373&lt;&gt;""),IF(D373="",0,D373)+IF(E373="",0,E373),"")</f>
+        <f>IF(OR(D389&lt;&gt;"",E389&lt;&gt;""),IF(D389="",0,D389)+IF(E389="",0,E389),"")</f>
         <v/>
       </c>
       <c r="G389" s="14" t="n"/>
@@ -61932,7 +62208,7 @@
       <c r="D390" s="27" t="n"/>
       <c r="E390" s="28" t="n"/>
       <c r="F390" s="15">
-        <f>IF(OR(D374&lt;&gt;"",E374&lt;&gt;""),IF(D374="",0,D374)+IF(E374="",0,E374),"")</f>
+        <f>IF(OR(D390&lt;&gt;"",E390&lt;&gt;""),IF(D390="",0,D390)+IF(E390="",0,E390),"")</f>
         <v/>
       </c>
       <c r="G390" s="14" t="n"/>
@@ -61948,7 +62224,7 @@
       <c r="D391" s="27" t="n"/>
       <c r="E391" s="28" t="n"/>
       <c r="F391" s="15">
-        <f>IF(OR(D375&lt;&gt;"",E375&lt;&gt;""),IF(D375="",0,D375)+IF(E375="",0,E375),"")</f>
+        <f>IF(OR(D391&lt;&gt;"",E391&lt;&gt;""),IF(D391="",0,D391)+IF(E391="",0,E391),"")</f>
         <v/>
       </c>
       <c r="G391" s="14" t="n"/>
@@ -61964,7 +62240,7 @@
       <c r="D392" s="27" t="n"/>
       <c r="E392" s="28" t="n"/>
       <c r="F392" s="15">
-        <f>IF(OR(D376&lt;&gt;"",E376&lt;&gt;""),IF(D376="",0,D376)+IF(E376="",0,E376),"")</f>
+        <f>IF(OR(D392&lt;&gt;"",E392&lt;&gt;""),IF(D392="",0,D392)+IF(E392="",0,E392),"")</f>
         <v/>
       </c>
       <c r="G392" s="14" t="n"/>
@@ -61980,7 +62256,7 @@
       <c r="D393" s="27" t="n"/>
       <c r="E393" s="28" t="n"/>
       <c r="F393" s="15">
-        <f>IF(OR(D377&lt;&gt;"",E377&lt;&gt;""),IF(D377="",0,D377)+IF(E377="",0,E377),"")</f>
+        <f>IF(OR(D393&lt;&gt;"",E393&lt;&gt;""),IF(D393="",0,D393)+IF(E393="",0,E393),"")</f>
         <v/>
       </c>
       <c r="G393" s="14" t="n"/>
@@ -61996,7 +62272,7 @@
       <c r="D394" s="27" t="n"/>
       <c r="E394" s="28" t="n"/>
       <c r="F394" s="15">
-        <f>IF(OR(D378&lt;&gt;"",E378&lt;&gt;""),IF(D378="",0,D378)+IF(E378="",0,E378),"")</f>
+        <f>IF(OR(D394&lt;&gt;"",E394&lt;&gt;""),IF(D394="",0,D394)+IF(E394="",0,E394),"")</f>
         <v/>
       </c>
       <c r="G394" s="14" t="n"/>
@@ -62012,7 +62288,7 @@
       <c r="D395" s="27" t="n"/>
       <c r="E395" s="28" t="n"/>
       <c r="F395" s="15">
-        <f>IF(OR(D379&lt;&gt;"",E379&lt;&gt;""),IF(D379="",0,D379)+IF(E379="",0,E379),"")</f>
+        <f>IF(OR(D395&lt;&gt;"",E395&lt;&gt;""),IF(D395="",0,D395)+IF(E395="",0,E395),"")</f>
         <v/>
       </c>
       <c r="G395" s="14" t="n"/>

</xml_diff>

<commit_message>
Load Sol Café Illy October almacén expense ($232,140).
Add COMIDA · Café Illy to Almacen Detalle (Importe Sol, Octubre) and regenerate SOL master.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -62049,15 +62049,27 @@
           <t>Octubre</t>
         </is>
       </c>
-      <c r="B398" s="17" t="n"/>
-      <c r="C398" s="14" t="n"/>
-      <c r="D398" s="27" t="n"/>
+      <c r="B398" s="17" t="n">
+        <v>46326</v>
+      </c>
+      <c r="C398" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · Café Illy</t>
+        </is>
+      </c>
+      <c r="D398" s="27" t="n">
+        <v>232140</v>
+      </c>
       <c r="E398" s="28" t="n"/>
       <c r="F398" s="15">
-        <f>IF(OR(D382&lt;&gt;"",E382&lt;&gt;""),IF(D382="",0,D382)+IF(E382="",0,E382),"")</f>
-        <v/>
-      </c>
-      <c r="G398" s="14" t="n"/>
+        <f>IF(OR(D398&lt;&gt;"",E398&lt;&gt;""),IF(D398="",0,D398)+IF(E398="",0,E398),"")</f>
+        <v/>
+      </c>
+      <c r="G398" s="14" t="inlineStr">
+        <is>
+          <t>Sol · COMIDA · Café Illy · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="399">
       <c r="A399" s="14" t="inlineStr">
@@ -62070,7 +62082,7 @@
       <c r="D399" s="27" t="n"/>
       <c r="E399" s="28" t="n"/>
       <c r="F399" s="15">
-        <f>IF(OR(D383&lt;&gt;"",E383&lt;&gt;""),IF(D383="",0,D383)+IF(E383="",0,E383),"")</f>
+        <f>IF(OR(D399&lt;&gt;"",E399&lt;&gt;""),IF(D399="",0,D399)+IF(E399="",0,E399),"")</f>
         <v/>
       </c>
       <c r="G399" s="14" t="n"/>
@@ -62086,7 +62098,7 @@
       <c r="D400" s="27" t="n"/>
       <c r="E400" s="28" t="n"/>
       <c r="F400" s="15">
-        <f>IF(OR(D384&lt;&gt;"",E384&lt;&gt;""),IF(D384="",0,D384)+IF(E384="",0,E384),"")</f>
+        <f>IF(OR(D400&lt;&gt;"",E400&lt;&gt;""),IF(D400="",0,D400)+IF(E400="",0,E400),"")</f>
         <v/>
       </c>
       <c r="G400" s="14" t="n"/>
@@ -62102,7 +62114,7 @@
       <c r="D401" s="27" t="n"/>
       <c r="E401" s="28" t="n"/>
       <c r="F401" s="15">
-        <f>IF(OR(D385&lt;&gt;"",E385&lt;&gt;""),IF(D385="",0,D385)+IF(E385="",0,E385),"")</f>
+        <f>IF(OR(D401&lt;&gt;"",E401&lt;&gt;""),IF(D401="",0,D401)+IF(E401="",0,E401),"")</f>
         <v/>
       </c>
       <c r="G401" s="14" t="n"/>
@@ -62118,7 +62130,7 @@
       <c r="D402" s="27" t="n"/>
       <c r="E402" s="28" t="n"/>
       <c r="F402" s="15">
-        <f>IF(OR(D386&lt;&gt;"",E386&lt;&gt;""),IF(D386="",0,D386)+IF(E386="",0,E386),"")</f>
+        <f>IF(OR(D402&lt;&gt;"",E402&lt;&gt;""),IF(D402="",0,D402)+IF(E402="",0,E402),"")</f>
         <v/>
       </c>
       <c r="G402" s="14" t="n"/>
@@ -62134,7 +62146,7 @@
       <c r="D403" s="27" t="n"/>
       <c r="E403" s="28" t="n"/>
       <c r="F403" s="15">
-        <f>IF(OR(D387&lt;&gt;"",E387&lt;&gt;""),IF(D387="",0,D387)+IF(E387="",0,E387),"")</f>
+        <f>IF(OR(D403&lt;&gt;"",E403&lt;&gt;""),IF(D403="",0,D403)+IF(E403="",0,E403),"")</f>
         <v/>
       </c>
       <c r="G403" s="14" t="n"/>
@@ -62150,7 +62162,7 @@
       <c r="D404" s="27" t="n"/>
       <c r="E404" s="28" t="n"/>
       <c r="F404" s="15">
-        <f>IF(OR(D388&lt;&gt;"",E388&lt;&gt;""),IF(D388="",0,D388)+IF(E388="",0,E388),"")</f>
+        <f>IF(OR(D404&lt;&gt;"",E404&lt;&gt;""),IF(D404="",0,D404)+IF(E404="",0,E404),"")</f>
         <v/>
       </c>
       <c r="G404" s="14" t="n"/>
@@ -62166,7 +62178,7 @@
       <c r="D405" s="27" t="n"/>
       <c r="E405" s="28" t="n"/>
       <c r="F405" s="15">
-        <f>IF(OR(D389&lt;&gt;"",E389&lt;&gt;""),IF(D389="",0,D389)+IF(E389="",0,E389),"")</f>
+        <f>IF(OR(D405&lt;&gt;"",E405&lt;&gt;""),IF(D405="",0,D405)+IF(E405="",0,E405),"")</f>
         <v/>
       </c>
       <c r="G405" s="14" t="n"/>
@@ -62182,7 +62194,7 @@
       <c r="D406" s="27" t="n"/>
       <c r="E406" s="28" t="n"/>
       <c r="F406" s="15">
-        <f>IF(OR(D390&lt;&gt;"",E390&lt;&gt;""),IF(D390="",0,D390)+IF(E390="",0,E390),"")</f>
+        <f>IF(OR(D406&lt;&gt;"",E406&lt;&gt;""),IF(D406="",0,D406)+IF(E406="",0,E406),"")</f>
         <v/>
       </c>
       <c r="G406" s="14" t="n"/>
@@ -62198,7 +62210,7 @@
       <c r="D407" s="27" t="n"/>
       <c r="E407" s="28" t="n"/>
       <c r="F407" s="15">
-        <f>IF(OR(D391&lt;&gt;"",E391&lt;&gt;""),IF(D391="",0,D391)+IF(E391="",0,E391),"")</f>
+        <f>IF(OR(D407&lt;&gt;"",E407&lt;&gt;""),IF(D407="",0,D407)+IF(E407="",0,E407),"")</f>
         <v/>
       </c>
       <c r="G407" s="14" t="n"/>
@@ -62214,7 +62226,7 @@
       <c r="D408" s="27" t="n"/>
       <c r="E408" s="28" t="n"/>
       <c r="F408" s="15">
-        <f>IF(OR(D392&lt;&gt;"",E392&lt;&gt;""),IF(D392="",0,D392)+IF(E392="",0,E392),"")</f>
+        <f>IF(OR(D408&lt;&gt;"",E408&lt;&gt;""),IF(D408="",0,D408)+IF(E408="",0,E408),"")</f>
         <v/>
       </c>
       <c r="G408" s="14" t="n"/>
@@ -62230,7 +62242,7 @@
       <c r="D409" s="27" t="n"/>
       <c r="E409" s="28" t="n"/>
       <c r="F409" s="15">
-        <f>IF(OR(D393&lt;&gt;"",E393&lt;&gt;""),IF(D393="",0,D393)+IF(E393="",0,E393),"")</f>
+        <f>IF(OR(D409&lt;&gt;"",E409&lt;&gt;""),IF(D409="",0,D409)+IF(E409="",0,E409),"")</f>
         <v/>
       </c>
       <c r="G409" s="14" t="n"/>
@@ -62246,7 +62258,7 @@
       <c r="D410" s="27" t="n"/>
       <c r="E410" s="28" t="n"/>
       <c r="F410" s="15">
-        <f>IF(OR(D394&lt;&gt;"",E394&lt;&gt;""),IF(D394="",0,D394)+IF(E394="",0,E394),"")</f>
+        <f>IF(OR(D410&lt;&gt;"",E410&lt;&gt;""),IF(D410="",0,D410)+IF(E410="",0,E410),"")</f>
         <v/>
       </c>
       <c r="G410" s="14" t="n"/>
@@ -62262,7 +62274,7 @@
       <c r="D411" s="27" t="n"/>
       <c r="E411" s="28" t="n"/>
       <c r="F411" s="15">
-        <f>IF(OR(D395&lt;&gt;"",E395&lt;&gt;""),IF(D395="",0,D395)+IF(E395="",0,E395),"")</f>
+        <f>IF(OR(D411&lt;&gt;"",E411&lt;&gt;""),IF(D411="",0,D411)+IF(E411="",0,E411),"")</f>
         <v/>
       </c>
       <c r="G411" s="14" t="n"/>
@@ -62278,7 +62290,7 @@
       <c r="D412" s="27" t="n"/>
       <c r="E412" s="28" t="n"/>
       <c r="F412" s="15">
-        <f>IF(OR(D396&lt;&gt;"",E396&lt;&gt;""),IF(D396="",0,D396)+IF(E396="",0,E396),"")</f>
+        <f>IF(OR(D412&lt;&gt;"",E412&lt;&gt;""),IF(D412="",0,D412)+IF(E412="",0,E412),"")</f>
         <v/>
       </c>
       <c r="G412" s="14" t="n"/>
@@ -62294,7 +62306,7 @@
       <c r="D413" s="27" t="n"/>
       <c r="E413" s="28" t="n"/>
       <c r="F413" s="15">
-        <f>IF(OR(D397&lt;&gt;"",E397&lt;&gt;""),IF(D397="",0,D397)+IF(E397="",0,E397),"")</f>
+        <f>IF(OR(D413&lt;&gt;"",E413&lt;&gt;""),IF(D413="",0,D413)+IF(E413="",0,E413),"")</f>
         <v/>
       </c>
       <c r="G413" s="14" t="n"/>
@@ -62310,7 +62322,7 @@
       <c r="D414" s="27" t="n"/>
       <c r="E414" s="28" t="n"/>
       <c r="F414" s="15">
-        <f>IF(OR(D398&lt;&gt;"",E398&lt;&gt;""),IF(D398="",0,D398)+IF(E398="",0,E398),"")</f>
+        <f>IF(OR(D414&lt;&gt;"",E414&lt;&gt;""),IF(D414="",0,D414)+IF(E414="",0,E414),"")</f>
         <v/>
       </c>
       <c r="G414" s="14" t="n"/>
@@ -62326,7 +62338,7 @@
       <c r="D415" s="27" t="n"/>
       <c r="E415" s="28" t="n"/>
       <c r="F415" s="15">
-        <f>IF(OR(D399&lt;&gt;"",E399&lt;&gt;""),IF(D399="",0,D399)+IF(E399="",0,E399),"")</f>
+        <f>IF(OR(D415&lt;&gt;"",E415&lt;&gt;""),IF(D415="",0,D415)+IF(E415="",0,E415),"")</f>
         <v/>
       </c>
       <c r="G415" s="14" t="n"/>
@@ -62342,7 +62354,7 @@
       <c r="D416" s="27" t="n"/>
       <c r="E416" s="28" t="n"/>
       <c r="F416" s="15">
-        <f>IF(OR(D400&lt;&gt;"",E400&lt;&gt;""),IF(D400="",0,D400)+IF(E400="",0,E400),"")</f>
+        <f>IF(OR(D416&lt;&gt;"",E416&lt;&gt;""),IF(D416="",0,D416)+IF(E416="",0,E416),"")</f>
         <v/>
       </c>
       <c r="G416" s="14" t="n"/>
@@ -62358,7 +62370,7 @@
       <c r="D417" s="27" t="n"/>
       <c r="E417" s="28" t="n"/>
       <c r="F417" s="15">
-        <f>IF(OR(D401&lt;&gt;"",E401&lt;&gt;""),IF(D401="",0,D401)+IF(E401="",0,E401),"")</f>
+        <f>IF(OR(D417&lt;&gt;"",E417&lt;&gt;""),IF(D417="",0,D417)+IF(E417="",0,E417),"")</f>
         <v/>
       </c>
       <c r="G417" s="14" t="n"/>
@@ -62374,7 +62386,7 @@
       <c r="D418" s="27" t="n"/>
       <c r="E418" s="28" t="n"/>
       <c r="F418" s="15">
-        <f>IF(OR(D402&lt;&gt;"",E402&lt;&gt;""),IF(D402="",0,D402)+IF(E402="",0,E402),"")</f>
+        <f>IF(OR(D418&lt;&gt;"",E418&lt;&gt;""),IF(D418="",0,D418)+IF(E418="",0,E418),"")</f>
         <v/>
       </c>
       <c r="G418" s="14" t="n"/>
@@ -62390,7 +62402,7 @@
       <c r="D419" s="27" t="n"/>
       <c r="E419" s="28" t="n"/>
       <c r="F419" s="15">
-        <f>IF(OR(D403&lt;&gt;"",E403&lt;&gt;""),IF(D403="",0,D403)+IF(E403="",0,E403),"")</f>
+        <f>IF(OR(D419&lt;&gt;"",E419&lt;&gt;""),IF(D419="",0,D419)+IF(E419="",0,E419),"")</f>
         <v/>
       </c>
       <c r="G419" s="14" t="n"/>
@@ -62406,7 +62418,7 @@
       <c r="D420" s="27" t="n"/>
       <c r="E420" s="28" t="n"/>
       <c r="F420" s="15">
-        <f>IF(OR(D404&lt;&gt;"",E404&lt;&gt;""),IF(D404="",0,D404)+IF(E404="",0,E404),"")</f>
+        <f>IF(OR(D420&lt;&gt;"",E420&lt;&gt;""),IF(D420="",0,D420)+IF(E420="",0,E420),"")</f>
         <v/>
       </c>
       <c r="G420" s="14" t="n"/>
@@ -62422,7 +62434,7 @@
       <c r="D421" s="27" t="n"/>
       <c r="E421" s="28" t="n"/>
       <c r="F421" s="15">
-        <f>IF(OR(D405&lt;&gt;"",E405&lt;&gt;""),IF(D405="",0,D405)+IF(E405="",0,E405),"")</f>
+        <f>IF(OR(D421&lt;&gt;"",E421&lt;&gt;""),IF(D421="",0,D421)+IF(E421="",0,E421),"")</f>
         <v/>
       </c>
       <c r="G421" s="14" t="n"/>
@@ -62438,7 +62450,7 @@
       <c r="D422" s="27" t="n"/>
       <c r="E422" s="28" t="n"/>
       <c r="F422" s="15">
-        <f>IF(OR(D406&lt;&gt;"",E406&lt;&gt;""),IF(D406="",0,D406)+IF(E406="",0,E406),"")</f>
+        <f>IF(OR(D422&lt;&gt;"",E422&lt;&gt;""),IF(D422="",0,D422)+IF(E422="",0,E422),"")</f>
         <v/>
       </c>
       <c r="G422" s="14" t="n"/>
@@ -62454,7 +62466,7 @@
       <c r="D423" s="27" t="n"/>
       <c r="E423" s="28" t="n"/>
       <c r="F423" s="15">
-        <f>IF(OR(D407&lt;&gt;"",E407&lt;&gt;""),IF(D407="",0,D407)+IF(E407="",0,E407),"")</f>
+        <f>IF(OR(D423&lt;&gt;"",E423&lt;&gt;""),IF(D423="",0,D423)+IF(E423="",0,E423),"")</f>
         <v/>
       </c>
       <c r="G423" s="14" t="n"/>
@@ -62470,7 +62482,7 @@
       <c r="D424" s="27" t="n"/>
       <c r="E424" s="28" t="n"/>
       <c r="F424" s="15">
-        <f>IF(OR(D408&lt;&gt;"",E408&lt;&gt;""),IF(D408="",0,D408)+IF(E408="",0,E408),"")</f>
+        <f>IF(OR(D424&lt;&gt;"",E424&lt;&gt;""),IF(D424="",0,D424)+IF(E424="",0,E424),"")</f>
         <v/>
       </c>
       <c r="G424" s="14" t="n"/>
@@ -62486,7 +62498,7 @@
       <c r="D425" s="27" t="n"/>
       <c r="E425" s="28" t="n"/>
       <c r="F425" s="15">
-        <f>IF(OR(D409&lt;&gt;"",E409&lt;&gt;""),IF(D409="",0,D409)+IF(E409="",0,E409),"")</f>
+        <f>IF(OR(D425&lt;&gt;"",E425&lt;&gt;""),IF(D425="",0,D425)+IF(E425="",0,E425),"")</f>
         <v/>
       </c>
       <c r="G425" s="14" t="n"/>
@@ -62502,7 +62514,7 @@
       <c r="D426" s="27" t="n"/>
       <c r="E426" s="28" t="n"/>
       <c r="F426" s="15">
-        <f>IF(OR(D410&lt;&gt;"",E410&lt;&gt;""),IF(D410="",0,D410)+IF(E410="",0,E410),"")</f>
+        <f>IF(OR(D426&lt;&gt;"",E426&lt;&gt;""),IF(D426="",0,D426)+IF(E426="",0,E426),"")</f>
         <v/>
       </c>
       <c r="G426" s="14" t="n"/>
@@ -62518,7 +62530,7 @@
       <c r="D427" s="27" t="n"/>
       <c r="E427" s="28" t="n"/>
       <c r="F427" s="15">
-        <f>IF(OR(D411&lt;&gt;"",E411&lt;&gt;""),IF(D411="",0,D411)+IF(E411="",0,E411),"")</f>
+        <f>IF(OR(D427&lt;&gt;"",E427&lt;&gt;""),IF(D427="",0,D427)+IF(E427="",0,E427),"")</f>
         <v/>
       </c>
       <c r="G427" s="14" t="n"/>
@@ -62534,7 +62546,7 @@
       <c r="D428" s="27" t="n"/>
       <c r="E428" s="28" t="n"/>
       <c r="F428" s="15">
-        <f>IF(OR(D412&lt;&gt;"",E412&lt;&gt;""),IF(D412="",0,D412)+IF(E412="",0,E412),"")</f>
+        <f>IF(OR(D428&lt;&gt;"",E428&lt;&gt;""),IF(D428="",0,D428)+IF(E428="",0,E428),"")</f>
         <v/>
       </c>
       <c r="G428" s="14" t="n"/>
@@ -62550,7 +62562,7 @@
       <c r="D429" s="27" t="n"/>
       <c r="E429" s="28" t="n"/>
       <c r="F429" s="15">
-        <f>IF(OR(D413&lt;&gt;"",E413&lt;&gt;""),IF(D413="",0,D413)+IF(E413="",0,E413),"")</f>
+        <f>IF(OR(D429&lt;&gt;"",E429&lt;&gt;""),IF(D429="",0,D429)+IF(E429="",0,E429),"")</f>
         <v/>
       </c>
       <c r="G429" s="14" t="n"/>
@@ -62566,7 +62578,7 @@
       <c r="D430" s="27" t="n"/>
       <c r="E430" s="28" t="n"/>
       <c r="F430" s="15">
-        <f>IF(OR(D414&lt;&gt;"",E414&lt;&gt;""),IF(D414="",0,D414)+IF(E414="",0,E414),"")</f>
+        <f>IF(OR(D430&lt;&gt;"",E430&lt;&gt;""),IF(D430="",0,D430)+IF(E430="",0,E430),"")</f>
         <v/>
       </c>
       <c r="G430" s="14" t="n"/>
@@ -62582,7 +62594,7 @@
       <c r="D431" s="27" t="n"/>
       <c r="E431" s="28" t="n"/>
       <c r="F431" s="15">
-        <f>IF(OR(D415&lt;&gt;"",E415&lt;&gt;""),IF(D415="",0,D415)+IF(E415="",0,E415),"")</f>
+        <f>IF(OR(D431&lt;&gt;"",E431&lt;&gt;""),IF(D431="",0,D431)+IF(E431="",0,E431),"")</f>
         <v/>
       </c>
       <c r="G431" s="14" t="n"/>
@@ -62598,7 +62610,7 @@
       <c r="D432" s="27" t="n"/>
       <c r="E432" s="28" t="n"/>
       <c r="F432" s="15">
-        <f>IF(OR(D416&lt;&gt;"",E416&lt;&gt;""),IF(D416="",0,D416)+IF(E416="",0,E416),"")</f>
+        <f>IF(OR(D432&lt;&gt;"",E432&lt;&gt;""),IF(D432="",0,D432)+IF(E432="",0,E432),"")</f>
         <v/>
       </c>
       <c r="G432" s="14" t="n"/>
@@ -62614,7 +62626,7 @@
       <c r="D433" s="27" t="n"/>
       <c r="E433" s="28" t="n"/>
       <c r="F433" s="15">
-        <f>IF(OR(D417&lt;&gt;"",E417&lt;&gt;""),IF(D417="",0,D417)+IF(E417="",0,E417),"")</f>
+        <f>IF(OR(D433&lt;&gt;"",E433&lt;&gt;""),IF(D433="",0,D433)+IF(E433="",0,E433),"")</f>
         <v/>
       </c>
       <c r="G433" s="14" t="n"/>
@@ -62630,7 +62642,7 @@
       <c r="D434" s="27" t="n"/>
       <c r="E434" s="28" t="n"/>
       <c r="F434" s="15">
-        <f>IF(OR(D418&lt;&gt;"",E418&lt;&gt;""),IF(D418="",0,D418)+IF(E418="",0,E418),"")</f>
+        <f>IF(OR(D434&lt;&gt;"",E434&lt;&gt;""),IF(D434="",0,D434)+IF(E434="",0,E434),"")</f>
         <v/>
       </c>
       <c r="G434" s="14" t="n"/>
@@ -62646,7 +62658,7 @@
       <c r="D435" s="27" t="n"/>
       <c r="E435" s="28" t="n"/>
       <c r="F435" s="15">
-        <f>IF(OR(D419&lt;&gt;"",E419&lt;&gt;""),IF(D419="",0,D419)+IF(E419="",0,E419),"")</f>
+        <f>IF(OR(D435&lt;&gt;"",E435&lt;&gt;""),IF(D435="",0,D435)+IF(E435="",0,E435),"")</f>
         <v/>
       </c>
       <c r="G435" s="14" t="n"/>
@@ -62662,7 +62674,7 @@
       <c r="D436" s="27" t="n"/>
       <c r="E436" s="28" t="n"/>
       <c r="F436" s="15">
-        <f>IF(OR(D420&lt;&gt;"",E420&lt;&gt;""),IF(D420="",0,D420)+IF(E420="",0,E420),"")</f>
+        <f>IF(OR(D436&lt;&gt;"",E436&lt;&gt;""),IF(D436="",0,D436)+IF(E436="",0,E436),"")</f>
         <v/>
       </c>
       <c r="G436" s="14" t="n"/>
@@ -62678,7 +62690,7 @@
       <c r="D437" s="27" t="n"/>
       <c r="E437" s="28" t="n"/>
       <c r="F437" s="15">
-        <f>IF(OR(D421&lt;&gt;"",E421&lt;&gt;""),IF(D421="",0,D421)+IF(E421="",0,E421),"")</f>
+        <f>IF(OR(D437&lt;&gt;"",E437&lt;&gt;""),IF(D437="",0,D437)+IF(E437="",0,E437),"")</f>
         <v/>
       </c>
       <c r="G437" s="14" t="n"/>

</xml_diff>

<commit_message>
Add Chris September COMIDA · pollo $10,140 to Almacen Detalle.
Second pollo line for Chris (alongside existing $10,295); Septiembre Importe Chris total now $237,104.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -62027,15 +62027,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B379" s="17" t="n"/>
-      <c r="C379" s="14" t="n"/>
+      <c r="B379" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C379" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · pollo</t>
+        </is>
+      </c>
       <c r="D379" s="27" t="n"/>
-      <c r="E379" s="28" t="n"/>
+      <c r="E379" s="28" t="n">
+        <v>10140</v>
+      </c>
       <c r="F379" s="15">
         <f>IF(OR(D379&lt;&gt;"",E379&lt;&gt;""),IF(D379="",0,D379)+IF(E379="",0,E379),"")</f>
         <v/>
       </c>
-      <c r="G379" s="14" t="n"/>
+      <c r="G379" s="14" t="inlineStr">
+        <is>
+          <t>Chris · COMIDA · pollo · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="380">
       <c r="A380" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Load Mercado Pago Gmail purchases into CIUDAD Almacén and GPS.
Extract Aug–Oct (plus key May/Jun/Jul gaps) payment emails: Sodastream and Pescadería to Almacen Detalle; Copetin, travel, vestimenta, farmacia and other clear GPS items; skip TC MP multi-cuota and MP No Gasto. Add classification report and harden SOL supermercado classifier.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -3641,7 +3641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F828"/>
+  <dimension ref="A1:F850"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25746,6 +25746,622 @@
       <c r="F828" s="34" t="inlineStr">
         <is>
           <t>SALUD · Vitaminas · Promarine · TC Mercado Pago · C.04/06 · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" s="52" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>COMIDA · Oficina</t>
+        </is>
+      </c>
+      <c r="D829" t="n">
+        <v>11010</v>
+      </c>
+      <c r="E829" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F829" t="inlineStr">
+        <is>
+          <t>COMIDA · Oficina · Copetin Catering · Gmail MP · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" s="52" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>COMIDA · Oficina</t>
+        </is>
+      </c>
+      <c r="D830" t="n">
+        <v>13600</v>
+      </c>
+      <c r="E830" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F830" t="inlineStr">
+        <is>
+          <t>COMIDA · Oficina · Copetin Catering · Gmail MP · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" s="52" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>COMIDA · Oficina</t>
+        </is>
+      </c>
+      <c r="D831" t="n">
+        <v>4080</v>
+      </c>
+      <c r="E831" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F831" t="inlineStr">
+        <is>
+          <t>COMIDA · Oficina · Copetin Catering · Gmail MP · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" s="52" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B832" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D832" t="n">
+        <v>350580</v>
+      </c>
+      <c r="E832" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F832" t="inlineStr">
+        <is>
+          <t>COMPRAS · CENTRAL STORE · Gmail MP · REVISAR · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" s="52" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D833" t="n">
+        <v>176000</v>
+      </c>
+      <c r="E833" t="inlineStr">
+        <is>
+          <t>BBVA Crédito</t>
+        </is>
+      </c>
+      <c r="F833" t="inlineStr">
+        <is>
+          <t>COMPRAS · Gibiana Cova · Gmail MP · BBVA 1 cuota · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" s="52" t="n">
+        <v>46239</v>
+      </c>
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>VESTIMENTA</t>
+        </is>
+      </c>
+      <c r="D834" t="n">
+        <v>152000</v>
+      </c>
+      <c r="E834" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F834" t="inlineStr">
+        <is>
+          <t>VESTIMENTA · Renová tu vestidor · Gmail MP · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" s="52" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B835" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>SALUD</t>
+        </is>
+      </c>
+      <c r="D835" t="n">
+        <v>22222</v>
+      </c>
+      <c r="E835" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F835" t="inlineStr">
+        <is>
+          <t>SALUD · Siendo Consciencia · Gmail MP · REVISAR · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" s="52" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D836" t="n">
+        <v>24000</v>
+      </c>
+      <c r="E836" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F836" t="inlineStr">
+        <is>
+          <t>COMPRAS · Lorena Ferreyra · Gmail MP · REVISAR · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" s="52" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D837" t="n">
+        <v>75000</v>
+      </c>
+      <c r="E837" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F837" t="inlineStr">
+        <is>
+          <t>COMPRAS · Lorena Ferreyra · Gmail MP · REVISAR · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" s="52" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B838" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C838" t="inlineStr">
+        <is>
+          <t>SALUD</t>
+        </is>
+      </c>
+      <c r="D838" t="n">
+        <v>356000</v>
+      </c>
+      <c r="E838" t="inlineStr">
+        <is>
+          <t>BBVA Crédito</t>
+        </is>
+      </c>
+      <c r="F838" t="inlineStr">
+        <is>
+          <t>SALUD · Reiki · Gmail MP · BBVA 1 cuota · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" s="52" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B839" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C839" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D839" t="n">
+        <v>27000</v>
+      </c>
+      <c r="E839" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F839" t="inlineStr">
+        <is>
+          <t>COMPRAS · Karen · Gmail MP · REVISAR · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" s="52" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B840" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C840" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D840" t="n">
+        <v>57725</v>
+      </c>
+      <c r="E840" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F840" t="inlineStr">
+        <is>
+          <t>COMPRAS · Juan Cornacchini · Gmail MP · REVISAR · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" s="52" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B841" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C841" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D841" t="n">
+        <v>30000</v>
+      </c>
+      <c r="E841" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F841" t="inlineStr">
+        <is>
+          <t>COMPRAS · Bitgenia · Gmail MP · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" s="52" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B842" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C842" t="inlineStr">
+        <is>
+          <t>VESTIMENTA</t>
+        </is>
+      </c>
+      <c r="D842" t="n">
+        <v>719990</v>
+      </c>
+      <c r="E842" t="inlineStr">
+        <is>
+          <t>BBVA Crédito</t>
+        </is>
+      </c>
+      <c r="F842" t="inlineStr">
+        <is>
+          <t>VESTIMENTA · Itsclassic · Gmail MP · BBVA 1 cuota · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" s="52" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C843" t="inlineStr">
+        <is>
+          <t>EDUCACIÓN</t>
+        </is>
+      </c>
+      <c r="D843" t="n">
+        <v>127196</v>
+      </c>
+      <c r="E843" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F843" t="inlineStr">
+        <is>
+          <t>EDUCACIÓN · EducaciónIT · Gmail MP · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" s="52" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C844" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D844" t="n">
+        <v>89998</v>
+      </c>
+      <c r="E844" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F844" t="inlineStr">
+        <is>
+          <t>COMPRAS · Yenny El Ateneo · Gmail MP · libros · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" s="52" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="C845" t="inlineStr">
+        <is>
+          <t>FARMACIA SALUD</t>
+        </is>
+      </c>
+      <c r="D845" t="n">
+        <v>17038</v>
+      </c>
+      <c r="E845" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F845" t="inlineStr">
+        <is>
+          <t>FARMACIA SALUD · Hiperfarmacéutica Temperley · Gmail MP · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" s="52" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="C846" t="inlineStr">
+        <is>
+          <t>VIAJES</t>
+        </is>
+      </c>
+      <c r="D846" t="n">
+        <v>1430000</v>
+      </c>
+      <c r="E846" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F846" t="inlineStr">
+        <is>
+          <t>VIAJES · MARPATAG SRL · Gmail MP · TC MP 1 cuota · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" s="52" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr">
+        <is>
+          <t>PELUQUERÍA</t>
+        </is>
+      </c>
+      <c r="D847" t="n">
+        <v>7000</v>
+      </c>
+      <c r="E847" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F847" t="inlineStr">
+        <is>
+          <t>PELUQUERÍA · Soy lashista · Gmail MP · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" s="52" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr">
+        <is>
+          <t>PELUQUERÍA</t>
+        </is>
+      </c>
+      <c r="D848" t="n">
+        <v>7000</v>
+      </c>
+      <c r="E848" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F848" t="inlineStr">
+        <is>
+          <t>PELUQUERÍA · Soy lashista · Gmail MP · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" s="52" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr">
+        <is>
+          <t>VIAJES</t>
+        </is>
+      </c>
+      <c r="D849" t="n">
+        <v>1143000</v>
+      </c>
+      <c r="E849" t="inlineStr">
+        <is>
+          <t>BBVA Crédito</t>
+        </is>
+      </c>
+      <c r="F849" t="inlineStr">
+        <is>
+          <t>VIAJES · Patagonia Chic Excursiones · Gmail MP · BBVA 1 cuota · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" s="52" t="n">
+        <v>46215</v>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D850" t="n">
+        <v>27000</v>
+      </c>
+      <c r="E850" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F850" t="inlineStr">
+        <is>
+          <t>COMPRAS · Karen · Gmail MP · REVISAR · gasto personal Sol</t>
         </is>
       </c>
     </row>
@@ -57624,6 +58240,7 @@
       </c>
       <c r="G176" s="22" t="n"/>
     </row>
+    <row r="177"/>
     <row r="178">
       <c r="A178" s="14" t="inlineStr">
         <is>
@@ -58386,15 +59003,27 @@
           <t>Mayo</t>
         </is>
       </c>
-      <c r="B205" s="17" t="n"/>
-      <c r="C205" s="14" t="n"/>
-      <c r="D205" s="27" t="n"/>
+      <c r="B205" s="17" t="n">
+        <v>46153</v>
+      </c>
+      <c r="C205" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · Pescadería Belgrano</t>
+        </is>
+      </c>
+      <c r="D205" s="27" t="n">
+        <v>24852</v>
+      </c>
       <c r="E205" s="28" t="n"/>
       <c r="F205" s="15">
-        <f>IF(OR(D200&lt;&gt;"",E200&lt;&gt;""),IF(D200="",0,D200)+IF(E200="",0,E200),"")</f>
-        <v/>
-      </c>
-      <c r="G205" s="14" t="n"/>
+        <f>IF(OR(D205&lt;&gt;"",E205&lt;&gt;""),IF(D205="",0,D205)+IF(E205="",0,E205),"")</f>
+        <v/>
+      </c>
+      <c r="G205" s="14" t="inlineStr">
+        <is>
+          <t>Gmail MP · COMIDA · Pescadería Belgrano · dinero disponible</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="14" t="inlineStr">
@@ -58906,6 +59535,7 @@
       </c>
       <c r="G228" s="22" t="n"/>
     </row>
+    <row r="229"/>
     <row r="230">
       <c r="A230" s="14" t="inlineStr">
         <is>
@@ -59556,15 +60186,27 @@
           <t>Junio</t>
         </is>
       </c>
-      <c r="B253" s="17" t="n"/>
-      <c r="C253" s="14" t="n"/>
-      <c r="D253" s="27" t="n"/>
+      <c r="B253" s="17" t="n">
+        <v>46175</v>
+      </c>
+      <c r="C253" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · Pescadería Belgrano</t>
+        </is>
+      </c>
+      <c r="D253" s="27" t="n">
+        <v>32046</v>
+      </c>
       <c r="E253" s="28" t="n"/>
       <c r="F253" s="15">
-        <f>IF(OR(D238&lt;&gt;"",E238&lt;&gt;""),IF(D238="",0,D238)+IF(E238="",0,E238),"")</f>
-        <v/>
-      </c>
-      <c r="G253" s="14" t="n"/>
+        <f>IF(OR(D253&lt;&gt;"",E253&lt;&gt;""),IF(D253="",0,D253)+IF(E253="",0,E253),"")</f>
+        <v/>
+      </c>
+      <c r="G253" s="14" t="inlineStr">
+        <is>
+          <t>Gmail MP · COMIDA · Pescadería Belgrano · dinero disponible</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="14" t="inlineStr">
@@ -59944,6 +60586,7 @@
       </c>
       <c r="G273" s="22" t="n"/>
     </row>
+    <row r="274"/>
     <row r="275">
       <c r="A275" s="14" t="inlineStr">
         <is>
@@ -60711,6 +61354,7 @@
       </c>
       <c r="G312" s="22" t="n"/>
     </row>
+    <row r="313"/>
     <row r="314">
       <c r="A314" s="14" t="inlineStr">
         <is>
@@ -61377,21 +62021,34 @@
       </c>
       <c r="G354" s="22" t="n"/>
     </row>
+    <row r="355"/>
     <row r="356">
       <c r="A356" s="14" t="inlineStr">
         <is>
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B356" s="17" t="n"/>
-      <c r="C356" s="14" t="n"/>
-      <c r="D356" s="27" t="n"/>
+      <c r="B356" s="17" t="n">
+        <v>46269</v>
+      </c>
+      <c r="C356" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · Pescadería Belgrano</t>
+        </is>
+      </c>
+      <c r="D356" s="27" t="n">
+        <v>6213</v>
+      </c>
       <c r="E356" s="28" t="n"/>
       <c r="F356" s="15">
-        <f>IF(OR(D340&lt;&gt;"",E340&lt;&gt;""),IF(D340="",0,D340)+IF(E340="",0,E340),"")</f>
-        <v/>
-      </c>
-      <c r="G356" s="14" t="n"/>
+        <f>IF(OR(D356&lt;&gt;"",E356&lt;&gt;""),IF(D356="",0,D356)+IF(E356="",0,E356),"")</f>
+        <v/>
+      </c>
+      <c r="G356" s="14" t="inlineStr">
+        <is>
+          <t>Gmail MP · COMIDA · Pescadería Belgrano · dinero disponible</t>
+        </is>
+      </c>
     </row>
     <row r="357">
       <c r="A357" s="14" t="inlineStr">
@@ -61399,15 +62056,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B357" s="17" t="n"/>
-      <c r="C357" s="14" t="n"/>
-      <c r="D357" s="27" t="n"/>
+      <c r="B357" s="17" t="n">
+        <v>46273</v>
+      </c>
+      <c r="C357" s="14" t="inlineStr">
+        <is>
+          <t>REPUESTOS · Sodastream</t>
+        </is>
+      </c>
+      <c r="D357" s="27" t="n">
+        <v>88659</v>
+      </c>
       <c r="E357" s="28" t="n"/>
       <c r="F357" s="15">
-        <f>IF(OR(D341&lt;&gt;"",E341&lt;&gt;""),IF(D341="",0,D341)+IF(E341="",0,E341),"")</f>
-        <v/>
-      </c>
-      <c r="G357" s="14" t="n"/>
+        <f>IF(OR(D357&lt;&gt;"",E357&lt;&gt;""),IF(D357="",0,D357)+IF(E357="",0,E357),"")</f>
+        <v/>
+      </c>
+      <c r="G357" s="14" t="inlineStr">
+        <is>
+          <t>Gmail MP · REPUESTOS · Sodastream · dinero disponible</t>
+        </is>
+      </c>
     </row>
     <row r="358">
       <c r="A358" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Consolidate September 2026: add Almacén Chris and refresh summary.
Expand Almacen Detalle September slots, load Chris line items ($237,104), retarget matrix TOTAL row refs, regenerate SOL master, and update RESUMEN_SEPTIEMBRE_2026 (TOTAL CASA $2,342,021).

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -1257,19 +1257,19 @@
         <v/>
       </c>
       <c r="L13" s="5">
-        <f>'Almacen Detalle'!D396</f>
+        <f>'Almacen Detalle'!D426</f>
         <v/>
       </c>
       <c r="M13" s="5">
-        <f>'Almacen Detalle'!D438</f>
+        <f>'Almacen Detalle'!D468</f>
         <v/>
       </c>
       <c r="N13" s="5">
-        <f>'Almacen Detalle'!D480</f>
+        <f>'Almacen Detalle'!D510</f>
         <v/>
       </c>
       <c r="O13" s="5">
-        <f>'Almacen Detalle'!D522</f>
+        <f>'Almacen Detalle'!D552</f>
         <v/>
       </c>
       <c r="P13" s="7">
@@ -1326,19 +1326,19 @@
         <v/>
       </c>
       <c r="L14" s="9">
-        <f>'Almacen Detalle'!E396</f>
+        <f>'Almacen Detalle'!E426</f>
         <v/>
       </c>
       <c r="M14" s="9">
-        <f>'Almacen Detalle'!E438</f>
+        <f>'Almacen Detalle'!E468</f>
         <v/>
       </c>
       <c r="N14" s="9">
-        <f>'Almacen Detalle'!E480</f>
+        <f>'Almacen Detalle'!E510</f>
         <v/>
       </c>
       <c r="O14" s="9">
-        <f>'Almacen Detalle'!E522</f>
+        <f>'Almacen Detalle'!E552</f>
         <v/>
       </c>
       <c r="P14" s="7">
@@ -57128,7 +57128,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G524"/>
+  <dimension ref="A1:G799"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -58408,11 +58408,11 @@
         </is>
       </c>
       <c r="D47" s="7">
-        <f>SUMIFS($D$4:$D$600,$A$4:$A$600,"Enero")</f>
+        <f>SUMIFS($D$4:$D$800,$A$4:$A$800,"Enero")</f>
         <v/>
       </c>
       <c r="E47" s="7">
-        <f>SUMIFS($E$4:$E$600,$A$4:$A$600,"Enero")</f>
+        <f>SUMIFS($E$4:$E$800,$A$4:$A$800,"Enero")</f>
         <v/>
       </c>
       <c r="F47" s="7">
@@ -59513,11 +59513,11 @@
         </is>
       </c>
       <c r="D87" s="7">
-        <f>SUMIFS($D$4:$D$600,$A$4:$A$600,"Febrero")</f>
+        <f>SUMIFS($D$4:$D$800,$A$4:$A$800,"Febrero")</f>
         <v/>
       </c>
       <c r="E87" s="7">
-        <f>SUMIFS($E$4:$E$600,$A$4:$A$600,"Febrero")</f>
+        <f>SUMIFS($E$4:$E$800,$A$4:$A$800,"Febrero")</f>
         <v/>
       </c>
       <c r="F87" s="7">
@@ -60598,11 +60598,11 @@
         </is>
       </c>
       <c r="D131" s="7">
-        <f>SUMIFS($D$4:$D$600,$A$4:$A$600,"Marzo")</f>
+        <f>SUMIFS($D$4:$D$800,$A$4:$A$800,"Marzo")</f>
         <v/>
       </c>
       <c r="E131" s="7">
-        <f>SUMIFS($E$4:$E$600,$A$4:$A$600,"Marzo")</f>
+        <f>SUMIFS($E$4:$E$800,$A$4:$A$800,"Marzo")</f>
         <v/>
       </c>
       <c r="F131" s="7">
@@ -61675,11 +61675,11 @@
         </is>
       </c>
       <c r="D176" s="7">
-        <f>SUMIFS($D$4:$D$600,$A$4:$A$600,"Abril")</f>
+        <f>SUMIFS($D$4:$D$800,$A$4:$A$800,"Abril")</f>
         <v/>
       </c>
       <c r="E176" s="7">
-        <f>SUMIFS($E$4:$E$600,$A$4:$A$600,"Abril")</f>
+        <f>SUMIFS($E$4:$E$800,$A$4:$A$800,"Abril")</f>
         <v/>
       </c>
       <c r="F176" s="7">
@@ -61688,6 +61688,7 @@
       </c>
       <c r="G176" s="22" t="n"/>
     </row>
+    <row r="177"/>
     <row r="178">
       <c r="A178" s="14" t="inlineStr">
         <is>
@@ -62957,11 +62958,11 @@
         </is>
       </c>
       <c r="D228" s="7">
-        <f>SUMIFS($D$4:$D$600,$A$4:$A$600,"Mayo")</f>
+        <f>SUMIFS($D$4:$D$800,$A$4:$A$800,"Mayo")</f>
         <v/>
       </c>
       <c r="E228" s="7">
-        <f>SUMIFS($E$4:$E$600,$A$4:$A$600,"Mayo")</f>
+        <f>SUMIFS($E$4:$E$800,$A$4:$A$800,"Mayo")</f>
         <v/>
       </c>
       <c r="F228" s="7">
@@ -62970,6 +62971,7 @@
       </c>
       <c r="G228" s="22" t="n"/>
     </row>
+    <row r="229"/>
     <row r="230">
       <c r="A230" s="14" t="inlineStr">
         <is>
@@ -63995,11 +63997,11 @@
         </is>
       </c>
       <c r="D273" s="7">
-        <f>SUMIFS($D$4:$D$600,$A$4:$A$600,"Junio")</f>
+        <f>SUMIFS($D$4:$D$800,$A$4:$A$800,"Junio")</f>
         <v/>
       </c>
       <c r="E273" s="7">
-        <f>SUMIFS($E$4:$E$600,$A$4:$A$600,"Junio")</f>
+        <f>SUMIFS($E$4:$E$800,$A$4:$A$800,"Junio")</f>
         <v/>
       </c>
       <c r="F273" s="7">
@@ -64008,6 +64010,7 @@
       </c>
       <c r="G273" s="22" t="n"/>
     </row>
+    <row r="274"/>
     <row r="275">
       <c r="A275" s="14" t="inlineStr">
         <is>
@@ -64762,11 +64765,11 @@
         </is>
       </c>
       <c r="D312" s="7">
-        <f>SUMIFS($D$4:$D$600,$A$4:$A$600,"Julio")</f>
+        <f>SUMIFS($D$4:$D$800,$A$4:$A$800,"Julio")</f>
         <v/>
       </c>
       <c r="E312" s="7">
-        <f>SUMIFS($E$4:$E$600,$A$4:$A$600,"Julio")</f>
+        <f>SUMIFS($E$4:$E$800,$A$4:$A$800,"Julio")</f>
         <v/>
       </c>
       <c r="F312" s="7">
@@ -64775,6 +64778,7 @@
       </c>
       <c r="G312" s="22" t="n"/>
     </row>
+    <row r="313"/>
     <row r="314">
       <c r="A314" s="14" t="inlineStr">
         <is>
@@ -65428,11 +65432,11 @@
         </is>
       </c>
       <c r="D354" s="7">
-        <f>SUMIFS($D$4:$D$600,$A$4:$A$600,"Agosto")</f>
+        <f>SUMIFS($D$4:$D$800,$A$4:$A$800,"Agosto")</f>
         <v/>
       </c>
       <c r="E354" s="7">
-        <f>SUMIFS($E$4:$E$600,$A$4:$A$600,"Agosto")</f>
+        <f>SUMIFS($E$4:$E$800,$A$4:$A$800,"Agosto")</f>
         <v/>
       </c>
       <c r="F354" s="7">
@@ -65441,6 +65445,7 @@
       </c>
       <c r="G354" s="22" t="n"/>
     </row>
+    <row r="355"/>
     <row r="356">
       <c r="A356" s="14" t="inlineStr">
         <is>
@@ -65460,7 +65465,7 @@
       </c>
       <c r="E356" s="28" t="n"/>
       <c r="F356" s="15">
-        <f>IF(OR(D340&lt;&gt;"",E340&lt;&gt;""),IF(D340="",0,D340)+IF(E340="",0,E340),"")</f>
+        <f>IF(OR(D356&lt;&gt;"",E356&lt;&gt;""),IF(D356="",0,D356)+IF(E356="",0,E356),"")</f>
         <v/>
       </c>
       <c r="G356" s="14" t="inlineStr">
@@ -65488,7 +65493,7 @@
       </c>
       <c r="E357" s="28" t="n"/>
       <c r="F357" s="15">
-        <f>IF(OR(D341&lt;&gt;"",E341&lt;&gt;""),IF(D341="",0,D341)+IF(E341="",0,E341),"")</f>
+        <f>IF(OR(D357&lt;&gt;"",E357&lt;&gt;""),IF(D357="",0,D357)+IF(E357="",0,E357),"")</f>
         <v/>
       </c>
       <c r="G357" s="14" t="inlineStr">
@@ -65516,7 +65521,7 @@
       </c>
       <c r="E358" s="28" t="n"/>
       <c r="F358" s="15">
-        <f>IF(OR(D342&lt;&gt;"",E342&lt;&gt;""),IF(D342="",0,D342)+IF(E342="",0,E342),"")</f>
+        <f>IF(OR(D358&lt;&gt;"",E358&lt;&gt;""),IF(D358="",0,D358)+IF(E358="",0,E358),"")</f>
         <v/>
       </c>
       <c r="G358" s="14" t="inlineStr">
@@ -66268,15 +66273,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B386" s="17" t="n"/>
-      <c r="C386" s="14" t="n"/>
+      <c r="B386" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C386" s="14" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Coto</t>
+        </is>
+      </c>
       <c r="D386" s="27" t="n"/>
-      <c r="E386" s="28" t="n"/>
+      <c r="E386" s="28" t="n">
+        <v>11436</v>
+      </c>
       <c r="F386" s="15">
-        <f>IF(OR(D370&lt;&gt;"",E370&lt;&gt;""),IF(D370="",0,D370)+IF(E370="",0,E370),"")</f>
+        <f>IF(OR(D386&lt;&gt;"",E386&lt;&gt;""),IF(D386="",0,D386)+IF(E386="",0,E386),"")</f>
         <v/>
       </c>
-      <c r="G386" s="14" t="n"/>
+      <c r="G386" s="14" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Coto · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="387">
       <c r="A387" s="14" t="inlineStr">
@@ -66284,15 +66301,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B387" s="17" t="n"/>
-      <c r="C387" s="14" t="n"/>
+      <c r="B387" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C387" s="14" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Día</t>
+        </is>
+      </c>
       <c r="D387" s="27" t="n"/>
-      <c r="E387" s="28" t="n"/>
+      <c r="E387" s="28" t="n">
+        <v>7264</v>
+      </c>
       <c r="F387" s="15">
-        <f>IF(OR(D371&lt;&gt;"",E371&lt;&gt;""),IF(D371="",0,D371)+IF(E371="",0,E371),"")</f>
+        <f>IF(OR(D387&lt;&gt;"",E387&lt;&gt;""),IF(D387="",0,D387)+IF(E387="",0,E387),"")</f>
         <v/>
       </c>
-      <c r="G387" s="14" t="n"/>
+      <c r="G387" s="14" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Día · SUPERDIA · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="388">
       <c r="A388" s="14" t="inlineStr">
@@ -66300,15 +66329,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B388" s="17" t="n"/>
-      <c r="C388" s="14" t="n"/>
+      <c r="B388" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C388" s="14" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Coto</t>
+        </is>
+      </c>
       <c r="D388" s="27" t="n"/>
-      <c r="E388" s="28" t="n"/>
+      <c r="E388" s="28" t="n">
+        <v>10000</v>
+      </c>
       <c r="F388" s="15">
-        <f>IF(OR(D372&lt;&gt;"",E372&lt;&gt;""),IF(D372="",0,D372)+IF(E372="",0,E372),"")</f>
+        <f>IF(OR(D388&lt;&gt;"",E388&lt;&gt;""),IF(D388="",0,D388)+IF(E388="",0,E388),"")</f>
         <v/>
       </c>
-      <c r="G388" s="14" t="n"/>
+      <c r="G388" s="14" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Coto · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="389">
       <c r="A389" s="14" t="inlineStr">
@@ -66316,15 +66357,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B389" s="17" t="n"/>
-      <c r="C389" s="14" t="n"/>
+      <c r="B389" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C389" s="14" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Coto</t>
+        </is>
+      </c>
       <c r="D389" s="27" t="n"/>
-      <c r="E389" s="28" t="n"/>
+      <c r="E389" s="28" t="n">
+        <v>11993</v>
+      </c>
       <c r="F389" s="15">
-        <f>IF(OR(D373&lt;&gt;"",E373&lt;&gt;""),IF(D373="",0,D373)+IF(E373="",0,E373),"")</f>
+        <f>IF(OR(D389&lt;&gt;"",E389&lt;&gt;""),IF(D389="",0,D389)+IF(E389="",0,E389),"")</f>
         <v/>
       </c>
-      <c r="G389" s="14" t="n"/>
+      <c r="G389" s="14" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Coto · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="390">
       <c r="A390" s="14" t="inlineStr">
@@ -66332,15 +66385,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B390" s="17" t="n"/>
-      <c r="C390" s="14" t="n"/>
+      <c r="B390" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C390" s="14" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Día</t>
+        </is>
+      </c>
       <c r="D390" s="27" t="n"/>
-      <c r="E390" s="28" t="n"/>
+      <c r="E390" s="28" t="n">
+        <v>9980</v>
+      </c>
       <c r="F390" s="15">
-        <f>IF(OR(D374&lt;&gt;"",E374&lt;&gt;""),IF(D374="",0,D374)+IF(E374="",0,E374),"")</f>
+        <f>IF(OR(D390&lt;&gt;"",E390&lt;&gt;""),IF(D390="",0,D390)+IF(E390="",0,E390),"")</f>
         <v/>
       </c>
-      <c r="G390" s="14" t="n"/>
+      <c r="G390" s="14" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Día · SUPERDIA · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="391">
       <c r="A391" s="14" t="inlineStr">
@@ -66348,15 +66413,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B391" s="17" t="n"/>
-      <c r="C391" s="14" t="n"/>
+      <c r="B391" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C391" s="14" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Día</t>
+        </is>
+      </c>
       <c r="D391" s="27" t="n"/>
-      <c r="E391" s="28" t="n"/>
+      <c r="E391" s="28" t="n">
+        <v>4152</v>
+      </c>
       <c r="F391" s="15">
-        <f>IF(OR(D375&lt;&gt;"",E375&lt;&gt;""),IF(D375="",0,D375)+IF(E375="",0,E375),"")</f>
+        <f>IF(OR(D391&lt;&gt;"",E391&lt;&gt;""),IF(D391="",0,D391)+IF(E391="",0,E391),"")</f>
         <v/>
       </c>
-      <c r="G391" s="14" t="n"/>
+      <c r="G391" s="14" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Día · SUPERDIA · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="392">
       <c r="A392" s="14" t="inlineStr">
@@ -66364,15 +66441,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B392" s="17" t="n"/>
-      <c r="C392" s="14" t="n"/>
+      <c r="B392" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C392" s="14" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Día</t>
+        </is>
+      </c>
       <c r="D392" s="27" t="n"/>
-      <c r="E392" s="28" t="n"/>
+      <c r="E392" s="28" t="n">
+        <v>7488</v>
+      </c>
       <c r="F392" s="15">
-        <f>IF(OR(D376&lt;&gt;"",E376&lt;&gt;""),IF(D376="",0,D376)+IF(E376="",0,E376),"")</f>
+        <f>IF(OR(D392&lt;&gt;"",E392&lt;&gt;""),IF(D392="",0,D392)+IF(E392="",0,E392),"")</f>
         <v/>
       </c>
-      <c r="G392" s="14" t="n"/>
+      <c r="G392" s="14" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Día · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="393">
       <c r="A393" s="14" t="inlineStr">
@@ -66380,15 +66469,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B393" s="17" t="n"/>
-      <c r="C393" s="14" t="n"/>
+      <c r="B393" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C393" s="14" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Coto</t>
+        </is>
+      </c>
       <c r="D393" s="27" t="n"/>
-      <c r="E393" s="28" t="n"/>
+      <c r="E393" s="28" t="n">
+        <v>1999</v>
+      </c>
       <c r="F393" s="15">
-        <f>IF(OR(D377&lt;&gt;"",E377&lt;&gt;""),IF(D377="",0,D377)+IF(E377="",0,E377),"")</f>
+        <f>IF(OR(D393&lt;&gt;"",E393&lt;&gt;""),IF(D393="",0,D393)+IF(E393="",0,E393),"")</f>
         <v/>
       </c>
-      <c r="G393" s="14" t="n"/>
+      <c r="G393" s="14" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Coto · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="394">
       <c r="A394" s="14" t="inlineStr">
@@ -66396,15 +66497,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B394" s="17" t="n"/>
-      <c r="C394" s="14" t="n"/>
+      <c r="B394" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C394" s="14" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Día</t>
+        </is>
+      </c>
       <c r="D394" s="27" t="n"/>
-      <c r="E394" s="28" t="n"/>
+      <c r="E394" s="28" t="n">
+        <v>5680</v>
+      </c>
       <c r="F394" s="15">
-        <f>IF(OR(D378&lt;&gt;"",E378&lt;&gt;""),IF(D378="",0,D378)+IF(E378="",0,E378),"")</f>
+        <f>IF(OR(D394&lt;&gt;"",E394&lt;&gt;""),IF(D394="",0,D394)+IF(E394="",0,E394),"")</f>
         <v/>
       </c>
-      <c r="G394" s="14" t="n"/>
+      <c r="G394" s="14" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Día · sin fecha día · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="395">
       <c r="A395" s="14" t="inlineStr">
@@ -66412,522 +66525,609 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B395" s="17" t="n"/>
-      <c r="C395" s="14" t="n"/>
+      <c r="B395" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C395" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · VERDULERÍA</t>
+        </is>
+      </c>
       <c r="D395" s="27" t="n"/>
-      <c r="E395" s="28" t="n"/>
+      <c r="E395" s="28" t="n">
+        <v>4101</v>
+      </c>
       <c r="F395" s="15">
-        <f>IF(OR(D379&lt;&gt;"",E379&lt;&gt;""),IF(D379="",0,D379)+IF(E379="",0,E379),"")</f>
-        <v/>
-      </c>
-      <c r="G395" s="14" t="n"/>
-    </row>
-    <row r="396">
-      <c r="A396" s="10" t="inlineStr">
-        <is>
-          <t>TOTAL SEPTIEMBRE</t>
-        </is>
-      </c>
-      <c r="B396" s="22" t="n"/>
-      <c r="C396" s="29" t="inlineStr">
-        <is>
-          <t>Totales mes →</t>
-        </is>
-      </c>
-      <c r="D396" s="7">
-        <f>SUMIFS($D$4:$D$600,$A$4:$A$600,"Septiembre")</f>
-        <v/>
-      </c>
-      <c r="E396" s="7">
-        <f>SUMIFS($E$4:$E$600,$A$4:$A$600,"Septiembre")</f>
-        <v/>
-      </c>
-      <c r="F396" s="7">
-        <f>D396+E396</f>
-        <v/>
-      </c>
-      <c r="G396" s="22" t="n"/>
-    </row>
-    <row r="398">
-      <c r="A398" s="14" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B398" s="17" t="n"/>
-      <c r="C398" s="14" t="n"/>
-      <c r="D398" s="27" t="n"/>
-      <c r="E398" s="28" t="n"/>
-      <c r="F398" s="15">
-        <f>IF(OR(D382&lt;&gt;"",E382&lt;&gt;""),IF(D382="",0,D382)+IF(E382="",0,E382),"")</f>
-        <v/>
-      </c>
-      <c r="G398" s="14" t="n"/>
-    </row>
-    <row r="399">
-      <c r="A399" s="14" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B399" s="17" t="n"/>
-      <c r="C399" s="14" t="n"/>
-      <c r="D399" s="27" t="n"/>
-      <c r="E399" s="28" t="n"/>
-      <c r="F399" s="15">
-        <f>IF(OR(D383&lt;&gt;"",E383&lt;&gt;""),IF(D383="",0,D383)+IF(E383="",0,E383),"")</f>
-        <v/>
-      </c>
-      <c r="G399" s="14" t="n"/>
-    </row>
-    <row r="400">
-      <c r="A400" s="14" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B400" s="17" t="n"/>
-      <c r="C400" s="14" t="n"/>
-      <c r="D400" s="27" t="n"/>
-      <c r="E400" s="28" t="n"/>
-      <c r="F400" s="15">
-        <f>IF(OR(D384&lt;&gt;"",E384&lt;&gt;""),IF(D384="",0,D384)+IF(E384="",0,E384),"")</f>
-        <v/>
-      </c>
-      <c r="G400" s="14" t="n"/>
-    </row>
-    <row r="401">
-      <c r="A401" s="14" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B401" s="17" t="n"/>
-      <c r="C401" s="14" t="n"/>
-      <c r="D401" s="27" t="n"/>
-      <c r="E401" s="28" t="n"/>
-      <c r="F401" s="15">
-        <f>IF(OR(D385&lt;&gt;"",E385&lt;&gt;""),IF(D385="",0,D385)+IF(E385="",0,E385),"")</f>
-        <v/>
-      </c>
-      <c r="G401" s="14" t="n"/>
-    </row>
-    <row r="402">
-      <c r="A402" s="14" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B402" s="17" t="n"/>
-      <c r="C402" s="14" t="n"/>
-      <c r="D402" s="27" t="n"/>
-      <c r="E402" s="28" t="n"/>
-      <c r="F402" s="15">
-        <f>IF(OR(D386&lt;&gt;"",E386&lt;&gt;""),IF(D386="",0,D386)+IF(E386="",0,E386),"")</f>
-        <v/>
-      </c>
-      <c r="G402" s="14" t="n"/>
-    </row>
-    <row r="403">
-      <c r="A403" s="14" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B403" s="17" t="n"/>
-      <c r="C403" s="14" t="n"/>
-      <c r="D403" s="27" t="n"/>
-      <c r="E403" s="28" t="n"/>
-      <c r="F403" s="15">
-        <f>IF(OR(D387&lt;&gt;"",E387&lt;&gt;""),IF(D387="",0,D387)+IF(E387="",0,E387),"")</f>
-        <v/>
-      </c>
-      <c r="G403" s="14" t="n"/>
-    </row>
-    <row r="404">
-      <c r="A404" s="14" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B404" s="17" t="n"/>
-      <c r="C404" s="14" t="n"/>
-      <c r="D404" s="27" t="n"/>
-      <c r="E404" s="28" t="n"/>
-      <c r="F404" s="15">
-        <f>IF(OR(D388&lt;&gt;"",E388&lt;&gt;""),IF(D388="",0,D388)+IF(E388="",0,E388),"")</f>
-        <v/>
-      </c>
-      <c r="G404" s="14" t="n"/>
-    </row>
-    <row r="405">
-      <c r="A405" s="14" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B405" s="17" t="n"/>
-      <c r="C405" s="14" t="n"/>
-      <c r="D405" s="27" t="n"/>
-      <c r="E405" s="28" t="n"/>
-      <c r="F405" s="15">
-        <f>IF(OR(D389&lt;&gt;"",E389&lt;&gt;""),IF(D389="",0,D389)+IF(E389="",0,E389),"")</f>
-        <v/>
-      </c>
-      <c r="G405" s="14" t="n"/>
-    </row>
-    <row r="406">
-      <c r="A406" s="14" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B406" s="17" t="n"/>
-      <c r="C406" s="14" t="n"/>
-      <c r="D406" s="27" t="n"/>
-      <c r="E406" s="28" t="n"/>
-      <c r="F406" s="15">
-        <f>IF(OR(D390&lt;&gt;"",E390&lt;&gt;""),IF(D390="",0,D390)+IF(E390="",0,E390),"")</f>
-        <v/>
-      </c>
-      <c r="G406" s="14" t="n"/>
-    </row>
-    <row r="407">
-      <c r="A407" s="14" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B407" s="17" t="n"/>
-      <c r="C407" s="14" t="n"/>
-      <c r="D407" s="27" t="n"/>
-      <c r="E407" s="28" t="n"/>
-      <c r="F407" s="15">
-        <f>IF(OR(D391&lt;&gt;"",E391&lt;&gt;""),IF(D391="",0,D391)+IF(E391="",0,E391),"")</f>
-        <v/>
-      </c>
-      <c r="G407" s="14" t="n"/>
-    </row>
-    <row r="408">
-      <c r="A408" s="14" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B408" s="17" t="n"/>
-      <c r="C408" s="14" t="n"/>
-      <c r="D408" s="27" t="n"/>
-      <c r="E408" s="28" t="n"/>
-      <c r="F408" s="15">
-        <f>IF(OR(D392&lt;&gt;"",E392&lt;&gt;""),IF(D392="",0,D392)+IF(E392="",0,E392),"")</f>
-        <v/>
-      </c>
-      <c r="G408" s="14" t="n"/>
-    </row>
-    <row r="409">
-      <c r="A409" s="14" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B409" s="17" t="n"/>
-      <c r="C409" s="14" t="n"/>
-      <c r="D409" s="27" t="n"/>
-      <c r="E409" s="28" t="n"/>
-      <c r="F409" s="15">
-        <f>IF(OR(D393&lt;&gt;"",E393&lt;&gt;""),IF(D393="",0,D393)+IF(E393="",0,E393),"")</f>
-        <v/>
-      </c>
-      <c r="G409" s="14" t="n"/>
-    </row>
-    <row r="410">
-      <c r="A410" s="14" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B410" s="17" t="n"/>
-      <c r="C410" s="14" t="n"/>
-      <c r="D410" s="27" t="n"/>
-      <c r="E410" s="28" t="n"/>
-      <c r="F410" s="15">
-        <f>IF(OR(D394&lt;&gt;"",E394&lt;&gt;""),IF(D394="",0,D394)+IF(E394="",0,E394),"")</f>
-        <v/>
-      </c>
-      <c r="G410" s="14" t="n"/>
-    </row>
-    <row r="411">
-      <c r="A411" s="14" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B411" s="17" t="n"/>
-      <c r="C411" s="14" t="n"/>
-      <c r="D411" s="27" t="n"/>
-      <c r="E411" s="28" t="n"/>
-      <c r="F411" s="15">
         <f>IF(OR(D395&lt;&gt;"",E395&lt;&gt;""),IF(D395="",0,D395)+IF(E395="",0,E395),"")</f>
         <v/>
       </c>
-      <c r="G411" s="14" t="n"/>
-    </row>
-    <row r="412">
-      <c r="A412" s="14" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B412" s="17" t="n"/>
-      <c r="C412" s="14" t="n"/>
-      <c r="D412" s="27" t="n"/>
-      <c r="E412" s="28" t="n"/>
-      <c r="F412" s="15">
+      <c r="G395" s="14" t="inlineStr">
+        <is>
+          <t>Chris · COMIDA · VERDULERÍA · sin fecha día · REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="B396" s="52" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Coto</t>
+        </is>
+      </c>
+      <c r="E396" t="n">
+        <v>7610</v>
+      </c>
+      <c r="F396">
         <f>IF(OR(D396&lt;&gt;"",E396&lt;&gt;""),IF(D396="",0,D396)+IF(E396="",0,E396),"")</f>
         <v/>
       </c>
-      <c r="G412" s="14" t="n"/>
-    </row>
-    <row r="413">
-      <c r="A413" s="14" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B413" s="17" t="n"/>
-      <c r="C413" s="14" t="n"/>
-      <c r="D413" s="27" t="n"/>
-      <c r="E413" s="28" t="n"/>
-      <c r="F413" s="15">
+      <c r="G396" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Coto · sin fecha día · REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="B397" s="52" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Día</t>
+        </is>
+      </c>
+      <c r="E397" t="n">
+        <v>4796</v>
+      </c>
+      <c r="F397">
         <f>IF(OR(D397&lt;&gt;"",E397&lt;&gt;""),IF(D397="",0,D397)+IF(E397="",0,E397),"")</f>
         <v/>
       </c>
-      <c r="G413" s="14" t="n"/>
-    </row>
-    <row r="414">
-      <c r="A414" s="14" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B414" s="17" t="n"/>
-      <c r="C414" s="14" t="n"/>
-      <c r="D414" s="27" t="n"/>
-      <c r="E414" s="28" t="n"/>
-      <c r="F414" s="15">
+      <c r="G397" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Día · sin fecha día · REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="B398" s="52" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Día</t>
+        </is>
+      </c>
+      <c r="E398" t="n">
+        <v>3952</v>
+      </c>
+      <c r="F398">
         <f>IF(OR(D398&lt;&gt;"",E398&lt;&gt;""),IF(D398="",0,D398)+IF(E398="",0,E398),"")</f>
         <v/>
       </c>
-      <c r="G414" s="14" t="n"/>
-    </row>
-    <row r="415">
-      <c r="A415" s="14" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B415" s="17" t="n"/>
-      <c r="C415" s="14" t="n"/>
-      <c r="D415" s="27" t="n"/>
-      <c r="E415" s="28" t="n"/>
-      <c r="F415" s="15">
+      <c r="G398" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Día · sin fecha día · REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="B399" s="52" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>COMIDA · pollo</t>
+        </is>
+      </c>
+      <c r="E399" t="n">
+        <v>10295</v>
+      </c>
+      <c r="F399">
         <f>IF(OR(D399&lt;&gt;"",E399&lt;&gt;""),IF(D399="",0,D399)+IF(E399="",0,E399),"")</f>
         <v/>
       </c>
-      <c r="G415" s="14" t="n"/>
-    </row>
-    <row r="416">
-      <c r="A416" s="14" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B416" s="17" t="n"/>
-      <c r="C416" s="14" t="n"/>
-      <c r="D416" s="27" t="n"/>
-      <c r="E416" s="28" t="n"/>
-      <c r="F416" s="15">
+      <c r="G399" t="inlineStr">
+        <is>
+          <t>Chris · COMIDA · pollo · sin fecha día · REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="B400" s="52" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Día</t>
+        </is>
+      </c>
+      <c r="E400" t="n">
+        <v>6480</v>
+      </c>
+      <c r="F400">
         <f>IF(OR(D400&lt;&gt;"",E400&lt;&gt;""),IF(D400="",0,D400)+IF(E400="",0,E400),"")</f>
         <v/>
       </c>
-      <c r="G416" s="14" t="n"/>
-    </row>
-    <row r="417">
-      <c r="A417" s="14" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B417" s="17" t="n"/>
-      <c r="C417" s="14" t="n"/>
-      <c r="D417" s="27" t="n"/>
-      <c r="E417" s="28" t="n"/>
-      <c r="F417" s="15">
+      <c r="G400" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Día · sin fecha día · REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="B401" s="52" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Día</t>
+        </is>
+      </c>
+      <c r="E401" t="n">
+        <v>4739</v>
+      </c>
+      <c r="F401">
         <f>IF(OR(D401&lt;&gt;"",E401&lt;&gt;""),IF(D401="",0,D401)+IF(E401="",0,E401),"")</f>
         <v/>
       </c>
-      <c r="G417" s="14" t="n"/>
-    </row>
-    <row r="418">
-      <c r="A418" s="14" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B418" s="17" t="n"/>
-      <c r="C418" s="14" t="n"/>
-      <c r="D418" s="27" t="n"/>
-      <c r="E418" s="28" t="n"/>
-      <c r="F418" s="15">
+      <c r="G401" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Día · sin fecha día · REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="B402" s="52" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>PEDIDOS YA · COMIDA</t>
+        </is>
+      </c>
+      <c r="E402" t="n">
+        <v>23424</v>
+      </c>
+      <c r="F402">
         <f>IF(OR(D402&lt;&gt;"",E402&lt;&gt;""),IF(D402="",0,D402)+IF(E402="",0,E402),"")</f>
         <v/>
       </c>
-      <c r="G418" s="14" t="n"/>
-    </row>
-    <row r="419">
-      <c r="A419" s="14" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B419" s="17" t="n"/>
-      <c r="C419" s="14" t="n"/>
-      <c r="D419" s="27" t="n"/>
-      <c r="E419" s="28" t="n"/>
-      <c r="F419" s="15">
+      <c r="G402" t="inlineStr">
+        <is>
+          <t>Chris · PEDIDOS YA · COMIDA · sin fecha día · REVISAR · confirmar si Market</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="B403" s="52" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Día</t>
+        </is>
+      </c>
+      <c r="E403" t="n">
+        <v>7439</v>
+      </c>
+      <c r="F403">
         <f>IF(OR(D403&lt;&gt;"",E403&lt;&gt;""),IF(D403="",0,D403)+IF(E403="",0,E403),"")</f>
         <v/>
       </c>
-      <c r="G419" s="14" t="n"/>
-    </row>
-    <row r="420">
-      <c r="A420" s="14" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B420" s="17" t="n"/>
-      <c r="C420" s="14" t="n"/>
-      <c r="D420" s="27" t="n"/>
-      <c r="E420" s="28" t="n"/>
-      <c r="F420" s="15">
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Día · sin fecha día · REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="B404" s="52" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Día</t>
+        </is>
+      </c>
+      <c r="E404" t="n">
+        <v>5716</v>
+      </c>
+      <c r="F404">
         <f>IF(OR(D404&lt;&gt;"",E404&lt;&gt;""),IF(D404="",0,D404)+IF(E404="",0,E404),"")</f>
         <v/>
       </c>
-      <c r="G420" s="14" t="n"/>
-    </row>
-    <row r="421">
-      <c r="A421" s="14" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B421" s="17" t="n"/>
-      <c r="C421" s="14" t="n"/>
-      <c r="D421" s="27" t="n"/>
-      <c r="E421" s="28" t="n"/>
-      <c r="F421" s="15">
+      <c r="G404" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Día · sin fecha día · REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="B405" s="52" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Día</t>
+        </is>
+      </c>
+      <c r="E405" t="n">
+        <v>3768</v>
+      </c>
+      <c r="F405">
         <f>IF(OR(D405&lt;&gt;"",E405&lt;&gt;""),IF(D405="",0,D405)+IF(E405="",0,E405),"")</f>
         <v/>
       </c>
-      <c r="G421" s="14" t="n"/>
-    </row>
-    <row r="422">
-      <c r="A422" s="14" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B422" s="17" t="n"/>
-      <c r="C422" s="14" t="n"/>
-      <c r="D422" s="27" t="n"/>
-      <c r="E422" s="28" t="n"/>
-      <c r="F422" s="15">
+      <c r="G405" t="inlineStr">
+        <is>
+          <t>Chris · SUPERMERCADO · Día · sin fecha día · REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="B406" s="52" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>COMIDA · Vinos</t>
+        </is>
+      </c>
+      <c r="E406" t="n">
+        <v>17780</v>
+      </c>
+      <c r="F406">
         <f>IF(OR(D406&lt;&gt;"",E406&lt;&gt;""),IF(D406="",0,D406)+IF(E406="",0,E406),"")</f>
         <v/>
       </c>
-      <c r="G422" s="14" t="n"/>
-    </row>
-    <row r="423">
-      <c r="A423" s="14" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B423" s="17" t="n"/>
-      <c r="C423" s="14" t="n"/>
-      <c r="D423" s="27" t="n"/>
-      <c r="E423" s="28" t="n"/>
-      <c r="F423" s="15">
+      <c r="G406" t="inlineStr">
+        <is>
+          <t>Chris · COMIDA · Vinos · sin fecha día · REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="B407" s="52" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>REVISAR · sin comercio</t>
+        </is>
+      </c>
+      <c r="E407" t="n">
+        <v>48960</v>
+      </c>
+      <c r="F407">
         <f>IF(OR(D407&lt;&gt;"",E407&lt;&gt;""),IF(D407="",0,D407)+IF(E407="",0,E407),"")</f>
         <v/>
       </c>
-      <c r="G423" s="14" t="n"/>
-    </row>
-    <row r="424">
-      <c r="A424" s="14" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B424" s="17" t="n"/>
-      <c r="C424" s="14" t="n"/>
-      <c r="D424" s="27" t="n"/>
-      <c r="E424" s="28" t="n"/>
-      <c r="F424" s="15">
+      <c r="G407" t="inlineStr">
+        <is>
+          <t>Chris · REVISAR · monto sin comercio en listado · sin fecha día</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="B408" s="52" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>COMIDA · VERDULERÍA</t>
+        </is>
+      </c>
+      <c r="E408" t="n">
+        <v>7912</v>
+      </c>
+      <c r="F408">
         <f>IF(OR(D408&lt;&gt;"",E408&lt;&gt;""),IF(D408="",0,D408)+IF(E408="",0,E408),"")</f>
         <v/>
       </c>
-      <c r="G424" s="14" t="n"/>
-    </row>
-    <row r="425">
-      <c r="A425" s="14" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B425" s="17" t="n"/>
-      <c r="C425" s="14" t="n"/>
-      <c r="D425" s="27" t="n"/>
-      <c r="E425" s="28" t="n"/>
-      <c r="F425" s="15">
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>Chris · COMIDA · VERDULERÍA · sin fecha día · REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="B409" s="52" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>COMIDA · pollo</t>
+        </is>
+      </c>
+      <c r="E409" t="n">
+        <v>10140</v>
+      </c>
+      <c r="F409">
         <f>IF(OR(D409&lt;&gt;"",E409&lt;&gt;""),IF(D409="",0,D409)+IF(E409="",0,E409),"")</f>
         <v/>
       </c>
-      <c r="G425" s="14" t="n"/>
-    </row>
-    <row r="426">
-      <c r="A426" s="14" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B426" s="17" t="n"/>
-      <c r="C426" s="14" t="n"/>
-      <c r="D426" s="27" t="n"/>
-      <c r="E426" s="28" t="n"/>
-      <c r="F426" s="15">
+      <c r="G409" t="inlineStr">
+        <is>
+          <t>Chris · COMIDA · pollo · sin fecha día · REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="F410">
         <f>IF(OR(D410&lt;&gt;"",E410&lt;&gt;""),IF(D410="",0,D410)+IF(E410="",0,E410),"")</f>
         <v/>
       </c>
-      <c r="G426" s="14" t="n"/>
-    </row>
-    <row r="427">
-      <c r="A427" s="14" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B427" s="17" t="n"/>
-      <c r="C427" s="14" t="n"/>
-      <c r="D427" s="27" t="n"/>
-      <c r="E427" s="28" t="n"/>
-      <c r="F427" s="15">
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="F411">
         <f>IF(OR(D411&lt;&gt;"",E411&lt;&gt;""),IF(D411="",0,D411)+IF(E411="",0,E411),"")</f>
         <v/>
       </c>
-      <c r="G427" s="14" t="n"/>
-    </row>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="F412">
+        <f>IF(OR(D412&lt;&gt;"",E412&lt;&gt;""),IF(D412="",0,D412)+IF(E412="",0,E412),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="F413">
+        <f>IF(OR(D413&lt;&gt;"",E413&lt;&gt;""),IF(D413="",0,D413)+IF(E413="",0,E413),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="F414">
+        <f>IF(OR(D414&lt;&gt;"",E414&lt;&gt;""),IF(D414="",0,D414)+IF(E414="",0,E414),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="F415">
+        <f>IF(OR(D415&lt;&gt;"",E415&lt;&gt;""),IF(D415="",0,D415)+IF(E415="",0,E415),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="F416">
+        <f>IF(OR(D416&lt;&gt;"",E416&lt;&gt;""),IF(D416="",0,D416)+IF(E416="",0,E416),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="F417">
+        <f>IF(OR(D417&lt;&gt;"",E417&lt;&gt;""),IF(D417="",0,D417)+IF(E417="",0,E417),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="F418">
+        <f>IF(OR(D418&lt;&gt;"",E418&lt;&gt;""),IF(D418="",0,D418)+IF(E418="",0,E418),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="F419">
+        <f>IF(OR(D419&lt;&gt;"",E419&lt;&gt;""),IF(D419="",0,D419)+IF(E419="",0,E419),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="F420">
+        <f>IF(OR(D420&lt;&gt;"",E420&lt;&gt;""),IF(D420="",0,D420)+IF(E420="",0,E420),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="F421">
+        <f>IF(OR(D421&lt;&gt;"",E421&lt;&gt;""),IF(D421="",0,D421)+IF(E421="",0,E421),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="F422">
+        <f>IF(OR(D422&lt;&gt;"",E422&lt;&gt;""),IF(D422="",0,D422)+IF(E422="",0,E422),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="F423">
+        <f>IF(OR(D423&lt;&gt;"",E423&lt;&gt;""),IF(D423="",0,D423)+IF(E423="",0,E423),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="F424">
+        <f>IF(OR(D424&lt;&gt;"",E424&lt;&gt;""),IF(D424="",0,D424)+IF(E424="",0,E424),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="F425">
+        <f>IF(OR(D425&lt;&gt;"",E425&lt;&gt;""),IF(D425="",0,D425)+IF(E425="",0,E425),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" s="10" t="inlineStr">
+        <is>
+          <t>TOTAL SEPTIEMBRE</t>
+        </is>
+      </c>
+      <c r="B426" s="22" t="n"/>
+      <c r="C426" s="29" t="inlineStr">
+        <is>
+          <t>Totales mes →</t>
+        </is>
+      </c>
+      <c r="D426" s="7">
+        <f>SUMIFS($D$4:$D$800,$A$4:$A$800,"Septiembre")</f>
+        <v/>
+      </c>
+      <c r="E426" s="7">
+        <f>SUMIFS($E$4:$E$800,$A$4:$A$800,"Septiembre")</f>
+        <v/>
+      </c>
+      <c r="F426" s="7">
+        <f>D426+E426</f>
+        <v/>
+      </c>
+      <c r="G426" s="22" t="n"/>
+    </row>
+    <row r="427"/>
     <row r="428">
       <c r="A428" s="14" t="inlineStr">
         <is>
@@ -66939,7 +67139,7 @@
       <c r="D428" s="27" t="n"/>
       <c r="E428" s="28" t="n"/>
       <c r="F428" s="15">
-        <f>IF(OR(D412&lt;&gt;"",E412&lt;&gt;""),IF(D412="",0,D412)+IF(E412="",0,E412),"")</f>
+        <f>IF(OR(D382&lt;&gt;"",E382&lt;&gt;""),IF(D382="",0,D382)+IF(E382="",0,E382),"")</f>
         <v/>
       </c>
       <c r="G428" s="14" t="n"/>
@@ -66955,7 +67155,7 @@
       <c r="D429" s="27" t="n"/>
       <c r="E429" s="28" t="n"/>
       <c r="F429" s="15">
-        <f>IF(OR(D413&lt;&gt;"",E413&lt;&gt;""),IF(D413="",0,D413)+IF(E413="",0,E413),"")</f>
+        <f>IF(OR(D383&lt;&gt;"",E383&lt;&gt;""),IF(D383="",0,D383)+IF(E383="",0,E383),"")</f>
         <v/>
       </c>
       <c r="G429" s="14" t="n"/>
@@ -66971,7 +67171,7 @@
       <c r="D430" s="27" t="n"/>
       <c r="E430" s="28" t="n"/>
       <c r="F430" s="15">
-        <f>IF(OR(D414&lt;&gt;"",E414&lt;&gt;""),IF(D414="",0,D414)+IF(E414="",0,E414),"")</f>
+        <f>IF(OR(D384&lt;&gt;"",E384&lt;&gt;""),IF(D384="",0,D384)+IF(E384="",0,E384),"")</f>
         <v/>
       </c>
       <c r="G430" s="14" t="n"/>
@@ -66987,7 +67187,7 @@
       <c r="D431" s="27" t="n"/>
       <c r="E431" s="28" t="n"/>
       <c r="F431" s="15">
-        <f>IF(OR(D415&lt;&gt;"",E415&lt;&gt;""),IF(D415="",0,D415)+IF(E415="",0,E415),"")</f>
+        <f>IF(OR(D385&lt;&gt;"",E385&lt;&gt;""),IF(D385="",0,D385)+IF(E385="",0,E385),"")</f>
         <v/>
       </c>
       <c r="G431" s="14" t="n"/>
@@ -67003,7 +67203,7 @@
       <c r="D432" s="27" t="n"/>
       <c r="E432" s="28" t="n"/>
       <c r="F432" s="15">
-        <f>IF(OR(D416&lt;&gt;"",E416&lt;&gt;""),IF(D416="",0,D416)+IF(E416="",0,E416),"")</f>
+        <f>IF(OR(D386&lt;&gt;"",E386&lt;&gt;""),IF(D386="",0,D386)+IF(E386="",0,E386),"")</f>
         <v/>
       </c>
       <c r="G432" s="14" t="n"/>
@@ -67019,7 +67219,7 @@
       <c r="D433" s="27" t="n"/>
       <c r="E433" s="28" t="n"/>
       <c r="F433" s="15">
-        <f>IF(OR(D417&lt;&gt;"",E417&lt;&gt;""),IF(D417="",0,D417)+IF(E417="",0,E417),"")</f>
+        <f>IF(OR(D387&lt;&gt;"",E387&lt;&gt;""),IF(D387="",0,D387)+IF(E387="",0,E387),"")</f>
         <v/>
       </c>
       <c r="G433" s="14" t="n"/>
@@ -67035,7 +67235,7 @@
       <c r="D434" s="27" t="n"/>
       <c r="E434" s="28" t="n"/>
       <c r="F434" s="15">
-        <f>IF(OR(D418&lt;&gt;"",E418&lt;&gt;""),IF(D418="",0,D418)+IF(E418="",0,E418),"")</f>
+        <f>IF(OR(D388&lt;&gt;"",E388&lt;&gt;""),IF(D388="",0,D388)+IF(E388="",0,E388),"")</f>
         <v/>
       </c>
       <c r="G434" s="14" t="n"/>
@@ -67051,7 +67251,7 @@
       <c r="D435" s="27" t="n"/>
       <c r="E435" s="28" t="n"/>
       <c r="F435" s="15">
-        <f>IF(OR(D419&lt;&gt;"",E419&lt;&gt;""),IF(D419="",0,D419)+IF(E419="",0,E419),"")</f>
+        <f>IF(OR(D389&lt;&gt;"",E389&lt;&gt;""),IF(D389="",0,D389)+IF(E389="",0,E389),"")</f>
         <v/>
       </c>
       <c r="G435" s="14" t="n"/>
@@ -67067,7 +67267,7 @@
       <c r="D436" s="27" t="n"/>
       <c r="E436" s="28" t="n"/>
       <c r="F436" s="15">
-        <f>IF(OR(D420&lt;&gt;"",E420&lt;&gt;""),IF(D420="",0,D420)+IF(E420="",0,E420),"")</f>
+        <f>IF(OR(D390&lt;&gt;"",E390&lt;&gt;""),IF(D390="",0,D390)+IF(E390="",0,E390),"")</f>
         <v/>
       </c>
       <c r="G436" s="14" t="n"/>
@@ -67083,41 +67283,47 @@
       <c r="D437" s="27" t="n"/>
       <c r="E437" s="28" t="n"/>
       <c r="F437" s="15">
-        <f>IF(OR(D421&lt;&gt;"",E421&lt;&gt;""),IF(D421="",0,D421)+IF(E421="",0,E421),"")</f>
+        <f>IF(OR(D391&lt;&gt;"",E391&lt;&gt;""),IF(D391="",0,D391)+IF(E391="",0,E391),"")</f>
         <v/>
       </c>
       <c r="G437" s="14" t="n"/>
     </row>
     <row r="438">
-      <c r="A438" s="10" t="inlineStr">
-        <is>
-          <t>TOTAL OCTUBRE</t>
-        </is>
-      </c>
-      <c r="B438" s="22" t="n"/>
-      <c r="C438" s="29" t="inlineStr">
-        <is>
-          <t>Totales mes →</t>
-        </is>
-      </c>
-      <c r="D438" s="7">
-        <f>SUMIFS($D$4:$D$600,$A$4:$A$600,"Octubre")</f>
+      <c r="A438" s="14" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="B438" s="17" t="n"/>
+      <c r="C438" s="14" t="n"/>
+      <c r="D438" s="27" t="n"/>
+      <c r="E438" s="28" t="n"/>
+      <c r="F438" s="15">
+        <f>IF(OR(D392&lt;&gt;"",E392&lt;&gt;""),IF(D392="",0,D392)+IF(E392="",0,E392),"")</f>
         <v/>
       </c>
-      <c r="E438" s="7">
-        <f>SUMIFS($E$4:$E$600,$A$4:$A$600,"Octubre")</f>
+      <c r="G438" s="14" t="n"/>
+    </row>
+    <row r="439">
+      <c r="A439" s="14" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="B439" s="17" t="n"/>
+      <c r="C439" s="14" t="n"/>
+      <c r="D439" s="27" t="n"/>
+      <c r="E439" s="28" t="n"/>
+      <c r="F439" s="15">
+        <f>IF(OR(D393&lt;&gt;"",E393&lt;&gt;""),IF(D393="",0,D393)+IF(E393="",0,E393),"")</f>
         <v/>
       </c>
-      <c r="F438" s="7">
-        <f>D438+E438</f>
-        <v/>
-      </c>
-      <c r="G438" s="22" t="n"/>
+      <c r="G439" s="14" t="n"/>
     </row>
     <row r="440">
       <c r="A440" s="14" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B440" s="17" t="n"/>
@@ -67125,7 +67331,7 @@
       <c r="D440" s="27" t="n"/>
       <c r="E440" s="28" t="n"/>
       <c r="F440" s="15">
-        <f>IF(OR(D424&lt;&gt;"",E424&lt;&gt;""),IF(D424="",0,D424)+IF(E424="",0,E424),"")</f>
+        <f>IF(OR(D394&lt;&gt;"",E394&lt;&gt;""),IF(D394="",0,D394)+IF(E394="",0,E394),"")</f>
         <v/>
       </c>
       <c r="G440" s="14" t="n"/>
@@ -67133,7 +67339,7 @@
     <row r="441">
       <c r="A441" s="14" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B441" s="17" t="n"/>
@@ -67141,7 +67347,7 @@
       <c r="D441" s="27" t="n"/>
       <c r="E441" s="28" t="n"/>
       <c r="F441" s="15">
-        <f>IF(OR(D425&lt;&gt;"",E425&lt;&gt;""),IF(D425="",0,D425)+IF(E425="",0,E425),"")</f>
+        <f>IF(OR(D395&lt;&gt;"",E395&lt;&gt;""),IF(D395="",0,D395)+IF(E395="",0,E395),"")</f>
         <v/>
       </c>
       <c r="G441" s="14" t="n"/>
@@ -67149,7 +67355,7 @@
     <row r="442">
       <c r="A442" s="14" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B442" s="17" t="n"/>
@@ -67157,7 +67363,7 @@
       <c r="D442" s="27" t="n"/>
       <c r="E442" s="28" t="n"/>
       <c r="F442" s="15">
-        <f>IF(OR(D426&lt;&gt;"",E426&lt;&gt;""),IF(D426="",0,D426)+IF(E426="",0,E426),"")</f>
+        <f>IF(OR(D396&lt;&gt;"",E396&lt;&gt;""),IF(D396="",0,D396)+IF(E396="",0,E396),"")</f>
         <v/>
       </c>
       <c r="G442" s="14" t="n"/>
@@ -67165,7 +67371,7 @@
     <row r="443">
       <c r="A443" s="14" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B443" s="17" t="n"/>
@@ -67173,7 +67379,7 @@
       <c r="D443" s="27" t="n"/>
       <c r="E443" s="28" t="n"/>
       <c r="F443" s="15">
-        <f>IF(OR(D427&lt;&gt;"",E427&lt;&gt;""),IF(D427="",0,D427)+IF(E427="",0,E427),"")</f>
+        <f>IF(OR(D397&lt;&gt;"",E397&lt;&gt;""),IF(D397="",0,D397)+IF(E397="",0,E397),"")</f>
         <v/>
       </c>
       <c r="G443" s="14" t="n"/>
@@ -67181,7 +67387,7 @@
     <row r="444">
       <c r="A444" s="14" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B444" s="17" t="n"/>
@@ -67189,7 +67395,7 @@
       <c r="D444" s="27" t="n"/>
       <c r="E444" s="28" t="n"/>
       <c r="F444" s="15">
-        <f>IF(OR(D428&lt;&gt;"",E428&lt;&gt;""),IF(D428="",0,D428)+IF(E428="",0,E428),"")</f>
+        <f>IF(OR(D398&lt;&gt;"",E398&lt;&gt;""),IF(D398="",0,D398)+IF(E398="",0,E398),"")</f>
         <v/>
       </c>
       <c r="G444" s="14" t="n"/>
@@ -67197,7 +67403,7 @@
     <row r="445">
       <c r="A445" s="14" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B445" s="17" t="n"/>
@@ -67205,7 +67411,7 @@
       <c r="D445" s="27" t="n"/>
       <c r="E445" s="28" t="n"/>
       <c r="F445" s="15">
-        <f>IF(OR(D429&lt;&gt;"",E429&lt;&gt;""),IF(D429="",0,D429)+IF(E429="",0,E429),"")</f>
+        <f>IF(OR(D399&lt;&gt;"",E399&lt;&gt;""),IF(D399="",0,D399)+IF(E399="",0,E399),"")</f>
         <v/>
       </c>
       <c r="G445" s="14" t="n"/>
@@ -67213,7 +67419,7 @@
     <row r="446">
       <c r="A446" s="14" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B446" s="17" t="n"/>
@@ -67221,7 +67427,7 @@
       <c r="D446" s="27" t="n"/>
       <c r="E446" s="28" t="n"/>
       <c r="F446" s="15">
-        <f>IF(OR(D430&lt;&gt;"",E430&lt;&gt;""),IF(D430="",0,D430)+IF(E430="",0,E430),"")</f>
+        <f>IF(OR(D400&lt;&gt;"",E400&lt;&gt;""),IF(D400="",0,D400)+IF(E400="",0,E400),"")</f>
         <v/>
       </c>
       <c r="G446" s="14" t="n"/>
@@ -67229,7 +67435,7 @@
     <row r="447">
       <c r="A447" s="14" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B447" s="17" t="n"/>
@@ -67237,7 +67443,7 @@
       <c r="D447" s="27" t="n"/>
       <c r="E447" s="28" t="n"/>
       <c r="F447" s="15">
-        <f>IF(OR(D431&lt;&gt;"",E431&lt;&gt;""),IF(D431="",0,D431)+IF(E431="",0,E431),"")</f>
+        <f>IF(OR(D401&lt;&gt;"",E401&lt;&gt;""),IF(D401="",0,D401)+IF(E401="",0,E401),"")</f>
         <v/>
       </c>
       <c r="G447" s="14" t="n"/>
@@ -67245,7 +67451,7 @@
     <row r="448">
       <c r="A448" s="14" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B448" s="17" t="n"/>
@@ -67253,7 +67459,7 @@
       <c r="D448" s="27" t="n"/>
       <c r="E448" s="28" t="n"/>
       <c r="F448" s="15">
-        <f>IF(OR(D432&lt;&gt;"",E432&lt;&gt;""),IF(D432="",0,D432)+IF(E432="",0,E432),"")</f>
+        <f>IF(OR(D402&lt;&gt;"",E402&lt;&gt;""),IF(D402="",0,D402)+IF(E402="",0,E402),"")</f>
         <v/>
       </c>
       <c r="G448" s="14" t="n"/>
@@ -67261,7 +67467,7 @@
     <row r="449">
       <c r="A449" s="14" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B449" s="17" t="n"/>
@@ -67269,7 +67475,7 @@
       <c r="D449" s="27" t="n"/>
       <c r="E449" s="28" t="n"/>
       <c r="F449" s="15">
-        <f>IF(OR(D433&lt;&gt;"",E433&lt;&gt;""),IF(D433="",0,D433)+IF(E433="",0,E433),"")</f>
+        <f>IF(OR(D403&lt;&gt;"",E403&lt;&gt;""),IF(D403="",0,D403)+IF(E403="",0,E403),"")</f>
         <v/>
       </c>
       <c r="G449" s="14" t="n"/>
@@ -67277,7 +67483,7 @@
     <row r="450">
       <c r="A450" s="14" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B450" s="17" t="n"/>
@@ -67285,7 +67491,7 @@
       <c r="D450" s="27" t="n"/>
       <c r="E450" s="28" t="n"/>
       <c r="F450" s="15">
-        <f>IF(OR(D434&lt;&gt;"",E434&lt;&gt;""),IF(D434="",0,D434)+IF(E434="",0,E434),"")</f>
+        <f>IF(OR(D404&lt;&gt;"",E404&lt;&gt;""),IF(D404="",0,D404)+IF(E404="",0,E404),"")</f>
         <v/>
       </c>
       <c r="G450" s="14" t="n"/>
@@ -67293,7 +67499,7 @@
     <row r="451">
       <c r="A451" s="14" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B451" s="17" t="n"/>
@@ -67301,7 +67507,7 @@
       <c r="D451" s="27" t="n"/>
       <c r="E451" s="28" t="n"/>
       <c r="F451" s="15">
-        <f>IF(OR(D435&lt;&gt;"",E435&lt;&gt;""),IF(D435="",0,D435)+IF(E435="",0,E435),"")</f>
+        <f>IF(OR(D405&lt;&gt;"",E405&lt;&gt;""),IF(D405="",0,D405)+IF(E405="",0,E405),"")</f>
         <v/>
       </c>
       <c r="G451" s="14" t="n"/>
@@ -67309,7 +67515,7 @@
     <row r="452">
       <c r="A452" s="14" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B452" s="17" t="n"/>
@@ -67317,7 +67523,7 @@
       <c r="D452" s="27" t="n"/>
       <c r="E452" s="28" t="n"/>
       <c r="F452" s="15">
-        <f>IF(OR(D436&lt;&gt;"",E436&lt;&gt;""),IF(D436="",0,D436)+IF(E436="",0,E436),"")</f>
+        <f>IF(OR(D406&lt;&gt;"",E406&lt;&gt;""),IF(D406="",0,D406)+IF(E406="",0,E406),"")</f>
         <v/>
       </c>
       <c r="G452" s="14" t="n"/>
@@ -67325,7 +67531,7 @@
     <row r="453">
       <c r="A453" s="14" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B453" s="17" t="n"/>
@@ -67333,7 +67539,7 @@
       <c r="D453" s="27" t="n"/>
       <c r="E453" s="28" t="n"/>
       <c r="F453" s="15">
-        <f>IF(OR(D437&lt;&gt;"",E437&lt;&gt;""),IF(D437="",0,D437)+IF(E437="",0,E437),"")</f>
+        <f>IF(OR(D407&lt;&gt;"",E407&lt;&gt;""),IF(D407="",0,D407)+IF(E407="",0,E407),"")</f>
         <v/>
       </c>
       <c r="G453" s="14" t="n"/>
@@ -67341,7 +67547,7 @@
     <row r="454">
       <c r="A454" s="14" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B454" s="17" t="n"/>
@@ -67349,7 +67555,7 @@
       <c r="D454" s="27" t="n"/>
       <c r="E454" s="28" t="n"/>
       <c r="F454" s="15">
-        <f>IF(OR(D438&lt;&gt;"",E438&lt;&gt;""),IF(D438="",0,D438)+IF(E438="",0,E438),"")</f>
+        <f>IF(OR(D408&lt;&gt;"",E408&lt;&gt;""),IF(D408="",0,D408)+IF(E408="",0,E408),"")</f>
         <v/>
       </c>
       <c r="G454" s="14" t="n"/>
@@ -67357,7 +67563,7 @@
     <row r="455">
       <c r="A455" s="14" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B455" s="17" t="n"/>
@@ -67365,7 +67571,7 @@
       <c r="D455" s="27" t="n"/>
       <c r="E455" s="28" t="n"/>
       <c r="F455" s="15">
-        <f>IF(OR(D439&lt;&gt;"",E439&lt;&gt;""),IF(D439="",0,D439)+IF(E439="",0,E439),"")</f>
+        <f>IF(OR(D409&lt;&gt;"",E409&lt;&gt;""),IF(D409="",0,D409)+IF(E409="",0,E409),"")</f>
         <v/>
       </c>
       <c r="G455" s="14" t="n"/>
@@ -67373,7 +67579,7 @@
     <row r="456">
       <c r="A456" s="14" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B456" s="17" t="n"/>
@@ -67381,7 +67587,7 @@
       <c r="D456" s="27" t="n"/>
       <c r="E456" s="28" t="n"/>
       <c r="F456" s="15">
-        <f>IF(OR(D440&lt;&gt;"",E440&lt;&gt;""),IF(D440="",0,D440)+IF(E440="",0,E440),"")</f>
+        <f>IF(OR(D410&lt;&gt;"",E410&lt;&gt;""),IF(D410="",0,D410)+IF(E410="",0,E410),"")</f>
         <v/>
       </c>
       <c r="G456" s="14" t="n"/>
@@ -67389,7 +67595,7 @@
     <row r="457">
       <c r="A457" s="14" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B457" s="17" t="n"/>
@@ -67397,7 +67603,7 @@
       <c r="D457" s="27" t="n"/>
       <c r="E457" s="28" t="n"/>
       <c r="F457" s="15">
-        <f>IF(OR(D441&lt;&gt;"",E441&lt;&gt;""),IF(D441="",0,D441)+IF(E441="",0,E441),"")</f>
+        <f>IF(OR(D411&lt;&gt;"",E411&lt;&gt;""),IF(D411="",0,D411)+IF(E411="",0,E411),"")</f>
         <v/>
       </c>
       <c r="G457" s="14" t="n"/>
@@ -67405,7 +67611,7 @@
     <row r="458">
       <c r="A458" s="14" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B458" s="17" t="n"/>
@@ -67413,7 +67619,7 @@
       <c r="D458" s="27" t="n"/>
       <c r="E458" s="28" t="n"/>
       <c r="F458" s="15">
-        <f>IF(OR(D442&lt;&gt;"",E442&lt;&gt;""),IF(D442="",0,D442)+IF(E442="",0,E442),"")</f>
+        <f>IF(OR(D412&lt;&gt;"",E412&lt;&gt;""),IF(D412="",0,D412)+IF(E412="",0,E412),"")</f>
         <v/>
       </c>
       <c r="G458" s="14" t="n"/>
@@ -67421,7 +67627,7 @@
     <row r="459">
       <c r="A459" s="14" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B459" s="17" t="n"/>
@@ -67429,7 +67635,7 @@
       <c r="D459" s="27" t="n"/>
       <c r="E459" s="28" t="n"/>
       <c r="F459" s="15">
-        <f>IF(OR(D443&lt;&gt;"",E443&lt;&gt;""),IF(D443="",0,D443)+IF(E443="",0,E443),"")</f>
+        <f>IF(OR(D413&lt;&gt;"",E413&lt;&gt;""),IF(D413="",0,D413)+IF(E413="",0,E413),"")</f>
         <v/>
       </c>
       <c r="G459" s="14" t="n"/>
@@ -67437,7 +67643,7 @@
     <row r="460">
       <c r="A460" s="14" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B460" s="17" t="n"/>
@@ -67445,7 +67651,7 @@
       <c r="D460" s="27" t="n"/>
       <c r="E460" s="28" t="n"/>
       <c r="F460" s="15">
-        <f>IF(OR(D444&lt;&gt;"",E444&lt;&gt;""),IF(D444="",0,D444)+IF(E444="",0,E444),"")</f>
+        <f>IF(OR(D414&lt;&gt;"",E414&lt;&gt;""),IF(D414="",0,D414)+IF(E414="",0,E414),"")</f>
         <v/>
       </c>
       <c r="G460" s="14" t="n"/>
@@ -67453,7 +67659,7 @@
     <row r="461">
       <c r="A461" s="14" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B461" s="17" t="n"/>
@@ -67461,7 +67667,7 @@
       <c r="D461" s="27" t="n"/>
       <c r="E461" s="28" t="n"/>
       <c r="F461" s="15">
-        <f>IF(OR(D445&lt;&gt;"",E445&lt;&gt;""),IF(D445="",0,D445)+IF(E445="",0,E445),"")</f>
+        <f>IF(OR(D415&lt;&gt;"",E415&lt;&gt;""),IF(D415="",0,D415)+IF(E415="",0,E415),"")</f>
         <v/>
       </c>
       <c r="G461" s="14" t="n"/>
@@ -67469,7 +67675,7 @@
     <row r="462">
       <c r="A462" s="14" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B462" s="17" t="n"/>
@@ -67477,7 +67683,7 @@
       <c r="D462" s="27" t="n"/>
       <c r="E462" s="28" t="n"/>
       <c r="F462" s="15">
-        <f>IF(OR(D446&lt;&gt;"",E446&lt;&gt;""),IF(D446="",0,D446)+IF(E446="",0,E446),"")</f>
+        <f>IF(OR(D416&lt;&gt;"",E416&lt;&gt;""),IF(D416="",0,D416)+IF(E416="",0,E416),"")</f>
         <v/>
       </c>
       <c r="G462" s="14" t="n"/>
@@ -67485,7 +67691,7 @@
     <row r="463">
       <c r="A463" s="14" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B463" s="17" t="n"/>
@@ -67493,7 +67699,7 @@
       <c r="D463" s="27" t="n"/>
       <c r="E463" s="28" t="n"/>
       <c r="F463" s="15">
-        <f>IF(OR(D447&lt;&gt;"",E447&lt;&gt;""),IF(D447="",0,D447)+IF(E447="",0,E447),"")</f>
+        <f>IF(OR(D417&lt;&gt;"",E417&lt;&gt;""),IF(D417="",0,D417)+IF(E417="",0,E417),"")</f>
         <v/>
       </c>
       <c r="G463" s="14" t="n"/>
@@ -67501,7 +67707,7 @@
     <row r="464">
       <c r="A464" s="14" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B464" s="17" t="n"/>
@@ -67509,7 +67715,7 @@
       <c r="D464" s="27" t="n"/>
       <c r="E464" s="28" t="n"/>
       <c r="F464" s="15">
-        <f>IF(OR(D448&lt;&gt;"",E448&lt;&gt;""),IF(D448="",0,D448)+IF(E448="",0,E448),"")</f>
+        <f>IF(OR(D418&lt;&gt;"",E418&lt;&gt;""),IF(D418="",0,D418)+IF(E418="",0,E418),"")</f>
         <v/>
       </c>
       <c r="G464" s="14" t="n"/>
@@ -67517,7 +67723,7 @@
     <row r="465">
       <c r="A465" s="14" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B465" s="17" t="n"/>
@@ -67525,7 +67731,7 @@
       <c r="D465" s="27" t="n"/>
       <c r="E465" s="28" t="n"/>
       <c r="F465" s="15">
-        <f>IF(OR(D449&lt;&gt;"",E449&lt;&gt;""),IF(D449="",0,D449)+IF(E449="",0,E449),"")</f>
+        <f>IF(OR(D419&lt;&gt;"",E419&lt;&gt;""),IF(D419="",0,D419)+IF(E419="",0,E419),"")</f>
         <v/>
       </c>
       <c r="G465" s="14" t="n"/>
@@ -67533,7 +67739,7 @@
     <row r="466">
       <c r="A466" s="14" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B466" s="17" t="n"/>
@@ -67541,7 +67747,7 @@
       <c r="D466" s="27" t="n"/>
       <c r="E466" s="28" t="n"/>
       <c r="F466" s="15">
-        <f>IF(OR(D450&lt;&gt;"",E450&lt;&gt;""),IF(D450="",0,D450)+IF(E450="",0,E450),"")</f>
+        <f>IF(OR(D420&lt;&gt;"",E420&lt;&gt;""),IF(D420="",0,D420)+IF(E420="",0,E420),"")</f>
         <v/>
       </c>
       <c r="G466" s="14" t="n"/>
@@ -67549,7 +67755,7 @@
     <row r="467">
       <c r="A467" s="14" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B467" s="17" t="n"/>
@@ -67557,43 +67763,38 @@
       <c r="D467" s="27" t="n"/>
       <c r="E467" s="28" t="n"/>
       <c r="F467" s="15">
-        <f>IF(OR(D451&lt;&gt;"",E451&lt;&gt;""),IF(D451="",0,D451)+IF(E451="",0,E451),"")</f>
+        <f>IF(OR(D421&lt;&gt;"",E421&lt;&gt;""),IF(D421="",0,D421)+IF(E421="",0,E421),"")</f>
         <v/>
       </c>
       <c r="G467" s="14" t="n"/>
     </row>
     <row r="468">
-      <c r="A468" s="14" t="inlineStr">
-        <is>
-          <t>Noviembre</t>
-        </is>
-      </c>
-      <c r="B468" s="17" t="n"/>
-      <c r="C468" s="14" t="n"/>
-      <c r="D468" s="27" t="n"/>
-      <c r="E468" s="28" t="n"/>
-      <c r="F468" s="15">
-        <f>IF(OR(D452&lt;&gt;"",E452&lt;&gt;""),IF(D452="",0,D452)+IF(E452="",0,E452),"")</f>
+      <c r="A468" s="10" t="inlineStr">
+        <is>
+          <t>TOTAL OCTUBRE</t>
+        </is>
+      </c>
+      <c r="B468" s="22" t="n"/>
+      <c r="C468" s="29" t="inlineStr">
+        <is>
+          <t>Totales mes →</t>
+        </is>
+      </c>
+      <c r="D468" s="7">
+        <f>SUMIFS($D$4:$D$800,$A$4:$A$800,"Octubre")</f>
         <v/>
       </c>
-      <c r="G468" s="14" t="n"/>
-    </row>
-    <row r="469">
-      <c r="A469" s="14" t="inlineStr">
-        <is>
-          <t>Noviembre</t>
-        </is>
-      </c>
-      <c r="B469" s="17" t="n"/>
-      <c r="C469" s="14" t="n"/>
-      <c r="D469" s="27" t="n"/>
-      <c r="E469" s="28" t="n"/>
-      <c r="F469" s="15">
-        <f>IF(OR(D453&lt;&gt;"",E453&lt;&gt;""),IF(D453="",0,D453)+IF(E453="",0,E453),"")</f>
+      <c r="E468" s="7">
+        <f>SUMIFS($E$4:$E$800,$A$4:$A$800,"Octubre")</f>
         <v/>
       </c>
-      <c r="G469" s="14" t="n"/>
-    </row>
+      <c r="F468" s="7">
+        <f>D468+E468</f>
+        <v/>
+      </c>
+      <c r="G468" s="22" t="n"/>
+    </row>
+    <row r="469"/>
     <row r="470">
       <c r="A470" s="14" t="inlineStr">
         <is>
@@ -67605,7 +67806,7 @@
       <c r="D470" s="27" t="n"/>
       <c r="E470" s="28" t="n"/>
       <c r="F470" s="15">
-        <f>IF(OR(D454&lt;&gt;"",E454&lt;&gt;""),IF(D454="",0,D454)+IF(E454="",0,E454),"")</f>
+        <f>IF(OR(D424&lt;&gt;"",E424&lt;&gt;""),IF(D424="",0,D424)+IF(E424="",0,E424),"")</f>
         <v/>
       </c>
       <c r="G470" s="14" t="n"/>
@@ -67621,7 +67822,7 @@
       <c r="D471" s="27" t="n"/>
       <c r="E471" s="28" t="n"/>
       <c r="F471" s="15">
-        <f>IF(OR(D455&lt;&gt;"",E455&lt;&gt;""),IF(D455="",0,D455)+IF(E455="",0,E455),"")</f>
+        <f>IF(OR(D425&lt;&gt;"",E425&lt;&gt;""),IF(D425="",0,D425)+IF(E425="",0,E425),"")</f>
         <v/>
       </c>
       <c r="G471" s="14" t="n"/>
@@ -67637,7 +67838,7 @@
       <c r="D472" s="27" t="n"/>
       <c r="E472" s="28" t="n"/>
       <c r="F472" s="15">
-        <f>IF(OR(D456&lt;&gt;"",E456&lt;&gt;""),IF(D456="",0,D456)+IF(E456="",0,E456),"")</f>
+        <f>IF(OR(D426&lt;&gt;"",E426&lt;&gt;""),IF(D426="",0,D426)+IF(E426="",0,E426),"")</f>
         <v/>
       </c>
       <c r="G472" s="14" t="n"/>
@@ -67653,7 +67854,7 @@
       <c r="D473" s="27" t="n"/>
       <c r="E473" s="28" t="n"/>
       <c r="F473" s="15">
-        <f>IF(OR(D457&lt;&gt;"",E457&lt;&gt;""),IF(D457="",0,D457)+IF(E457="",0,E457),"")</f>
+        <f>IF(OR(D427&lt;&gt;"",E427&lt;&gt;""),IF(D427="",0,D427)+IF(E427="",0,E427),"")</f>
         <v/>
       </c>
       <c r="G473" s="14" t="n"/>
@@ -67669,7 +67870,7 @@
       <c r="D474" s="27" t="n"/>
       <c r="E474" s="28" t="n"/>
       <c r="F474" s="15">
-        <f>IF(OR(D458&lt;&gt;"",E458&lt;&gt;""),IF(D458="",0,D458)+IF(E458="",0,E458),"")</f>
+        <f>IF(OR(D428&lt;&gt;"",E428&lt;&gt;""),IF(D428="",0,D428)+IF(E428="",0,E428),"")</f>
         <v/>
       </c>
       <c r="G474" s="14" t="n"/>
@@ -67685,7 +67886,7 @@
       <c r="D475" s="27" t="n"/>
       <c r="E475" s="28" t="n"/>
       <c r="F475" s="15">
-        <f>IF(OR(D459&lt;&gt;"",E459&lt;&gt;""),IF(D459="",0,D459)+IF(E459="",0,E459),"")</f>
+        <f>IF(OR(D429&lt;&gt;"",E429&lt;&gt;""),IF(D429="",0,D429)+IF(E429="",0,E429),"")</f>
         <v/>
       </c>
       <c r="G475" s="14" t="n"/>
@@ -67701,7 +67902,7 @@
       <c r="D476" s="27" t="n"/>
       <c r="E476" s="28" t="n"/>
       <c r="F476" s="15">
-        <f>IF(OR(D460&lt;&gt;"",E460&lt;&gt;""),IF(D460="",0,D460)+IF(E460="",0,E460),"")</f>
+        <f>IF(OR(D430&lt;&gt;"",E430&lt;&gt;""),IF(D430="",0,D430)+IF(E430="",0,E430),"")</f>
         <v/>
       </c>
       <c r="G476" s="14" t="n"/>
@@ -67717,7 +67918,7 @@
       <c r="D477" s="27" t="n"/>
       <c r="E477" s="28" t="n"/>
       <c r="F477" s="15">
-        <f>IF(OR(D461&lt;&gt;"",E461&lt;&gt;""),IF(D461="",0,D461)+IF(E461="",0,E461),"")</f>
+        <f>IF(OR(D431&lt;&gt;"",E431&lt;&gt;""),IF(D431="",0,D431)+IF(E431="",0,E431),"")</f>
         <v/>
       </c>
       <c r="G477" s="14" t="n"/>
@@ -67733,7 +67934,7 @@
       <c r="D478" s="27" t="n"/>
       <c r="E478" s="28" t="n"/>
       <c r="F478" s="15">
-        <f>IF(OR(D462&lt;&gt;"",E462&lt;&gt;""),IF(D462="",0,D462)+IF(E462="",0,E462),"")</f>
+        <f>IF(OR(D432&lt;&gt;"",E432&lt;&gt;""),IF(D432="",0,D432)+IF(E432="",0,E432),"")</f>
         <v/>
       </c>
       <c r="G478" s="14" t="n"/>
@@ -67749,41 +67950,47 @@
       <c r="D479" s="27" t="n"/>
       <c r="E479" s="28" t="n"/>
       <c r="F479" s="15">
-        <f>IF(OR(D463&lt;&gt;"",E463&lt;&gt;""),IF(D463="",0,D463)+IF(E463="",0,E463),"")</f>
+        <f>IF(OR(D433&lt;&gt;"",E433&lt;&gt;""),IF(D433="",0,D433)+IF(E433="",0,E433),"")</f>
         <v/>
       </c>
       <c r="G479" s="14" t="n"/>
     </row>
     <row r="480">
-      <c r="A480" s="10" t="inlineStr">
-        <is>
-          <t>TOTAL NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="B480" s="22" t="n"/>
-      <c r="C480" s="29" t="inlineStr">
-        <is>
-          <t>Totales mes →</t>
-        </is>
-      </c>
-      <c r="D480" s="7">
-        <f>SUMIFS($D$4:$D$600,$A$4:$A$600,"Noviembre")</f>
+      <c r="A480" s="14" t="inlineStr">
+        <is>
+          <t>Noviembre</t>
+        </is>
+      </c>
+      <c r="B480" s="17" t="n"/>
+      <c r="C480" s="14" t="n"/>
+      <c r="D480" s="27" t="n"/>
+      <c r="E480" s="28" t="n"/>
+      <c r="F480" s="15">
+        <f>IF(OR(D434&lt;&gt;"",E434&lt;&gt;""),IF(D434="",0,D434)+IF(E434="",0,E434),"")</f>
         <v/>
       </c>
-      <c r="E480" s="7">
-        <f>SUMIFS($E$4:$E$600,$A$4:$A$600,"Noviembre")</f>
+      <c r="G480" s="14" t="n"/>
+    </row>
+    <row r="481">
+      <c r="A481" s="14" t="inlineStr">
+        <is>
+          <t>Noviembre</t>
+        </is>
+      </c>
+      <c r="B481" s="17" t="n"/>
+      <c r="C481" s="14" t="n"/>
+      <c r="D481" s="27" t="n"/>
+      <c r="E481" s="28" t="n"/>
+      <c r="F481" s="15">
+        <f>IF(OR(D435&lt;&gt;"",E435&lt;&gt;""),IF(D435="",0,D435)+IF(E435="",0,E435),"")</f>
         <v/>
       </c>
-      <c r="F480" s="7">
-        <f>D480+E480</f>
-        <v/>
-      </c>
-      <c r="G480" s="22" t="n"/>
+      <c r="G481" s="14" t="n"/>
     </row>
     <row r="482">
       <c r="A482" s="14" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B482" s="17" t="n"/>
@@ -67791,7 +67998,7 @@
       <c r="D482" s="27" t="n"/>
       <c r="E482" s="28" t="n"/>
       <c r="F482" s="15">
-        <f>IF(OR(D466&lt;&gt;"",E466&lt;&gt;""),IF(D466="",0,D466)+IF(E466="",0,E466),"")</f>
+        <f>IF(OR(D436&lt;&gt;"",E436&lt;&gt;""),IF(D436="",0,D436)+IF(E436="",0,E436),"")</f>
         <v/>
       </c>
       <c r="G482" s="14" t="n"/>
@@ -67799,7 +68006,7 @@
     <row r="483">
       <c r="A483" s="14" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B483" s="17" t="n"/>
@@ -67807,7 +68014,7 @@
       <c r="D483" s="27" t="n"/>
       <c r="E483" s="28" t="n"/>
       <c r="F483" s="15">
-        <f>IF(OR(D467&lt;&gt;"",E467&lt;&gt;""),IF(D467="",0,D467)+IF(E467="",0,E467),"")</f>
+        <f>IF(OR(D437&lt;&gt;"",E437&lt;&gt;""),IF(D437="",0,D437)+IF(E437="",0,E437),"")</f>
         <v/>
       </c>
       <c r="G483" s="14" t="n"/>
@@ -67815,7 +68022,7 @@
     <row r="484">
       <c r="A484" s="14" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B484" s="17" t="n"/>
@@ -67823,7 +68030,7 @@
       <c r="D484" s="27" t="n"/>
       <c r="E484" s="28" t="n"/>
       <c r="F484" s="15">
-        <f>IF(OR(D468&lt;&gt;"",E468&lt;&gt;""),IF(D468="",0,D468)+IF(E468="",0,E468),"")</f>
+        <f>IF(OR(D438&lt;&gt;"",E438&lt;&gt;""),IF(D438="",0,D438)+IF(E438="",0,E438),"")</f>
         <v/>
       </c>
       <c r="G484" s="14" t="n"/>
@@ -67831,7 +68038,7 @@
     <row r="485">
       <c r="A485" s="14" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B485" s="17" t="n"/>
@@ -67839,7 +68046,7 @@
       <c r="D485" s="27" t="n"/>
       <c r="E485" s="28" t="n"/>
       <c r="F485" s="15">
-        <f>IF(OR(D469&lt;&gt;"",E469&lt;&gt;""),IF(D469="",0,D469)+IF(E469="",0,E469),"")</f>
+        <f>IF(OR(D439&lt;&gt;"",E439&lt;&gt;""),IF(D439="",0,D439)+IF(E439="",0,E439),"")</f>
         <v/>
       </c>
       <c r="G485" s="14" t="n"/>
@@ -67847,7 +68054,7 @@
     <row r="486">
       <c r="A486" s="14" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B486" s="17" t="n"/>
@@ -67855,7 +68062,7 @@
       <c r="D486" s="27" t="n"/>
       <c r="E486" s="28" t="n"/>
       <c r="F486" s="15">
-        <f>IF(OR(D470&lt;&gt;"",E470&lt;&gt;""),IF(D470="",0,D470)+IF(E470="",0,E470),"")</f>
+        <f>IF(OR(D440&lt;&gt;"",E440&lt;&gt;""),IF(D440="",0,D440)+IF(E440="",0,E440),"")</f>
         <v/>
       </c>
       <c r="G486" s="14" t="n"/>
@@ -67863,7 +68070,7 @@
     <row r="487">
       <c r="A487" s="14" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B487" s="17" t="n"/>
@@ -67871,7 +68078,7 @@
       <c r="D487" s="27" t="n"/>
       <c r="E487" s="28" t="n"/>
       <c r="F487" s="15">
-        <f>IF(OR(D471&lt;&gt;"",E471&lt;&gt;""),IF(D471="",0,D471)+IF(E471="",0,E471),"")</f>
+        <f>IF(OR(D441&lt;&gt;"",E441&lt;&gt;""),IF(D441="",0,D441)+IF(E441="",0,E441),"")</f>
         <v/>
       </c>
       <c r="G487" s="14" t="n"/>
@@ -67879,7 +68086,7 @@
     <row r="488">
       <c r="A488" s="14" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B488" s="17" t="n"/>
@@ -67887,7 +68094,7 @@
       <c r="D488" s="27" t="n"/>
       <c r="E488" s="28" t="n"/>
       <c r="F488" s="15">
-        <f>IF(OR(D472&lt;&gt;"",E472&lt;&gt;""),IF(D472="",0,D472)+IF(E472="",0,E472),"")</f>
+        <f>IF(OR(D442&lt;&gt;"",E442&lt;&gt;""),IF(D442="",0,D442)+IF(E442="",0,E442),"")</f>
         <v/>
       </c>
       <c r="G488" s="14" t="n"/>
@@ -67895,7 +68102,7 @@
     <row r="489">
       <c r="A489" s="14" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B489" s="17" t="n"/>
@@ -67903,7 +68110,7 @@
       <c r="D489" s="27" t="n"/>
       <c r="E489" s="28" t="n"/>
       <c r="F489" s="15">
-        <f>IF(OR(D473&lt;&gt;"",E473&lt;&gt;""),IF(D473="",0,D473)+IF(E473="",0,E473),"")</f>
+        <f>IF(OR(D443&lt;&gt;"",E443&lt;&gt;""),IF(D443="",0,D443)+IF(E443="",0,E443),"")</f>
         <v/>
       </c>
       <c r="G489" s="14" t="n"/>
@@ -67911,7 +68118,7 @@
     <row r="490">
       <c r="A490" s="14" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B490" s="17" t="n"/>
@@ -67919,7 +68126,7 @@
       <c r="D490" s="27" t="n"/>
       <c r="E490" s="28" t="n"/>
       <c r="F490" s="15">
-        <f>IF(OR(D474&lt;&gt;"",E474&lt;&gt;""),IF(D474="",0,D474)+IF(E474="",0,E474),"")</f>
+        <f>IF(OR(D444&lt;&gt;"",E444&lt;&gt;""),IF(D444="",0,D444)+IF(E444="",0,E444),"")</f>
         <v/>
       </c>
       <c r="G490" s="14" t="n"/>
@@ -67927,7 +68134,7 @@
     <row r="491">
       <c r="A491" s="14" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B491" s="17" t="n"/>
@@ -67935,7 +68142,7 @@
       <c r="D491" s="27" t="n"/>
       <c r="E491" s="28" t="n"/>
       <c r="F491" s="15">
-        <f>IF(OR(D475&lt;&gt;"",E475&lt;&gt;""),IF(D475="",0,D475)+IF(E475="",0,E475),"")</f>
+        <f>IF(OR(D445&lt;&gt;"",E445&lt;&gt;""),IF(D445="",0,D445)+IF(E445="",0,E445),"")</f>
         <v/>
       </c>
       <c r="G491" s="14" t="n"/>
@@ -67943,7 +68150,7 @@
     <row r="492">
       <c r="A492" s="14" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B492" s="17" t="n"/>
@@ -67951,7 +68158,7 @@
       <c r="D492" s="27" t="n"/>
       <c r="E492" s="28" t="n"/>
       <c r="F492" s="15">
-        <f>IF(OR(D476&lt;&gt;"",E476&lt;&gt;""),IF(D476="",0,D476)+IF(E476="",0,E476),"")</f>
+        <f>IF(OR(D446&lt;&gt;"",E446&lt;&gt;""),IF(D446="",0,D446)+IF(E446="",0,E446),"")</f>
         <v/>
       </c>
       <c r="G492" s="14" t="n"/>
@@ -67959,7 +68166,7 @@
     <row r="493">
       <c r="A493" s="14" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B493" s="17" t="n"/>
@@ -67967,7 +68174,7 @@
       <c r="D493" s="27" t="n"/>
       <c r="E493" s="28" t="n"/>
       <c r="F493" s="15">
-        <f>IF(OR(D477&lt;&gt;"",E477&lt;&gt;""),IF(D477="",0,D477)+IF(E477="",0,E477),"")</f>
+        <f>IF(OR(D447&lt;&gt;"",E447&lt;&gt;""),IF(D447="",0,D447)+IF(E447="",0,E447),"")</f>
         <v/>
       </c>
       <c r="G493" s="14" t="n"/>
@@ -67975,7 +68182,7 @@
     <row r="494">
       <c r="A494" s="14" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B494" s="17" t="n"/>
@@ -67983,7 +68190,7 @@
       <c r="D494" s="27" t="n"/>
       <c r="E494" s="28" t="n"/>
       <c r="F494" s="15">
-        <f>IF(OR(D478&lt;&gt;"",E478&lt;&gt;""),IF(D478="",0,D478)+IF(E478="",0,E478),"")</f>
+        <f>IF(OR(D448&lt;&gt;"",E448&lt;&gt;""),IF(D448="",0,D448)+IF(E448="",0,E448),"")</f>
         <v/>
       </c>
       <c r="G494" s="14" t="n"/>
@@ -67991,7 +68198,7 @@
     <row r="495">
       <c r="A495" s="14" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B495" s="17" t="n"/>
@@ -67999,7 +68206,7 @@
       <c r="D495" s="27" t="n"/>
       <c r="E495" s="28" t="n"/>
       <c r="F495" s="15">
-        <f>IF(OR(D479&lt;&gt;"",E479&lt;&gt;""),IF(D479="",0,D479)+IF(E479="",0,E479),"")</f>
+        <f>IF(OR(D449&lt;&gt;"",E449&lt;&gt;""),IF(D449="",0,D449)+IF(E449="",0,E449),"")</f>
         <v/>
       </c>
       <c r="G495" s="14" t="n"/>
@@ -68007,7 +68214,7 @@
     <row r="496">
       <c r="A496" s="14" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B496" s="17" t="n"/>
@@ -68015,7 +68222,7 @@
       <c r="D496" s="27" t="n"/>
       <c r="E496" s="28" t="n"/>
       <c r="F496" s="15">
-        <f>IF(OR(D480&lt;&gt;"",E480&lt;&gt;""),IF(D480="",0,D480)+IF(E480="",0,E480),"")</f>
+        <f>IF(OR(D450&lt;&gt;"",E450&lt;&gt;""),IF(D450="",0,D450)+IF(E450="",0,E450),"")</f>
         <v/>
       </c>
       <c r="G496" s="14" t="n"/>
@@ -68023,7 +68230,7 @@
     <row r="497">
       <c r="A497" s="14" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B497" s="17" t="n"/>
@@ -68031,7 +68238,7 @@
       <c r="D497" s="27" t="n"/>
       <c r="E497" s="28" t="n"/>
       <c r="F497" s="15">
-        <f>IF(OR(D481&lt;&gt;"",E481&lt;&gt;""),IF(D481="",0,D481)+IF(E481="",0,E481),"")</f>
+        <f>IF(OR(D451&lt;&gt;"",E451&lt;&gt;""),IF(D451="",0,D451)+IF(E451="",0,E451),"")</f>
         <v/>
       </c>
       <c r="G497" s="14" t="n"/>
@@ -68039,7 +68246,7 @@
     <row r="498">
       <c r="A498" s="14" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B498" s="17" t="n"/>
@@ -68047,7 +68254,7 @@
       <c r="D498" s="27" t="n"/>
       <c r="E498" s="28" t="n"/>
       <c r="F498" s="15">
-        <f>IF(OR(D482&lt;&gt;"",E482&lt;&gt;""),IF(D482="",0,D482)+IF(E482="",0,E482),"")</f>
+        <f>IF(OR(D452&lt;&gt;"",E452&lt;&gt;""),IF(D452="",0,D452)+IF(E452="",0,E452),"")</f>
         <v/>
       </c>
       <c r="G498" s="14" t="n"/>
@@ -68055,7 +68262,7 @@
     <row r="499">
       <c r="A499" s="14" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B499" s="17" t="n"/>
@@ -68063,7 +68270,7 @@
       <c r="D499" s="27" t="n"/>
       <c r="E499" s="28" t="n"/>
       <c r="F499" s="15">
-        <f>IF(OR(D483&lt;&gt;"",E483&lt;&gt;""),IF(D483="",0,D483)+IF(E483="",0,E483),"")</f>
+        <f>IF(OR(D453&lt;&gt;"",E453&lt;&gt;""),IF(D453="",0,D453)+IF(E453="",0,E453),"")</f>
         <v/>
       </c>
       <c r="G499" s="14" t="n"/>
@@ -68071,7 +68278,7 @@
     <row r="500">
       <c r="A500" s="14" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B500" s="17" t="n"/>
@@ -68079,7 +68286,7 @@
       <c r="D500" s="27" t="n"/>
       <c r="E500" s="28" t="n"/>
       <c r="F500" s="15">
-        <f>IF(OR(D484&lt;&gt;"",E484&lt;&gt;""),IF(D484="",0,D484)+IF(E484="",0,E484),"")</f>
+        <f>IF(OR(D454&lt;&gt;"",E454&lt;&gt;""),IF(D454="",0,D454)+IF(E454="",0,E454),"")</f>
         <v/>
       </c>
       <c r="G500" s="14" t="n"/>
@@ -68087,7 +68294,7 @@
     <row r="501">
       <c r="A501" s="14" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B501" s="17" t="n"/>
@@ -68095,7 +68302,7 @@
       <c r="D501" s="27" t="n"/>
       <c r="E501" s="28" t="n"/>
       <c r="F501" s="15">
-        <f>IF(OR(D485&lt;&gt;"",E485&lt;&gt;""),IF(D485="",0,D485)+IF(E485="",0,E485),"")</f>
+        <f>IF(OR(D455&lt;&gt;"",E455&lt;&gt;""),IF(D455="",0,D455)+IF(E455="",0,E455),"")</f>
         <v/>
       </c>
       <c r="G501" s="14" t="n"/>
@@ -68103,7 +68310,7 @@
     <row r="502">
       <c r="A502" s="14" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B502" s="17" t="n"/>
@@ -68111,7 +68318,7 @@
       <c r="D502" s="27" t="n"/>
       <c r="E502" s="28" t="n"/>
       <c r="F502" s="15">
-        <f>IF(OR(D486&lt;&gt;"",E486&lt;&gt;""),IF(D486="",0,D486)+IF(E486="",0,E486),"")</f>
+        <f>IF(OR(D456&lt;&gt;"",E456&lt;&gt;""),IF(D456="",0,D456)+IF(E456="",0,E456),"")</f>
         <v/>
       </c>
       <c r="G502" s="14" t="n"/>
@@ -68119,7 +68326,7 @@
     <row r="503">
       <c r="A503" s="14" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B503" s="17" t="n"/>
@@ -68127,7 +68334,7 @@
       <c r="D503" s="27" t="n"/>
       <c r="E503" s="28" t="n"/>
       <c r="F503" s="15">
-        <f>IF(OR(D487&lt;&gt;"",E487&lt;&gt;""),IF(D487="",0,D487)+IF(E487="",0,E487),"")</f>
+        <f>IF(OR(D457&lt;&gt;"",E457&lt;&gt;""),IF(D457="",0,D457)+IF(E457="",0,E457),"")</f>
         <v/>
       </c>
       <c r="G503" s="14" t="n"/>
@@ -68135,7 +68342,7 @@
     <row r="504">
       <c r="A504" s="14" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B504" s="17" t="n"/>
@@ -68143,7 +68350,7 @@
       <c r="D504" s="27" t="n"/>
       <c r="E504" s="28" t="n"/>
       <c r="F504" s="15">
-        <f>IF(OR(D488&lt;&gt;"",E488&lt;&gt;""),IF(D488="",0,D488)+IF(E488="",0,E488),"")</f>
+        <f>IF(OR(D458&lt;&gt;"",E458&lt;&gt;""),IF(D458="",0,D458)+IF(E458="",0,E458),"")</f>
         <v/>
       </c>
       <c r="G504" s="14" t="n"/>
@@ -68151,7 +68358,7 @@
     <row r="505">
       <c r="A505" s="14" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B505" s="17" t="n"/>
@@ -68159,7 +68366,7 @@
       <c r="D505" s="27" t="n"/>
       <c r="E505" s="28" t="n"/>
       <c r="F505" s="15">
-        <f>IF(OR(D489&lt;&gt;"",E489&lt;&gt;""),IF(D489="",0,D489)+IF(E489="",0,E489),"")</f>
+        <f>IF(OR(D459&lt;&gt;"",E459&lt;&gt;""),IF(D459="",0,D459)+IF(E459="",0,E459),"")</f>
         <v/>
       </c>
       <c r="G505" s="14" t="n"/>
@@ -68167,7 +68374,7 @@
     <row r="506">
       <c r="A506" s="14" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B506" s="17" t="n"/>
@@ -68175,7 +68382,7 @@
       <c r="D506" s="27" t="n"/>
       <c r="E506" s="28" t="n"/>
       <c r="F506" s="15">
-        <f>IF(OR(D490&lt;&gt;"",E490&lt;&gt;""),IF(D490="",0,D490)+IF(E490="",0,E490),"")</f>
+        <f>IF(OR(D460&lt;&gt;"",E460&lt;&gt;""),IF(D460="",0,D460)+IF(E460="",0,E460),"")</f>
         <v/>
       </c>
       <c r="G506" s="14" t="n"/>
@@ -68183,7 +68390,7 @@
     <row r="507">
       <c r="A507" s="14" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B507" s="17" t="n"/>
@@ -68191,7 +68398,7 @@
       <c r="D507" s="27" t="n"/>
       <c r="E507" s="28" t="n"/>
       <c r="F507" s="15">
-        <f>IF(OR(D491&lt;&gt;"",E491&lt;&gt;""),IF(D491="",0,D491)+IF(E491="",0,E491),"")</f>
+        <f>IF(OR(D461&lt;&gt;"",E461&lt;&gt;""),IF(D461="",0,D461)+IF(E461="",0,E461),"")</f>
         <v/>
       </c>
       <c r="G507" s="14" t="n"/>
@@ -68199,7 +68406,7 @@
     <row r="508">
       <c r="A508" s="14" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B508" s="17" t="n"/>
@@ -68207,7 +68414,7 @@
       <c r="D508" s="27" t="n"/>
       <c r="E508" s="28" t="n"/>
       <c r="F508" s="15">
-        <f>IF(OR(D492&lt;&gt;"",E492&lt;&gt;""),IF(D492="",0,D492)+IF(E492="",0,E492),"")</f>
+        <f>IF(OR(D462&lt;&gt;"",E462&lt;&gt;""),IF(D462="",0,D462)+IF(E462="",0,E462),"")</f>
         <v/>
       </c>
       <c r="G508" s="14" t="n"/>
@@ -68215,7 +68422,7 @@
     <row r="509">
       <c r="A509" s="14" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B509" s="17" t="n"/>
@@ -68223,43 +68430,38 @@
       <c r="D509" s="27" t="n"/>
       <c r="E509" s="28" t="n"/>
       <c r="F509" s="15">
-        <f>IF(OR(D493&lt;&gt;"",E493&lt;&gt;""),IF(D493="",0,D493)+IF(E493="",0,E493),"")</f>
+        <f>IF(OR(D463&lt;&gt;"",E463&lt;&gt;""),IF(D463="",0,D463)+IF(E463="",0,E463),"")</f>
         <v/>
       </c>
       <c r="G509" s="14" t="n"/>
     </row>
     <row r="510">
-      <c r="A510" s="14" t="inlineStr">
-        <is>
-          <t>Diciembre</t>
-        </is>
-      </c>
-      <c r="B510" s="17" t="n"/>
-      <c r="C510" s="14" t="n"/>
-      <c r="D510" s="27" t="n"/>
-      <c r="E510" s="28" t="n"/>
-      <c r="F510" s="15">
-        <f>IF(OR(D494&lt;&gt;"",E494&lt;&gt;""),IF(D494="",0,D494)+IF(E494="",0,E494),"")</f>
+      <c r="A510" s="10" t="inlineStr">
+        <is>
+          <t>TOTAL NOVIEMBRE</t>
+        </is>
+      </c>
+      <c r="B510" s="22" t="n"/>
+      <c r="C510" s="29" t="inlineStr">
+        <is>
+          <t>Totales mes →</t>
+        </is>
+      </c>
+      <c r="D510" s="7">
+        <f>SUMIFS($D$4:$D$800,$A$4:$A$800,"Noviembre")</f>
         <v/>
       </c>
-      <c r="G510" s="14" t="n"/>
-    </row>
-    <row r="511">
-      <c r="A511" s="14" t="inlineStr">
-        <is>
-          <t>Diciembre</t>
-        </is>
-      </c>
-      <c r="B511" s="17" t="n"/>
-      <c r="C511" s="14" t="n"/>
-      <c r="D511" s="27" t="n"/>
-      <c r="E511" s="28" t="n"/>
-      <c r="F511" s="15">
-        <f>IF(OR(D495&lt;&gt;"",E495&lt;&gt;""),IF(D495="",0,D495)+IF(E495="",0,E495),"")</f>
+      <c r="E510" s="7">
+        <f>SUMIFS($E$4:$E$800,$A$4:$A$800,"Noviembre")</f>
         <v/>
       </c>
-      <c r="G511" s="14" t="n"/>
-    </row>
+      <c r="F510" s="7">
+        <f>D510+E510</f>
+        <v/>
+      </c>
+      <c r="G510" s="22" t="n"/>
+    </row>
+    <row r="511"/>
     <row r="512">
       <c r="A512" s="14" t="inlineStr">
         <is>
@@ -68271,7 +68473,7 @@
       <c r="D512" s="27" t="n"/>
       <c r="E512" s="28" t="n"/>
       <c r="F512" s="15">
-        <f>IF(OR(D496&lt;&gt;"",E496&lt;&gt;""),IF(D496="",0,D496)+IF(E496="",0,E496),"")</f>
+        <f>IF(OR(D466&lt;&gt;"",E466&lt;&gt;""),IF(D466="",0,D466)+IF(E466="",0,E466),"")</f>
         <v/>
       </c>
       <c r="G512" s="14" t="n"/>
@@ -68287,7 +68489,7 @@
       <c r="D513" s="27" t="n"/>
       <c r="E513" s="28" t="n"/>
       <c r="F513" s="15">
-        <f>IF(OR(D497&lt;&gt;"",E497&lt;&gt;""),IF(D497="",0,D497)+IF(E497="",0,E497),"")</f>
+        <f>IF(OR(D467&lt;&gt;"",E467&lt;&gt;""),IF(D467="",0,D467)+IF(E467="",0,E467),"")</f>
         <v/>
       </c>
       <c r="G513" s="14" t="n"/>
@@ -68303,7 +68505,7 @@
       <c r="D514" s="27" t="n"/>
       <c r="E514" s="28" t="n"/>
       <c r="F514" s="15">
-        <f>IF(OR(D498&lt;&gt;"",E498&lt;&gt;""),IF(D498="",0,D498)+IF(E498="",0,E498),"")</f>
+        <f>IF(OR(D468&lt;&gt;"",E468&lt;&gt;""),IF(D468="",0,D468)+IF(E468="",0,E468),"")</f>
         <v/>
       </c>
       <c r="G514" s="14" t="n"/>
@@ -68319,7 +68521,7 @@
       <c r="D515" s="27" t="n"/>
       <c r="E515" s="28" t="n"/>
       <c r="F515" s="15">
-        <f>IF(OR(D499&lt;&gt;"",E499&lt;&gt;""),IF(D499="",0,D499)+IF(E499="",0,E499),"")</f>
+        <f>IF(OR(D469&lt;&gt;"",E469&lt;&gt;""),IF(D469="",0,D469)+IF(E469="",0,E469),"")</f>
         <v/>
       </c>
       <c r="G515" s="14" t="n"/>
@@ -68335,7 +68537,7 @@
       <c r="D516" s="27" t="n"/>
       <c r="E516" s="28" t="n"/>
       <c r="F516" s="15">
-        <f>IF(OR(D500&lt;&gt;"",E500&lt;&gt;""),IF(D500="",0,D500)+IF(E500="",0,E500),"")</f>
+        <f>IF(OR(D470&lt;&gt;"",E470&lt;&gt;""),IF(D470="",0,D470)+IF(E470="",0,E470),"")</f>
         <v/>
       </c>
       <c r="G516" s="14" t="n"/>
@@ -68351,7 +68553,7 @@
       <c r="D517" s="27" t="n"/>
       <c r="E517" s="28" t="n"/>
       <c r="F517" s="15">
-        <f>IF(OR(D501&lt;&gt;"",E501&lt;&gt;""),IF(D501="",0,D501)+IF(E501="",0,E501),"")</f>
+        <f>IF(OR(D471&lt;&gt;"",E471&lt;&gt;""),IF(D471="",0,D471)+IF(E471="",0,E471),"")</f>
         <v/>
       </c>
       <c r="G517" s="14" t="n"/>
@@ -68367,7 +68569,7 @@
       <c r="D518" s="27" t="n"/>
       <c r="E518" s="28" t="n"/>
       <c r="F518" s="15">
-        <f>IF(OR(D502&lt;&gt;"",E502&lt;&gt;""),IF(D502="",0,D502)+IF(E502="",0,E502),"")</f>
+        <f>IF(OR(D472&lt;&gt;"",E472&lt;&gt;""),IF(D472="",0,D472)+IF(E472="",0,E472),"")</f>
         <v/>
       </c>
       <c r="G518" s="14" t="n"/>
@@ -68383,7 +68585,7 @@
       <c r="D519" s="27" t="n"/>
       <c r="E519" s="28" t="n"/>
       <c r="F519" s="15">
-        <f>IF(OR(D503&lt;&gt;"",E503&lt;&gt;""),IF(D503="",0,D503)+IF(E503="",0,E503),"")</f>
+        <f>IF(OR(D473&lt;&gt;"",E473&lt;&gt;""),IF(D473="",0,D473)+IF(E473="",0,E473),"")</f>
         <v/>
       </c>
       <c r="G519" s="14" t="n"/>
@@ -68399,7 +68601,7 @@
       <c r="D520" s="27" t="n"/>
       <c r="E520" s="28" t="n"/>
       <c r="F520" s="15">
-        <f>IF(OR(D504&lt;&gt;"",E504&lt;&gt;""),IF(D504="",0,D504)+IF(E504="",0,E504),"")</f>
+        <f>IF(OR(D474&lt;&gt;"",E474&lt;&gt;""),IF(D474="",0,D474)+IF(E474="",0,E474),"")</f>
         <v/>
       </c>
       <c r="G520" s="14" t="n"/>
@@ -68415,91 +68617,816 @@
       <c r="D521" s="27" t="n"/>
       <c r="E521" s="28" t="n"/>
       <c r="F521" s="15">
+        <f>IF(OR(D475&lt;&gt;"",E475&lt;&gt;""),IF(D475="",0,D475)+IF(E475="",0,E475),"")</f>
+        <v/>
+      </c>
+      <c r="G521" s="14" t="n"/>
+    </row>
+    <row r="522">
+      <c r="A522" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B522" s="17" t="n"/>
+      <c r="C522" s="14" t="n"/>
+      <c r="D522" s="27" t="n"/>
+      <c r="E522" s="28" t="n"/>
+      <c r="F522" s="15">
+        <f>IF(OR(D476&lt;&gt;"",E476&lt;&gt;""),IF(D476="",0,D476)+IF(E476="",0,E476),"")</f>
+        <v/>
+      </c>
+      <c r="G522" s="14" t="n"/>
+    </row>
+    <row r="523">
+      <c r="A523" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B523" s="17" t="n"/>
+      <c r="C523" s="14" t="n"/>
+      <c r="D523" s="27" t="n"/>
+      <c r="E523" s="28" t="n"/>
+      <c r="F523" s="15">
+        <f>IF(OR(D477&lt;&gt;"",E477&lt;&gt;""),IF(D477="",0,D477)+IF(E477="",0,E477),"")</f>
+        <v/>
+      </c>
+      <c r="G523" s="14" t="n"/>
+    </row>
+    <row r="524">
+      <c r="A524" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B524" s="17" t="n"/>
+      <c r="C524" s="14" t="n"/>
+      <c r="D524" s="27" t="n"/>
+      <c r="E524" s="28" t="n"/>
+      <c r="F524" s="15">
+        <f>IF(OR(D478&lt;&gt;"",E478&lt;&gt;""),IF(D478="",0,D478)+IF(E478="",0,E478),"")</f>
+        <v/>
+      </c>
+      <c r="G524" s="14" t="n"/>
+    </row>
+    <row r="525">
+      <c r="A525" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B525" s="17" t="n"/>
+      <c r="C525" s="14" t="n"/>
+      <c r="D525" s="27" t="n"/>
+      <c r="E525" s="28" t="n"/>
+      <c r="F525" s="15">
+        <f>IF(OR(D479&lt;&gt;"",E479&lt;&gt;""),IF(D479="",0,D479)+IF(E479="",0,E479),"")</f>
+        <v/>
+      </c>
+      <c r="G525" s="14" t="n"/>
+    </row>
+    <row r="526">
+      <c r="A526" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B526" s="17" t="n"/>
+      <c r="C526" s="14" t="n"/>
+      <c r="D526" s="27" t="n"/>
+      <c r="E526" s="28" t="n"/>
+      <c r="F526" s="15">
+        <f>IF(OR(D480&lt;&gt;"",E480&lt;&gt;""),IF(D480="",0,D480)+IF(E480="",0,E480),"")</f>
+        <v/>
+      </c>
+      <c r="G526" s="14" t="n"/>
+    </row>
+    <row r="527">
+      <c r="A527" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B527" s="17" t="n"/>
+      <c r="C527" s="14" t="n"/>
+      <c r="D527" s="27" t="n"/>
+      <c r="E527" s="28" t="n"/>
+      <c r="F527" s="15">
+        <f>IF(OR(D481&lt;&gt;"",E481&lt;&gt;""),IF(D481="",0,D481)+IF(E481="",0,E481),"")</f>
+        <v/>
+      </c>
+      <c r="G527" s="14" t="n"/>
+    </row>
+    <row r="528">
+      <c r="A528" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B528" s="17" t="n"/>
+      <c r="C528" s="14" t="n"/>
+      <c r="D528" s="27" t="n"/>
+      <c r="E528" s="28" t="n"/>
+      <c r="F528" s="15">
+        <f>IF(OR(D482&lt;&gt;"",E482&lt;&gt;""),IF(D482="",0,D482)+IF(E482="",0,E482),"")</f>
+        <v/>
+      </c>
+      <c r="G528" s="14" t="n"/>
+    </row>
+    <row r="529">
+      <c r="A529" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B529" s="17" t="n"/>
+      <c r="C529" s="14" t="n"/>
+      <c r="D529" s="27" t="n"/>
+      <c r="E529" s="28" t="n"/>
+      <c r="F529" s="15">
+        <f>IF(OR(D483&lt;&gt;"",E483&lt;&gt;""),IF(D483="",0,D483)+IF(E483="",0,E483),"")</f>
+        <v/>
+      </c>
+      <c r="G529" s="14" t="n"/>
+    </row>
+    <row r="530">
+      <c r="A530" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B530" s="17" t="n"/>
+      <c r="C530" s="14" t="n"/>
+      <c r="D530" s="27" t="n"/>
+      <c r="E530" s="28" t="n"/>
+      <c r="F530" s="15">
+        <f>IF(OR(D484&lt;&gt;"",E484&lt;&gt;""),IF(D484="",0,D484)+IF(E484="",0,E484),"")</f>
+        <v/>
+      </c>
+      <c r="G530" s="14" t="n"/>
+    </row>
+    <row r="531">
+      <c r="A531" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B531" s="17" t="n"/>
+      <c r="C531" s="14" t="n"/>
+      <c r="D531" s="27" t="n"/>
+      <c r="E531" s="28" t="n"/>
+      <c r="F531" s="15">
+        <f>IF(OR(D485&lt;&gt;"",E485&lt;&gt;""),IF(D485="",0,D485)+IF(E485="",0,E485),"")</f>
+        <v/>
+      </c>
+      <c r="G531" s="14" t="n"/>
+    </row>
+    <row r="532">
+      <c r="A532" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B532" s="17" t="n"/>
+      <c r="C532" s="14" t="n"/>
+      <c r="D532" s="27" t="n"/>
+      <c r="E532" s="28" t="n"/>
+      <c r="F532" s="15">
+        <f>IF(OR(D486&lt;&gt;"",E486&lt;&gt;""),IF(D486="",0,D486)+IF(E486="",0,E486),"")</f>
+        <v/>
+      </c>
+      <c r="G532" s="14" t="n"/>
+    </row>
+    <row r="533">
+      <c r="A533" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B533" s="17" t="n"/>
+      <c r="C533" s="14" t="n"/>
+      <c r="D533" s="27" t="n"/>
+      <c r="E533" s="28" t="n"/>
+      <c r="F533" s="15">
+        <f>IF(OR(D487&lt;&gt;"",E487&lt;&gt;""),IF(D487="",0,D487)+IF(E487="",0,E487),"")</f>
+        <v/>
+      </c>
+      <c r="G533" s="14" t="n"/>
+    </row>
+    <row r="534">
+      <c r="A534" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B534" s="17" t="n"/>
+      <c r="C534" s="14" t="n"/>
+      <c r="D534" s="27" t="n"/>
+      <c r="E534" s="28" t="n"/>
+      <c r="F534" s="15">
+        <f>IF(OR(D488&lt;&gt;"",E488&lt;&gt;""),IF(D488="",0,D488)+IF(E488="",0,E488),"")</f>
+        <v/>
+      </c>
+      <c r="G534" s="14" t="n"/>
+    </row>
+    <row r="535">
+      <c r="A535" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B535" s="17" t="n"/>
+      <c r="C535" s="14" t="n"/>
+      <c r="D535" s="27" t="n"/>
+      <c r="E535" s="28" t="n"/>
+      <c r="F535" s="15">
+        <f>IF(OR(D489&lt;&gt;"",E489&lt;&gt;""),IF(D489="",0,D489)+IF(E489="",0,E489),"")</f>
+        <v/>
+      </c>
+      <c r="G535" s="14" t="n"/>
+    </row>
+    <row r="536">
+      <c r="A536" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B536" s="17" t="n"/>
+      <c r="C536" s="14" t="n"/>
+      <c r="D536" s="27" t="n"/>
+      <c r="E536" s="28" t="n"/>
+      <c r="F536" s="15">
+        <f>IF(OR(D490&lt;&gt;"",E490&lt;&gt;""),IF(D490="",0,D490)+IF(E490="",0,E490),"")</f>
+        <v/>
+      </c>
+      <c r="G536" s="14" t="n"/>
+    </row>
+    <row r="537">
+      <c r="A537" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B537" s="17" t="n"/>
+      <c r="C537" s="14" t="n"/>
+      <c r="D537" s="27" t="n"/>
+      <c r="E537" s="28" t="n"/>
+      <c r="F537" s="15">
+        <f>IF(OR(D491&lt;&gt;"",E491&lt;&gt;""),IF(D491="",0,D491)+IF(E491="",0,E491),"")</f>
+        <v/>
+      </c>
+      <c r="G537" s="14" t="n"/>
+    </row>
+    <row r="538">
+      <c r="A538" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B538" s="17" t="n"/>
+      <c r="C538" s="14" t="n"/>
+      <c r="D538" s="27" t="n"/>
+      <c r="E538" s="28" t="n"/>
+      <c r="F538" s="15">
+        <f>IF(OR(D492&lt;&gt;"",E492&lt;&gt;""),IF(D492="",0,D492)+IF(E492="",0,E492),"")</f>
+        <v/>
+      </c>
+      <c r="G538" s="14" t="n"/>
+    </row>
+    <row r="539">
+      <c r="A539" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B539" s="17" t="n"/>
+      <c r="C539" s="14" t="n"/>
+      <c r="D539" s="27" t="n"/>
+      <c r="E539" s="28" t="n"/>
+      <c r="F539" s="15">
+        <f>IF(OR(D493&lt;&gt;"",E493&lt;&gt;""),IF(D493="",0,D493)+IF(E493="",0,E493),"")</f>
+        <v/>
+      </c>
+      <c r="G539" s="14" t="n"/>
+    </row>
+    <row r="540">
+      <c r="A540" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B540" s="17" t="n"/>
+      <c r="C540" s="14" t="n"/>
+      <c r="D540" s="27" t="n"/>
+      <c r="E540" s="28" t="n"/>
+      <c r="F540" s="15">
+        <f>IF(OR(D494&lt;&gt;"",E494&lt;&gt;""),IF(D494="",0,D494)+IF(E494="",0,E494),"")</f>
+        <v/>
+      </c>
+      <c r="G540" s="14" t="n"/>
+    </row>
+    <row r="541">
+      <c r="A541" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B541" s="17" t="n"/>
+      <c r="C541" s="14" t="n"/>
+      <c r="D541" s="27" t="n"/>
+      <c r="E541" s="28" t="n"/>
+      <c r="F541" s="15">
+        <f>IF(OR(D495&lt;&gt;"",E495&lt;&gt;""),IF(D495="",0,D495)+IF(E495="",0,E495),"")</f>
+        <v/>
+      </c>
+      <c r="G541" s="14" t="n"/>
+    </row>
+    <row r="542">
+      <c r="A542" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B542" s="17" t="n"/>
+      <c r="C542" s="14" t="n"/>
+      <c r="D542" s="27" t="n"/>
+      <c r="E542" s="28" t="n"/>
+      <c r="F542" s="15">
+        <f>IF(OR(D496&lt;&gt;"",E496&lt;&gt;""),IF(D496="",0,D496)+IF(E496="",0,E496),"")</f>
+        <v/>
+      </c>
+      <c r="G542" s="14" t="n"/>
+    </row>
+    <row r="543">
+      <c r="A543" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B543" s="17" t="n"/>
+      <c r="C543" s="14" t="n"/>
+      <c r="D543" s="27" t="n"/>
+      <c r="E543" s="28" t="n"/>
+      <c r="F543" s="15">
+        <f>IF(OR(D497&lt;&gt;"",E497&lt;&gt;""),IF(D497="",0,D497)+IF(E497="",0,E497),"")</f>
+        <v/>
+      </c>
+      <c r="G543" s="14" t="n"/>
+    </row>
+    <row r="544">
+      <c r="A544" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B544" s="17" t="n"/>
+      <c r="C544" s="14" t="n"/>
+      <c r="D544" s="27" t="n"/>
+      <c r="E544" s="28" t="n"/>
+      <c r="F544" s="15">
+        <f>IF(OR(D498&lt;&gt;"",E498&lt;&gt;""),IF(D498="",0,D498)+IF(E498="",0,E498),"")</f>
+        <v/>
+      </c>
+      <c r="G544" s="14" t="n"/>
+    </row>
+    <row r="545">
+      <c r="A545" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B545" s="17" t="n"/>
+      <c r="C545" s="14" t="n"/>
+      <c r="D545" s="27" t="n"/>
+      <c r="E545" s="28" t="n"/>
+      <c r="F545" s="15">
+        <f>IF(OR(D499&lt;&gt;"",E499&lt;&gt;""),IF(D499="",0,D499)+IF(E499="",0,E499),"")</f>
+        <v/>
+      </c>
+      <c r="G545" s="14" t="n"/>
+    </row>
+    <row r="546">
+      <c r="A546" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B546" s="17" t="n"/>
+      <c r="C546" s="14" t="n"/>
+      <c r="D546" s="27" t="n"/>
+      <c r="E546" s="28" t="n"/>
+      <c r="F546" s="15">
+        <f>IF(OR(D500&lt;&gt;"",E500&lt;&gt;""),IF(D500="",0,D500)+IF(E500="",0,E500),"")</f>
+        <v/>
+      </c>
+      <c r="G546" s="14" t="n"/>
+    </row>
+    <row r="547">
+      <c r="A547" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B547" s="17" t="n"/>
+      <c r="C547" s="14" t="n"/>
+      <c r="D547" s="27" t="n"/>
+      <c r="E547" s="28" t="n"/>
+      <c r="F547" s="15">
+        <f>IF(OR(D501&lt;&gt;"",E501&lt;&gt;""),IF(D501="",0,D501)+IF(E501="",0,E501),"")</f>
+        <v/>
+      </c>
+      <c r="G547" s="14" t="n"/>
+    </row>
+    <row r="548">
+      <c r="A548" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B548" s="17" t="n"/>
+      <c r="C548" s="14" t="n"/>
+      <c r="D548" s="27" t="n"/>
+      <c r="E548" s="28" t="n"/>
+      <c r="F548" s="15">
+        <f>IF(OR(D502&lt;&gt;"",E502&lt;&gt;""),IF(D502="",0,D502)+IF(E502="",0,E502),"")</f>
+        <v/>
+      </c>
+      <c r="G548" s="14" t="n"/>
+    </row>
+    <row r="549">
+      <c r="A549" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B549" s="17" t="n"/>
+      <c r="C549" s="14" t="n"/>
+      <c r="D549" s="27" t="n"/>
+      <c r="E549" s="28" t="n"/>
+      <c r="F549" s="15">
+        <f>IF(OR(D503&lt;&gt;"",E503&lt;&gt;""),IF(D503="",0,D503)+IF(E503="",0,E503),"")</f>
+        <v/>
+      </c>
+      <c r="G549" s="14" t="n"/>
+    </row>
+    <row r="550">
+      <c r="A550" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B550" s="17" t="n"/>
+      <c r="C550" s="14" t="n"/>
+      <c r="D550" s="27" t="n"/>
+      <c r="E550" s="28" t="n"/>
+      <c r="F550" s="15">
+        <f>IF(OR(D504&lt;&gt;"",E504&lt;&gt;""),IF(D504="",0,D504)+IF(E504="",0,E504),"")</f>
+        <v/>
+      </c>
+      <c r="G550" s="14" t="n"/>
+    </row>
+    <row r="551">
+      <c r="A551" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B551" s="17" t="n"/>
+      <c r="C551" s="14" t="n"/>
+      <c r="D551" s="27" t="n"/>
+      <c r="E551" s="28" t="n"/>
+      <c r="F551" s="15">
         <f>IF(OR(D505&lt;&gt;"",E505&lt;&gt;""),IF(D505="",0,D505)+IF(E505="",0,E505),"")</f>
         <v/>
       </c>
-      <c r="G521" s="14" t="n"/>
-    </row>
-    <row r="522">
-      <c r="A522" s="10" t="inlineStr">
+      <c r="G551" s="14" t="n"/>
+    </row>
+    <row r="552">
+      <c r="A552" s="10" t="inlineStr">
         <is>
           <t>TOTAL DICIEMBRE</t>
         </is>
       </c>
-      <c r="B522" s="22" t="n"/>
-      <c r="C522" s="29" t="inlineStr">
+      <c r="B552" s="22" t="n"/>
+      <c r="C552" s="29" t="inlineStr">
         <is>
           <t>Totales mes →</t>
         </is>
       </c>
-      <c r="D522" s="7">
-        <f>SUMIFS($D$4:$D$600,$A$4:$A$600,"Diciembre")</f>
+      <c r="D552" s="7">
+        <f>SUMIFS($D$4:$D$800,$A$4:$A$800,"Diciembre")</f>
         <v/>
       </c>
-      <c r="E522" s="7">
-        <f>SUMIFS($E$4:$E$600,$A$4:$A$600,"Diciembre")</f>
+      <c r="E552" s="7">
+        <f>SUMIFS($E$4:$E$800,$A$4:$A$800,"Diciembre")</f>
         <v/>
       </c>
-      <c r="F522" s="7">
-        <f>D522+E522</f>
+      <c r="F552" s="7">
+        <f>D552+E552</f>
         <v/>
       </c>
-      <c r="G522" s="22" t="n"/>
-    </row>
-    <row r="523">
-      <c r="A523" t="inlineStr">
+      <c r="G552" s="22" t="n"/>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
         <is>
           <t>Enero</t>
         </is>
       </c>
-      <c r="B523" s="54" t="n">
+      <c r="B553" s="54" t="n">
         <v>46034</v>
       </c>
-      <c r="C523" t="inlineStr">
+      <c r="C553" t="inlineStr">
         <is>
           <t>SUPERMERCADO · Coto</t>
         </is>
       </c>
-      <c r="D523" t="n">
+      <c r="D553" t="n">
         <v>337644</v>
       </c>
-      <c r="F523">
+      <c r="F553">
         <f>IF(OR(D523&lt;&gt;"",E523&lt;&gt;""),IF(D523="",0,D523)+IF(E523="",0,E523),"")</f>
         <v/>
       </c>
-      <c r="G523" t="inlineStr">
+      <c r="G553" t="inlineStr">
         <is>
           <t>SUPERMERCADO · Coto · TC Mercado Pago · compra 2025-12-22</t>
         </is>
       </c>
     </row>
-    <row r="524">
-      <c r="A524" t="inlineStr">
+    <row r="554">
+      <c r="A554" t="inlineStr">
         <is>
           <t>Enero</t>
         </is>
       </c>
-      <c r="B524" s="54" t="n">
+      <c r="B554" s="54" t="n">
         <v>46034</v>
       </c>
-      <c r="C524" t="inlineStr">
+      <c r="C554" t="inlineStr">
         <is>
           <t>SUPERMERCADO · Coto</t>
         </is>
       </c>
-      <c r="D524" t="n">
+      <c r="D554" t="n">
         <v>-49597</v>
       </c>
-      <c r="F524">
+      <c r="F554">
         <f>IF(OR(D524&lt;&gt;"",E524&lt;&gt;""),IF(D524="",0,D524)+IF(E524="",0,E524),"")</f>
         <v/>
       </c>
-      <c r="G524" t="inlineStr">
+      <c r="G554" t="inlineStr">
         <is>
           <t>REEMBOLSO · SUPERMERCADO · Coto · TC Mercado Pago · compra 2025-12-23</t>
         </is>
       </c>
     </row>
+    <row r="555"/>
+    <row r="556"/>
+    <row r="557"/>
+    <row r="558"/>
+    <row r="559"/>
+    <row r="560"/>
+    <row r="561"/>
+    <row r="562"/>
+    <row r="563"/>
+    <row r="564"/>
+    <row r="565"/>
+    <row r="566"/>
+    <row r="567"/>
+    <row r="568"/>
+    <row r="569"/>
+    <row r="570"/>
+    <row r="571"/>
+    <row r="572"/>
+    <row r="573"/>
+    <row r="574"/>
+    <row r="575"/>
+    <row r="576"/>
+    <row r="577"/>
+    <row r="578"/>
+    <row r="579"/>
+    <row r="580"/>
+    <row r="581"/>
+    <row r="582"/>
+    <row r="583"/>
+    <row r="584"/>
+    <row r="585"/>
+    <row r="586"/>
+    <row r="587"/>
+    <row r="588"/>
+    <row r="589"/>
+    <row r="590"/>
+    <row r="591"/>
+    <row r="592"/>
+    <row r="593"/>
+    <row r="594"/>
+    <row r="595"/>
+    <row r="596"/>
+    <row r="597"/>
+    <row r="598"/>
+    <row r="599"/>
+    <row r="600"/>
+    <row r="601"/>
+    <row r="602"/>
+    <row r="603"/>
+    <row r="604"/>
+    <row r="605"/>
+    <row r="606"/>
+    <row r="607"/>
+    <row r="608"/>
+    <row r="609"/>
+    <row r="610"/>
+    <row r="611"/>
+    <row r="612"/>
+    <row r="613"/>
+    <row r="614"/>
+    <row r="615"/>
+    <row r="616"/>
+    <row r="617"/>
+    <row r="618"/>
+    <row r="619"/>
+    <row r="620"/>
+    <row r="621"/>
+    <row r="622"/>
+    <row r="623"/>
+    <row r="624"/>
+    <row r="625"/>
+    <row r="626"/>
+    <row r="627"/>
+    <row r="628"/>
+    <row r="629"/>
+    <row r="630"/>
+    <row r="631"/>
+    <row r="632"/>
+    <row r="633"/>
+    <row r="634"/>
+    <row r="635"/>
+    <row r="636"/>
+    <row r="637"/>
+    <row r="638"/>
+    <row r="639"/>
+    <row r="640"/>
+    <row r="641"/>
+    <row r="642"/>
+    <row r="643"/>
+    <row r="644"/>
+    <row r="645"/>
+    <row r="646"/>
+    <row r="647"/>
+    <row r="648"/>
+    <row r="649"/>
+    <row r="650"/>
+    <row r="651"/>
+    <row r="652"/>
+    <row r="653"/>
+    <row r="654"/>
+    <row r="655"/>
+    <row r="656"/>
+    <row r="657"/>
+    <row r="658"/>
+    <row r="659"/>
+    <row r="660"/>
+    <row r="661"/>
+    <row r="662"/>
+    <row r="663"/>
+    <row r="664"/>
+    <row r="665"/>
+    <row r="666"/>
+    <row r="667"/>
+    <row r="668"/>
+    <row r="669"/>
+    <row r="670"/>
+    <row r="671"/>
+    <row r="672"/>
+    <row r="673"/>
+    <row r="674"/>
+    <row r="675"/>
+    <row r="676"/>
+    <row r="677"/>
+    <row r="678"/>
+    <row r="679"/>
+    <row r="680"/>
+    <row r="681"/>
+    <row r="682"/>
+    <row r="683"/>
+    <row r="684"/>
+    <row r="685"/>
+    <row r="686"/>
+    <row r="687"/>
+    <row r="688"/>
+    <row r="689"/>
+    <row r="690"/>
+    <row r="691"/>
+    <row r="692"/>
+    <row r="693"/>
+    <row r="694"/>
+    <row r="695"/>
+    <row r="696"/>
+    <row r="697"/>
+    <row r="698"/>
+    <row r="699"/>
+    <row r="700"/>
+    <row r="701"/>
+    <row r="702"/>
+    <row r="703"/>
+    <row r="704"/>
+    <row r="705"/>
+    <row r="706"/>
+    <row r="707"/>
+    <row r="708"/>
+    <row r="709"/>
+    <row r="710"/>
+    <row r="711"/>
+    <row r="712"/>
+    <row r="713"/>
+    <row r="714"/>
+    <row r="715"/>
+    <row r="716"/>
+    <row r="717"/>
+    <row r="718"/>
+    <row r="719"/>
+    <row r="720"/>
+    <row r="721"/>
+    <row r="722"/>
+    <row r="723"/>
+    <row r="724"/>
+    <row r="725"/>
+    <row r="726"/>
+    <row r="727"/>
+    <row r="728"/>
+    <row r="729"/>
+    <row r="730"/>
+    <row r="731"/>
+    <row r="732"/>
+    <row r="733"/>
+    <row r="734"/>
+    <row r="735"/>
+    <row r="736"/>
+    <row r="737"/>
+    <row r="738"/>
+    <row r="739"/>
+    <row r="740"/>
+    <row r="741"/>
+    <row r="742"/>
+    <row r="743"/>
+    <row r="744"/>
+    <row r="745"/>
+    <row r="746"/>
+    <row r="747"/>
+    <row r="748"/>
+    <row r="749"/>
+    <row r="750"/>
+    <row r="751"/>
+    <row r="752"/>
+    <row r="753"/>
+    <row r="754"/>
+    <row r="755"/>
+    <row r="756"/>
+    <row r="757"/>
+    <row r="758"/>
+    <row r="759"/>
+    <row r="760"/>
+    <row r="761"/>
+    <row r="762"/>
+    <row r="763"/>
+    <row r="764"/>
+    <row r="765"/>
+    <row r="766"/>
+    <row r="767"/>
+    <row r="768"/>
+    <row r="769"/>
+    <row r="770"/>
+    <row r="771"/>
+    <row r="772"/>
+    <row r="773"/>
+    <row r="774"/>
+    <row r="775"/>
+    <row r="776"/>
+    <row r="777"/>
+    <row r="778"/>
+    <row r="779"/>
+    <row r="780"/>
+    <row r="781"/>
+    <row r="782"/>
+    <row r="783"/>
+    <row r="784"/>
+    <row r="785"/>
+    <row r="786"/>
+    <row r="787"/>
+    <row r="788"/>
+    <row r="789"/>
+    <row r="790"/>
+    <row r="791"/>
+    <row r="792"/>
+    <row r="793"/>
+    <row r="794"/>
+    <row r="795"/>
+    <row r="796"/>
+    <row r="797"/>
+    <row r="798"/>
+    <row r="799"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Load CIUDAD July expensas $300,850 from Gmail Sent (10/08).
Payment to Consorcio De Propiet / Patagonia for período julio (liquidación De Filippo UF 2 1-A). Fill matrix Julio, Detalle and Expensas Consorcios; correct Mayo/Junio period labels on prior Detalle rows.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -870,7 +870,9 @@
       <c r="I5" s="5" t="n">
         <v>273500</v>
       </c>
-      <c r="J5" s="5" t="n"/>
+      <c r="J5" s="5" t="n">
+        <v>300850</v>
+      </c>
       <c r="K5" s="5" t="n">
         <v>300850</v>
       </c>
@@ -2861,13 +2863,37 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="17" t="n"/>
-      <c r="B48" s="14" t="n"/>
-      <c r="C48" s="14" t="n"/>
-      <c r="D48" s="14" t="n"/>
-      <c r="E48" s="15" t="n"/>
-      <c r="F48" s="14" t="n"/>
-      <c r="G48" s="14" t="n"/>
+      <c r="A48" s="17" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B48" s="14" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C48" s="14" t="inlineStr">
+        <is>
+          <t>Consorcio De Propiet</t>
+        </is>
+      </c>
+      <c r="D48" s="14" t="inlineStr">
+        <is>
+          <t>CIUDAD 1132</t>
+        </is>
+      </c>
+      <c r="E48" s="15" t="n">
+        <v>300850</v>
+      </c>
+      <c r="F48" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Transferencia enviada</t>
+        </is>
+      </c>
+      <c r="G48" s="14" t="inlineStr">
+        <is>
+          <t>Pago de Expensas · CIUDAD 1132 · Patagonia CBU 0340116900116010765007 / CUIL 30714962473 · período julio 2026 (Gmail Sent 10/08 · op 173005218278)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="17" t="n"/>
@@ -57128,7 +57154,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G799"/>
+  <dimension ref="A1:G554"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -61688,7 +61714,6 @@
       </c>
       <c r="G176" s="22" t="n"/>
     </row>
-    <row r="177"/>
     <row r="178">
       <c r="A178" s="14" t="inlineStr">
         <is>
@@ -62971,7 +62996,6 @@
       </c>
       <c r="G228" s="22" t="n"/>
     </row>
-    <row r="229"/>
     <row r="230">
       <c r="A230" s="14" t="inlineStr">
         <is>
@@ -64010,7 +64034,6 @@
       </c>
       <c r="G273" s="22" t="n"/>
     </row>
-    <row r="274"/>
     <row r="275">
       <c r="A275" s="14" t="inlineStr">
         <is>
@@ -64778,7 +64801,6 @@
       </c>
       <c r="G312" s="22" t="n"/>
     </row>
-    <row r="313"/>
     <row r="314">
       <c r="A314" s="14" t="inlineStr">
         <is>
@@ -65445,7 +65467,6 @@
       </c>
       <c r="G354" s="22" t="n"/>
     </row>
-    <row r="355"/>
     <row r="356">
       <c r="A356" s="14" t="inlineStr">
         <is>
@@ -67127,7 +67148,6 @@
       </c>
       <c r="G426" s="22" t="n"/>
     </row>
-    <row r="427"/>
     <row r="428">
       <c r="A428" s="14" t="inlineStr">
         <is>
@@ -67794,7 +67814,6 @@
       </c>
       <c r="G468" s="22" t="n"/>
     </row>
-    <row r="469"/>
     <row r="470">
       <c r="A470" s="14" t="inlineStr">
         <is>
@@ -68461,7 +68480,6 @@
       </c>
       <c r="G510" s="22" t="n"/>
     </row>
-    <row r="511"/>
     <row r="512">
       <c r="A512" s="14" t="inlineStr">
         <is>
@@ -69182,251 +69200,6 @@
         </is>
       </c>
     </row>
-    <row r="555"/>
-    <row r="556"/>
-    <row r="557"/>
-    <row r="558"/>
-    <row r="559"/>
-    <row r="560"/>
-    <row r="561"/>
-    <row r="562"/>
-    <row r="563"/>
-    <row r="564"/>
-    <row r="565"/>
-    <row r="566"/>
-    <row r="567"/>
-    <row r="568"/>
-    <row r="569"/>
-    <row r="570"/>
-    <row r="571"/>
-    <row r="572"/>
-    <row r="573"/>
-    <row r="574"/>
-    <row r="575"/>
-    <row r="576"/>
-    <row r="577"/>
-    <row r="578"/>
-    <row r="579"/>
-    <row r="580"/>
-    <row r="581"/>
-    <row r="582"/>
-    <row r="583"/>
-    <row r="584"/>
-    <row r="585"/>
-    <row r="586"/>
-    <row r="587"/>
-    <row r="588"/>
-    <row r="589"/>
-    <row r="590"/>
-    <row r="591"/>
-    <row r="592"/>
-    <row r="593"/>
-    <row r="594"/>
-    <row r="595"/>
-    <row r="596"/>
-    <row r="597"/>
-    <row r="598"/>
-    <row r="599"/>
-    <row r="600"/>
-    <row r="601"/>
-    <row r="602"/>
-    <row r="603"/>
-    <row r="604"/>
-    <row r="605"/>
-    <row r="606"/>
-    <row r="607"/>
-    <row r="608"/>
-    <row r="609"/>
-    <row r="610"/>
-    <row r="611"/>
-    <row r="612"/>
-    <row r="613"/>
-    <row r="614"/>
-    <row r="615"/>
-    <row r="616"/>
-    <row r="617"/>
-    <row r="618"/>
-    <row r="619"/>
-    <row r="620"/>
-    <row r="621"/>
-    <row r="622"/>
-    <row r="623"/>
-    <row r="624"/>
-    <row r="625"/>
-    <row r="626"/>
-    <row r="627"/>
-    <row r="628"/>
-    <row r="629"/>
-    <row r="630"/>
-    <row r="631"/>
-    <row r="632"/>
-    <row r="633"/>
-    <row r="634"/>
-    <row r="635"/>
-    <row r="636"/>
-    <row r="637"/>
-    <row r="638"/>
-    <row r="639"/>
-    <row r="640"/>
-    <row r="641"/>
-    <row r="642"/>
-    <row r="643"/>
-    <row r="644"/>
-    <row r="645"/>
-    <row r="646"/>
-    <row r="647"/>
-    <row r="648"/>
-    <row r="649"/>
-    <row r="650"/>
-    <row r="651"/>
-    <row r="652"/>
-    <row r="653"/>
-    <row r="654"/>
-    <row r="655"/>
-    <row r="656"/>
-    <row r="657"/>
-    <row r="658"/>
-    <row r="659"/>
-    <row r="660"/>
-    <row r="661"/>
-    <row r="662"/>
-    <row r="663"/>
-    <row r="664"/>
-    <row r="665"/>
-    <row r="666"/>
-    <row r="667"/>
-    <row r="668"/>
-    <row r="669"/>
-    <row r="670"/>
-    <row r="671"/>
-    <row r="672"/>
-    <row r="673"/>
-    <row r="674"/>
-    <row r="675"/>
-    <row r="676"/>
-    <row r="677"/>
-    <row r="678"/>
-    <row r="679"/>
-    <row r="680"/>
-    <row r="681"/>
-    <row r="682"/>
-    <row r="683"/>
-    <row r="684"/>
-    <row r="685"/>
-    <row r="686"/>
-    <row r="687"/>
-    <row r="688"/>
-    <row r="689"/>
-    <row r="690"/>
-    <row r="691"/>
-    <row r="692"/>
-    <row r="693"/>
-    <row r="694"/>
-    <row r="695"/>
-    <row r="696"/>
-    <row r="697"/>
-    <row r="698"/>
-    <row r="699"/>
-    <row r="700"/>
-    <row r="701"/>
-    <row r="702"/>
-    <row r="703"/>
-    <row r="704"/>
-    <row r="705"/>
-    <row r="706"/>
-    <row r="707"/>
-    <row r="708"/>
-    <row r="709"/>
-    <row r="710"/>
-    <row r="711"/>
-    <row r="712"/>
-    <row r="713"/>
-    <row r="714"/>
-    <row r="715"/>
-    <row r="716"/>
-    <row r="717"/>
-    <row r="718"/>
-    <row r="719"/>
-    <row r="720"/>
-    <row r="721"/>
-    <row r="722"/>
-    <row r="723"/>
-    <row r="724"/>
-    <row r="725"/>
-    <row r="726"/>
-    <row r="727"/>
-    <row r="728"/>
-    <row r="729"/>
-    <row r="730"/>
-    <row r="731"/>
-    <row r="732"/>
-    <row r="733"/>
-    <row r="734"/>
-    <row r="735"/>
-    <row r="736"/>
-    <row r="737"/>
-    <row r="738"/>
-    <row r="739"/>
-    <row r="740"/>
-    <row r="741"/>
-    <row r="742"/>
-    <row r="743"/>
-    <row r="744"/>
-    <row r="745"/>
-    <row r="746"/>
-    <row r="747"/>
-    <row r="748"/>
-    <row r="749"/>
-    <row r="750"/>
-    <row r="751"/>
-    <row r="752"/>
-    <row r="753"/>
-    <row r="754"/>
-    <row r="755"/>
-    <row r="756"/>
-    <row r="757"/>
-    <row r="758"/>
-    <row r="759"/>
-    <row r="760"/>
-    <row r="761"/>
-    <row r="762"/>
-    <row r="763"/>
-    <row r="764"/>
-    <row r="765"/>
-    <row r="766"/>
-    <row r="767"/>
-    <row r="768"/>
-    <row r="769"/>
-    <row r="770"/>
-    <row r="771"/>
-    <row r="772"/>
-    <row r="773"/>
-    <row r="774"/>
-    <row r="775"/>
-    <row r="776"/>
-    <row r="777"/>
-    <row r="778"/>
-    <row r="779"/>
-    <row r="780"/>
-    <row r="781"/>
-    <row r="782"/>
-    <row r="783"/>
-    <row r="784"/>
-    <row r="785"/>
-    <row r="786"/>
-    <row r="787"/>
-    <row r="788"/>
-    <row r="789"/>
-    <row r="790"/>
-    <row r="791"/>
-    <row r="792"/>
-    <row r="793"/>
-    <row r="794"/>
-    <row r="795"/>
-    <row r="796"/>
-    <row r="797"/>
-    <row r="798"/>
-    <row r="799"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -69438,7 +69211,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I81"/>
+  <dimension ref="A1:I82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -69966,7 +69739,7 @@
       <c r="G17" s="18" t="inlineStr"/>
       <c r="H17" s="14" t="inlineStr">
         <is>
-          <t>PENDIENTE — no se encontró el monto</t>
+          <t>Consorcio de Propietarios · Pagado · Gmail Sent 7-abr</t>
         </is>
       </c>
       <c r="I17" s="14" t="inlineStr">
@@ -70108,37 +69881,15 @@
       <c r="I21" s="14" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="17" t="n">
-        <v>46143</v>
-      </c>
-      <c r="B22" s="14" t="inlineStr">
-        <is>
-          <t>Expensas</t>
-        </is>
-      </c>
-      <c r="C22" s="14" t="inlineStr">
-        <is>
-          <t>Expensas — Mayo 2026</t>
-        </is>
-      </c>
+      <c r="A22" s="17" t="n"/>
+      <c r="B22" s="14" t="n"/>
+      <c r="C22" s="14" t="n"/>
       <c r="D22" s="15" t="n"/>
-      <c r="E22" s="14" t="inlineStr">
-        <is>
-          <t>Transferencia</t>
-        </is>
-      </c>
-      <c r="F22" s="18" t="inlineStr"/>
-      <c r="G22" s="18" t="inlineStr"/>
-      <c r="H22" s="14" t="inlineStr">
-        <is>
-          <t>PENDIENTE — no se encontró el monto</t>
-        </is>
-      </c>
-      <c r="I22" s="14" t="inlineStr">
-        <is>
-          <t>Mayo</t>
-        </is>
-      </c>
+      <c r="E22" s="14" t="n"/>
+      <c r="F22" s="18" t="n"/>
+      <c r="G22" s="18" t="n"/>
+      <c r="H22" s="14" t="n"/>
+      <c r="I22" s="14" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="17" t="n">
@@ -70419,7 +70170,7 @@
       </c>
       <c r="C31" s="14" t="inlineStr">
         <is>
-          <t>Expensas — Junio 2026</t>
+          <t>Expensas — Mayo 2026 (pago Gmail Sent 10/06)</t>
         </is>
       </c>
       <c r="D31" s="15" t="n">
@@ -70434,12 +70185,12 @@
       <c r="G31" s="18" t="inlineStr"/>
       <c r="H31" s="14" t="inlineStr">
         <is>
-          <t>Consorcio de Propietarios · Pagado</t>
+          <t>Período mayo · Consorcio De Propietarios · Pagado · Gmail Sent</t>
         </is>
       </c>
       <c r="I31" s="14" t="inlineStr">
         <is>
-          <t>Junio</t>
+          <t>Mayo</t>
         </is>
       </c>
     </row>
@@ -70524,7 +70275,7 @@
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>Expensas — Julio 2026</t>
+          <t>Expensas — Junio 2026 (pago Gmail Sent 09/07)</t>
         </is>
       </c>
       <c r="D34" s="15" t="n">
@@ -70539,12 +70290,12 @@
       <c r="G34" s="18" t="inlineStr"/>
       <c r="H34" s="14" t="inlineStr">
         <is>
-          <t>Consorcio de Propietarios · Pagado</t>
+          <t>Período junio · Consorcio De Propietarios · Pagado · Gmail Sent</t>
         </is>
       </c>
       <c r="I34" s="14" t="inlineStr">
         <is>
-          <t>Julio</t>
+          <t>Junio</t>
         </is>
       </c>
     </row>
@@ -71963,6 +71714,39 @@
       <c r="I81" t="inlineStr">
         <is>
           <t>Septiembre</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="52" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Expensas</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Expensas — Julio 2026 (pago Gmail Sent 10/08)</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>300850</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Transferencia</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Período julio · De Filippo · UF 2 1-A · pagado 10/08 · Gmail Sent · op MP 173005218278</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Julio</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fill August CIUDAD gaps: utilities, limpieza, partial almacén.
Set Telecentro 31999, Metrogas 73187, ABL 41344, Limpieza 567080; update July limpieza to 653120; add verdulería Sol and Chris almacén lump; document remaining August gaps.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -925,7 +925,7 @@
         <v>31999</v>
       </c>
       <c r="K6" s="9" t="n">
-        <v>50000</v>
+        <v>31999</v>
       </c>
       <c r="L6" s="9" t="n">
         <v>69659</v>
@@ -979,7 +979,9 @@
         <v>30643</v>
       </c>
       <c r="J7" s="5" t="n"/>
-      <c r="K7" s="5" t="n"/>
+      <c r="K7" s="5" t="n">
+        <v>73187</v>
+      </c>
       <c r="L7" s="5" t="n">
         <v>105839</v>
       </c>
@@ -1069,7 +1071,9 @@
       <c r="J9" s="5" t="n">
         <v>26175</v>
       </c>
-      <c r="K9" s="5" t="n"/>
+      <c r="K9" s="5" t="n">
+        <v>41344</v>
+      </c>
       <c r="L9" s="5" t="n">
         <v>27635</v>
       </c>
@@ -1116,9 +1120,11 @@
         <v>876981</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>400640</v>
-      </c>
-      <c r="K10" s="9" t="n"/>
+        <v>653120</v>
+      </c>
+      <c r="K10" s="9" t="n">
+        <v>567080</v>
+      </c>
       <c r="L10" s="9" t="n">
         <v>835200</v>
       </c>
@@ -64807,15 +64813,27 @@
           <t>Agosto</t>
         </is>
       </c>
-      <c r="B314" s="17" t="n"/>
-      <c r="C314" s="14" t="n"/>
-      <c r="D314" s="27" t="n"/>
+      <c r="B314" s="17" t="n">
+        <v>46245</v>
+      </c>
+      <c r="C314" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · VERDULERÍA</t>
+        </is>
+      </c>
+      <c r="D314" s="27" t="n">
+        <v>8900</v>
+      </c>
       <c r="E314" s="28" t="n"/>
       <c r="F314" s="15">
-        <f>IF(OR(D298&lt;&gt;"",E298&lt;&gt;""),IF(D298="",0,D298)+IF(E298="",0,E298),"")</f>
+        <f>IF(OR(D314&lt;&gt;"",E314&lt;&gt;""),IF(D314="",0,D314)+IF(E314="",0,E314),"")</f>
         <v/>
       </c>
-      <c r="G314" s="14" t="n"/>
+      <c r="G314" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · VERDULERÍA · Agosto</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" s="14" t="inlineStr">
@@ -64823,15 +64841,27 @@
           <t>Agosto</t>
         </is>
       </c>
-      <c r="B315" s="17" t="n"/>
-      <c r="C315" s="14" t="n"/>
+      <c r="B315" s="17" t="n">
+        <v>46265</v>
+      </c>
+      <c r="C315" s="14" t="inlineStr">
+        <is>
+          <t>Almacén</t>
+        </is>
+      </c>
       <c r="D315" s="27" t="n"/>
-      <c r="E315" s="28" t="n"/>
+      <c r="E315" s="28" t="n">
+        <v>80000</v>
+      </c>
       <c r="F315" s="15">
-        <f>IF(OR(D299&lt;&gt;"",E299&lt;&gt;""),IF(D299="",0,D299)+IF(E299="",0,E299),"")</f>
+        <f>IF(OR(D315&lt;&gt;"",E315&lt;&gt;""),IF(D315="",0,D315)+IF(E315="",0,E315),"")</f>
         <v/>
       </c>
-      <c r="G315" s="14" t="n"/>
+      <c r="G315" s="14" t="inlineStr">
+        <is>
+          <t>ALMACEN CHRIS · total agosto (sin desglose) · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="316">
       <c r="A316" s="14" t="inlineStr">
@@ -64844,7 +64874,7 @@
       <c r="D316" s="27" t="n"/>
       <c r="E316" s="28" t="n"/>
       <c r="F316" s="15">
-        <f>IF(OR(D300&lt;&gt;"",E300&lt;&gt;""),IF(D300="",0,D300)+IF(E300="",0,E300),"")</f>
+        <f>IF(OR(D316&lt;&gt;"",E316&lt;&gt;""),IF(D316="",0,D316)+IF(E316="",0,E316),"")</f>
         <v/>
       </c>
       <c r="G316" s="14" t="n"/>
@@ -64860,7 +64890,7 @@
       <c r="D317" s="27" t="n"/>
       <c r="E317" s="28" t="n"/>
       <c r="F317" s="15">
-        <f>IF(OR(D301&lt;&gt;"",E301&lt;&gt;""),IF(D301="",0,D301)+IF(E301="",0,E301),"")</f>
+        <f>IF(OR(D317&lt;&gt;"",E317&lt;&gt;""),IF(D317="",0,D317)+IF(E317="",0,E317),"")</f>
         <v/>
       </c>
       <c r="G317" s="14" t="n"/>
@@ -64876,7 +64906,7 @@
       <c r="D318" s="27" t="n"/>
       <c r="E318" s="28" t="n"/>
       <c r="F318" s="15">
-        <f>IF(OR(D302&lt;&gt;"",E302&lt;&gt;""),IF(D302="",0,D302)+IF(E302="",0,E302),"")</f>
+        <f>IF(OR(D318&lt;&gt;"",E318&lt;&gt;""),IF(D318="",0,D318)+IF(E318="",0,E318),"")</f>
         <v/>
       </c>
       <c r="G318" s="14" t="n"/>
@@ -64892,7 +64922,7 @@
       <c r="D319" s="27" t="n"/>
       <c r="E319" s="28" t="n"/>
       <c r="F319" s="15">
-        <f>IF(OR(D303&lt;&gt;"",E303&lt;&gt;""),IF(D303="",0,D303)+IF(E303="",0,E303),"")</f>
+        <f>IF(OR(D319&lt;&gt;"",E319&lt;&gt;""),IF(D319="",0,D319)+IF(E319="",0,E319),"")</f>
         <v/>
       </c>
       <c r="G319" s="14" t="n"/>
@@ -64908,7 +64938,7 @@
       <c r="D320" s="27" t="n"/>
       <c r="E320" s="28" t="n"/>
       <c r="F320" s="15">
-        <f>IF(OR(D304&lt;&gt;"",E304&lt;&gt;""),IF(D304="",0,D304)+IF(E304="",0,E304),"")</f>
+        <f>IF(OR(D320&lt;&gt;"",E320&lt;&gt;""),IF(D320="",0,D320)+IF(E320="",0,E320),"")</f>
         <v/>
       </c>
       <c r="G320" s="14" t="n"/>
@@ -64924,7 +64954,7 @@
       <c r="D321" s="27" t="n"/>
       <c r="E321" s="28" t="n"/>
       <c r="F321" s="15">
-        <f>IF(OR(D305&lt;&gt;"",E305&lt;&gt;""),IF(D305="",0,D305)+IF(E305="",0,E305),"")</f>
+        <f>IF(OR(D321&lt;&gt;"",E321&lt;&gt;""),IF(D321="",0,D321)+IF(E321="",0,E321),"")</f>
         <v/>
       </c>
       <c r="G321" s="14" t="n"/>
@@ -64940,7 +64970,7 @@
       <c r="D322" s="27" t="n"/>
       <c r="E322" s="28" t="n"/>
       <c r="F322" s="15">
-        <f>IF(OR(D306&lt;&gt;"",E306&lt;&gt;""),IF(D306="",0,D306)+IF(E306="",0,E306),"")</f>
+        <f>IF(OR(D322&lt;&gt;"",E322&lt;&gt;""),IF(D322="",0,D322)+IF(E322="",0,E322),"")</f>
         <v/>
       </c>
       <c r="G322" s="14" t="n"/>
@@ -64956,7 +64986,7 @@
       <c r="D323" s="27" t="n"/>
       <c r="E323" s="28" t="n"/>
       <c r="F323" s="15">
-        <f>IF(OR(D307&lt;&gt;"",E307&lt;&gt;""),IF(D307="",0,D307)+IF(E307="",0,E307),"")</f>
+        <f>IF(OR(D323&lt;&gt;"",E323&lt;&gt;""),IF(D323="",0,D323)+IF(E323="",0,E323),"")</f>
         <v/>
       </c>
       <c r="G323" s="14" t="n"/>
@@ -64972,7 +65002,7 @@
       <c r="D324" s="27" t="n"/>
       <c r="E324" s="28" t="n"/>
       <c r="F324" s="15">
-        <f>IF(OR(D308&lt;&gt;"",E308&lt;&gt;""),IF(D308="",0,D308)+IF(E308="",0,E308),"")</f>
+        <f>IF(OR(D324&lt;&gt;"",E324&lt;&gt;""),IF(D324="",0,D324)+IF(E324="",0,E324),"")</f>
         <v/>
       </c>
       <c r="G324" s="14" t="n"/>
@@ -64988,7 +65018,7 @@
       <c r="D325" s="27" t="n"/>
       <c r="E325" s="28" t="n"/>
       <c r="F325" s="15">
-        <f>IF(OR(D309&lt;&gt;"",E309&lt;&gt;""),IF(D309="",0,D309)+IF(E309="",0,E309),"")</f>
+        <f>IF(OR(D325&lt;&gt;"",E325&lt;&gt;""),IF(D325="",0,D325)+IF(E325="",0,E325),"")</f>
         <v/>
       </c>
       <c r="G325" s="14" t="n"/>
@@ -65004,7 +65034,7 @@
       <c r="D326" s="27" t="n"/>
       <c r="E326" s="28" t="n"/>
       <c r="F326" s="15">
-        <f>IF(OR(D310&lt;&gt;"",E310&lt;&gt;""),IF(D310="",0,D310)+IF(E310="",0,E310),"")</f>
+        <f>IF(OR(D326&lt;&gt;"",E326&lt;&gt;""),IF(D326="",0,D326)+IF(E326="",0,E326),"")</f>
         <v/>
       </c>
       <c r="G326" s="14" t="n"/>
@@ -65020,7 +65050,7 @@
       <c r="D327" s="27" t="n"/>
       <c r="E327" s="28" t="n"/>
       <c r="F327" s="15">
-        <f>IF(OR(D311&lt;&gt;"",E311&lt;&gt;""),IF(D311="",0,D311)+IF(E311="",0,E311),"")</f>
+        <f>IF(OR(D327&lt;&gt;"",E327&lt;&gt;""),IF(D327="",0,D327)+IF(E327="",0,E327),"")</f>
         <v/>
       </c>
       <c r="G327" s="14" t="n"/>
@@ -65036,7 +65066,7 @@
       <c r="D328" s="27" t="n"/>
       <c r="E328" s="28" t="n"/>
       <c r="F328" s="15">
-        <f>IF(OR(D312&lt;&gt;"",E312&lt;&gt;""),IF(D312="",0,D312)+IF(E312="",0,E312),"")</f>
+        <f>IF(OR(D328&lt;&gt;"",E328&lt;&gt;""),IF(D328="",0,D328)+IF(E328="",0,E328),"")</f>
         <v/>
       </c>
       <c r="G328" s="14" t="n"/>
@@ -65052,7 +65082,7 @@
       <c r="D329" s="27" t="n"/>
       <c r="E329" s="28" t="n"/>
       <c r="F329" s="15">
-        <f>IF(OR(D313&lt;&gt;"",E313&lt;&gt;""),IF(D313="",0,D313)+IF(E313="",0,E313),"")</f>
+        <f>IF(OR(D329&lt;&gt;"",E329&lt;&gt;""),IF(D329="",0,D329)+IF(E329="",0,E329),"")</f>
         <v/>
       </c>
       <c r="G329" s="14" t="n"/>
@@ -65068,7 +65098,7 @@
       <c r="D330" s="27" t="n"/>
       <c r="E330" s="28" t="n"/>
       <c r="F330" s="15">
-        <f>IF(OR(D314&lt;&gt;"",E314&lt;&gt;""),IF(D314="",0,D314)+IF(E314="",0,E314),"")</f>
+        <f>IF(OR(D330&lt;&gt;"",E330&lt;&gt;""),IF(D330="",0,D330)+IF(E330="",0,E330),"")</f>
         <v/>
       </c>
       <c r="G330" s="14" t="n"/>
@@ -65084,7 +65114,7 @@
       <c r="D331" s="27" t="n"/>
       <c r="E331" s="28" t="n"/>
       <c r="F331" s="15">
-        <f>IF(OR(D315&lt;&gt;"",E315&lt;&gt;""),IF(D315="",0,D315)+IF(E315="",0,E315),"")</f>
+        <f>IF(OR(D331&lt;&gt;"",E331&lt;&gt;""),IF(D331="",0,D331)+IF(E331="",0,E331),"")</f>
         <v/>
       </c>
       <c r="G331" s="14" t="n"/>
@@ -65100,7 +65130,7 @@
       <c r="D332" s="27" t="n"/>
       <c r="E332" s="28" t="n"/>
       <c r="F332" s="15">
-        <f>IF(OR(D316&lt;&gt;"",E316&lt;&gt;""),IF(D316="",0,D316)+IF(E316="",0,E316),"")</f>
+        <f>IF(OR(D332&lt;&gt;"",E332&lt;&gt;""),IF(D332="",0,D332)+IF(E332="",0,E332),"")</f>
         <v/>
       </c>
       <c r="G332" s="14" t="n"/>
@@ -65116,7 +65146,7 @@
       <c r="D333" s="27" t="n"/>
       <c r="E333" s="28" t="n"/>
       <c r="F333" s="15">
-        <f>IF(OR(D317&lt;&gt;"",E317&lt;&gt;""),IF(D317="",0,D317)+IF(E317="",0,E317),"")</f>
+        <f>IF(OR(D333&lt;&gt;"",E333&lt;&gt;""),IF(D333="",0,D333)+IF(E333="",0,E333),"")</f>
         <v/>
       </c>
       <c r="G333" s="14" t="n"/>
@@ -65132,7 +65162,7 @@
       <c r="D334" s="27" t="n"/>
       <c r="E334" s="28" t="n"/>
       <c r="F334" s="15">
-        <f>IF(OR(D318&lt;&gt;"",E318&lt;&gt;""),IF(D318="",0,D318)+IF(E318="",0,E318),"")</f>
+        <f>IF(OR(D334&lt;&gt;"",E334&lt;&gt;""),IF(D334="",0,D334)+IF(E334="",0,E334),"")</f>
         <v/>
       </c>
       <c r="G334" s="14" t="n"/>
@@ -65148,7 +65178,7 @@
       <c r="D335" s="27" t="n"/>
       <c r="E335" s="28" t="n"/>
       <c r="F335" s="15">
-        <f>IF(OR(D319&lt;&gt;"",E319&lt;&gt;""),IF(D319="",0,D319)+IF(E319="",0,E319),"")</f>
+        <f>IF(OR(D335&lt;&gt;"",E335&lt;&gt;""),IF(D335="",0,D335)+IF(E335="",0,E335),"")</f>
         <v/>
       </c>
       <c r="G335" s="14" t="n"/>
@@ -65164,7 +65194,7 @@
       <c r="D336" s="27" t="n"/>
       <c r="E336" s="28" t="n"/>
       <c r="F336" s="15">
-        <f>IF(OR(D320&lt;&gt;"",E320&lt;&gt;""),IF(D320="",0,D320)+IF(E320="",0,E320),"")</f>
+        <f>IF(OR(D336&lt;&gt;"",E336&lt;&gt;""),IF(D336="",0,D336)+IF(E336="",0,E336),"")</f>
         <v/>
       </c>
       <c r="G336" s="14" t="n"/>
@@ -65180,7 +65210,7 @@
       <c r="D337" s="27" t="n"/>
       <c r="E337" s="28" t="n"/>
       <c r="F337" s="15">
-        <f>IF(OR(D321&lt;&gt;"",E321&lt;&gt;""),IF(D321="",0,D321)+IF(E321="",0,E321),"")</f>
+        <f>IF(OR(D337&lt;&gt;"",E337&lt;&gt;""),IF(D337="",0,D337)+IF(E337="",0,E337),"")</f>
         <v/>
       </c>
       <c r="G337" s="14" t="n"/>
@@ -65196,7 +65226,7 @@
       <c r="D338" s="27" t="n"/>
       <c r="E338" s="28" t="n"/>
       <c r="F338" s="15">
-        <f>IF(OR(D322&lt;&gt;"",E322&lt;&gt;""),IF(D322="",0,D322)+IF(E322="",0,E322),"")</f>
+        <f>IF(OR(D338&lt;&gt;"",E338&lt;&gt;""),IF(D338="",0,D338)+IF(E338="",0,E338),"")</f>
         <v/>
       </c>
       <c r="G338" s="14" t="n"/>
@@ -65212,7 +65242,7 @@
       <c r="D339" s="27" t="n"/>
       <c r="E339" s="28" t="n"/>
       <c r="F339" s="15">
-        <f>IF(OR(D323&lt;&gt;"",E323&lt;&gt;""),IF(D323="",0,D323)+IF(E323="",0,E323),"")</f>
+        <f>IF(OR(D339&lt;&gt;"",E339&lt;&gt;""),IF(D339="",0,D339)+IF(E339="",0,E339),"")</f>
         <v/>
       </c>
       <c r="G339" s="14" t="n"/>
@@ -65228,7 +65258,7 @@
       <c r="D340" s="27" t="n"/>
       <c r="E340" s="28" t="n"/>
       <c r="F340" s="15">
-        <f>IF(OR(D324&lt;&gt;"",E324&lt;&gt;""),IF(D324="",0,D324)+IF(E324="",0,E324),"")</f>
+        <f>IF(OR(D340&lt;&gt;"",E340&lt;&gt;""),IF(D340="",0,D340)+IF(E340="",0,E340),"")</f>
         <v/>
       </c>
       <c r="G340" s="14" t="n"/>
@@ -65244,7 +65274,7 @@
       <c r="D341" s="27" t="n"/>
       <c r="E341" s="28" t="n"/>
       <c r="F341" s="15">
-        <f>IF(OR(D325&lt;&gt;"",E325&lt;&gt;""),IF(D325="",0,D325)+IF(E325="",0,E325),"")</f>
+        <f>IF(OR(D341&lt;&gt;"",E341&lt;&gt;""),IF(D341="",0,D341)+IF(E341="",0,E341),"")</f>
         <v/>
       </c>
       <c r="G341" s="14" t="n"/>
@@ -65260,7 +65290,7 @@
       <c r="D342" s="27" t="n"/>
       <c r="E342" s="28" t="n"/>
       <c r="F342" s="15">
-        <f>IF(OR(D326&lt;&gt;"",E326&lt;&gt;""),IF(D326="",0,D326)+IF(E326="",0,E326),"")</f>
+        <f>IF(OR(D342&lt;&gt;"",E342&lt;&gt;""),IF(D342="",0,D342)+IF(E342="",0,E342),"")</f>
         <v/>
       </c>
       <c r="G342" s="14" t="n"/>
@@ -65276,7 +65306,7 @@
       <c r="D343" s="27" t="n"/>
       <c r="E343" s="28" t="n"/>
       <c r="F343" s="15">
-        <f>IF(OR(D327&lt;&gt;"",E327&lt;&gt;""),IF(D327="",0,D327)+IF(E327="",0,E327),"")</f>
+        <f>IF(OR(D343&lt;&gt;"",E343&lt;&gt;""),IF(D343="",0,D343)+IF(E343="",0,E343),"")</f>
         <v/>
       </c>
       <c r="G343" s="14" t="n"/>
@@ -65292,7 +65322,7 @@
       <c r="D344" s="27" t="n"/>
       <c r="E344" s="28" t="n"/>
       <c r="F344" s="15">
-        <f>IF(OR(D328&lt;&gt;"",E328&lt;&gt;""),IF(D328="",0,D328)+IF(E328="",0,E328),"")</f>
+        <f>IF(OR(D344&lt;&gt;"",E344&lt;&gt;""),IF(D344="",0,D344)+IF(E344="",0,E344),"")</f>
         <v/>
       </c>
       <c r="G344" s="14" t="n"/>
@@ -65308,7 +65338,7 @@
       <c r="D345" s="27" t="n"/>
       <c r="E345" s="28" t="n"/>
       <c r="F345" s="15">
-        <f>IF(OR(D329&lt;&gt;"",E329&lt;&gt;""),IF(D329="",0,D329)+IF(E329="",0,E329),"")</f>
+        <f>IF(OR(D345&lt;&gt;"",E345&lt;&gt;""),IF(D345="",0,D345)+IF(E345="",0,E345),"")</f>
         <v/>
       </c>
       <c r="G345" s="14" t="n"/>
@@ -65324,7 +65354,7 @@
       <c r="D346" s="27" t="n"/>
       <c r="E346" s="28" t="n"/>
       <c r="F346" s="15">
-        <f>IF(OR(D330&lt;&gt;"",E330&lt;&gt;""),IF(D330="",0,D330)+IF(E330="",0,E330),"")</f>
+        <f>IF(OR(D346&lt;&gt;"",E346&lt;&gt;""),IF(D346="",0,D346)+IF(E346="",0,E346),"")</f>
         <v/>
       </c>
       <c r="G346" s="14" t="n"/>
@@ -65340,7 +65370,7 @@
       <c r="D347" s="27" t="n"/>
       <c r="E347" s="28" t="n"/>
       <c r="F347" s="15">
-        <f>IF(OR(D331&lt;&gt;"",E331&lt;&gt;""),IF(D331="",0,D331)+IF(E331="",0,E331),"")</f>
+        <f>IF(OR(D347&lt;&gt;"",E347&lt;&gt;""),IF(D347="",0,D347)+IF(E347="",0,E347),"")</f>
         <v/>
       </c>
       <c r="G347" s="14" t="n"/>
@@ -65356,7 +65386,7 @@
       <c r="D348" s="27" t="n"/>
       <c r="E348" s="28" t="n"/>
       <c r="F348" s="15">
-        <f>IF(OR(D332&lt;&gt;"",E332&lt;&gt;""),IF(D332="",0,D332)+IF(E332="",0,E332),"")</f>
+        <f>IF(OR(D348&lt;&gt;"",E348&lt;&gt;""),IF(D348="",0,D348)+IF(E348="",0,E348),"")</f>
         <v/>
       </c>
       <c r="G348" s="14" t="n"/>
@@ -65372,7 +65402,7 @@
       <c r="D349" s="27" t="n"/>
       <c r="E349" s="28" t="n"/>
       <c r="F349" s="15">
-        <f>IF(OR(D333&lt;&gt;"",E333&lt;&gt;""),IF(D333="",0,D333)+IF(E333="",0,E333),"")</f>
+        <f>IF(OR(D349&lt;&gt;"",E349&lt;&gt;""),IF(D349="",0,D349)+IF(E349="",0,E349),"")</f>
         <v/>
       </c>
       <c r="G349" s="14" t="n"/>
@@ -65388,7 +65418,7 @@
       <c r="D350" s="27" t="n"/>
       <c r="E350" s="28" t="n"/>
       <c r="F350" s="15">
-        <f>IF(OR(D334&lt;&gt;"",E334&lt;&gt;""),IF(D334="",0,D334)+IF(E334="",0,E334),"")</f>
+        <f>IF(OR(D350&lt;&gt;"",E350&lt;&gt;""),IF(D350="",0,D350)+IF(E350="",0,E350),"")</f>
         <v/>
       </c>
       <c r="G350" s="14" t="n"/>
@@ -65404,7 +65434,7 @@
       <c r="D351" s="27" t="n"/>
       <c r="E351" s="28" t="n"/>
       <c r="F351" s="15">
-        <f>IF(OR(D335&lt;&gt;"",E335&lt;&gt;""),IF(D335="",0,D335)+IF(E335="",0,E335),"")</f>
+        <f>IF(OR(D351&lt;&gt;"",E351&lt;&gt;""),IF(D351="",0,D351)+IF(E351="",0,E351),"")</f>
         <v/>
       </c>
       <c r="G351" s="14" t="n"/>
@@ -65420,7 +65450,7 @@
       <c r="D352" s="27" t="n"/>
       <c r="E352" s="28" t="n"/>
       <c r="F352" s="15">
-        <f>IF(OR(D336&lt;&gt;"",E336&lt;&gt;""),IF(D336="",0,D336)+IF(E336="",0,E336),"")</f>
+        <f>IF(OR(D352&lt;&gt;"",E352&lt;&gt;""),IF(D352="",0,D352)+IF(E352="",0,E352),"")</f>
         <v/>
       </c>
       <c r="G352" s="14" t="n"/>
@@ -65436,7 +65466,7 @@
       <c r="D353" s="27" t="n"/>
       <c r="E353" s="28" t="n"/>
       <c r="F353" s="15">
-        <f>IF(OR(D337&lt;&gt;"",E337&lt;&gt;""),IF(D337="",0,D337)+IF(E337="",0,E337),"")</f>
+        <f>IF(OR(D353&lt;&gt;"",E353&lt;&gt;""),IF(D353="",0,D353)+IF(E353="",0,E353),"")</f>
         <v/>
       </c>
       <c r="G353" s="14" t="n"/>
@@ -69211,7 +69241,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I82"/>
+  <dimension ref="A1:I86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -70310,18 +70340,26 @@
       </c>
       <c r="C35" s="14" t="inlineStr">
         <is>
-          <t>Telecentro CIUDAD — servicio mensual 08/2026</t>
+          <t>Telecentro CIUDAD — cobro Visa *3200 24/07/2026 (agosto)</t>
         </is>
       </c>
       <c r="D35" s="15" t="n">
-        <v>50000</v>
-      </c>
-      <c r="E35" s="14" t="inlineStr"/>
-      <c r="F35" s="18" t="inlineStr"/>
+        <v>31999</v>
+      </c>
+      <c r="E35" s="14" t="inlineStr">
+        <is>
+          <t>BBVA Visa *3200</t>
+        </is>
+      </c>
+      <c r="F35" s="18" t="inlineStr">
+        <is>
+          <t>3491192</t>
+        </is>
+      </c>
       <c r="G35" s="18" t="inlineStr"/>
       <c r="H35" s="14" t="inlineStr">
         <is>
-          <t>Recurrente $50.000/mes hasta nuevo aviso</t>
+          <t>Aviso tarjeta Visa *3200 · ARS 31.999 · período agosto · reemplaza recurrente $50.000</t>
         </is>
       </c>
       <c r="I35" s="14" t="inlineStr">
@@ -71747,6 +71785,128 @@
       <c r="I82" t="inlineStr">
         <is>
           <t>Julio</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="52" t="n">
+        <v>46252</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Metrogas</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Metrogas CIUDAD · vence 18/08/2026 · emisión 05/08/2026 (débito automático; mes = vencimiento)</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>73187</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Débito automático BBVA Visa</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>30010996459</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>40049923</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>ceil desde $73.186,92 · período consumo 06/06–07/07/2026 · mes gasto = cobro/vencimiento</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="52" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>ABL</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Agip ABL GCBA · partida 397789 · CUOTA 08/2026</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>41344</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Dinero disponible</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>ceil desde $41.343,91 · 1° vto 14/08/2026 · CIUDAD 1132 · Sol paga MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="52" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>LIMPIEZA CASA</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>LIMPIEZA CASA — Agosto 2026</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>567080</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Dinero disponible</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Transferencia MP · Susana Carmen Ortiz consolidado (8/8 123240; 16/8 126240; 22/8 154800+3800; 29/8 150000+9000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="52" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>LIMPIEZA CASA</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>LIMPIEZA CASA — Julio 2026</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>653120</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Dinero disponible</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Transferencia MP · Susana Carmen Ortiz consolidado (5/7 9500+123240; 12/7 120240; 18/7 147660; 25/7 126240; 31/7 126240)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete July CIUDAD gaps: Chris almacén, Todo Tartas, Telecentro.
Add ALMACEN CHRIS $155,800 and missing Todo Tartas $57,600; supersede Telecentro July $50k placeholder in favor of BBVA debit $31,999; document July status.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -57160,7 +57160,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G554"/>
+  <dimension ref="A1:G799"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -61720,6 +61720,7 @@
       </c>
       <c r="G176" s="22" t="n"/>
     </row>
+    <row r="177"/>
     <row r="178">
       <c r="A178" s="14" t="inlineStr">
         <is>
@@ -63002,6 +63003,7 @@
       </c>
       <c r="G228" s="22" t="n"/>
     </row>
+    <row r="229"/>
     <row r="230">
       <c r="A230" s="14" t="inlineStr">
         <is>
@@ -64040,6 +64042,7 @@
       </c>
       <c r="G273" s="22" t="n"/>
     </row>
+    <row r="274"/>
     <row r="275">
       <c r="A275" s="14" t="inlineStr">
         <is>
@@ -64391,15 +64394,27 @@
           <t>Julio</t>
         </is>
       </c>
-      <c r="B288" s="17" t="n"/>
-      <c r="C288" s="14" t="n"/>
+      <c r="B288" s="17" t="n">
+        <v>46234</v>
+      </c>
+      <c r="C288" s="14" t="inlineStr">
+        <is>
+          <t>Almacén</t>
+        </is>
+      </c>
       <c r="D288" s="27" t="n"/>
-      <c r="E288" s="28" t="n"/>
+      <c r="E288" s="28" t="n">
+        <v>155800</v>
+      </c>
       <c r="F288" s="15">
-        <f>IF(OR(D273&lt;&gt;"",E273&lt;&gt;""),IF(D273="",0,D273)+IF(E273="",0,E273),"")</f>
+        <f>IF(OR(D288&lt;&gt;"",E288&lt;&gt;""),IF(D288="",0,D288)+IF(E288="",0,E288),"")</f>
         <v/>
       </c>
-      <c r="G288" s="14" t="n"/>
+      <c r="G288" s="14" t="inlineStr">
+        <is>
+          <t>ALMACEN CHRIS · total julio (sin desglose) · REVISAR</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" s="14" t="inlineStr">
@@ -64407,15 +64422,27 @@
           <t>Julio</t>
         </is>
       </c>
-      <c r="B289" s="17" t="n"/>
-      <c r="C289" s="14" t="n"/>
-      <c r="D289" s="27" t="n"/>
+      <c r="B289" s="17" t="n">
+        <v>46224</v>
+      </c>
+      <c r="C289" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · Todo Tartas</t>
+        </is>
+      </c>
+      <c r="D289" s="27" t="n">
+        <v>57600</v>
+      </c>
       <c r="E289" s="28" t="n"/>
       <c r="F289" s="15">
-        <f>IF(OR(D274&lt;&gt;"",E274&lt;&gt;""),IF(D274="",0,D274)+IF(E274="",0,E274),"")</f>
+        <f>IF(OR(D289&lt;&gt;"",E289&lt;&gt;""),IF(D289="",0,D289)+IF(E289="",0,E289),"")</f>
         <v/>
       </c>
-      <c r="G289" s="14" t="n"/>
+      <c r="G289" s="14" t="inlineStr">
+        <is>
+          <t>MP · panadería · ex `Todo Tartas`</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" s="14" t="inlineStr">
@@ -64428,7 +64455,7 @@
       <c r="D290" s="27" t="n"/>
       <c r="E290" s="28" t="n"/>
       <c r="F290" s="15">
-        <f>IF(OR(D275&lt;&gt;"",E275&lt;&gt;""),IF(D275="",0,D275)+IF(E275="",0,E275),"")</f>
+        <f>IF(OR(D290&lt;&gt;"",E290&lt;&gt;""),IF(D290="",0,D290)+IF(E290="",0,E290),"")</f>
         <v/>
       </c>
       <c r="G290" s="14" t="n"/>
@@ -64444,7 +64471,7 @@
       <c r="D291" s="27" t="n"/>
       <c r="E291" s="28" t="n"/>
       <c r="F291" s="15">
-        <f>IF(OR(D276&lt;&gt;"",E276&lt;&gt;""),IF(D276="",0,D276)+IF(E276="",0,E276),"")</f>
+        <f>IF(OR(D291&lt;&gt;"",E291&lt;&gt;""),IF(D291="",0,D291)+IF(E291="",0,E291),"")</f>
         <v/>
       </c>
       <c r="G291" s="14" t="n"/>
@@ -64460,7 +64487,7 @@
       <c r="D292" s="27" t="n"/>
       <c r="E292" s="28" t="n"/>
       <c r="F292" s="15">
-        <f>IF(OR(D277&lt;&gt;"",E277&lt;&gt;""),IF(D277="",0,D277)+IF(E277="",0,E277),"")</f>
+        <f>IF(OR(D292&lt;&gt;"",E292&lt;&gt;""),IF(D292="",0,D292)+IF(E292="",0,E292),"")</f>
         <v/>
       </c>
       <c r="G292" s="14" t="n"/>
@@ -64476,7 +64503,7 @@
       <c r="D293" s="27" t="n"/>
       <c r="E293" s="28" t="n"/>
       <c r="F293" s="15">
-        <f>IF(OR(D278&lt;&gt;"",E278&lt;&gt;""),IF(D278="",0,D278)+IF(E278="",0,E278),"")</f>
+        <f>IF(OR(D293&lt;&gt;"",E293&lt;&gt;""),IF(D293="",0,D293)+IF(E293="",0,E293),"")</f>
         <v/>
       </c>
       <c r="G293" s="14" t="n"/>
@@ -64492,7 +64519,7 @@
       <c r="D294" s="27" t="n"/>
       <c r="E294" s="28" t="n"/>
       <c r="F294" s="15">
-        <f>IF(OR(D279&lt;&gt;"",E279&lt;&gt;""),IF(D279="",0,D279)+IF(E279="",0,E279),"")</f>
+        <f>IF(OR(D294&lt;&gt;"",E294&lt;&gt;""),IF(D294="",0,D294)+IF(E294="",0,E294),"")</f>
         <v/>
       </c>
       <c r="G294" s="14" t="n"/>
@@ -64508,7 +64535,7 @@
       <c r="D295" s="27" t="n"/>
       <c r="E295" s="28" t="n"/>
       <c r="F295" s="15">
-        <f>IF(OR(D280&lt;&gt;"",E280&lt;&gt;""),IF(D280="",0,D280)+IF(E280="",0,E280),"")</f>
+        <f>IF(OR(D295&lt;&gt;"",E295&lt;&gt;""),IF(D295="",0,D295)+IF(E295="",0,E295),"")</f>
         <v/>
       </c>
       <c r="G295" s="14" t="n"/>
@@ -64524,7 +64551,7 @@
       <c r="D296" s="27" t="n"/>
       <c r="E296" s="28" t="n"/>
       <c r="F296" s="15">
-        <f>IF(OR(D281&lt;&gt;"",E281&lt;&gt;""),IF(D281="",0,D281)+IF(E281="",0,E281),"")</f>
+        <f>IF(OR(D296&lt;&gt;"",E296&lt;&gt;""),IF(D296="",0,D296)+IF(E296="",0,E296),"")</f>
         <v/>
       </c>
       <c r="G296" s="14" t="n"/>
@@ -64540,7 +64567,7 @@
       <c r="D297" s="27" t="n"/>
       <c r="E297" s="28" t="n"/>
       <c r="F297" s="15">
-        <f>IF(OR(D282&lt;&gt;"",E282&lt;&gt;""),IF(D282="",0,D282)+IF(E282="",0,E282),"")</f>
+        <f>IF(OR(D297&lt;&gt;"",E297&lt;&gt;""),IF(D297="",0,D297)+IF(E297="",0,E297),"")</f>
         <v/>
       </c>
       <c r="G297" s="14" t="n"/>
@@ -64556,7 +64583,7 @@
       <c r="D298" s="27" t="n"/>
       <c r="E298" s="28" t="n"/>
       <c r="F298" s="15">
-        <f>IF(OR(D283&lt;&gt;"",E283&lt;&gt;""),IF(D283="",0,D283)+IF(E283="",0,E283),"")</f>
+        <f>IF(OR(D298&lt;&gt;"",E298&lt;&gt;""),IF(D298="",0,D298)+IF(E298="",0,E298),"")</f>
         <v/>
       </c>
       <c r="G298" s="14" t="n"/>
@@ -64572,7 +64599,7 @@
       <c r="D299" s="27" t="n"/>
       <c r="E299" s="28" t="n"/>
       <c r="F299" s="15">
-        <f>IF(OR(D284&lt;&gt;"",E284&lt;&gt;""),IF(D284="",0,D284)+IF(E284="",0,E284),"")</f>
+        <f>IF(OR(D299&lt;&gt;"",E299&lt;&gt;""),IF(D299="",0,D299)+IF(E299="",0,E299),"")</f>
         <v/>
       </c>
       <c r="G299" s="14" t="n"/>
@@ -64588,7 +64615,7 @@
       <c r="D300" s="27" t="n"/>
       <c r="E300" s="28" t="n"/>
       <c r="F300" s="15">
-        <f>IF(OR(D285&lt;&gt;"",E285&lt;&gt;""),IF(D285="",0,D285)+IF(E285="",0,E285),"")</f>
+        <f>IF(OR(D300&lt;&gt;"",E300&lt;&gt;""),IF(D300="",0,D300)+IF(E300="",0,E300),"")</f>
         <v/>
       </c>
       <c r="G300" s="14" t="n"/>
@@ -64604,7 +64631,7 @@
       <c r="D301" s="27" t="n"/>
       <c r="E301" s="28" t="n"/>
       <c r="F301" s="15">
-        <f>IF(OR(D286&lt;&gt;"",E286&lt;&gt;""),IF(D286="",0,D286)+IF(E286="",0,E286),"")</f>
+        <f>IF(OR(D301&lt;&gt;"",E301&lt;&gt;""),IF(D301="",0,D301)+IF(E301="",0,E301),"")</f>
         <v/>
       </c>
       <c r="G301" s="14" t="n"/>
@@ -64620,7 +64647,7 @@
       <c r="D302" s="27" t="n"/>
       <c r="E302" s="28" t="n"/>
       <c r="F302" s="15">
-        <f>IF(OR(D287&lt;&gt;"",E287&lt;&gt;""),IF(D287="",0,D287)+IF(E287="",0,E287),"")</f>
+        <f>IF(OR(D302&lt;&gt;"",E302&lt;&gt;""),IF(D302="",0,D302)+IF(E302="",0,E302),"")</f>
         <v/>
       </c>
       <c r="G302" s="14" t="n"/>
@@ -64636,7 +64663,7 @@
       <c r="D303" s="27" t="n"/>
       <c r="E303" s="28" t="n"/>
       <c r="F303" s="15">
-        <f>IF(OR(D288&lt;&gt;"",E288&lt;&gt;""),IF(D288="",0,D288)+IF(E288="",0,E288),"")</f>
+        <f>IF(OR(D303&lt;&gt;"",E303&lt;&gt;""),IF(D303="",0,D303)+IF(E303="",0,E303),"")</f>
         <v/>
       </c>
       <c r="G303" s="14" t="n"/>
@@ -64652,7 +64679,7 @@
       <c r="D304" s="27" t="n"/>
       <c r="E304" s="28" t="n"/>
       <c r="F304" s="15">
-        <f>IF(OR(D289&lt;&gt;"",E289&lt;&gt;""),IF(D289="",0,D289)+IF(E289="",0,E289),"")</f>
+        <f>IF(OR(D304&lt;&gt;"",E304&lt;&gt;""),IF(D304="",0,D304)+IF(E304="",0,E304),"")</f>
         <v/>
       </c>
       <c r="G304" s="14" t="n"/>
@@ -64668,7 +64695,7 @@
       <c r="D305" s="27" t="n"/>
       <c r="E305" s="28" t="n"/>
       <c r="F305" s="15">
-        <f>IF(OR(D290&lt;&gt;"",E290&lt;&gt;""),IF(D290="",0,D290)+IF(E290="",0,E290),"")</f>
+        <f>IF(OR(D305&lt;&gt;"",E305&lt;&gt;""),IF(D305="",0,D305)+IF(E305="",0,E305),"")</f>
         <v/>
       </c>
       <c r="G305" s="14" t="n"/>
@@ -64684,7 +64711,7 @@
       <c r="D306" s="27" t="n"/>
       <c r="E306" s="28" t="n"/>
       <c r="F306" s="15">
-        <f>IF(OR(D291&lt;&gt;"",E291&lt;&gt;""),IF(D291="",0,D291)+IF(E291="",0,E291),"")</f>
+        <f>IF(OR(D306&lt;&gt;"",E306&lt;&gt;""),IF(D306="",0,D306)+IF(E306="",0,E306),"")</f>
         <v/>
       </c>
       <c r="G306" s="14" t="n"/>
@@ -64700,7 +64727,7 @@
       <c r="D307" s="27" t="n"/>
       <c r="E307" s="28" t="n"/>
       <c r="F307" s="15">
-        <f>IF(OR(D292&lt;&gt;"",E292&lt;&gt;""),IF(D292="",0,D292)+IF(E292="",0,E292),"")</f>
+        <f>IF(OR(D307&lt;&gt;"",E307&lt;&gt;""),IF(D307="",0,D307)+IF(E307="",0,E307),"")</f>
         <v/>
       </c>
       <c r="G307" s="14" t="n"/>
@@ -64716,7 +64743,7 @@
       <c r="D308" s="27" t="n"/>
       <c r="E308" s="28" t="n"/>
       <c r="F308" s="15">
-        <f>IF(OR(D293&lt;&gt;"",E293&lt;&gt;""),IF(D293="",0,D293)+IF(E293="",0,E293),"")</f>
+        <f>IF(OR(D308&lt;&gt;"",E308&lt;&gt;""),IF(D308="",0,D308)+IF(E308="",0,E308),"")</f>
         <v/>
       </c>
       <c r="G308" s="14" t="n"/>
@@ -64732,7 +64759,7 @@
       <c r="D309" s="27" t="n"/>
       <c r="E309" s="28" t="n"/>
       <c r="F309" s="15">
-        <f>IF(OR(D294&lt;&gt;"",E294&lt;&gt;""),IF(D294="",0,D294)+IF(E294="",0,E294),"")</f>
+        <f>IF(OR(D309&lt;&gt;"",E309&lt;&gt;""),IF(D309="",0,D309)+IF(E309="",0,E309),"")</f>
         <v/>
       </c>
       <c r="G309" s="14" t="n"/>
@@ -64748,7 +64775,7 @@
       <c r="D310" s="27" t="n"/>
       <c r="E310" s="28" t="n"/>
       <c r="F310" s="15">
-        <f>IF(OR(D295&lt;&gt;"",E295&lt;&gt;""),IF(D295="",0,D295)+IF(E295="",0,E295),"")</f>
+        <f>IF(OR(D310&lt;&gt;"",E310&lt;&gt;""),IF(D310="",0,D310)+IF(E310="",0,E310),"")</f>
         <v/>
       </c>
       <c r="G310" s="14" t="n"/>
@@ -64807,6 +64834,7 @@
       </c>
       <c r="G312" s="22" t="n"/>
     </row>
+    <row r="313"/>
     <row r="314">
       <c r="A314" s="14" t="inlineStr">
         <is>
@@ -65497,6 +65525,7 @@
       </c>
       <c r="G354" s="22" t="n"/>
     </row>
+    <row r="355"/>
     <row r="356">
       <c r="A356" s="14" t="inlineStr">
         <is>
@@ -67178,6 +67207,7 @@
       </c>
       <c r="G426" s="22" t="n"/>
     </row>
+    <row r="427"/>
     <row r="428">
       <c r="A428" s="14" t="inlineStr">
         <is>
@@ -67844,6 +67874,7 @@
       </c>
       <c r="G468" s="22" t="n"/>
     </row>
+    <row r="469"/>
     <row r="470">
       <c r="A470" s="14" t="inlineStr">
         <is>
@@ -68510,6 +68541,7 @@
       </c>
       <c r="G510" s="22" t="n"/>
     </row>
+    <row r="511"/>
     <row r="512">
       <c r="A512" s="14" t="inlineStr">
         <is>
@@ -69230,6 +69262,251 @@
         </is>
       </c>
     </row>
+    <row r="555"/>
+    <row r="556"/>
+    <row r="557"/>
+    <row r="558"/>
+    <row r="559"/>
+    <row r="560"/>
+    <row r="561"/>
+    <row r="562"/>
+    <row r="563"/>
+    <row r="564"/>
+    <row r="565"/>
+    <row r="566"/>
+    <row r="567"/>
+    <row r="568"/>
+    <row r="569"/>
+    <row r="570"/>
+    <row r="571"/>
+    <row r="572"/>
+    <row r="573"/>
+    <row r="574"/>
+    <row r="575"/>
+    <row r="576"/>
+    <row r="577"/>
+    <row r="578"/>
+    <row r="579"/>
+    <row r="580"/>
+    <row r="581"/>
+    <row r="582"/>
+    <row r="583"/>
+    <row r="584"/>
+    <row r="585"/>
+    <row r="586"/>
+    <row r="587"/>
+    <row r="588"/>
+    <row r="589"/>
+    <row r="590"/>
+    <row r="591"/>
+    <row r="592"/>
+    <row r="593"/>
+    <row r="594"/>
+    <row r="595"/>
+    <row r="596"/>
+    <row r="597"/>
+    <row r="598"/>
+    <row r="599"/>
+    <row r="600"/>
+    <row r="601"/>
+    <row r="602"/>
+    <row r="603"/>
+    <row r="604"/>
+    <row r="605"/>
+    <row r="606"/>
+    <row r="607"/>
+    <row r="608"/>
+    <row r="609"/>
+    <row r="610"/>
+    <row r="611"/>
+    <row r="612"/>
+    <row r="613"/>
+    <row r="614"/>
+    <row r="615"/>
+    <row r="616"/>
+    <row r="617"/>
+    <row r="618"/>
+    <row r="619"/>
+    <row r="620"/>
+    <row r="621"/>
+    <row r="622"/>
+    <row r="623"/>
+    <row r="624"/>
+    <row r="625"/>
+    <row r="626"/>
+    <row r="627"/>
+    <row r="628"/>
+    <row r="629"/>
+    <row r="630"/>
+    <row r="631"/>
+    <row r="632"/>
+    <row r="633"/>
+    <row r="634"/>
+    <row r="635"/>
+    <row r="636"/>
+    <row r="637"/>
+    <row r="638"/>
+    <row r="639"/>
+    <row r="640"/>
+    <row r="641"/>
+    <row r="642"/>
+    <row r="643"/>
+    <row r="644"/>
+    <row r="645"/>
+    <row r="646"/>
+    <row r="647"/>
+    <row r="648"/>
+    <row r="649"/>
+    <row r="650"/>
+    <row r="651"/>
+    <row r="652"/>
+    <row r="653"/>
+    <row r="654"/>
+    <row r="655"/>
+    <row r="656"/>
+    <row r="657"/>
+    <row r="658"/>
+    <row r="659"/>
+    <row r="660"/>
+    <row r="661"/>
+    <row r="662"/>
+    <row r="663"/>
+    <row r="664"/>
+    <row r="665"/>
+    <row r="666"/>
+    <row r="667"/>
+    <row r="668"/>
+    <row r="669"/>
+    <row r="670"/>
+    <row r="671"/>
+    <row r="672"/>
+    <row r="673"/>
+    <row r="674"/>
+    <row r="675"/>
+    <row r="676"/>
+    <row r="677"/>
+    <row r="678"/>
+    <row r="679"/>
+    <row r="680"/>
+    <row r="681"/>
+    <row r="682"/>
+    <row r="683"/>
+    <row r="684"/>
+    <row r="685"/>
+    <row r="686"/>
+    <row r="687"/>
+    <row r="688"/>
+    <row r="689"/>
+    <row r="690"/>
+    <row r="691"/>
+    <row r="692"/>
+    <row r="693"/>
+    <row r="694"/>
+    <row r="695"/>
+    <row r="696"/>
+    <row r="697"/>
+    <row r="698"/>
+    <row r="699"/>
+    <row r="700"/>
+    <row r="701"/>
+    <row r="702"/>
+    <row r="703"/>
+    <row r="704"/>
+    <row r="705"/>
+    <row r="706"/>
+    <row r="707"/>
+    <row r="708"/>
+    <row r="709"/>
+    <row r="710"/>
+    <row r="711"/>
+    <row r="712"/>
+    <row r="713"/>
+    <row r="714"/>
+    <row r="715"/>
+    <row r="716"/>
+    <row r="717"/>
+    <row r="718"/>
+    <row r="719"/>
+    <row r="720"/>
+    <row r="721"/>
+    <row r="722"/>
+    <row r="723"/>
+    <row r="724"/>
+    <row r="725"/>
+    <row r="726"/>
+    <row r="727"/>
+    <row r="728"/>
+    <row r="729"/>
+    <row r="730"/>
+    <row r="731"/>
+    <row r="732"/>
+    <row r="733"/>
+    <row r="734"/>
+    <row r="735"/>
+    <row r="736"/>
+    <row r="737"/>
+    <row r="738"/>
+    <row r="739"/>
+    <row r="740"/>
+    <row r="741"/>
+    <row r="742"/>
+    <row r="743"/>
+    <row r="744"/>
+    <row r="745"/>
+    <row r="746"/>
+    <row r="747"/>
+    <row r="748"/>
+    <row r="749"/>
+    <row r="750"/>
+    <row r="751"/>
+    <row r="752"/>
+    <row r="753"/>
+    <row r="754"/>
+    <row r="755"/>
+    <row r="756"/>
+    <row r="757"/>
+    <row r="758"/>
+    <row r="759"/>
+    <row r="760"/>
+    <row r="761"/>
+    <row r="762"/>
+    <row r="763"/>
+    <row r="764"/>
+    <row r="765"/>
+    <row r="766"/>
+    <row r="767"/>
+    <row r="768"/>
+    <row r="769"/>
+    <row r="770"/>
+    <row r="771"/>
+    <row r="772"/>
+    <row r="773"/>
+    <row r="774"/>
+    <row r="775"/>
+    <row r="776"/>
+    <row r="777"/>
+    <row r="778"/>
+    <row r="779"/>
+    <row r="780"/>
+    <row r="781"/>
+    <row r="782"/>
+    <row r="783"/>
+    <row r="784"/>
+    <row r="785"/>
+    <row r="786"/>
+    <row r="787"/>
+    <row r="788"/>
+    <row r="789"/>
+    <row r="790"/>
+    <row r="791"/>
+    <row r="792"/>
+    <row r="793"/>
+    <row r="794"/>
+    <row r="795"/>
+    <row r="796"/>
+    <row r="797"/>
+    <row r="798"/>
+    <row r="799"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -70274,18 +70551,16 @@
       </c>
       <c r="C33" s="14" t="inlineStr">
         <is>
-          <t>Telecentro CIUDAD — servicio mensual 07/2026</t>
-        </is>
-      </c>
-      <c r="D33" s="15" t="n">
-        <v>50000</v>
-      </c>
+          <t>(duplicado) ver fila débito BBVA 30/06 — no sumar</t>
+        </is>
+      </c>
+      <c r="D33" s="15" t="n"/>
       <c r="E33" s="14" t="inlineStr"/>
       <c r="F33" s="18" t="inlineStr"/>
       <c r="G33" s="18" t="inlineStr"/>
       <c r="H33" s="14" t="inlineStr">
         <is>
-          <t>Recurrente $50.000/mes hasta nuevo aviso</t>
+          <t>SUPERSEDE · Telecentro Julio está en Detalle débito 30/06 $31.999</t>
         </is>
       </c>
       <c r="I33" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Load Telecentro Gmail invoices into CIUDAD TV CABLE.
Replace $50k placeholders with official factura amounts (Apr–May, Sep–Oct),
map months to invoice period, and keep Nov/Dec empty until new mails arrive.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -913,10 +913,10 @@
         <v>39163</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>50000</v>
+        <v>46909</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>50000</v>
+        <v>47939</v>
       </c>
       <c r="I6" s="9" t="n">
         <v>48420</v>
@@ -928,17 +928,13 @@
         <v>31999</v>
       </c>
       <c r="L6" s="9" t="n">
+        <v>82364</v>
+      </c>
+      <c r="M6" s="9" t="n">
         <v>69659</v>
       </c>
-      <c r="M6" s="9" t="n">
-        <v>50000</v>
-      </c>
-      <c r="N6" s="9" t="n">
-        <v>50000</v>
-      </c>
-      <c r="O6" s="9" t="n">
-        <v>50000</v>
-      </c>
+      <c r="N6" s="9" t="n"/>
+      <c r="O6" s="9" t="n"/>
       <c r="P6" s="7">
         <f>SUM(D6:O6)</f>
         <v/>
@@ -1756,7 +1752,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>• Telecentro: $50.000 mensuales hasta nuevo aviso</t>
+          <t>• Telecentro: montos desde facturas Gmail (facturadigital@factura.telecentro.com.ar); mes = período de factura. Cliente 3491192. Nov/Dic sin factura aún.</t>
         </is>
       </c>
     </row>
@@ -57160,7 +57156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G799"/>
+  <dimension ref="A1:G554"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -61720,7 +61716,6 @@
       </c>
       <c r="G176" s="22" t="n"/>
     </row>
-    <row r="177"/>
     <row r="178">
       <c r="A178" s="14" t="inlineStr">
         <is>
@@ -63003,7 +62998,6 @@
       </c>
       <c r="G228" s="22" t="n"/>
     </row>
-    <row r="229"/>
     <row r="230">
       <c r="A230" s="14" t="inlineStr">
         <is>
@@ -64042,7 +64036,6 @@
       </c>
       <c r="G273" s="22" t="n"/>
     </row>
-    <row r="274"/>
     <row r="275">
       <c r="A275" s="14" t="inlineStr">
         <is>
@@ -64834,7 +64827,6 @@
       </c>
       <c r="G312" s="22" t="n"/>
     </row>
-    <row r="313"/>
     <row r="314">
       <c r="A314" s="14" t="inlineStr">
         <is>
@@ -65525,7 +65517,6 @@
       </c>
       <c r="G354" s="22" t="n"/>
     </row>
-    <row r="355"/>
     <row r="356">
       <c r="A356" s="14" t="inlineStr">
         <is>
@@ -67207,7 +67198,6 @@
       </c>
       <c r="G426" s="22" t="n"/>
     </row>
-    <row r="427"/>
     <row r="428">
       <c r="A428" s="14" t="inlineStr">
         <is>
@@ -67874,7 +67864,6 @@
       </c>
       <c r="G468" s="22" t="n"/>
     </row>
-    <row r="469"/>
     <row r="470">
       <c r="A470" s="14" t="inlineStr">
         <is>
@@ -68541,7 +68530,6 @@
       </c>
       <c r="G510" s="22" t="n"/>
     </row>
-    <row r="511"/>
     <row r="512">
       <c r="A512" s="14" t="inlineStr">
         <is>
@@ -69262,251 +69250,6 @@
         </is>
       </c>
     </row>
-    <row r="555"/>
-    <row r="556"/>
-    <row r="557"/>
-    <row r="558"/>
-    <row r="559"/>
-    <row r="560"/>
-    <row r="561"/>
-    <row r="562"/>
-    <row r="563"/>
-    <row r="564"/>
-    <row r="565"/>
-    <row r="566"/>
-    <row r="567"/>
-    <row r="568"/>
-    <row r="569"/>
-    <row r="570"/>
-    <row r="571"/>
-    <row r="572"/>
-    <row r="573"/>
-    <row r="574"/>
-    <row r="575"/>
-    <row r="576"/>
-    <row r="577"/>
-    <row r="578"/>
-    <row r="579"/>
-    <row r="580"/>
-    <row r="581"/>
-    <row r="582"/>
-    <row r="583"/>
-    <row r="584"/>
-    <row r="585"/>
-    <row r="586"/>
-    <row r="587"/>
-    <row r="588"/>
-    <row r="589"/>
-    <row r="590"/>
-    <row r="591"/>
-    <row r="592"/>
-    <row r="593"/>
-    <row r="594"/>
-    <row r="595"/>
-    <row r="596"/>
-    <row r="597"/>
-    <row r="598"/>
-    <row r="599"/>
-    <row r="600"/>
-    <row r="601"/>
-    <row r="602"/>
-    <row r="603"/>
-    <row r="604"/>
-    <row r="605"/>
-    <row r="606"/>
-    <row r="607"/>
-    <row r="608"/>
-    <row r="609"/>
-    <row r="610"/>
-    <row r="611"/>
-    <row r="612"/>
-    <row r="613"/>
-    <row r="614"/>
-    <row r="615"/>
-    <row r="616"/>
-    <row r="617"/>
-    <row r="618"/>
-    <row r="619"/>
-    <row r="620"/>
-    <row r="621"/>
-    <row r="622"/>
-    <row r="623"/>
-    <row r="624"/>
-    <row r="625"/>
-    <row r="626"/>
-    <row r="627"/>
-    <row r="628"/>
-    <row r="629"/>
-    <row r="630"/>
-    <row r="631"/>
-    <row r="632"/>
-    <row r="633"/>
-    <row r="634"/>
-    <row r="635"/>
-    <row r="636"/>
-    <row r="637"/>
-    <row r="638"/>
-    <row r="639"/>
-    <row r="640"/>
-    <row r="641"/>
-    <row r="642"/>
-    <row r="643"/>
-    <row r="644"/>
-    <row r="645"/>
-    <row r="646"/>
-    <row r="647"/>
-    <row r="648"/>
-    <row r="649"/>
-    <row r="650"/>
-    <row r="651"/>
-    <row r="652"/>
-    <row r="653"/>
-    <row r="654"/>
-    <row r="655"/>
-    <row r="656"/>
-    <row r="657"/>
-    <row r="658"/>
-    <row r="659"/>
-    <row r="660"/>
-    <row r="661"/>
-    <row r="662"/>
-    <row r="663"/>
-    <row r="664"/>
-    <row r="665"/>
-    <row r="666"/>
-    <row r="667"/>
-    <row r="668"/>
-    <row r="669"/>
-    <row r="670"/>
-    <row r="671"/>
-    <row r="672"/>
-    <row r="673"/>
-    <row r="674"/>
-    <row r="675"/>
-    <row r="676"/>
-    <row r="677"/>
-    <row r="678"/>
-    <row r="679"/>
-    <row r="680"/>
-    <row r="681"/>
-    <row r="682"/>
-    <row r="683"/>
-    <row r="684"/>
-    <row r="685"/>
-    <row r="686"/>
-    <row r="687"/>
-    <row r="688"/>
-    <row r="689"/>
-    <row r="690"/>
-    <row r="691"/>
-    <row r="692"/>
-    <row r="693"/>
-    <row r="694"/>
-    <row r="695"/>
-    <row r="696"/>
-    <row r="697"/>
-    <row r="698"/>
-    <row r="699"/>
-    <row r="700"/>
-    <row r="701"/>
-    <row r="702"/>
-    <row r="703"/>
-    <row r="704"/>
-    <row r="705"/>
-    <row r="706"/>
-    <row r="707"/>
-    <row r="708"/>
-    <row r="709"/>
-    <row r="710"/>
-    <row r="711"/>
-    <row r="712"/>
-    <row r="713"/>
-    <row r="714"/>
-    <row r="715"/>
-    <row r="716"/>
-    <row r="717"/>
-    <row r="718"/>
-    <row r="719"/>
-    <row r="720"/>
-    <row r="721"/>
-    <row r="722"/>
-    <row r="723"/>
-    <row r="724"/>
-    <row r="725"/>
-    <row r="726"/>
-    <row r="727"/>
-    <row r="728"/>
-    <row r="729"/>
-    <row r="730"/>
-    <row r="731"/>
-    <row r="732"/>
-    <row r="733"/>
-    <row r="734"/>
-    <row r="735"/>
-    <row r="736"/>
-    <row r="737"/>
-    <row r="738"/>
-    <row r="739"/>
-    <row r="740"/>
-    <row r="741"/>
-    <row r="742"/>
-    <row r="743"/>
-    <row r="744"/>
-    <row r="745"/>
-    <row r="746"/>
-    <row r="747"/>
-    <row r="748"/>
-    <row r="749"/>
-    <row r="750"/>
-    <row r="751"/>
-    <row r="752"/>
-    <row r="753"/>
-    <row r="754"/>
-    <row r="755"/>
-    <row r="756"/>
-    <row r="757"/>
-    <row r="758"/>
-    <row r="759"/>
-    <row r="760"/>
-    <row r="761"/>
-    <row r="762"/>
-    <row r="763"/>
-    <row r="764"/>
-    <row r="765"/>
-    <row r="766"/>
-    <row r="767"/>
-    <row r="768"/>
-    <row r="769"/>
-    <row r="770"/>
-    <row r="771"/>
-    <row r="772"/>
-    <row r="773"/>
-    <row r="774"/>
-    <row r="775"/>
-    <row r="776"/>
-    <row r="777"/>
-    <row r="778"/>
-    <row r="779"/>
-    <row r="780"/>
-    <row r="781"/>
-    <row r="782"/>
-    <row r="783"/>
-    <row r="784"/>
-    <row r="785"/>
-    <row r="786"/>
-    <row r="787"/>
-    <row r="788"/>
-    <row r="789"/>
-    <row r="790"/>
-    <row r="791"/>
-    <row r="792"/>
-    <row r="793"/>
-    <row r="794"/>
-    <row r="795"/>
-    <row r="796"/>
-    <row r="797"/>
-    <row r="798"/>
-    <row r="799"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -69634,11 +69377,15 @@
         <v>37984</v>
       </c>
       <c r="E5" s="14" t="inlineStr"/>
-      <c r="F5" s="18" t="inlineStr"/>
+      <c r="F5" s="18" t="inlineStr">
+        <is>
+          <t>3491192</t>
+        </is>
+      </c>
       <c r="G5" s="18" t="inlineStr"/>
       <c r="H5" s="14" t="inlineStr">
         <is>
-          <t>Recurrente $50.000/mes hasta nuevo aviso</t>
+          <t>Gmail factura 01/2026 $37.983,38 · cliente 3491192</t>
         </is>
       </c>
       <c r="I5" s="14" t="inlineStr">
@@ -69766,11 +69513,15 @@
         <v>38489</v>
       </c>
       <c r="E9" s="14" t="inlineStr"/>
-      <c r="F9" s="18" t="inlineStr"/>
+      <c r="F9" s="18" t="inlineStr">
+        <is>
+          <t>3491192</t>
+        </is>
+      </c>
       <c r="G9" s="18" t="inlineStr"/>
       <c r="H9" s="14" t="inlineStr">
         <is>
-          <t>Recurrente $50.000/mes hasta nuevo aviso</t>
+          <t>Gmail factura 02/2026 $38.489,00 · cliente 3491192</t>
         </is>
       </c>
       <c r="I9" s="14" t="inlineStr">
@@ -69898,11 +69649,15 @@
         <v>39163</v>
       </c>
       <c r="E13" s="14" t="inlineStr"/>
-      <c r="F13" s="18" t="inlineStr"/>
+      <c r="F13" s="18" t="inlineStr">
+        <is>
+          <t>3491192</t>
+        </is>
+      </c>
       <c r="G13" s="18" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
         <is>
-          <t>Recurrente $50.000/mes hasta nuevo aviso</t>
+          <t>Gmail factura 03/2026 $39.162,75 · cliente 3491192</t>
         </is>
       </c>
       <c r="I13" s="14" t="inlineStr">
@@ -70093,18 +69848,22 @@
       </c>
       <c r="C19" s="14" t="inlineStr">
         <is>
-          <t>Telecentro CIUDAD — servicio mensual 04/2026</t>
+          <t>Telecentro CIUDAD — 04/2026 (Gmail)</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>50000</v>
+        <v>46909</v>
       </c>
       <c r="E19" s="14" t="inlineStr"/>
-      <c r="F19" s="18" t="inlineStr"/>
+      <c r="F19" s="18" t="inlineStr">
+        <is>
+          <t>3491192</t>
+        </is>
+      </c>
       <c r="G19" s="18" t="inlineStr"/>
       <c r="H19" s="14" t="inlineStr">
         <is>
-          <t>Recurrente $50.000/mes hasta nuevo aviso</t>
+          <t>Gmail factura 04/2026 $46.909,00 · cliente 3491192</t>
         </is>
       </c>
       <c r="I19" s="14" t="inlineStr">
@@ -70236,18 +69995,22 @@
       </c>
       <c r="C24" s="14" t="inlineStr">
         <is>
-          <t>Telecentro CIUDAD — servicio mensual 05/2026</t>
+          <t>Telecentro CIUDAD — 05/2026 (Gmail)</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>50000</v>
+        <v>47939</v>
       </c>
       <c r="E24" s="14" t="inlineStr"/>
-      <c r="F24" s="18" t="inlineStr"/>
+      <c r="F24" s="18" t="inlineStr">
+        <is>
+          <t>3491192</t>
+        </is>
+      </c>
       <c r="G24" s="18" t="inlineStr"/>
       <c r="H24" s="14" t="inlineStr">
         <is>
-          <t>Recurrente $50.000/mes hasta nuevo aviso</t>
+          <t>Gmail factura 05/2026 $47.939,00 · cliente 3491192</t>
         </is>
       </c>
       <c r="I24" s="14" t="inlineStr">
@@ -70372,18 +70135,24 @@
       </c>
       <c r="C28" s="14" t="inlineStr">
         <is>
-          <t>Telecentro CIUDAD — servicio mensual 06/2026</t>
-        </is>
-      </c>
-      <c r="D28" s="15" t="n">
-        <v>50000</v>
-      </c>
-      <c r="E28" s="14" t="inlineStr"/>
-      <c r="F28" s="18" t="inlineStr"/>
+          <t>(duplicado) ver fila pago MP 17/06 — no sumar</t>
+        </is>
+      </c>
+      <c r="D28" s="15" t="n"/>
+      <c r="E28" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F28" s="18" t="inlineStr">
+        <is>
+          <t>3491192</t>
+        </is>
+      </c>
       <c r="G28" s="18" t="inlineStr"/>
       <c r="H28" s="14" t="inlineStr">
         <is>
-          <t>Recurrente $50.000/mes hasta nuevo aviso</t>
+          <t>SUPERSEDE · Telecentro Junio está en Detalle pago MP 17/06 $48.420 · Gmail factura 06/2026 $48.419,26</t>
         </is>
       </c>
       <c r="I28" s="14" t="inlineStr">
@@ -70560,7 +70329,7 @@
       <c r="G33" s="18" t="inlineStr"/>
       <c r="H33" s="14" t="inlineStr">
         <is>
-          <t>SUPERSEDE · Telecentro Julio está en Detalle débito 30/06 $31.999</t>
+          <t>SUPERSEDE · Telecentro Julio está en Detalle débito 30/06 $31.999 · Gmail factura 07/2026 $31.999,00</t>
         </is>
       </c>
       <c r="I33" s="14" t="inlineStr">
@@ -70615,7 +70384,7 @@
       </c>
       <c r="C35" s="14" t="inlineStr">
         <is>
-          <t>Telecentro CIUDAD — cobro Visa *3200 24/07/2026 (agosto)</t>
+          <t>Telecentro CIUDAD — 08/2026 (Gmail) · cobro Visa *3200 24/07/2026</t>
         </is>
       </c>
       <c r="D35" s="15" t="n">
@@ -70634,7 +70403,7 @@
       <c r="G35" s="18" t="inlineStr"/>
       <c r="H35" s="14" t="inlineStr">
         <is>
-          <t>Aviso tarjeta Visa *3200 · ARS 31.999 · período agosto · reemplaza recurrente $50.000</t>
+          <t>Gmail factura 08/2026 $31.999,00 · cobro 24/07 · reemplaza recurrente $50.000</t>
         </is>
       </c>
       <c r="I35" s="14" t="inlineStr">
@@ -70654,20 +70423,22 @@
       </c>
       <c r="C36" s="14" t="inlineStr">
         <is>
-          <t>(duplicado) ver fila débito BBVA 25/09 — no sumar</t>
-        </is>
-      </c>
-      <c r="D36" s="15" t="n"/>
-      <c r="E36" s="14" t="inlineStr">
-        <is>
-          <t>Débito BBVA</t>
-        </is>
-      </c>
-      <c r="F36" s="18" t="inlineStr"/>
+          <t>Telecentro CIUDAD — 09/2026 (Gmail)</t>
+        </is>
+      </c>
+      <c r="D36" s="15" t="n">
+        <v>82364</v>
+      </c>
+      <c r="E36" s="14" t="n"/>
+      <c r="F36" s="18" t="inlineStr">
+        <is>
+          <t>3491192</t>
+        </is>
+      </c>
       <c r="G36" s="18" t="inlineStr"/>
       <c r="H36" s="14" t="inlineStr">
         <is>
-          <t>SUPERSEDE · Telecentro Sept está en Detalle débito 25/09 $69.659</t>
+          <t>Gmail factura 09/2026 $82.363,35 · mes=período factura (no cobro Oct $69.659)</t>
         </is>
       </c>
       <c r="I36" s="14" t="inlineStr">
@@ -70687,18 +70458,24 @@
       </c>
       <c r="C37" s="14" t="inlineStr">
         <is>
-          <t>Telecentro CIUDAD — servicio mensual 10/2026</t>
-        </is>
-      </c>
-      <c r="D37" s="15" t="n">
-        <v>50000</v>
-      </c>
-      <c r="E37" s="14" t="inlineStr"/>
-      <c r="F37" s="18" t="inlineStr"/>
+          <t>(duplicado) ver fila débito BBVA 25/09 — no sumar</t>
+        </is>
+      </c>
+      <c r="D37" s="15" t="n"/>
+      <c r="E37" s="14" t="inlineStr">
+        <is>
+          <t>Débito BBVA</t>
+        </is>
+      </c>
+      <c r="F37" s="18" t="inlineStr">
+        <is>
+          <t>3491192</t>
+        </is>
+      </c>
       <c r="G37" s="18" t="inlineStr"/>
       <c r="H37" s="14" t="inlineStr">
         <is>
-          <t>Recurrente $50.000/mes hasta nuevo aviso</t>
+          <t>SUPERSEDE · Telecentro Octubre está en Detalle débito 25/09 $69.659 · Gmail factura 10/2026 $69.659,00</t>
         </is>
       </c>
       <c r="I37" s="14" t="inlineStr">
@@ -70718,18 +70495,16 @@
       </c>
       <c r="C38" s="14" t="inlineStr">
         <is>
-          <t>Telecentro CIUDAD — servicio mensual 11/2026</t>
-        </is>
-      </c>
-      <c r="D38" s="15" t="n">
-        <v>50000</v>
-      </c>
+          <t>Telecentro CIUDAD — sin factura Gmail aún (Noviembre)</t>
+        </is>
+      </c>
+      <c r="D38" s="15" t="n"/>
       <c r="E38" s="14" t="inlineStr"/>
       <c r="F38" s="18" t="inlineStr"/>
       <c r="G38" s="18" t="inlineStr"/>
       <c r="H38" s="14" t="inlineStr">
         <is>
-          <t>Recurrente $50.000/mes hasta nuevo aviso</t>
+          <t>Sin mail ¡Ya está disponible tu factura! — no cargar placeholder</t>
         </is>
       </c>
       <c r="I38" s="14" t="inlineStr">
@@ -70749,18 +70524,16 @@
       </c>
       <c r="C39" s="14" t="inlineStr">
         <is>
-          <t>Telecentro CIUDAD — servicio mensual 12/2026</t>
-        </is>
-      </c>
-      <c r="D39" s="15" t="n">
-        <v>50000</v>
-      </c>
+          <t>Telecentro CIUDAD — sin factura Gmail aún (Diciembre)</t>
+        </is>
+      </c>
+      <c r="D39" s="15" t="n"/>
       <c r="E39" s="14" t="inlineStr"/>
       <c r="F39" s="18" t="inlineStr"/>
       <c r="G39" s="18" t="inlineStr"/>
       <c r="H39" s="14" t="inlineStr">
         <is>
-          <t>Recurrente $50.000/mes hasta nuevo aviso</t>
+          <t>Sin mail ¡Ya está disponible tu factura! — no cargar placeholder</t>
         </is>
       </c>
       <c r="I39" s="14" t="inlineStr">
@@ -71722,6 +71495,16 @@
           <t>3491192</t>
         </is>
       </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Gmail factura 06/2026 $48.419,26 · pago MP; mes=Junio</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="53" t="n">
@@ -71750,6 +71533,16 @@
           <t>3491192</t>
         </is>
       </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Gmail factura 07/2026 $31.999,00 · débito BBVA; mes=Julio</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="63" t="n">
@@ -71854,14 +71647,19 @@
           <t>Débito BBVA</t>
         </is>
       </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>3491192</t>
+        </is>
+      </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>Gmail Telecentro 10/2026 $69.659 + Compra aprobada; mes=cobro</t>
+          <t>Gmail Telecentro 10/2026 $69.659 + Compra aprobada; mes=período factura Octubre (cobro 25/09)</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>Septiembre</t>
+          <t>Octubre</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Catalog all Mercado Pago Gmail movement emails for 2026.
Parse 146 payment/transfer/card emails, classify into CIUDAD/BONORINO/OHIGGINS/GPS/MP No Gasto, load missing Aug–Oct GPS rows, and mirror September card-summary payments.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -3812,7 +3812,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F943"/>
+  <dimension ref="A1:F957"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29031,6 +29031,398 @@
       <c r="F943" t="inlineStr">
         <is>
           <t>Sol Estética · Kelly · $86.000 · resumen oficial cuenta MP 1–30 sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" s="52" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B944" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C944" t="inlineStr">
+        <is>
+          <t>COMIDA · Oficina</t>
+        </is>
+      </c>
+      <c r="D944" t="n">
+        <v>11010</v>
+      </c>
+      <c r="E944" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F944" t="inlineStr">
+        <is>
+          <t>COMIDA · Oficina · Copetin Catering · Gmail Pago aprobado</t>
+        </is>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" s="52" t="n">
+        <v>46239</v>
+      </c>
+      <c r="B945" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C945" t="inlineStr">
+        <is>
+          <t>VESTIMENTA</t>
+        </is>
+      </c>
+      <c r="D945" t="n">
+        <v>152000</v>
+      </c>
+      <c r="E945" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F945" t="inlineStr">
+        <is>
+          <t>VESTIMENTA · Renová tu vestidor · Gmail Pago aprobado · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" s="52" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B946" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C946" t="inlineStr">
+        <is>
+          <t>SALUD</t>
+        </is>
+      </c>
+      <c r="D946" t="n">
+        <v>22222</v>
+      </c>
+      <c r="E946" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F946" t="inlineStr">
+        <is>
+          <t>SALUD · Siendo Consciencia · Gmail Pago aprobado · REVISAR ítem</t>
+        </is>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" s="52" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B947" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C947" t="inlineStr">
+        <is>
+          <t>SALUD</t>
+        </is>
+      </c>
+      <c r="D947" t="n">
+        <v>24000</v>
+      </c>
+      <c r="E947" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F947" t="inlineStr">
+        <is>
+          <t>SALUD · Lorena Ferreyra · Gmail Pago aprobado · REVISAR ítem</t>
+        </is>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948" s="52" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B948" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C948" t="inlineStr">
+        <is>
+          <t>SALUD</t>
+        </is>
+      </c>
+      <c r="D948" t="n">
+        <v>75000</v>
+      </c>
+      <c r="E948" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F948" t="inlineStr">
+        <is>
+          <t>SALUD · Lorena Ferreyra · Gmail Pago aprobado · REVISAR ítem</t>
+        </is>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" s="52" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B949" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C949" t="inlineStr">
+        <is>
+          <t>SALUD</t>
+        </is>
+      </c>
+      <c r="D949" t="n">
+        <v>356000</v>
+      </c>
+      <c r="E949" t="inlineStr">
+        <is>
+          <t>BBVA Crédito ****3200</t>
+        </is>
+      </c>
+      <c r="F949" t="inlineStr">
+        <is>
+          <t>SALUD · Reiki · Gmail Pago aprobado · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" s="52" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B950" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C950" t="inlineStr">
+        <is>
+          <t>COMIDA · Oficina</t>
+        </is>
+      </c>
+      <c r="D950" t="n">
+        <v>13600</v>
+      </c>
+      <c r="E950" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F950" t="inlineStr">
+        <is>
+          <t>COMIDA · Oficina · Copetin Catering · Gmail Pago aprobado</t>
+        </is>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" s="52" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B951" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C951" t="inlineStr">
+        <is>
+          <t>SALUD</t>
+        </is>
+      </c>
+      <c r="D951" t="n">
+        <v>27000</v>
+      </c>
+      <c r="E951" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F951" t="inlineStr">
+        <is>
+          <t>SALUD · Karen · Gmail Pago aprobado · REVISAR ítem</t>
+        </is>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" s="52" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B952" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C952" t="inlineStr">
+        <is>
+          <t>EDUCACIÓN</t>
+        </is>
+      </c>
+      <c r="D952" t="n">
+        <v>30000</v>
+      </c>
+      <c r="E952" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F952" t="inlineStr">
+        <is>
+          <t>EDUCACIÓN · Bitgenia · Gmail Pago aprobado · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" s="52" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B953" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C953" t="inlineStr">
+        <is>
+          <t>VESTIMENTA</t>
+        </is>
+      </c>
+      <c r="D953" t="n">
+        <v>176000</v>
+      </c>
+      <c r="E953" t="inlineStr">
+        <is>
+          <t>BBVA Crédito ****3200</t>
+        </is>
+      </c>
+      <c r="F953" t="inlineStr">
+        <is>
+          <t>VESTIMENTA · Gibiana Cova · Gmail Pago aprobado · distinto de transferencia $131.000 · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" s="52" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B954" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="C954" t="inlineStr">
+        <is>
+          <t>FARMACIA SALUD</t>
+        </is>
+      </c>
+      <c r="D954" t="n">
+        <v>17038</v>
+      </c>
+      <c r="E954" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F954" t="inlineStr">
+        <is>
+          <t>FARMACIA SALUD · Hiperfarmaceutica Temperley · Gmail Pago aprobado</t>
+        </is>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" s="52" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B955" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="C955" t="inlineStr">
+        <is>
+          <t>VIAJES</t>
+        </is>
+      </c>
+      <c r="D955" t="n">
+        <v>1430000</v>
+      </c>
+      <c r="E955" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F955" t="inlineStr">
+        <is>
+          <t>VIAJES · MARPATAG SRL · Gmail Pago aprobado · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" s="52" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B956" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="C956" t="inlineStr">
+        <is>
+          <t>PELUQUERÍA</t>
+        </is>
+      </c>
+      <c r="D956" t="n">
+        <v>7000</v>
+      </c>
+      <c r="E956" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F956" t="inlineStr">
+        <is>
+          <t>PELUQUERÍA · Soy lashista · Gmail Pago aprobado (2 mails mismo monto; se carga 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" s="52" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B957" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="C957" t="inlineStr">
+        <is>
+          <t>VIAJES</t>
+        </is>
+      </c>
+      <c r="D957" t="n">
+        <v>1143000</v>
+      </c>
+      <c r="E957" t="inlineStr">
+        <is>
+          <t>BBVA Crédito ****3200</t>
+        </is>
+      </c>
+      <c r="F957" t="inlineStr">
+        <is>
+          <t>VIAJES · Patagonia Chic Excursiones · Gmail Pago aprobado · 1 cuota · gasto personal Sol</t>
         </is>
       </c>
     </row>
@@ -73736,7 +74128,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H213"/>
+  <dimension ref="A1:H215"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -73763,6 +74155,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="45" t="inlineStr">
         <is>
@@ -73877,6 +74270,7 @@
         <v/>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="47" t="inlineStr">
         <is>
@@ -73892,6 +74286,7 @@
         <v/>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
         <is>
@@ -73908,6 +74303,8 @@
     </row>
     <row r="17"/>
     <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="51" t="inlineStr">
         <is>
@@ -73915,6 +74312,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="46" t="inlineStr">
         <is>
@@ -81164,6 +81562,62 @@
       <c r="H213" t="inlineStr">
         <is>
           <t>Reserva automática · − · op 180676447379 · NUNCA almacén · resumen oficial cuenta MP 1–30 sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="52" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Pago de resumen TC</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>Pagaste una parte del resumen de tu tarjeta · Gmail</t>
+        </is>
+      </c>
+      <c r="E214" t="n">
+        <v>1214000</v>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="52" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Pago de resumen TC</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>Pagaste una parte del resumen de tu tarjeta · Gmail</t>
+        </is>
+      </c>
+      <c r="E215" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>ARS</t>
         </is>
       </c>
     </row>
@@ -86185,7 +86639,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -86627,6 +87081,62 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="52" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Tarjeta de crédito</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>1214000</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Pago parcial resumen · Gmail · espejo MP No Gasto</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="52" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Tarjeta de crédito</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Pago parcial resumen · Gmail · espejo MP No Gasto</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mark MARPATAG and Patagonia Chic as Chris 50th birthday gift.
Keep both in Gasto Personal Sol · VIAJES with comment regalo Chris Cumple 50.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -29366,7 +29366,7 @@
       </c>
       <c r="F955" t="inlineStr">
         <is>
-          <t>VIAJES · MARPATAG SRL · Gmail Pago aprobado · gasto personal Sol</t>
+          <t>VIAJES · regalo Chris Cumple 50 · MARPATAG SRL · Gmail Pago aprobado · gasto personal Sol</t>
         </is>
       </c>
     </row>
@@ -29422,7 +29422,7 @@
       </c>
       <c r="F957" t="inlineStr">
         <is>
-          <t>VIAJES · Patagonia Chic Excursiones · Gmail Pago aprobado · 1 cuota · gasto personal Sol</t>
+          <t>VIAJES · regalo Chris Cumple 50 · Patagonia Chic Excursiones · Gmail Pago aprobado · 1 cuota · gasto personal Sol</t>
         </is>
       </c>
     </row>
@@ -74155,7 +74155,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="45" t="inlineStr">
         <is>
@@ -74270,7 +74269,6 @@
         <v/>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="47" t="inlineStr">
         <is>
@@ -74286,7 +74284,6 @@
         <v/>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
         <is>
@@ -74303,8 +74300,6 @@
     </row>
     <row r="17"/>
     <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="51" t="inlineStr">
         <is>
@@ -74312,7 +74307,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="46" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Classify Correo Oficial as GPS Courier.
Rename existing Jun/Sep rows, add Aug 20 $24.000 from Gmail, and drop ENVÍOS REVISAR for these payments.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -3812,7 +3812,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F957"/>
+  <dimension ref="A1:F958"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7848,7 +7848,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>ENVÍOS</t>
+          <t>Courier</t>
         </is>
       </c>
       <c r="D174" s="26" t="n">
@@ -7861,7 +7861,7 @@
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>envíos · gasto personal Sol</t>
+          <t>Courier · Correo Oficial · Gmail Pago aprobado · $22.500 · gasto personal Sol</t>
         </is>
       </c>
     </row>
@@ -8072,7 +8072,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>ENVÍOS</t>
+          <t>Courier</t>
         </is>
       </c>
       <c r="D182" s="26" t="n">
@@ -8085,7 +8085,7 @@
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>envíos · gasto personal Sol</t>
+          <t>Courier · Correo Oficial · Gmail Pago aprobado · $48.000 · gasto personal Sol</t>
         </is>
       </c>
     </row>
@@ -26214,7 +26214,7 @@
       </c>
       <c r="C842" t="inlineStr">
         <is>
-          <t>ENVÍOS</t>
+          <t>Courier</t>
         </is>
       </c>
       <c r="D842" t="n">
@@ -26227,7 +26227,7 @@
       </c>
       <c r="F842" t="inlineStr">
         <is>
-          <t>ENVÍOS · Correo Oficial · gasto personal Sol · dinero en cuenta MP screenshot</t>
+          <t>Courier · Correo Oficial · Gmail Pago aprobado · $24.000 · gasto personal Sol</t>
         </is>
       </c>
     </row>
@@ -29423,6 +29423,34 @@
       <c r="F957" t="inlineStr">
         <is>
           <t>VIAJES · regalo Chris Cumple 50 · Patagonia Chic Excursiones · Gmail Pago aprobado · 1 cuota · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" s="52" t="n">
+        <v>46254</v>
+      </c>
+      <c r="B958" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C958" t="inlineStr">
+        <is>
+          <t>Courier</t>
+        </is>
+      </c>
+      <c r="D958" t="n">
+        <v>24000</v>
+      </c>
+      <c r="E958" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F958" t="inlineStr">
+        <is>
+          <t>Courier · Correo Oficial · Gmail Pago aprobado · $24.000 · gasto personal Sol</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inventory AGIP ABL Gmail boletas by property.
Document CIUDAD partida 397789 digital bills and BBVA reminders; note no OHIGGINS boletas in this inbox; remove CIUDAD Detalle duplicates of OHIGGINS ABL.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -71321,12 +71321,10 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Agip ABL GCBA</t>
-        </is>
-      </c>
-      <c r="D52" s="26" t="n">
-        <v>88141</v>
-      </c>
+          <t>(no CIUDAD) ABL OHIGGINS partida 3016365 — ver OHIGGINS/Detalle</t>
+        </is>
+      </c>
+      <c r="D52" s="26" t="n"/>
       <c r="E52" t="inlineStr">
         <is>
           <t>Mercado Pago — Dinero disponible</t>
@@ -71334,7 +71332,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>ceil desde $88.140,38</t>
+          <t>SUPERSEDE · monto 88141 es OHIGGINS (&gt;80k) · no sumar a CIUDAD</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -71354,12 +71352,10 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Agip ABL GCBA</t>
-        </is>
-      </c>
-      <c r="D53" s="26" t="n">
-        <v>83757</v>
-      </c>
+          <t>(no CIUDAD) ABL OHIGGINS partida 3016365 — ver OHIGGINS/Detalle</t>
+        </is>
+      </c>
+      <c r="D53" s="26" t="n"/>
       <c r="E53" t="inlineStr">
         <is>
           <t>Mercado Pago — Dinero disponible</t>
@@ -71367,7 +71363,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>ceil desde $83.756,62</t>
+          <t>SUPERSEDE · monto 83757 es OHIGGINS (&gt;80k) · no sumar a CIUDAD</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">

</xml_diff>

<commit_message>
Reclassify Dr.Barf / Gibiana Cova as Almacén RAMON · Comida.
Move Aug $176k (BBVA) and Sep $131k (MP transfer) from GPS VESTIMENTA
into Almacen Detalle; supersede GPS rows and regenerate SOL maestro.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -26746,20 +26746,12 @@
       </c>
       <c r="C861" t="inlineStr">
         <is>
-          <t>TRANSFERENCIAS</t>
-        </is>
-      </c>
-      <c r="D861" t="n">
-        <v>131000</v>
-      </c>
-      <c r="E861" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
+          <t>MOVIDO → Almacén</t>
         </is>
       </c>
       <c r="F861" t="inlineStr">
         <is>
-          <t>Cova Abreu Gibiana Del Valle · Transferencia enviada · gasto personal Sol · dinero en cuenta MP screenshot</t>
+          <t>SUPERSEDE · DR BARF / Gibiana Cova → Almacen Detalle · RAMON · Comida (no GPS)</t>
         </is>
       </c>
     </row>
@@ -29297,20 +29289,12 @@
       </c>
       <c r="C953" t="inlineStr">
         <is>
-          <t>VESTIMENTA</t>
-        </is>
-      </c>
-      <c r="D953" t="n">
-        <v>176000</v>
-      </c>
-      <c r="E953" t="inlineStr">
-        <is>
-          <t>BBVA Crédito ****3200</t>
+          <t>MOVIDO → Almacén</t>
         </is>
       </c>
       <c r="F953" t="inlineStr">
         <is>
-          <t>VESTIMENTA · Gibiana Cova · Gmail Pago aprobado · distinto de transferencia $131.000 · gasto personal Sol</t>
+          <t>SUPERSEDE · DR BARF / Gibiana Cova → Almacen Detalle · RAMON · Comida (no GPS)</t>
         </is>
       </c>
     </row>
@@ -65309,15 +65293,27 @@
           <t>Agosto</t>
         </is>
       </c>
-      <c r="B316" s="17" t="n"/>
-      <c r="C316" s="14" t="n"/>
-      <c r="D316" s="27" t="n"/>
+      <c r="B316" s="17" t="n">
+        <v>46235</v>
+      </c>
+      <c r="C316" s="14" t="inlineStr">
+        <is>
+          <t>RAMON · Comida</t>
+        </is>
+      </c>
+      <c r="D316" s="27" t="n">
+        <v>176000</v>
+      </c>
       <c r="E316" s="28" t="n"/>
       <c r="F316" s="15">
         <f>IF(OR(D316&lt;&gt;"",E316&lt;&gt;""),IF(D316="",0,D316)+IF(E316="",0,E316),"")</f>
         <v/>
       </c>
-      <c r="G316" s="14" t="n"/>
+      <c r="G316" s="14" t="inlineStr">
+        <is>
+          <t>RAMON · Comida · DR BARF · Gibiana Cova · Gmail Pago aprobado BBVA · ALMACEN SOL</t>
+        </is>
+      </c>
     </row>
     <row r="317">
       <c r="A317" s="14" t="inlineStr">
@@ -67422,9 +67418,25 @@
           <t>Septiembre</t>
         </is>
       </c>
+      <c r="B410" s="52" t="n">
+        <v>46275</v>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>RAMON · Comida</t>
+        </is>
+      </c>
+      <c r="D410" t="n">
+        <v>131000</v>
+      </c>
       <c r="F410">
         <f>IF(OR(D410&lt;&gt;"",E410&lt;&gt;""),IF(D410="",0,D410)+IF(E410="",0,E410),"")</f>
         <v/>
+      </c>
+      <c r="G410" t="inlineStr">
+        <is>
+          <t>RAMON · Comida · DR BARF · Cova Abreu Gibiana Del Valle · transferencia MP · ALMACEN SOL</t>
+        </is>
       </c>
     </row>
     <row r="411">

</xml_diff>

<commit_message>
Load missing Almacén CIUDAD expenses found in Gmail audit.
Move Pescadería Belgrano May/Jun from GPS to Almacén; add Dr.Barf July
checkout, Gardiner and Paws August BBVA purchases; document August MP
settlement CSV still needed for QR/super gaps.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -7460,20 +7460,13 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>TRANSFERENCIAS</t>
-        </is>
-      </c>
-      <c r="D155" s="26" t="n">
-        <v>24852</v>
-      </c>
-      <c r="E155" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
+          <t>MOVIDO → Almacén</t>
+        </is>
+      </c>
+      <c r="D155" s="26" t="n"/>
       <c r="F155" t="inlineStr">
         <is>
-          <t>compra · gasto personal Sol (ex-PENDIENTE) · ex `Andres Di Pasqua`</t>
+          <t>SUPERSEDE · Pescadería Belgrano $24852 → Almacen Detalle · COMIDA · Pescadería Belgrano (no GPS)</t>
         </is>
       </c>
     </row>
@@ -7820,20 +7813,13 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>TRANSFERENCIAS</t>
-        </is>
-      </c>
-      <c r="D173" s="26" t="n">
-        <v>32046</v>
-      </c>
-      <c r="E173" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
+          <t>MOVIDO → Almacén</t>
+        </is>
+      </c>
+      <c r="D173" s="26" t="n"/>
       <c r="F173" t="inlineStr">
         <is>
-          <t>compra · gasto personal Sol (ex-PENDIENTE) · ex `Andres Di Pasqua`</t>
+          <t>SUPERSEDE · Pescadería Belgrano $32046 → Almacen Detalle · COMIDA · Pescadería Belgrano (no GPS)</t>
         </is>
       </c>
     </row>
@@ -62882,15 +62868,27 @@
           <t>Mayo</t>
         </is>
       </c>
-      <c r="B205" s="17" t="n"/>
-      <c r="C205" s="14" t="n"/>
-      <c r="D205" s="27" t="n"/>
+      <c r="B205" s="17" t="n">
+        <v>46153</v>
+      </c>
+      <c r="C205" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · Pescadería Belgrano</t>
+        </is>
+      </c>
+      <c r="D205" s="27" t="n">
+        <v>24852</v>
+      </c>
       <c r="E205" s="28" t="n"/>
       <c r="F205" s="15">
-        <f>IF(OR(D200&lt;&gt;"",E200&lt;&gt;""),IF(D200="",0,D200)+IF(E200="",0,E200),"")</f>
+        <f>IF(OR(D205&lt;&gt;"",E205&lt;&gt;""),IF(D205="",0,D205)+IF(E205="",0,E205),"")</f>
         <v/>
       </c>
-      <c r="G205" s="14" t="n"/>
+      <c r="G205" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · Pescadería Belgrano · Mercado Pago · Gmail Pago aprobado · movido desde GPS · ALMACEN SOL</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="14" t="inlineStr">
@@ -64052,15 +64050,27 @@
           <t>Junio</t>
         </is>
       </c>
-      <c r="B253" s="17" t="n"/>
-      <c r="C253" s="14" t="n"/>
-      <c r="D253" s="27" t="n"/>
+      <c r="B253" s="17" t="n">
+        <v>46175</v>
+      </c>
+      <c r="C253" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · Pescadería Belgrano</t>
+        </is>
+      </c>
+      <c r="D253" s="27" t="n">
+        <v>32046</v>
+      </c>
       <c r="E253" s="28" t="n"/>
       <c r="F253" s="15">
-        <f>IF(OR(D238&lt;&gt;"",E238&lt;&gt;""),IF(D238="",0,D238)+IF(E238="",0,E238),"")</f>
+        <f>IF(OR(D253&lt;&gt;"",E253&lt;&gt;""),IF(D253="",0,D253)+IF(E253="",0,E253),"")</f>
         <v/>
       </c>
-      <c r="G253" s="14" t="n"/>
+      <c r="G253" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · Pescadería Belgrano · Mercado Pago · Gmail Pago aprobado · movido desde GPS · ALMACEN SOL</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="14" t="inlineStr">
@@ -64847,15 +64857,27 @@
           <t>Julio</t>
         </is>
       </c>
-      <c r="B290" s="17" t="n"/>
-      <c r="C290" s="14" t="n"/>
-      <c r="D290" s="27" t="n"/>
+      <c r="B290" s="17" t="n">
+        <v>46207</v>
+      </c>
+      <c r="C290" s="14" t="inlineStr">
+        <is>
+          <t>RAMON · Comida</t>
+        </is>
+      </c>
+      <c r="D290" s="27" t="n">
+        <v>149500</v>
+      </c>
       <c r="E290" s="28" t="n"/>
       <c r="F290" s="15">
         <f>IF(OR(D290&lt;&gt;"",E290&lt;&gt;""),IF(D290="",0,D290)+IF(E290="",0,E290),"")</f>
         <v/>
       </c>
-      <c r="G290" s="14" t="n"/>
+      <c r="G290" s="14" t="inlineStr">
+        <is>
+          <t>RAMON · Comida · DR BARF · pedido #462 · checkout total $149.500 · Gmail Recibimos tu pago · ALMACEN SOL</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" s="14" t="inlineStr">
@@ -65321,15 +65343,27 @@
           <t>Agosto</t>
         </is>
       </c>
-      <c r="B317" s="17" t="n"/>
-      <c r="C317" s="14" t="n"/>
-      <c r="D317" s="27" t="n"/>
+      <c r="B317" s="17" t="n">
+        <v>46250</v>
+      </c>
+      <c r="C317" s="14" t="inlineStr">
+        <is>
+          <t>ENTRETENIMIENTO · Social</t>
+        </is>
+      </c>
+      <c r="D317" s="27" t="n">
+        <v>1060501</v>
+      </c>
       <c r="E317" s="28" t="n"/>
       <c r="F317" s="15">
         <f>IF(OR(D317&lt;&gt;"",E317&lt;&gt;""),IF(D317="",0,D317)+IF(E317="",0,E317),"")</f>
         <v/>
       </c>
-      <c r="G317" s="14" t="n"/>
+      <c r="G317" s="14" t="inlineStr">
+        <is>
+          <t>ENTRETENIMIENTO · Social · Gardiner Restaurant · BBVA VISA · Gmail Compra aprobada · mesa 9 · ALMACEN SOL</t>
+        </is>
+      </c>
     </row>
     <row r="318">
       <c r="A318" s="14" t="inlineStr">
@@ -65337,15 +65371,27 @@
           <t>Agosto</t>
         </is>
       </c>
-      <c r="B318" s="17" t="n"/>
-      <c r="C318" s="14" t="n"/>
-      <c r="D318" s="27" t="n"/>
+      <c r="B318" s="17" t="n">
+        <v>46256</v>
+      </c>
+      <c r="C318" s="14" t="inlineStr">
+        <is>
+          <t>RAMON · Otros</t>
+        </is>
+      </c>
+      <c r="D318" s="27" t="n">
+        <v>77200</v>
+      </c>
       <c r="E318" s="28" t="n"/>
       <c r="F318" s="15">
         <f>IF(OR(D318&lt;&gt;"",E318&lt;&gt;""),IF(D318="",0,D318)+IF(E318="",0,E318),"")</f>
         <v/>
       </c>
-      <c r="G318" s="14" t="n"/>
+      <c r="G318" s="14" t="inlineStr">
+        <is>
+          <t>RAMON · Otros · Paws Pet Market · BBVA VISA · 3 cuotas · Gmail Compra aprobada · ALMACEN SOL</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Sum forgotten Almacén items into September as AJUSTE SEPT.
Pescadería (incl. Andres Di Pasqua) stays Almacén CIUDAD; catch-up rows
keep original expense dates and note they were not reported in the
origin month due to error.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -4256,20 +4256,14 @@
       </c>
       <c r="C31" s="14" t="inlineStr">
         <is>
-          <t>TRANSFERENCIAS</t>
-        </is>
-      </c>
-      <c r="D31" s="15" t="n">
-        <v>12426</v>
-      </c>
-      <c r="E31" s="14" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
+          <t>MOVIDO → Almacén</t>
+        </is>
+      </c>
+      <c r="D31" s="15" t="n"/>
+      <c r="E31" s="14" t="n"/>
       <c r="F31" s="14" t="inlineStr">
         <is>
-          <t>compra · gasto personal Sol (ex-PENDIENTE) · ex `Andres Javier Di Pasqua`</t>
+          <t>SUPERSEDE · Pescadería Belgrano / Andres Javier Di Pasqua $12426 → Almacen Detalle · Septiembre AJUSTE (origen no rendido por error)</t>
         </is>
       </c>
     </row>
@@ -4944,20 +4938,14 @@
       </c>
       <c r="C57" s="14" t="inlineStr">
         <is>
-          <t>TRANSFERENCIAS</t>
-        </is>
-      </c>
-      <c r="D57" s="15" t="n">
-        <v>24852</v>
-      </c>
-      <c r="E57" s="14" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
+          <t>MOVIDO → Almacén</t>
+        </is>
+      </c>
+      <c r="D57" s="15" t="n"/>
+      <c r="E57" s="14" t="n"/>
       <c r="F57" s="14" t="inlineStr">
         <is>
-          <t>compra · gasto personal Sol (ex-PENDIENTE) · ex `Andres Javier Di Pasqua`</t>
+          <t>SUPERSEDE · Pescadería Belgrano / Andres Javier Di Pasqua $24852 → Almacen Detalle · Septiembre AJUSTE (origen no rendido por error)</t>
         </is>
       </c>
     </row>
@@ -7466,7 +7454,7 @@
       <c r="D155" s="26" t="n"/>
       <c r="F155" t="inlineStr">
         <is>
-          <t>SUPERSEDE · Pescadería Belgrano $24852 → Almacen Detalle · COMIDA · Pescadería Belgrano (no GPS)</t>
+          <t>SUPERSEDE · Pescadería Belgrano $24852 → Almacen Detalle · Septiembre AJUSTE · COMIDA · Pescadería Belgrano (no GPS)</t>
         </is>
       </c>
     </row>
@@ -7819,7 +7807,7 @@
       <c r="D173" s="26" t="n"/>
       <c r="F173" t="inlineStr">
         <is>
-          <t>SUPERSEDE · Pescadería Belgrano $32046 → Almacen Detalle · COMIDA · Pescadería Belgrano (no GPS)</t>
+          <t>SUPERSEDE · Pescadería Belgrano $32046 → Almacen Detalle · Septiembre AJUSTE · COMIDA · Pescadería Belgrano (no GPS)</t>
         </is>
       </c>
     </row>
@@ -62106,6 +62094,7 @@
       </c>
       <c r="G176" s="22" t="n"/>
     </row>
+    <row r="177"/>
     <row r="178">
       <c r="A178" s="14" t="inlineStr">
         <is>
@@ -62868,27 +62857,15 @@
           <t>Mayo</t>
         </is>
       </c>
-      <c r="B205" s="17" t="n">
-        <v>46153</v>
-      </c>
-      <c r="C205" s="14" t="inlineStr">
-        <is>
-          <t>COMIDA · Pescadería Belgrano</t>
-        </is>
-      </c>
-      <c r="D205" s="27" t="n">
-        <v>24852</v>
-      </c>
+      <c r="B205" s="17" t="n"/>
+      <c r="C205" s="14" t="n"/>
+      <c r="D205" s="27" t="n"/>
       <c r="E205" s="28" t="n"/>
       <c r="F205" s="15">
         <f>IF(OR(D205&lt;&gt;"",E205&lt;&gt;""),IF(D205="",0,D205)+IF(E205="",0,E205),"")</f>
         <v/>
       </c>
-      <c r="G205" s="14" t="inlineStr">
-        <is>
-          <t>COMIDA · Pescadería Belgrano · Mercado Pago · Gmail Pago aprobado · movido desde GPS · ALMACEN SOL</t>
-        </is>
-      </c>
+      <c r="G205" s="14" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="14" t="inlineStr">
@@ -63400,6 +63377,7 @@
       </c>
       <c r="G228" s="22" t="n"/>
     </row>
+    <row r="229"/>
     <row r="230">
       <c r="A230" s="14" t="inlineStr">
         <is>
@@ -64050,27 +64028,15 @@
           <t>Junio</t>
         </is>
       </c>
-      <c r="B253" s="17" t="n">
-        <v>46175</v>
-      </c>
-      <c r="C253" s="14" t="inlineStr">
-        <is>
-          <t>COMIDA · Pescadería Belgrano</t>
-        </is>
-      </c>
-      <c r="D253" s="27" t="n">
-        <v>32046</v>
-      </c>
+      <c r="B253" s="17" t="n"/>
+      <c r="C253" s="14" t="n"/>
+      <c r="D253" s="27" t="n"/>
       <c r="E253" s="28" t="n"/>
       <c r="F253" s="15">
         <f>IF(OR(D253&lt;&gt;"",E253&lt;&gt;""),IF(D253="",0,D253)+IF(E253="",0,E253),"")</f>
         <v/>
       </c>
-      <c r="G253" s="14" t="inlineStr">
-        <is>
-          <t>COMIDA · Pescadería Belgrano · Mercado Pago · Gmail Pago aprobado · movido desde GPS · ALMACEN SOL</t>
-        </is>
-      </c>
+      <c r="G253" s="14" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="14" t="inlineStr">
@@ -64450,6 +64416,7 @@
       </c>
       <c r="G273" s="22" t="n"/>
     </row>
+    <row r="274"/>
     <row r="275">
       <c r="A275" s="14" t="inlineStr">
         <is>
@@ -64857,27 +64824,15 @@
           <t>Julio</t>
         </is>
       </c>
-      <c r="B290" s="17" t="n">
-        <v>46207</v>
-      </c>
-      <c r="C290" s="14" t="inlineStr">
-        <is>
-          <t>RAMON · Comida</t>
-        </is>
-      </c>
-      <c r="D290" s="27" t="n">
-        <v>149500</v>
-      </c>
+      <c r="B290" s="17" t="n"/>
+      <c r="C290" s="14" t="n"/>
+      <c r="D290" s="27" t="n"/>
       <c r="E290" s="28" t="n"/>
       <c r="F290" s="15">
         <f>IF(OR(D290&lt;&gt;"",E290&lt;&gt;""),IF(D290="",0,D290)+IF(E290="",0,E290),"")</f>
         <v/>
       </c>
-      <c r="G290" s="14" t="inlineStr">
-        <is>
-          <t>RAMON · Comida · DR BARF · pedido #462 · checkout total $149.500 · Gmail Recibimos tu pago · ALMACEN SOL</t>
-        </is>
-      </c>
+      <c r="G290" s="14" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="14" t="inlineStr">
@@ -65253,6 +65208,7 @@
       </c>
       <c r="G312" s="22" t="n"/>
     </row>
+    <row r="313"/>
     <row r="314">
       <c r="A314" s="14" t="inlineStr">
         <is>
@@ -65315,27 +65271,15 @@
           <t>Agosto</t>
         </is>
       </c>
-      <c r="B316" s="17" t="n">
-        <v>46235</v>
-      </c>
-      <c r="C316" s="14" t="inlineStr">
-        <is>
-          <t>RAMON · Comida</t>
-        </is>
-      </c>
-      <c r="D316" s="27" t="n">
-        <v>176000</v>
-      </c>
+      <c r="B316" s="17" t="n"/>
+      <c r="C316" s="14" t="n"/>
+      <c r="D316" s="27" t="n"/>
       <c r="E316" s="28" t="n"/>
       <c r="F316" s="15">
         <f>IF(OR(D316&lt;&gt;"",E316&lt;&gt;""),IF(D316="",0,D316)+IF(E316="",0,E316),"")</f>
         <v/>
       </c>
-      <c r="G316" s="14" t="inlineStr">
-        <is>
-          <t>RAMON · Comida · DR BARF · Gibiana Cova · Gmail Pago aprobado BBVA · ALMACEN SOL</t>
-        </is>
-      </c>
+      <c r="G316" s="14" t="n"/>
     </row>
     <row r="317">
       <c r="A317" s="14" t="inlineStr">
@@ -65343,27 +65287,15 @@
           <t>Agosto</t>
         </is>
       </c>
-      <c r="B317" s="17" t="n">
-        <v>46250</v>
-      </c>
-      <c r="C317" s="14" t="inlineStr">
-        <is>
-          <t>ENTRETENIMIENTO · Social</t>
-        </is>
-      </c>
-      <c r="D317" s="27" t="n">
-        <v>1060501</v>
-      </c>
+      <c r="B317" s="17" t="n"/>
+      <c r="C317" s="14" t="n"/>
+      <c r="D317" s="27" t="n"/>
       <c r="E317" s="28" t="n"/>
       <c r="F317" s="15">
         <f>IF(OR(D317&lt;&gt;"",E317&lt;&gt;""),IF(D317="",0,D317)+IF(E317="",0,E317),"")</f>
         <v/>
       </c>
-      <c r="G317" s="14" t="inlineStr">
-        <is>
-          <t>ENTRETENIMIENTO · Social · Gardiner Restaurant · BBVA VISA · Gmail Compra aprobada · mesa 9 · ALMACEN SOL</t>
-        </is>
-      </c>
+      <c r="G317" s="14" t="n"/>
     </row>
     <row r="318">
       <c r="A318" s="14" t="inlineStr">
@@ -65371,27 +65303,15 @@
           <t>Agosto</t>
         </is>
       </c>
-      <c r="B318" s="17" t="n">
-        <v>46256</v>
-      </c>
-      <c r="C318" s="14" t="inlineStr">
-        <is>
-          <t>RAMON · Otros</t>
-        </is>
-      </c>
-      <c r="D318" s="27" t="n">
-        <v>77200</v>
-      </c>
+      <c r="B318" s="17" t="n"/>
+      <c r="C318" s="14" t="n"/>
+      <c r="D318" s="27" t="n"/>
       <c r="E318" s="28" t="n"/>
       <c r="F318" s="15">
         <f>IF(OR(D318&lt;&gt;"",E318&lt;&gt;""),IF(D318="",0,D318)+IF(E318="",0,E318),"")</f>
         <v/>
       </c>
-      <c r="G318" s="14" t="inlineStr">
-        <is>
-          <t>RAMON · Otros · Paws Pet Market · BBVA VISA · 3 cuotas · Gmail Compra aprobada · ALMACEN SOL</t>
-        </is>
-      </c>
+      <c r="G318" s="14" t="n"/>
     </row>
     <row r="319">
       <c r="A319" s="14" t="inlineStr">
@@ -65979,6 +65899,7 @@
       </c>
       <c r="G354" s="22" t="n"/>
     </row>
+    <row r="355"/>
     <row r="356">
       <c r="A356" s="14" t="inlineStr">
         <is>
@@ -66059,7 +65980,7 @@
       </c>
       <c r="G358" s="14" t="inlineStr">
         <is>
-          <t>COMIDA · Pescadería Belgrano · Mercado Pago · Gmail Pago aprobado · REVISAR vs settlement</t>
+          <t>COMIDA · Pescadería Belgrano · Mercado Pago · Gmail Pago aprobado · ALMACEN SOL (pescadería siempre Almacén CIUDAD)</t>
         </is>
       </c>
     </row>
@@ -67491,87 +67412,215 @@
           <t>Septiembre</t>
         </is>
       </c>
+      <c r="B411" s="52" t="n">
+        <v>46030</v>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>COMIDA · Pescadería Belgrano</t>
+        </is>
+      </c>
+      <c r="D411" t="n">
+        <v>12426</v>
+      </c>
       <c r="F411">
         <f>IF(OR(D411&lt;&gt;"",E411&lt;&gt;""),IF(D411="",0,D411)+IF(E411="",0,E411),"")</f>
         <v/>
       </c>
+      <c r="G411" t="inlineStr">
+        <is>
+          <t>AJUSTE SEPT · gasto origen Enero 08/01/2026 · no se pasó/rindió en el mes de origen por error · COMIDA · Pescadería Belgrano · Andres Javier Di Pasqua · MP cuenta · ALMACEN SOL</t>
+        </is>
+      </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
           <t>Septiembre</t>
         </is>
+      </c>
+      <c r="B412" s="52" t="n">
+        <v>46059</v>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>COMIDA · Pescadería Belgrano</t>
+        </is>
+      </c>
+      <c r="D412" t="n">
+        <v>24852</v>
       </c>
       <c r="F412">
         <f>IF(OR(D412&lt;&gt;"",E412&lt;&gt;""),IF(D412="",0,D412)+IF(E412="",0,E412),"")</f>
         <v/>
       </c>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t>AJUSTE SEPT · gasto origen Febrero 06/02/2026 · no se pasó/rindió en el mes de origen por error · COMIDA · Pescadería Belgrano · Andres Javier Di Pasqua · MP cuenta · ALMACEN SOL</t>
+        </is>
+      </c>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
           <t>Septiembre</t>
         </is>
+      </c>
+      <c r="B413" s="52" t="n">
+        <v>46153</v>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>COMIDA · Pescadería Belgrano</t>
+        </is>
+      </c>
+      <c r="D413" t="n">
+        <v>24852</v>
       </c>
       <c r="F413">
         <f>IF(OR(D413&lt;&gt;"",E413&lt;&gt;""),IF(D413="",0,D413)+IF(E413="",0,E413),"")</f>
         <v/>
       </c>
+      <c r="G413" t="inlineStr">
+        <is>
+          <t>AJUSTE SEPT · gasto origen Mayo 11/05/2026 · no se pasó/rindió en el mes de origen por error · COMIDA · Pescadería Belgrano · Mercado Pago · Gmail Pago aprobado · ALMACEN SOL</t>
+        </is>
+      </c>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
           <t>Septiembre</t>
         </is>
+      </c>
+      <c r="B414" s="52" t="n">
+        <v>46175</v>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>COMIDA · Pescadería Belgrano</t>
+        </is>
+      </c>
+      <c r="D414" t="n">
+        <v>32046</v>
       </c>
       <c r="F414">
         <f>IF(OR(D414&lt;&gt;"",E414&lt;&gt;""),IF(D414="",0,D414)+IF(E414="",0,E414),"")</f>
         <v/>
       </c>
+      <c r="G414" t="inlineStr">
+        <is>
+          <t>AJUSTE SEPT · gasto origen Junio 02/06/2026 · no se pasó/rindió en el mes de origen por error · COMIDA · Pescadería Belgrano · Mercado Pago · Gmail Pago aprobado · ALMACEN SOL</t>
+        </is>
+      </c>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
         <is>
           <t>Septiembre</t>
         </is>
+      </c>
+      <c r="B415" s="52" t="n">
+        <v>46207</v>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>RAMON · Comida</t>
+        </is>
+      </c>
+      <c r="D415" t="n">
+        <v>149500</v>
       </c>
       <c r="F415">
         <f>IF(OR(D415&lt;&gt;"",E415&lt;&gt;""),IF(D415="",0,D415)+IF(E415="",0,E415),"")</f>
         <v/>
       </c>
+      <c r="G415" t="inlineStr">
+        <is>
+          <t>AJUSTE SEPT · gasto origen Julio 04/07/2026 · no se pasó/rindió en el mes de origen por error · RAMON · Comida · DR BARF · pedido #462 · checkout $149.500 · ALMACEN SOL</t>
+        </is>
+      </c>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
         <is>
           <t>Septiembre</t>
         </is>
+      </c>
+      <c r="B416" s="52" t="n">
+        <v>46235</v>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>RAMON · Comida</t>
+        </is>
+      </c>
+      <c r="D416" t="n">
+        <v>176000</v>
       </c>
       <c r="F416">
         <f>IF(OR(D416&lt;&gt;"",E416&lt;&gt;""),IF(D416="",0,D416)+IF(E416="",0,E416),"")</f>
         <v/>
       </c>
+      <c r="G416" t="inlineStr">
+        <is>
+          <t>AJUSTE SEPT · gasto origen Agosto 01/08/2026 · no se pasó/rindió en el mes de origen por error · RAMON · Comida · DR BARF · Gibiana Cova · BBVA · ALMACEN SOL</t>
+        </is>
+      </c>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
           <t>Septiembre</t>
         </is>
+      </c>
+      <c r="B417" s="52" t="n">
+        <v>46250</v>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>ENTRETENIMIENTO · Social</t>
+        </is>
+      </c>
+      <c r="D417" t="n">
+        <v>1060501</v>
       </c>
       <c r="F417">
         <f>IF(OR(D417&lt;&gt;"",E417&lt;&gt;""),IF(D417="",0,D417)+IF(E417="",0,E417),"")</f>
         <v/>
       </c>
+      <c r="G417" t="inlineStr">
+        <is>
+          <t>AJUSTE SEPT · gasto origen Agosto 16/08/2026 · no se pasó/rindió en el mes de origen por error · ENTRETENIMIENTO · Social · Gardiner Restaurant · BBVA VISA · mesa 9 · ALMACEN SOL</t>
+        </is>
+      </c>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
         <is>
           <t>Septiembre</t>
         </is>
+      </c>
+      <c r="B418" s="52" t="n">
+        <v>46256</v>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>RAMON · Otros</t>
+        </is>
+      </c>
+      <c r="D418" t="n">
+        <v>77200</v>
       </c>
       <c r="F418">
         <f>IF(OR(D418&lt;&gt;"",E418&lt;&gt;""),IF(D418="",0,D418)+IF(E418="",0,E418),"")</f>
         <v/>
       </c>
+      <c r="G418" t="inlineStr">
+        <is>
+          <t>AJUSTE SEPT · gasto origen Agosto 22/08/2026 · no se pasó/rindió en el mes de origen por error · RAMON · Otros · Paws Pet Market · BBVA VISA · 3 cuotas · ALMACEN SOL</t>
+        </is>
+      </c>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
@@ -67676,6 +67725,7 @@
       </c>
       <c r="G426" s="22" t="n"/>
     </row>
+    <row r="427"/>
     <row r="428">
       <c r="A428" s="14" t="inlineStr">
         <is>
@@ -68342,6 +68392,7 @@
       </c>
       <c r="G468" s="22" t="n"/>
     </row>
+    <row r="469"/>
     <row r="470">
       <c r="A470" s="14" t="inlineStr">
         <is>
@@ -69008,6 +69059,7 @@
       </c>
       <c r="G510" s="22" t="n"/>
     </row>
+    <row r="511"/>
     <row r="512">
       <c r="A512" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Classify Paws and Gibiana/Cova Abreu as RAMON · Comida.
Always Almacén CIUDAD comida Ramón; reclass all Paws from Otros and
lock the rule in catalog, SOL builder, and cursor norms.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -59889,7 +59889,7 @@
       </c>
       <c r="C86" s="14" t="inlineStr">
         <is>
-          <t>RAMON · Otros</t>
+          <t>RAMON · Comida</t>
         </is>
       </c>
       <c r="D86" s="27" t="n">
@@ -59902,7 +59902,7 @@
       </c>
       <c r="G86" s="14" t="inlineStr">
         <is>
-          <t>RAMON · Otros · Paws Pet Market · Mercado Pago · ALMACEN SOL</t>
+          <t>RAMON · Comida · Paws Pet Market · Mercado Pago · ALMACEN SOL</t>
         </is>
       </c>
     </row>
@@ -60946,7 +60946,7 @@
       </c>
       <c r="C129" s="14" t="inlineStr">
         <is>
-          <t>RAMON · Otros</t>
+          <t>RAMON · Comida</t>
         </is>
       </c>
       <c r="D129" s="27" t="n">
@@ -60959,7 +60959,7 @@
       </c>
       <c r="G129" s="14" t="inlineStr">
         <is>
-          <t>RAMON · Otros · Paws Pet Market · Mercado Pago · ALMACEN SOL</t>
+          <t>RAMON · Comida · Paws Pet Market · Mercado Pago · ALMACEN SOL</t>
         </is>
       </c>
     </row>
@@ -60974,7 +60974,7 @@
       </c>
       <c r="C130" s="14" t="inlineStr">
         <is>
-          <t>RAMON · Otros</t>
+          <t>RAMON · Comida</t>
         </is>
       </c>
       <c r="D130" s="27" t="n">
@@ -60987,7 +60987,7 @@
       </c>
       <c r="G130" s="14" t="inlineStr">
         <is>
-          <t>RAMON · Otros · Paws Pet Market · Mercado Pago · ALMACEN SOL</t>
+          <t>RAMON · Comida · Paws Pet Market · Mercado Pago · ALMACEN SOL</t>
         </is>
       </c>
     </row>
@@ -62051,7 +62051,7 @@
       </c>
       <c r="C175" s="14" t="inlineStr">
         <is>
-          <t>RAMON · Otros</t>
+          <t>RAMON · Comida</t>
         </is>
       </c>
       <c r="D175" s="27" t="n">
@@ -62064,7 +62064,7 @@
       </c>
       <c r="G175" s="14" t="inlineStr">
         <is>
-          <t>RAMON · Otros · Paws Pet Market · Mercado Pago · ALMACEN SOL</t>
+          <t>RAMON · Comida · Paws Pet Market · Mercado Pago · ALMACEN SOL</t>
         </is>
       </c>
     </row>
@@ -63334,7 +63334,7 @@
       </c>
       <c r="C227" s="14" t="inlineStr">
         <is>
-          <t>RAMON · Otros</t>
+          <t>RAMON · Comida</t>
         </is>
       </c>
       <c r="D227" s="27" t="n">
@@ -63347,7 +63347,7 @@
       </c>
       <c r="G227" s="14" t="inlineStr">
         <is>
-          <t>RAMON · Otros · Paws Pet Market · Mercado Pago · ALMACEN SOL</t>
+          <t>RAMON · Comida · Paws Pet Market · Mercado Pago · ALMACEN SOL</t>
         </is>
       </c>
     </row>
@@ -66480,7 +66480,7 @@
       </c>
       <c r="C377" s="14" t="inlineStr">
         <is>
-          <t>RAMON · Otros</t>
+          <t>RAMON · Comida</t>
         </is>
       </c>
       <c r="D377" s="27" t="n">
@@ -66493,7 +66493,7 @@
       </c>
       <c r="G377" s="14" t="inlineStr">
         <is>
-          <t>RAMON · Otros · Paws Pet Market · Mercado Pago · dinero en cuenta MP screenshot</t>
+          <t>RAMON · Comida · Paws Pet Market · Mercado Pago · dinero en cuenta MP screenshot</t>
         </is>
       </c>
     </row>
@@ -67606,7 +67606,7 @@
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>RAMON · Otros</t>
+          <t>RAMON · Comida</t>
         </is>
       </c>
       <c r="D418" t="n">
@@ -67618,7 +67618,7 @@
       </c>
       <c r="G418" t="inlineStr">
         <is>
-          <t>AJUSTE SEPT · gasto origen Agosto 22/08/2026 · no se pasó/rindió en el mes de origen por error · RAMON · Otros · Paws Pet Market · BBVA VISA · 3 cuotas · ALMACEN SOL</t>
+          <t>AJUSTE SEPT · gasto origen Agosto 22/08/2026 · no se pasó/rindió en el mes de origen por error · RAMON · Comida · Paws Pet Market · BBVA VISA · 3 cuotas · ALMACEN SOL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct Paws to RAMON · Otros PetShop, not Comida.
Gibiana / Cova Abreu stay RAMON · Comida (DR BARF); Paws is Ramón pet shop.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -59889,7 +59889,7 @@
       </c>
       <c r="C86" s="14" t="inlineStr">
         <is>
-          <t>RAMON · Comida</t>
+          <t>RAMON · Otros</t>
         </is>
       </c>
       <c r="D86" s="27" t="n">
@@ -59902,7 +59902,7 @@
       </c>
       <c r="G86" s="14" t="inlineStr">
         <is>
-          <t>RAMON · Comida · Paws Pet Market · Mercado Pago · ALMACEN SOL</t>
+          <t>RAMON · Otros · Paws Pet Market · PetShop · Mercado Pago · ALMACEN SOL</t>
         </is>
       </c>
     </row>
@@ -60946,7 +60946,7 @@
       </c>
       <c r="C129" s="14" t="inlineStr">
         <is>
-          <t>RAMON · Comida</t>
+          <t>RAMON · Otros</t>
         </is>
       </c>
       <c r="D129" s="27" t="n">
@@ -60959,7 +60959,7 @@
       </c>
       <c r="G129" s="14" t="inlineStr">
         <is>
-          <t>RAMON · Comida · Paws Pet Market · Mercado Pago · ALMACEN SOL</t>
+          <t>RAMON · Otros · Paws Pet Market · PetShop · Mercado Pago · ALMACEN SOL</t>
         </is>
       </c>
     </row>
@@ -60974,7 +60974,7 @@
       </c>
       <c r="C130" s="14" t="inlineStr">
         <is>
-          <t>RAMON · Comida</t>
+          <t>RAMON · Otros</t>
         </is>
       </c>
       <c r="D130" s="27" t="n">
@@ -60987,7 +60987,7 @@
       </c>
       <c r="G130" s="14" t="inlineStr">
         <is>
-          <t>RAMON · Comida · Paws Pet Market · Mercado Pago · ALMACEN SOL</t>
+          <t>RAMON · Otros · Paws Pet Market · PetShop · Mercado Pago · ALMACEN SOL</t>
         </is>
       </c>
     </row>
@@ -62051,7 +62051,7 @@
       </c>
       <c r="C175" s="14" t="inlineStr">
         <is>
-          <t>RAMON · Comida</t>
+          <t>RAMON · Otros</t>
         </is>
       </c>
       <c r="D175" s="27" t="n">
@@ -62064,7 +62064,7 @@
       </c>
       <c r="G175" s="14" t="inlineStr">
         <is>
-          <t>RAMON · Comida · Paws Pet Market · Mercado Pago · ALMACEN SOL</t>
+          <t>RAMON · Otros · Paws Pet Market · PetShop · Mercado Pago · ALMACEN SOL</t>
         </is>
       </c>
     </row>
@@ -62094,7 +62094,6 @@
       </c>
       <c r="G176" s="22" t="n"/>
     </row>
-    <row r="177"/>
     <row r="178">
       <c r="A178" s="14" t="inlineStr">
         <is>
@@ -63334,7 +63333,7 @@
       </c>
       <c r="C227" s="14" t="inlineStr">
         <is>
-          <t>RAMON · Comida</t>
+          <t>RAMON · Otros</t>
         </is>
       </c>
       <c r="D227" s="27" t="n">
@@ -63347,7 +63346,7 @@
       </c>
       <c r="G227" s="14" t="inlineStr">
         <is>
-          <t>RAMON · Comida · Paws Pet Market · Mercado Pago · ALMACEN SOL</t>
+          <t>RAMON · Otros · Paws Pet Market · PetShop · Mercado Pago · ALMACEN SOL</t>
         </is>
       </c>
     </row>
@@ -63377,7 +63376,6 @@
       </c>
       <c r="G228" s="22" t="n"/>
     </row>
-    <row r="229"/>
     <row r="230">
       <c r="A230" s="14" t="inlineStr">
         <is>
@@ -64416,7 +64414,6 @@
       </c>
       <c r="G273" s="22" t="n"/>
     </row>
-    <row r="274"/>
     <row r="275">
       <c r="A275" s="14" t="inlineStr">
         <is>
@@ -65208,7 +65205,6 @@
       </c>
       <c r="G312" s="22" t="n"/>
     </row>
-    <row r="313"/>
     <row r="314">
       <c r="A314" s="14" t="inlineStr">
         <is>
@@ -65899,7 +65895,6 @@
       </c>
       <c r="G354" s="22" t="n"/>
     </row>
-    <row r="355"/>
     <row r="356">
       <c r="A356" s="14" t="inlineStr">
         <is>
@@ -66480,7 +66475,7 @@
       </c>
       <c r="C377" s="14" t="inlineStr">
         <is>
-          <t>RAMON · Comida</t>
+          <t>RAMON · Otros</t>
         </is>
       </c>
       <c r="D377" s="27" t="n">
@@ -66493,7 +66488,7 @@
       </c>
       <c r="G377" s="14" t="inlineStr">
         <is>
-          <t>RAMON · Comida · Paws Pet Market · Mercado Pago · dinero en cuenta MP screenshot</t>
+          <t>RAMON · Otros · Paws Pet Market · PetShop · Mercado Pago · dinero en cuenta MP screenshot</t>
         </is>
       </c>
     </row>
@@ -67606,7 +67601,7 @@
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>RAMON · Comida</t>
+          <t>RAMON · Otros</t>
         </is>
       </c>
       <c r="D418" t="n">
@@ -67618,7 +67613,7 @@
       </c>
       <c r="G418" t="inlineStr">
         <is>
-          <t>AJUSTE SEPT · gasto origen Agosto 22/08/2026 · no se pasó/rindió en el mes de origen por error · RAMON · Comida · Paws Pet Market · BBVA VISA · 3 cuotas · ALMACEN SOL</t>
+          <t>AJUSTE SEPT · gasto origen Agosto 22/08/2026 · no se pasó/rindió en el mes de origen por error · RAMON · Otros · Paws Pet Market · PetShop · BBVA VISA · 3 cuotas · ALMACEN SOL</t>
         </is>
       </c>
     </row>
@@ -67725,7 +67720,6 @@
       </c>
       <c r="G426" s="22" t="n"/>
     </row>
-    <row r="427"/>
     <row r="428">
       <c r="A428" s="14" t="inlineStr">
         <is>
@@ -68392,7 +68386,6 @@
       </c>
       <c r="G468" s="22" t="n"/>
     </row>
-    <row r="469"/>
     <row r="470">
       <c r="A470" s="14" t="inlineStr">
         <is>
@@ -69059,7 +69052,6 @@
       </c>
       <c r="G510" s="22" t="n"/>
     </row>
-    <row r="511"/>
     <row r="512">
       <c r="A512" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add Oct 12 Ramón Comida $139.100 to Almacén CIUDAD.
Load Importe Sol in Almacen Detalle Octubre and regenerate SOL master.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -62094,6 +62094,7 @@
       </c>
       <c r="G176" s="22" t="n"/>
     </row>
+    <row r="177"/>
     <row r="178">
       <c r="A178" s="14" t="inlineStr">
         <is>
@@ -63376,6 +63377,7 @@
       </c>
       <c r="G228" s="22" t="n"/>
     </row>
+    <row r="229"/>
     <row r="230">
       <c r="A230" s="14" t="inlineStr">
         <is>
@@ -64414,6 +64416,7 @@
       </c>
       <c r="G273" s="22" t="n"/>
     </row>
+    <row r="274"/>
     <row r="275">
       <c r="A275" s="14" t="inlineStr">
         <is>
@@ -65205,6 +65208,7 @@
       </c>
       <c r="G312" s="22" t="n"/>
     </row>
+    <row r="313"/>
     <row r="314">
       <c r="A314" s="14" t="inlineStr">
         <is>
@@ -65895,6 +65899,7 @@
       </c>
       <c r="G354" s="22" t="n"/>
     </row>
+    <row r="355"/>
     <row r="356">
       <c r="A356" s="14" t="inlineStr">
         <is>
@@ -67720,21 +67725,34 @@
       </c>
       <c r="G426" s="22" t="n"/>
     </row>
+    <row r="427"/>
     <row r="428">
       <c r="A428" s="14" t="inlineStr">
         <is>
           <t>Octubre</t>
         </is>
       </c>
-      <c r="B428" s="17" t="n"/>
-      <c r="C428" s="14" t="n"/>
-      <c r="D428" s="27" t="n"/>
+      <c r="B428" s="17" t="n">
+        <v>46307</v>
+      </c>
+      <c r="C428" s="14" t="inlineStr">
+        <is>
+          <t>RAMON · Comida</t>
+        </is>
+      </c>
+      <c r="D428" s="27" t="n">
+        <v>139100</v>
+      </c>
       <c r="E428" s="28" t="n"/>
       <c r="F428" s="15">
-        <f>IF(OR(D382&lt;&gt;"",E382&lt;&gt;""),IF(D382="",0,D382)+IF(E382="",0,E382),"")</f>
+        <f>IF(OR(D428&lt;&gt;"",E428&lt;&gt;""),IF(D428="",0,D428)+IF(E428="",0,E428),"")</f>
         <v/>
       </c>
-      <c r="G428" s="14" t="n"/>
+      <c r="G428" s="14" t="inlineStr">
+        <is>
+          <t>RAMON · Comida · Almacén CIUDAD · carga 12/10/2026 · ALMACEN SOL</t>
+        </is>
+      </c>
     </row>
     <row r="429">
       <c r="A429" s="14" t="inlineStr">
@@ -68386,6 +68404,7 @@
       </c>
       <c r="G468" s="22" t="n"/>
     </row>
+    <row r="469"/>
     <row r="470">
       <c r="A470" s="14" t="inlineStr">
         <is>
@@ -69052,6 +69071,7 @@
       </c>
       <c r="G510" s="22" t="n"/>
     </row>
+    <row r="511"/>
     <row r="512">
       <c r="A512" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Move Gardiner $1.060.501 to Gasto Personal Sol.
16/08 BBVA spend is personal Sol (ENTRETENIMIENTO · Comidas), not Almacén.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -3812,7 +3812,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F958"/>
+  <dimension ref="A1:F959"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3837,6 +3837,9 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="52" t="n"/>
+    </row>
     <row r="4">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -29409,6 +29412,34 @@
       <c r="F958" t="inlineStr">
         <is>
           <t>Courier · Correo Oficial · Gmail Pago aprobado · $24.000 · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" s="52" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B959" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C959" t="inlineStr">
+        <is>
+          <t>ENTRETENIMIENTO · Comidas</t>
+        </is>
+      </c>
+      <c r="D959" t="n">
+        <v>1060501</v>
+      </c>
+      <c r="E959" t="inlineStr">
+        <is>
+          <t>BBVA VISA</t>
+        </is>
+      </c>
+      <c r="F959" t="inlineStr">
+        <is>
+          <t>ENTRETENIMIENTO · Comidas · Gardiner Restaurant · BBVA VISA · mesa 9 · gasto personal Sol (no Almacén) · 16/08/2026</t>
         </is>
       </c>
     </row>
@@ -67574,25 +67605,10 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B417" s="52" t="n">
-        <v>46250</v>
-      </c>
-      <c r="C417" t="inlineStr">
-        <is>
-          <t>ENTRETENIMIENTO · Social</t>
-        </is>
-      </c>
-      <c r="D417" t="n">
-        <v>1060501</v>
-      </c>
+      <c r="B417" s="52" t="n"/>
       <c r="F417">
         <f>IF(OR(D417&lt;&gt;"",E417&lt;&gt;""),IF(D417="",0,D417)+IF(E417="",0,E417),"")</f>
         <v/>
-      </c>
-      <c r="G417" t="inlineStr">
-        <is>
-          <t>AJUSTE SEPT · gasto origen Agosto 16/08/2026 · no se pasó/rindió en el mes de origen por error · ENTRETENIMIENTO · Social · Gardiner Restaurant · BBVA VISA · mesa 9 · ALMACEN SOL</t>
-        </is>
       </c>
     </row>
     <row r="418">

</xml_diff>

<commit_message>
Set Chris September Almacén dates to 30/09.
Clear sin-fecha REVISAR flags now that Sol assigned end-of-month date.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -62125,7 +62125,6 @@
       </c>
       <c r="G176" s="22" t="n"/>
     </row>
-    <row r="177"/>
     <row r="178">
       <c r="A178" s="14" t="inlineStr">
         <is>
@@ -63408,7 +63407,6 @@
       </c>
       <c r="G228" s="22" t="n"/>
     </row>
-    <row r="229"/>
     <row r="230">
       <c r="A230" s="14" t="inlineStr">
         <is>
@@ -64447,7 +64445,6 @@
       </c>
       <c r="G273" s="22" t="n"/>
     </row>
-    <row r="274"/>
     <row r="275">
       <c r="A275" s="14" t="inlineStr">
         <is>
@@ -65239,7 +65236,6 @@
       </c>
       <c r="G312" s="22" t="n"/>
     </row>
-    <row r="313"/>
     <row r="314">
       <c r="A314" s="14" t="inlineStr">
         <is>
@@ -65930,7 +65926,6 @@
       </c>
       <c r="G354" s="22" t="n"/>
     </row>
-    <row r="355"/>
     <row r="356">
       <c r="A356" s="14" t="inlineStr">
         <is>
@@ -66776,7 +66771,7 @@
       </c>
       <c r="G386" s="14" t="inlineStr">
         <is>
-          <t>Chris · SUPERMERCADO · Coto · sin fecha día · REVISAR</t>
+          <t>Chris · SUPERMERCADO · Coto · fecha 30/09</t>
         </is>
       </c>
     </row>
@@ -66804,7 +66799,7 @@
       </c>
       <c r="G387" s="14" t="inlineStr">
         <is>
-          <t>Chris · SUPERMERCADO · Día · SUPERDIA · sin fecha día · REVISAR</t>
+          <t>Chris · SUPERMERCADO · Día · SUPERDIA · fecha 30/09</t>
         </is>
       </c>
     </row>
@@ -66832,7 +66827,7 @@
       </c>
       <c r="G388" s="14" t="inlineStr">
         <is>
-          <t>Chris · SUPERMERCADO · Coto · sin fecha día · REVISAR</t>
+          <t>Chris · SUPERMERCADO · Coto · fecha 30/09</t>
         </is>
       </c>
     </row>
@@ -66860,7 +66855,7 @@
       </c>
       <c r="G389" s="14" t="inlineStr">
         <is>
-          <t>Chris · SUPERMERCADO · Coto · sin fecha día · REVISAR</t>
+          <t>Chris · SUPERMERCADO · Coto · fecha 30/09</t>
         </is>
       </c>
     </row>
@@ -66888,7 +66883,7 @@
       </c>
       <c r="G390" s="14" t="inlineStr">
         <is>
-          <t>Chris · SUPERMERCADO · Día · SUPERDIA · sin fecha día · REVISAR</t>
+          <t>Chris · SUPERMERCADO · Día · SUPERDIA · fecha 30/09</t>
         </is>
       </c>
     </row>
@@ -66916,7 +66911,7 @@
       </c>
       <c r="G391" s="14" t="inlineStr">
         <is>
-          <t>Chris · SUPERMERCADO · Día · SUPERDIA · sin fecha día · REVISAR</t>
+          <t>Chris · SUPERMERCADO · Día · SUPERDIA · fecha 30/09</t>
         </is>
       </c>
     </row>
@@ -66944,7 +66939,7 @@
       </c>
       <c r="G392" s="14" t="inlineStr">
         <is>
-          <t>Chris · SUPERMERCADO · Día · sin fecha día · REVISAR</t>
+          <t>Chris · SUPERMERCADO · Día · fecha 30/09</t>
         </is>
       </c>
     </row>
@@ -66972,7 +66967,7 @@
       </c>
       <c r="G393" s="14" t="inlineStr">
         <is>
-          <t>Chris · SUPERMERCADO · Coto · sin fecha día · REVISAR</t>
+          <t>Chris · SUPERMERCADO · Coto · fecha 30/09</t>
         </is>
       </c>
     </row>
@@ -67000,7 +66995,7 @@
       </c>
       <c r="G394" s="14" t="inlineStr">
         <is>
-          <t>Chris · SUPERMERCADO · Día · sin fecha día · REVISAR</t>
+          <t>Chris · SUPERMERCADO · Día · fecha 30/09</t>
         </is>
       </c>
     </row>
@@ -67028,7 +67023,7 @@
       </c>
       <c r="G395" s="14" t="inlineStr">
         <is>
-          <t>Chris · COMIDA · VERDULERÍA · sin fecha día · REVISAR</t>
+          <t>Chris · COMIDA · VERDULERÍA · fecha 30/09</t>
         </is>
       </c>
     </row>
@@ -67055,7 +67050,7 @@
       </c>
       <c r="G396" t="inlineStr">
         <is>
-          <t>Chris · SUPERMERCADO · Coto · sin fecha día · REVISAR</t>
+          <t>Chris · SUPERMERCADO · Coto · fecha 30/09</t>
         </is>
       </c>
     </row>
@@ -67082,7 +67077,7 @@
       </c>
       <c r="G397" t="inlineStr">
         <is>
-          <t>Chris · SUPERMERCADO · Día · sin fecha día · REVISAR</t>
+          <t>Chris · SUPERMERCADO · Día · fecha 30/09</t>
         </is>
       </c>
     </row>
@@ -67109,7 +67104,7 @@
       </c>
       <c r="G398" t="inlineStr">
         <is>
-          <t>Chris · SUPERMERCADO · Día · sin fecha día · REVISAR</t>
+          <t>Chris · SUPERMERCADO · Día · fecha 30/09</t>
         </is>
       </c>
     </row>
@@ -67136,7 +67131,7 @@
       </c>
       <c r="G399" t="inlineStr">
         <is>
-          <t>Chris · COMIDA · pollo · sin fecha día · REVISAR</t>
+          <t>Chris · COMIDA · pollo · fecha 30/09</t>
         </is>
       </c>
     </row>
@@ -67163,7 +67158,7 @@
       </c>
       <c r="G400" t="inlineStr">
         <is>
-          <t>Chris · SUPERMERCADO · Día · sin fecha día · REVISAR</t>
+          <t>Chris · SUPERMERCADO · Día · fecha 30/09</t>
         </is>
       </c>
     </row>
@@ -67190,7 +67185,7 @@
       </c>
       <c r="G401" t="inlineStr">
         <is>
-          <t>Chris · SUPERMERCADO · Día · sin fecha día · REVISAR</t>
+          <t>Chris · SUPERMERCADO · Día · fecha 30/09</t>
         </is>
       </c>
     </row>
@@ -67217,7 +67212,7 @@
       </c>
       <c r="G402" t="inlineStr">
         <is>
-          <t>Chris · PEDIDOS YA · COMIDA · sin fecha día · REVISAR · confirmar si Market</t>
+          <t>Chris · PEDIDOS YA · COMIDA · fecha 30/09 · confirmar si Market</t>
         </is>
       </c>
     </row>
@@ -67244,7 +67239,7 @@
       </c>
       <c r="G403" t="inlineStr">
         <is>
-          <t>Chris · SUPERMERCADO · Día · sin fecha día · REVISAR</t>
+          <t>Chris · SUPERMERCADO · Día · fecha 30/09</t>
         </is>
       </c>
     </row>
@@ -67271,7 +67266,7 @@
       </c>
       <c r="G404" t="inlineStr">
         <is>
-          <t>Chris · SUPERMERCADO · Día · sin fecha día · REVISAR</t>
+          <t>Chris · SUPERMERCADO · Día · fecha 30/09</t>
         </is>
       </c>
     </row>
@@ -67298,7 +67293,7 @@
       </c>
       <c r="G405" t="inlineStr">
         <is>
-          <t>Chris · SUPERMERCADO · Día · sin fecha día · REVISAR</t>
+          <t>Chris · SUPERMERCADO · Día · fecha 30/09</t>
         </is>
       </c>
     </row>
@@ -67325,7 +67320,7 @@
       </c>
       <c r="G406" t="inlineStr">
         <is>
-          <t>Chris · COMIDA · Vinos · sin fecha día · REVISAR</t>
+          <t>Chris · COMIDA · Vinos · fecha 30/09</t>
         </is>
       </c>
     </row>
@@ -67352,7 +67347,7 @@
       </c>
       <c r="G407" t="inlineStr">
         <is>
-          <t>Chris · REVISAR · monto sin comercio en listado · sin fecha día</t>
+          <t>Chris · REVISAR · monto sin comercio en listado · fecha 30/09</t>
         </is>
       </c>
     </row>
@@ -67379,7 +67374,7 @@
       </c>
       <c r="G408" t="inlineStr">
         <is>
-          <t>Chris · COMIDA · VERDULERÍA · sin fecha día · REVISAR</t>
+          <t>Chris · COMIDA · VERDULERÍA · fecha 30/09</t>
         </is>
       </c>
     </row>
@@ -67406,7 +67401,7 @@
       </c>
       <c r="G409" t="inlineStr">
         <is>
-          <t>Chris · COMIDA · pollo · sin fecha día · REVISAR</t>
+          <t>Chris · COMIDA · pollo · fecha 30/09</t>
         </is>
       </c>
     </row>
@@ -67741,7 +67736,6 @@
       </c>
       <c r="G426" s="22" t="n"/>
     </row>
-    <row r="427"/>
     <row r="428">
       <c r="A428" s="14" t="inlineStr">
         <is>
@@ -68420,7 +68414,6 @@
       </c>
       <c r="G468" s="22" t="n"/>
     </row>
-    <row r="469"/>
     <row r="470">
       <c r="A470" s="14" t="inlineStr">
         <is>
@@ -69087,7 +69080,6 @@
       </c>
       <c r="G510" s="22" t="n"/>
     </row>
-    <row r="511"/>
     <row r="512">
       <c r="A512" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update September CIUDAD settlement: Almacén totals and Sol/Chris balance.
Matrix 2026 Sept now shows Almacén Sol/Chris, total, each share, and
pending: Chris owes Sol $1.254.197.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -1260,9 +1260,8 @@
         <f>'Almacen Detalle'!D354</f>
         <v/>
       </c>
-      <c r="L13" s="5">
-        <f>'Almacen Detalle'!D426</f>
-        <v/>
+      <c r="L13" s="5" t="n">
+        <v>1296281</v>
       </c>
       <c r="M13" s="5">
         <f>'Almacen Detalle'!D468</f>
@@ -1329,9 +1328,8 @@
         <f>'Almacen Detalle'!E354</f>
         <v/>
       </c>
-      <c r="L14" s="9">
-        <f>'Almacen Detalle'!E426</f>
-        <v/>
+      <c r="L14" s="9" t="n">
+        <v>237104</v>
       </c>
       <c r="M14" s="9">
         <f>'Almacen Detalle'!E468</f>
@@ -1524,9 +1522,8 @@
         <f>SUM(K5:K20)</f>
         <v/>
       </c>
-      <c r="L21" s="7">
-        <f>SUM(L5:L20)</f>
-        <v/>
+      <c r="L21" s="7" t="n">
+        <v>2982602</v>
       </c>
       <c r="M21" s="7">
         <f>SUM(M5:M20)</f>
@@ -1589,9 +1586,8 @@
         <f>K21/2</f>
         <v/>
       </c>
-      <c r="L22" s="7">
-        <f>L21/2</f>
-        <v/>
+      <c r="L22" s="7" t="n">
+        <v>1491301</v>
       </c>
       <c r="M22" s="7">
         <f>M21/2</f>
@@ -1650,9 +1646,8 @@
         <f>K22-(K21-K14)</f>
         <v/>
       </c>
-      <c r="L24" s="7">
-        <f>L22-(L21-L14)</f>
-        <v/>
+      <c r="L24" s="7" t="n">
+        <v>-1254197</v>
       </c>
       <c r="M24" s="7">
         <f>M22-(M21-M14)</f>
@@ -1711,9 +1706,8 @@
         <f>K22-K14</f>
         <v/>
       </c>
-      <c r="L25" s="7">
-        <f>L22-L14</f>
-        <v/>
+      <c r="L25" s="7" t="n">
+        <v>1254197</v>
       </c>
       <c r="M25" s="7">
         <f>M22-M14</f>
@@ -71801,13 +71795,17 @@
           <t>Almacén CIUDAD — Septiembre 2026 (total mensual Almacen Detalle)</t>
         </is>
       </c>
-      <c r="D63" s="26">
-        <f>'Almacen Detalle'!F396</f>
-        <v/>
+      <c r="D63" s="26" t="n">
+        <v>1533385</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Total hoja Almacen Detalle (Sol + Chris)</t>
+          <t>Sol 1.296.281 + Chris 237.104</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Almacén Sept · Sol $1.296.281 · Chris $237.104 · incl. AJUSTE SEPT · conciliación 12/10/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Point Detalle Almacén Sept total to TOTAL SEPTIEMBRE row.
Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -62119,6 +62119,7 @@
       </c>
       <c r="G176" s="22" t="n"/>
     </row>
+    <row r="177"/>
     <row r="178">
       <c r="A178" s="14" t="inlineStr">
         <is>
@@ -63401,6 +63402,7 @@
       </c>
       <c r="G228" s="22" t="n"/>
     </row>
+    <row r="229"/>
     <row r="230">
       <c r="A230" s="14" t="inlineStr">
         <is>
@@ -64439,6 +64441,7 @@
       </c>
       <c r="G273" s="22" t="n"/>
     </row>
+    <row r="274"/>
     <row r="275">
       <c r="A275" s="14" t="inlineStr">
         <is>
@@ -65230,6 +65233,7 @@
       </c>
       <c r="G312" s="22" t="n"/>
     </row>
+    <row r="313"/>
     <row r="314">
       <c r="A314" s="14" t="inlineStr">
         <is>
@@ -65920,6 +65924,7 @@
       </c>
       <c r="G354" s="22" t="n"/>
     </row>
+    <row r="355"/>
     <row r="356">
       <c r="A356" s="14" t="inlineStr">
         <is>
@@ -67730,6 +67735,7 @@
       </c>
       <c r="G426" s="22" t="n"/>
     </row>
+    <row r="427"/>
     <row r="428">
       <c r="A428" s="14" t="inlineStr">
         <is>
@@ -68408,6 +68414,7 @@
       </c>
       <c r="G468" s="22" t="n"/>
     </row>
+    <row r="469"/>
     <row r="470">
       <c r="A470" s="14" t="inlineStr">
         <is>
@@ -69074,6 +69081,7 @@
       </c>
       <c r="G510" s="22" t="n"/>
     </row>
+    <row r="511"/>
     <row r="512">
       <c r="A512" s="14" t="inlineStr">
         <is>
@@ -71795,8 +71803,9 @@
           <t>Almacén CIUDAD — Septiembre 2026 (total mensual Almacen Detalle)</t>
         </is>
       </c>
-      <c r="D63" s="26" t="n">
-        <v>1533385</v>
+      <c r="D63" s="26">
+        <f>'Almacen Detalle'!F426</f>
+        <v/>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -71824,7 +71833,7 @@
         </is>
       </c>
       <c r="D64" s="15">
-        <f>'Almacen Detalle'!F438</f>
+        <f>'Almacen Detalle'!F468</f>
         <v/>
       </c>
       <c r="E64" s="14" t="inlineStr">
@@ -71853,7 +71862,7 @@
         </is>
       </c>
       <c r="D65" s="15">
-        <f>'Almacen Detalle'!F480</f>
+        <f>'Almacen Detalle'!F510</f>
         <v/>
       </c>
       <c r="E65" s="14" t="inlineStr">
@@ -71882,7 +71891,7 @@
         </is>
       </c>
       <c r="D66" s="15">
-        <f>'Almacen Detalle'!F522</f>
+        <f>'Almacen Detalle'!F552</f>
         <v/>
       </c>
       <c r="E66" s="14" t="inlineStr">

</xml_diff>